<commit_message>
Bilan 2025 : suppression de la colonne Preuve de paiement
La colonne « Facture » est conservee mais laissee vide (a cocher a la main),
la colonne « Remarque » passe en K.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D4:L43"/>
+  <dimension ref="D1:K43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -755,10 +755,11 @@
     <col width="47.28515625" customWidth="1" min="8" max="8"/>
     <col width="8.42578125" bestFit="1" customWidth="1" min="9" max="9"/>
     <col width="7.7109375" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="19.140625" bestFit="1" customWidth="1" min="11" max="11"/>
-    <col width="26.42578125" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="26.42578125" bestFit="1" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="15.75" customHeight="1" thickBot="1"/>
     <row r="4">
       <c r="D4" s="1" t="inlineStr">
@@ -813,11 +814,6 @@
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>Preuve de paiement</t>
-        </is>
-      </c>
-      <c r="L5" s="10" t="inlineStr">
-        <is>
           <t>Remarque</t>
         </is>
       </c>
@@ -844,17 +840,8 @@
       <c r="I6" s="32" t="n">
         <v>26</v>
       </c>
-      <c r="J6" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J6" s="28" t="n"/>
       <c r="K6" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L6" s="28" t="inlineStr">
         <is>
           <t>Paiement du 31-12-2024 comptabilisé le 01-01-2025 — Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
         </is>
@@ -878,17 +865,8 @@
       <c r="I7" s="32" t="n">
         <v>2250</v>
       </c>
-      <c r="J7" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J7" s="28" t="n"/>
       <c r="K7" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L7" s="28" t="inlineStr">
         <is>
           <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
         </is>
@@ -912,17 +890,8 @@
       <c r="I8" s="32" t="n">
         <v>330.88</v>
       </c>
-      <c r="J8" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J8" s="28" t="n"/>
       <c r="K8" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L8" s="28" t="inlineStr">
         <is>
           <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
         </is>
@@ -940,17 +909,8 @@
       <c r="I9" s="32" t="n">
         <v>8.4</v>
       </c>
-      <c r="J9" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K9" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L9" s="28" t="n"/>
+      <c r="J9" s="28" t="n"/>
+      <c r="K9" s="28" t="n"/>
     </row>
     <row r="10">
       <c r="E10" s="16" t="n"/>
@@ -964,17 +924,8 @@
       <c r="I10" s="32" t="n">
         <v>256.99</v>
       </c>
-      <c r="J10" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J10" s="28" t="n"/>
       <c r="K10" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L10" s="28" t="inlineStr">
         <is>
           <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
         </is>
@@ -992,17 +943,8 @@
       <c r="I11" s="32" t="n">
         <v>149.1</v>
       </c>
-      <c r="J11" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J11" s="28" t="n"/>
       <c r="K11" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L11" s="28" t="inlineStr">
         <is>
           <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
         </is>
@@ -1020,17 +962,8 @@
       <c r="I12" s="32" t="n">
         <v>82.98999999999999</v>
       </c>
-      <c r="J12" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J12" s="28" t="n"/>
       <c r="K12" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L12" s="28" t="inlineStr">
         <is>
           <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage (82,98 encodé en 2024)</t>
         </is>
@@ -1048,17 +981,8 @@
       <c r="I13" s="32" t="n">
         <v>22.9</v>
       </c>
-      <c r="J13" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J13" s="28" t="n"/>
       <c r="K13" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L13" s="28" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
         </is>
@@ -1076,17 +1000,8 @@
       <c r="I14" s="32" t="n">
         <v>5.69</v>
       </c>
-      <c r="J14" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="K14" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L14" s="28" t="n"/>
+      <c r="J14" s="28" t="n"/>
+      <c r="K14" s="28" t="n"/>
     </row>
     <row r="15">
       <c r="E15" s="16" t="n"/>
@@ -1100,17 +1015,8 @@
       <c r="I15" s="32" t="n">
         <v>1.35</v>
       </c>
-      <c r="J15" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K15" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L15" s="28" t="n"/>
+      <c r="J15" s="28" t="n"/>
+      <c r="K15" s="28" t="n"/>
     </row>
     <row r="16">
       <c r="E16" s="16" t="n"/>
@@ -1124,17 +1030,8 @@
       <c r="I16" s="32" t="n">
         <v>62.79</v>
       </c>
-      <c r="J16" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J16" s="28" t="n"/>
       <c r="K16" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L16" s="28" t="inlineStr">
         <is>
           <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
         </is>
@@ -1152,17 +1049,8 @@
       <c r="I17" s="32" t="n">
         <v>724.12</v>
       </c>
-      <c r="J17" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K17" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L17" s="28" t="n"/>
+      <c r="J17" s="28" t="n"/>
+      <c r="K17" s="28" t="n"/>
     </row>
     <row r="18">
       <c r="E18" s="16" t="n"/>
@@ -1176,17 +1064,8 @@
       <c r="I18" s="32" t="n">
         <v>11.25</v>
       </c>
-      <c r="J18" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K18" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L18" s="28" t="n"/>
+      <c r="J18" s="28" t="n"/>
+      <c r="K18" s="28" t="n"/>
     </row>
     <row r="19">
       <c r="E19" s="16" t="n"/>
@@ -1200,17 +1079,8 @@
       <c r="I19" s="32" t="n">
         <v>431.25</v>
       </c>
-      <c r="J19" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J19" s="28" t="n"/>
       <c r="K19" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L19" s="28" t="inlineStr">
         <is>
           <t>Paiement par domiciliation (AG Insurance)</t>
         </is>
@@ -1228,17 +1098,8 @@
       <c r="I20" s="32" t="n">
         <v>22</v>
       </c>
-      <c r="J20" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K20" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L20" s="28" t="n"/>
+      <c r="J20" s="28" t="n"/>
+      <c r="K20" s="28" t="n"/>
     </row>
     <row r="21">
       <c r="E21" s="16" t="n"/>
@@ -1252,17 +1113,8 @@
       <c r="I21" s="32" t="n">
         <v>66.72</v>
       </c>
-      <c r="J21" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J21" s="28" t="n"/>
       <c r="K21" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L21" s="28" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
         </is>
@@ -1280,17 +1132,8 @@
       <c r="I22" s="32" t="n">
         <v>22.5</v>
       </c>
-      <c r="J22" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J22" s="28" t="n"/>
       <c r="K22" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L22" s="28" t="inlineStr">
         <is>
           <t>Parking Centraal Anvers</t>
         </is>
@@ -1308,17 +1151,8 @@
       <c r="I23" s="32" t="n">
         <v>1.8</v>
       </c>
-      <c r="J23" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J23" s="28" t="n"/>
       <c r="K23" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L23" s="28" t="inlineStr">
         <is>
           <t>Commune Saint-Josse</t>
         </is>
@@ -1336,17 +1170,8 @@
       <c r="I24" s="32" t="n">
         <v>256.99</v>
       </c>
-      <c r="J24" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="K24" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L24" s="28" t="n"/>
+      <c r="J24" s="28" t="n"/>
+      <c r="K24" s="28" t="n"/>
     </row>
     <row r="25">
       <c r="E25" s="16" t="n"/>
@@ -1360,17 +1185,8 @@
       <c r="I25" s="32" t="n">
         <v>159.1</v>
       </c>
-      <c r="J25" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="K25" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L25" s="28" t="n"/>
+      <c r="J25" s="28" t="n"/>
+      <c r="K25" s="28" t="n"/>
     </row>
     <row r="26">
       <c r="E26" s="16" t="n"/>
@@ -1384,17 +1200,8 @@
       <c r="I26" s="32" t="n">
         <v>1.6</v>
       </c>
-      <c r="J26" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J26" s="28" t="n"/>
       <c r="K26" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L26" s="28" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
         </is>
@@ -1412,17 +1219,8 @@
       <c r="I27" s="32" t="n">
         <v>71.13</v>
       </c>
-      <c r="J27" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J27" s="28" t="n"/>
       <c r="K27" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L27" s="28" t="inlineStr">
         <is>
           <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
         </is>
@@ -1440,17 +1238,8 @@
       <c r="I28" s="32" t="n">
         <v>27.9</v>
       </c>
-      <c r="J28" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J28" s="28" t="n"/>
       <c r="K28" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L28" s="28" t="inlineStr">
         <is>
           <t>Domiciliation Autoroutes du Sud de la France</t>
         </is>
@@ -1468,17 +1257,8 @@
       <c r="I29" s="32" t="n">
         <v>7.2</v>
       </c>
-      <c r="J29" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J29" s="28" t="n"/>
       <c r="K29" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L29" s="28" t="inlineStr">
         <is>
           <t>Parking Rogier</t>
         </is>
@@ -1496,17 +1276,8 @@
       <c r="I30" s="32" t="n">
         <v>2.68</v>
       </c>
-      <c r="J30" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K30" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L30" s="28" t="n"/>
+      <c r="J30" s="28" t="n"/>
+      <c r="K30" s="28" t="n"/>
     </row>
     <row r="31">
       <c r="E31" s="16" t="n"/>
@@ -1520,17 +1291,8 @@
       <c r="I31" s="32" t="n">
         <v>1100</v>
       </c>
-      <c r="J31" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J31" s="28" t="n"/>
       <c r="K31" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L31" s="28" t="inlineStr">
         <is>
           <t>Facture de l'agence à joindre</t>
         </is>
@@ -1548,17 +1310,8 @@
       <c r="I32" s="32" t="n">
         <v>2250</v>
       </c>
-      <c r="J32" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="K32" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L32" s="28" t="n"/>
+      <c r="J32" s="28" t="n"/>
+      <c r="K32" s="28" t="n"/>
     </row>
     <row r="33">
       <c r="E33" s="16" t="n"/>
@@ -1572,17 +1325,8 @@
       <c r="I33" s="32" t="n">
         <v>42</v>
       </c>
-      <c r="J33" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J33" s="28" t="n"/>
       <c r="K33" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L33" s="28" t="inlineStr">
         <is>
           <t>Complément — facture à joindre</t>
         </is>
@@ -1600,17 +1344,8 @@
       <c r="I34" s="32" t="n">
         <v>69.44</v>
       </c>
-      <c r="J34" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J34" s="28" t="n"/>
       <c r="K34" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L34" s="28" t="inlineStr">
         <is>
           <t>Lukoil Wezembeek</t>
         </is>
@@ -1628,17 +1363,8 @@
       <c r="I35" s="32" t="n">
         <v>4517.28</v>
       </c>
-      <c r="J35" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J35" s="28" t="n"/>
       <c r="K35" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L35" s="28" t="inlineStr">
         <is>
           <t>Communication 202/9987/63859</t>
         </is>
@@ -1656,17 +1382,8 @@
       <c r="I36" s="32" t="n">
         <v>1125.3</v>
       </c>
-      <c r="J36" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J36" s="28" t="n"/>
       <c r="K36" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L36" s="28" t="inlineStr">
         <is>
           <t>Facture 20240512</t>
         </is>
@@ -1684,17 +1401,8 @@
       <c r="I37" s="32" t="n">
         <v>331.52</v>
       </c>
-      <c r="J37" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="K37" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L37" s="28" t="n"/>
+      <c r="J37" s="28" t="n"/>
+      <c r="K37" s="28" t="n"/>
     </row>
     <row r="38">
       <c r="E38" s="16" t="n"/>
@@ -1708,17 +1416,8 @@
       <c r="I38" s="32" t="n">
         <v>290.4</v>
       </c>
-      <c r="J38" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J38" s="28" t="n"/>
       <c r="K38" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L38" s="28" t="inlineStr">
         <is>
           <t>Facture 20240616</t>
         </is>
@@ -1736,17 +1435,8 @@
       <c r="I39" s="32" t="n">
         <v>242</v>
       </c>
-      <c r="J39" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+      <c r="J39" s="28" t="n"/>
       <c r="K39" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L39" s="28" t="inlineStr">
         <is>
           <t>Facture 20240705</t>
         </is>
@@ -1764,17 +1454,8 @@
       <c r="I40" s="32" t="n">
         <v>70.18000000000001</v>
       </c>
-      <c r="J40" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="K40" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L40" s="28" t="n"/>
+      <c r="J40" s="28" t="n"/>
+      <c r="K40" s="28" t="n"/>
     </row>
     <row r="41">
       <c r="G41" s="33" t="n"/>

</xml_diff>

<commit_message>
Bilan 2025 : exclusion des operations deja reprises en 2024
Les 7 operations de l'extrait 2025-001 se rapportant a decembre 2024 et deja
encodees dans le bilan 2024 sont retirees de janvier 2025 :
entree LAM2415 (4.743,17) et depenses Repas Topogigio (26,00),
precompte salarial decembre 2024 (2.250,00), SD Worx (330,88),
Electrabel (256,99), Telenet (149,10), Proximus (82,99).

Janvier 2025 : 2 entrees = 12.328,20 / 29 depenses = 11.945,49.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K43"/>
+  <dimension ref="D1:K37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -826,76 +826,62 @@
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>LAM2415</t>
+          <t>LAM2501</t>
         </is>
       </c>
       <c r="G6" s="31" t="n">
-        <v>4743.17</v>
+        <v>5328.2</v>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Repas Topogigio</t>
+          <t>Collation - Plouf et Baballe</t>
         </is>
       </c>
       <c r="I6" s="32" t="n">
-        <v>26</v>
+        <v>8.4</v>
       </c>
       <c r="J6" s="28" t="n"/>
-      <c r="K6" s="28" t="inlineStr">
-        <is>
-          <t>Paiement du 31-12-2024 comptabilisé le 01-01-2025 — Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
-        </is>
-      </c>
+      <c r="K6" s="28" t="n"/>
     </row>
     <row r="7">
       <c r="E7" s="16" t="n"/>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>LAM2501</t>
+          <t>LAM2502</t>
         </is>
       </c>
       <c r="G7" s="31" t="n">
-        <v>5328.2</v>
+        <v>7000</v>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Précompte salarial décembre 2024 Thibault Duchène</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="I7" s="32" t="n">
-        <v>2250</v>
+        <v>22.9</v>
       </c>
       <c r="J7" s="28" t="n"/>
       <c r="K7" s="28" t="inlineStr">
         <is>
-          <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="E8" s="16" t="n"/>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>LAM2502</t>
-        </is>
-      </c>
-      <c r="G8" s="31" t="n">
-        <v>7000</v>
-      </c>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="31" t="n"/>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>SD Worx</t>
+          <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
       <c r="I8" s="32" t="n">
-        <v>330.88</v>
+        <v>5.69</v>
       </c>
       <c r="J8" s="28" t="n"/>
-      <c r="K8" s="28" t="inlineStr">
-        <is>
-          <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
-        </is>
-      </c>
+      <c r="K8" s="28" t="n"/>
     </row>
     <row r="9">
       <c r="E9" s="16" t="n"/>
@@ -903,11 +889,11 @@
       <c r="G9" s="31" t="n"/>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Collation - Plouf et Baballe</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="I9" s="32" t="n">
-        <v>8.4</v>
+        <v>1.35</v>
       </c>
       <c r="J9" s="28" t="n"/>
       <c r="K9" s="28" t="n"/>
@@ -918,16 +904,16 @@
       <c r="G10" s="31" t="n"/>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Electrabel</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="I10" s="32" t="n">
-        <v>256.99</v>
+        <v>62.79</v>
       </c>
       <c r="J10" s="28" t="n"/>
       <c r="K10" s="28" t="inlineStr">
         <is>
-          <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
+          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
         </is>
       </c>
     </row>
@@ -937,18 +923,14 @@
       <c r="G11" s="31" t="n"/>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Telenet</t>
+          <t>Crédit voiture</t>
         </is>
       </c>
       <c r="I11" s="32" t="n">
-        <v>149.1</v>
+        <v>724.12</v>
       </c>
       <c r="J11" s="28" t="n"/>
-      <c r="K11" s="28" t="inlineStr">
-        <is>
-          <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage</t>
-        </is>
-      </c>
+      <c r="K11" s="28" t="n"/>
     </row>
     <row r="12">
       <c r="E12" s="16" t="n"/>
@@ -956,18 +938,14 @@
       <c r="G12" s="31" t="n"/>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>Proximus</t>
+          <t>Frais bancaires trimestriels</t>
         </is>
       </c>
       <c r="I12" s="32" t="n">
-        <v>82.98999999999999</v>
+        <v>11.25</v>
       </c>
       <c r="J12" s="28" t="n"/>
-      <c r="K12" s="28" t="inlineStr">
-        <is>
-          <t>Déjà repris dans le bilan 2024 (décembre) — à vérifier pour éviter un double comptage (82,98 encodé en 2024)</t>
-        </is>
-      </c>
+      <c r="K12" s="28" t="n"/>
     </row>
     <row r="13">
       <c r="E13" s="16" t="n"/>
@@ -975,16 +953,16 @@
       <c r="G13" s="31" t="n"/>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Assurance voiture</t>
         </is>
       </c>
       <c r="I13" s="32" t="n">
-        <v>22.9</v>
+        <v>431.25</v>
       </c>
       <c r="J13" s="28" t="n"/>
       <c r="K13" s="28" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Paiement par domiciliation (AG Insurance)</t>
         </is>
       </c>
     </row>
@@ -994,11 +972,11 @@
       <c r="G14" s="31" t="n"/>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Réception marchandise - FEDEX</t>
+          <t>Repas Topogigio</t>
         </is>
       </c>
       <c r="I14" s="32" t="n">
-        <v>5.69</v>
+        <v>22</v>
       </c>
       <c r="J14" s="28" t="n"/>
       <c r="K14" s="28" t="n"/>
@@ -1009,14 +987,18 @@
       <c r="G15" s="31" t="n"/>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="I15" s="32" t="n">
-        <v>1.35</v>
+        <v>66.72</v>
       </c>
       <c r="J15" s="28" t="n"/>
-      <c r="K15" s="28" t="n"/>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="E16" s="16" t="n"/>
@@ -1024,16 +1006,16 @@
       <c r="G16" s="31" t="n"/>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="I16" s="32" t="n">
-        <v>62.79</v>
+        <v>22.5</v>
       </c>
       <c r="J16" s="28" t="n"/>
       <c r="K16" s="28" t="inlineStr">
         <is>
-          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
+          <t>Parking Centraal Anvers</t>
         </is>
       </c>
     </row>
@@ -1043,14 +1025,18 @@
       <c r="G17" s="31" t="n"/>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>Crédit voiture</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="I17" s="32" t="n">
-        <v>724.12</v>
+        <v>1.8</v>
       </c>
       <c r="J17" s="28" t="n"/>
-      <c r="K17" s="28" t="n"/>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>Commune Saint-Josse</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="E18" s="16" t="n"/>
@@ -1058,11 +1044,11 @@
       <c r="G18" s="31" t="n"/>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Frais bancaires trimestriels</t>
+          <t>Electrabel</t>
         </is>
       </c>
       <c r="I18" s="32" t="n">
-        <v>11.25</v>
+        <v>256.99</v>
       </c>
       <c r="J18" s="28" t="n"/>
       <c r="K18" s="28" t="n"/>
@@ -1073,18 +1059,14 @@
       <c r="G19" s="31" t="n"/>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>Assurance voiture</t>
+          <t>Telenet</t>
         </is>
       </c>
       <c r="I19" s="32" t="n">
-        <v>431.25</v>
+        <v>159.1</v>
       </c>
       <c r="J19" s="28" t="n"/>
-      <c r="K19" s="28" t="inlineStr">
-        <is>
-          <t>Paiement par domiciliation (AG Insurance)</t>
-        </is>
-      </c>
+      <c r="K19" s="28" t="n"/>
     </row>
     <row r="20">
       <c r="E20" s="16" t="n"/>
@@ -1092,14 +1074,18 @@
       <c r="G20" s="31" t="n"/>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Repas Topogigio</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="I20" s="32" t="n">
-        <v>22</v>
+        <v>1.6</v>
       </c>
       <c r="J20" s="28" t="n"/>
-      <c r="K20" s="28" t="n"/>
+      <c r="K20" s="28" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="E21" s="16" t="n"/>
@@ -1111,12 +1097,12 @@
         </is>
       </c>
       <c r="I21" s="32" t="n">
-        <v>66.72</v>
+        <v>71.13</v>
       </c>
       <c r="J21" s="28" t="n"/>
       <c r="K21" s="28" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
         </is>
       </c>
     </row>
@@ -1126,16 +1112,16 @@
       <c r="G22" s="31" t="n"/>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Péage autoroute France</t>
         </is>
       </c>
       <c r="I22" s="32" t="n">
-        <v>22.5</v>
+        <v>27.9</v>
       </c>
       <c r="J22" s="28" t="n"/>
       <c r="K22" s="28" t="inlineStr">
         <is>
-          <t>Parking Centraal Anvers</t>
+          <t>Domiciliation Autoroutes du Sud de la France</t>
         </is>
       </c>
     </row>
@@ -1149,12 +1135,12 @@
         </is>
       </c>
       <c r="I23" s="32" t="n">
-        <v>1.8</v>
+        <v>7.2</v>
       </c>
       <c r="J23" s="28" t="n"/>
       <c r="K23" s="28" t="inlineStr">
         <is>
-          <t>Commune Saint-Josse</t>
+          <t>Parking Rogier</t>
         </is>
       </c>
     </row>
@@ -1164,11 +1150,11 @@
       <c r="G24" s="31" t="n"/>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t>Electrabel</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="I24" s="32" t="n">
-        <v>256.99</v>
+        <v>2.68</v>
       </c>
       <c r="J24" s="28" t="n"/>
       <c r="K24" s="28" t="n"/>
@@ -1179,14 +1165,18 @@
       <c r="G25" s="31" t="n"/>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Telenet</t>
+          <t>Billets d'avion Pérou - Translatina Travel</t>
         </is>
       </c>
       <c r="I25" s="32" t="n">
-        <v>159.1</v>
+        <v>1100</v>
       </c>
       <c r="J25" s="28" t="n"/>
-      <c r="K25" s="28" t="n"/>
+      <c r="K25" s="28" t="inlineStr">
+        <is>
+          <t>Facture de l'agence à joindre</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="E26" s="16" t="n"/>
@@ -1194,18 +1184,14 @@
       <c r="G26" s="31" t="n"/>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Précompte salarial janvier 2025 Thibault Duchène</t>
         </is>
       </c>
       <c r="I26" s="32" t="n">
-        <v>1.6</v>
+        <v>2250</v>
       </c>
       <c r="J26" s="28" t="n"/>
-      <c r="K26" s="28" t="inlineStr">
-        <is>
-          <t>Woluwe-Saint-Lambert</t>
-        </is>
-      </c>
+      <c r="K26" s="28" t="n"/>
     </row>
     <row r="27">
       <c r="E27" s="16" t="n"/>
@@ -1213,16 +1199,16 @@
       <c r="G27" s="31" t="n"/>
       <c r="H27" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Billets d'avion Pérou - Translatina Travel</t>
         </is>
       </c>
       <c r="I27" s="32" t="n">
-        <v>71.13</v>
+        <v>42</v>
       </c>
       <c r="J27" s="28" t="n"/>
       <c r="K27" s="28" t="inlineStr">
         <is>
-          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
+          <t>Complément — facture à joindre</t>
         </is>
       </c>
     </row>
@@ -1232,16 +1218,16 @@
       <c r="G28" s="31" t="n"/>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>Péage autoroute France</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="I28" s="32" t="n">
-        <v>27.9</v>
+        <v>69.44</v>
       </c>
       <c r="J28" s="28" t="n"/>
       <c r="K28" s="28" t="inlineStr">
         <is>
-          <t>Domiciliation Autoroutes du Sud de la France</t>
+          <t>Lukoil Wezembeek</t>
         </is>
       </c>
     </row>
@@ -1251,16 +1237,16 @@
       <c r="G29" s="31" t="n"/>
       <c r="H29" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Impôt des sociétés</t>
         </is>
       </c>
       <c r="I29" s="32" t="n">
-        <v>7.2</v>
+        <v>4517.28</v>
       </c>
       <c r="J29" s="28" t="n"/>
       <c r="K29" s="28" t="inlineStr">
         <is>
-          <t>Parking Rogier</t>
+          <t>Communication 202/9987/63859</t>
         </is>
       </c>
     </row>
@@ -1270,14 +1256,18 @@
       <c r="G30" s="31" t="n"/>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Frais comptable BDH</t>
         </is>
       </c>
       <c r="I30" s="32" t="n">
-        <v>2.68</v>
+        <v>1125.3</v>
       </c>
       <c r="J30" s="28" t="n"/>
-      <c r="K30" s="28" t="n"/>
+      <c r="K30" s="28" t="inlineStr">
+        <is>
+          <t>Facture 20240512</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="E31" s="16" t="n"/>
@@ -1285,18 +1275,14 @@
       <c r="G31" s="31" t="n"/>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t>Billets d'avion Pérou - Translatina Travel</t>
+          <t>SD Worx</t>
         </is>
       </c>
       <c r="I31" s="32" t="n">
-        <v>1100</v>
+        <v>331.52</v>
       </c>
       <c r="J31" s="28" t="n"/>
-      <c r="K31" s="28" t="inlineStr">
-        <is>
-          <t>Facture de l'agence à joindre</t>
-        </is>
-      </c>
+      <c r="K31" s="28" t="n"/>
     </row>
     <row r="32">
       <c r="E32" s="16" t="n"/>
@@ -1304,14 +1290,18 @@
       <c r="G32" s="31" t="n"/>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t>Précompte salarial janvier 2025 Thibault Duchène</t>
+          <t>Frais comptable BDH</t>
         </is>
       </c>
       <c r="I32" s="32" t="n">
-        <v>2250</v>
+        <v>290.4</v>
       </c>
       <c r="J32" s="28" t="n"/>
-      <c r="K32" s="28" t="n"/>
+      <c r="K32" s="28" t="inlineStr">
+        <is>
+          <t>Facture 20240616</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="E33" s="16" t="n"/>
@@ -1319,16 +1309,16 @@
       <c r="G33" s="31" t="n"/>
       <c r="H33" s="13" t="inlineStr">
         <is>
-          <t>Billets d'avion Pérou - Translatina Travel</t>
+          <t>Frais comptable BDH</t>
         </is>
       </c>
       <c r="I33" s="32" t="n">
-        <v>42</v>
+        <v>242</v>
       </c>
       <c r="J33" s="28" t="n"/>
       <c r="K33" s="28" t="inlineStr">
         <is>
-          <t>Complément — facture à joindre</t>
+          <t>Facture 20240705</t>
         </is>
       </c>
     </row>
@@ -1338,140 +1328,30 @@
       <c r="G34" s="31" t="n"/>
       <c r="H34" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Proximus</t>
         </is>
       </c>
       <c r="I34" s="32" t="n">
-        <v>69.44</v>
+        <v>70.18000000000001</v>
       </c>
       <c r="J34" s="28" t="n"/>
-      <c r="K34" s="28" t="inlineStr">
-        <is>
-          <t>Lukoil Wezembeek</t>
-        </is>
-      </c>
+      <c r="K34" s="28" t="n"/>
     </row>
     <row r="35">
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="17" t="n"/>
-      <c r="G35" s="31" t="n"/>
-      <c r="H35" s="13" t="inlineStr">
-        <is>
-          <t>Impôt des sociétés</t>
-        </is>
-      </c>
-      <c r="I35" s="32" t="n">
-        <v>4517.28</v>
-      </c>
-      <c r="J35" s="28" t="n"/>
-      <c r="K35" s="28" t="inlineStr">
-        <is>
-          <t>Communication 202/9987/63859</t>
-        </is>
-      </c>
+      <c r="G35" s="33" t="n"/>
+      <c r="I35" s="33" t="n"/>
     </row>
     <row r="36">
-      <c r="E36" s="16" t="n"/>
-      <c r="F36" s="17" t="n"/>
-      <c r="G36" s="31" t="n"/>
-      <c r="H36" s="13" t="inlineStr">
-        <is>
-          <t>Frais comptable BDH</t>
-        </is>
-      </c>
-      <c r="I36" s="32" t="n">
-        <v>1125.3</v>
-      </c>
-      <c r="J36" s="28" t="n"/>
-      <c r="K36" s="28" t="inlineStr">
-        <is>
-          <t>Facture 20240512</t>
-        </is>
-      </c>
+      <c r="G36" s="33" t="n"/>
+      <c r="I36" s="33" t="n"/>
     </row>
     <row r="37">
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="17" t="n"/>
-      <c r="G37" s="31" t="n"/>
-      <c r="H37" s="13" t="inlineStr">
-        <is>
-          <t>SD Worx</t>
-        </is>
-      </c>
-      <c r="I37" s="32" t="n">
-        <v>331.52</v>
-      </c>
-      <c r="J37" s="28" t="n"/>
-      <c r="K37" s="28" t="n"/>
-    </row>
-    <row r="38">
-      <c r="E38" s="16" t="n"/>
-      <c r="F38" s="17" t="n"/>
-      <c r="G38" s="31" t="n"/>
-      <c r="H38" s="13" t="inlineStr">
-        <is>
-          <t>Frais comptable BDH</t>
-        </is>
-      </c>
-      <c r="I38" s="32" t="n">
-        <v>290.4</v>
-      </c>
-      <c r="J38" s="28" t="n"/>
-      <c r="K38" s="28" t="inlineStr">
-        <is>
-          <t>Facture 20240616</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="E39" s="16" t="n"/>
-      <c r="F39" s="17" t="n"/>
-      <c r="G39" s="31" t="n"/>
-      <c r="H39" s="13" t="inlineStr">
-        <is>
-          <t>Frais comptable BDH</t>
-        </is>
-      </c>
-      <c r="I39" s="32" t="n">
-        <v>242</v>
-      </c>
-      <c r="J39" s="28" t="n"/>
-      <c r="K39" s="28" t="inlineStr">
-        <is>
-          <t>Facture 20240705</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="E40" s="16" t="n"/>
-      <c r="F40" s="17" t="n"/>
-      <c r="G40" s="31" t="n"/>
-      <c r="H40" s="13" t="inlineStr">
-        <is>
-          <t>Proximus</t>
-        </is>
-      </c>
-      <c r="I40" s="32" t="n">
-        <v>70.18000000000001</v>
-      </c>
-      <c r="J40" s="28" t="n"/>
-      <c r="K40" s="28" t="n"/>
-    </row>
-    <row r="41">
-      <c r="G41" s="33" t="n"/>
-      <c r="I41" s="33" t="n"/>
-    </row>
-    <row r="42">
-      <c r="G42" s="33" t="n"/>
-      <c r="I42" s="33" t="n"/>
-    </row>
-    <row r="43">
-      <c r="G43" s="33">
-        <f>SUM(G6:G40)</f>
+      <c r="G37" s="33">
+        <f>SUM(G6:G34)</f>
         <v/>
       </c>
-      <c r="I43" s="33">
-        <f>SUM(I6:I40)</f>
+      <c r="I37" s="33">
+        <f>SUM(I6:I34)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : ajout de fevrier
Extrait BNP Paribas Fortis n 2025-002 (operations 0039 a 0066).
2 entrees = 5.401,99 / 26 depenses = 6.341,76.
Rapprochement exact : 3.407,94 + 5.401,99 - 6.341,76 = 2.468,17.

La colonne Remarque est desormais plafonnee a 60 de large avec retour a la
ligne automatique.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -313,7 +313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -347,7 +347,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -745,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K37"/>
+  <dimension ref="D1:K65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -755,7 +762,7 @@
     <col width="47.28515625" customWidth="1" min="8" max="8"/>
     <col width="8.42578125" bestFit="1" customWidth="1" min="9" max="9"/>
     <col width="7.7109375" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="52" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="60" bestFit="1" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -841,7 +848,7 @@
         <v>8.4</v>
       </c>
       <c r="J6" s="28" t="n"/>
-      <c r="K6" s="28" t="n"/>
+      <c r="K6" s="33" t="n"/>
     </row>
     <row r="7">
       <c r="E7" s="16" t="n"/>
@@ -862,7 +869,7 @@
         <v>22.9</v>
       </c>
       <c r="J7" s="28" t="n"/>
-      <c r="K7" s="28" t="inlineStr">
+      <c r="K7" s="33" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
         </is>
@@ -881,7 +888,7 @@
         <v>5.69</v>
       </c>
       <c r="J8" s="28" t="n"/>
-      <c r="K8" s="28" t="n"/>
+      <c r="K8" s="33" t="n"/>
     </row>
     <row r="9">
       <c r="E9" s="16" t="n"/>
@@ -896,7 +903,7 @@
         <v>1.35</v>
       </c>
       <c r="J9" s="28" t="n"/>
-      <c r="K9" s="28" t="n"/>
+      <c r="K9" s="33" t="n"/>
     </row>
     <row r="10">
       <c r="E10" s="16" t="n"/>
@@ -911,7 +918,7 @@
         <v>62.79</v>
       </c>
       <c r="J10" s="28" t="n"/>
-      <c r="K10" s="28" t="inlineStr">
+      <c r="K10" s="33" t="inlineStr">
         <is>
           <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
         </is>
@@ -930,7 +937,7 @@
         <v>724.12</v>
       </c>
       <c r="J11" s="28" t="n"/>
-      <c r="K11" s="28" t="n"/>
+      <c r="K11" s="33" t="n"/>
     </row>
     <row r="12">
       <c r="E12" s="16" t="n"/>
@@ -945,7 +952,7 @@
         <v>11.25</v>
       </c>
       <c r="J12" s="28" t="n"/>
-      <c r="K12" s="28" t="n"/>
+      <c r="K12" s="33" t="n"/>
     </row>
     <row r="13">
       <c r="E13" s="16" t="n"/>
@@ -960,7 +967,7 @@
         <v>431.25</v>
       </c>
       <c r="J13" s="28" t="n"/>
-      <c r="K13" s="28" t="inlineStr">
+      <c r="K13" s="33" t="inlineStr">
         <is>
           <t>Paiement par domiciliation (AG Insurance)</t>
         </is>
@@ -979,7 +986,7 @@
         <v>22</v>
       </c>
       <c r="J14" s="28" t="n"/>
-      <c r="K14" s="28" t="n"/>
+      <c r="K14" s="33" t="n"/>
     </row>
     <row r="15">
       <c r="E15" s="16" t="n"/>
@@ -994,7 +1001,7 @@
         <v>66.72</v>
       </c>
       <c r="J15" s="28" t="n"/>
-      <c r="K15" s="28" t="inlineStr">
+      <c r="K15" s="33" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
         </is>
@@ -1013,7 +1020,7 @@
         <v>22.5</v>
       </c>
       <c r="J16" s="28" t="n"/>
-      <c r="K16" s="28" t="inlineStr">
+      <c r="K16" s="33" t="inlineStr">
         <is>
           <t>Parking Centraal Anvers</t>
         </is>
@@ -1032,7 +1039,7 @@
         <v>1.8</v>
       </c>
       <c r="J17" s="28" t="n"/>
-      <c r="K17" s="28" t="inlineStr">
+      <c r="K17" s="33" t="inlineStr">
         <is>
           <t>Commune Saint-Josse</t>
         </is>
@@ -1051,7 +1058,7 @@
         <v>256.99</v>
       </c>
       <c r="J18" s="28" t="n"/>
-      <c r="K18" s="28" t="n"/>
+      <c r="K18" s="33" t="n"/>
     </row>
     <row r="19">
       <c r="E19" s="16" t="n"/>
@@ -1066,7 +1073,7 @@
         <v>159.1</v>
       </c>
       <c r="J19" s="28" t="n"/>
-      <c r="K19" s="28" t="n"/>
+      <c r="K19" s="33" t="n"/>
     </row>
     <row r="20">
       <c r="E20" s="16" t="n"/>
@@ -1081,7 +1088,7 @@
         <v>1.6</v>
       </c>
       <c r="J20" s="28" t="n"/>
-      <c r="K20" s="28" t="inlineStr">
+      <c r="K20" s="33" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
         </is>
@@ -1100,7 +1107,7 @@
         <v>71.13</v>
       </c>
       <c r="J21" s="28" t="n"/>
-      <c r="K21" s="28" t="inlineStr">
+      <c r="K21" s="33" t="inlineStr">
         <is>
           <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
         </is>
@@ -1119,7 +1126,7 @@
         <v>27.9</v>
       </c>
       <c r="J22" s="28" t="n"/>
-      <c r="K22" s="28" t="inlineStr">
+      <c r="K22" s="33" t="inlineStr">
         <is>
           <t>Domiciliation Autoroutes du Sud de la France</t>
         </is>
@@ -1138,7 +1145,7 @@
         <v>7.2</v>
       </c>
       <c r="J23" s="28" t="n"/>
-      <c r="K23" s="28" t="inlineStr">
+      <c r="K23" s="33" t="inlineStr">
         <is>
           <t>Parking Rogier</t>
         </is>
@@ -1157,7 +1164,7 @@
         <v>2.68</v>
       </c>
       <c r="J24" s="28" t="n"/>
-      <c r="K24" s="28" t="n"/>
+      <c r="K24" s="33" t="n"/>
     </row>
     <row r="25">
       <c r="E25" s="16" t="n"/>
@@ -1172,7 +1179,7 @@
         <v>1100</v>
       </c>
       <c r="J25" s="28" t="n"/>
-      <c r="K25" s="28" t="inlineStr">
+      <c r="K25" s="33" t="inlineStr">
         <is>
           <t>Facture de l'agence à joindre</t>
         </is>
@@ -1191,7 +1198,7 @@
         <v>2250</v>
       </c>
       <c r="J26" s="28" t="n"/>
-      <c r="K26" s="28" t="n"/>
+      <c r="K26" s="33" t="n"/>
     </row>
     <row r="27">
       <c r="E27" s="16" t="n"/>
@@ -1206,7 +1213,7 @@
         <v>42</v>
       </c>
       <c r="J27" s="28" t="n"/>
-      <c r="K27" s="28" t="inlineStr">
+      <c r="K27" s="33" t="inlineStr">
         <is>
           <t>Complément — facture à joindre</t>
         </is>
@@ -1225,7 +1232,7 @@
         <v>69.44</v>
       </c>
       <c r="J28" s="28" t="n"/>
-      <c r="K28" s="28" t="inlineStr">
+      <c r="K28" s="33" t="inlineStr">
         <is>
           <t>Lukoil Wezembeek</t>
         </is>
@@ -1244,7 +1251,7 @@
         <v>4517.28</v>
       </c>
       <c r="J29" s="28" t="n"/>
-      <c r="K29" s="28" t="inlineStr">
+      <c r="K29" s="33" t="inlineStr">
         <is>
           <t>Communication 202/9987/63859</t>
         </is>
@@ -1263,7 +1270,7 @@
         <v>1125.3</v>
       </c>
       <c r="J30" s="28" t="n"/>
-      <c r="K30" s="28" t="inlineStr">
+      <c r="K30" s="33" t="inlineStr">
         <is>
           <t>Facture 20240512</t>
         </is>
@@ -1282,7 +1289,7 @@
         <v>331.52</v>
       </c>
       <c r="J31" s="28" t="n"/>
-      <c r="K31" s="28" t="n"/>
+      <c r="K31" s="33" t="n"/>
     </row>
     <row r="32">
       <c r="E32" s="16" t="n"/>
@@ -1297,7 +1304,7 @@
         <v>290.4</v>
       </c>
       <c r="J32" s="28" t="n"/>
-      <c r="K32" s="28" t="inlineStr">
+      <c r="K32" s="33" t="inlineStr">
         <is>
           <t>Facture 20240616</t>
         </is>
@@ -1316,7 +1323,7 @@
         <v>242</v>
       </c>
       <c r="J33" s="28" t="n"/>
-      <c r="K33" s="28" t="inlineStr">
+      <c r="K33" s="33" t="inlineStr">
         <is>
           <t>Facture 20240705</t>
         </is>
@@ -1335,27 +1342,505 @@
         <v>70.18000000000001</v>
       </c>
       <c r="J34" s="28" t="n"/>
-      <c r="K34" s="28" t="n"/>
+      <c r="K34" s="33" t="n"/>
     </row>
     <row r="35">
-      <c r="G35" s="33" t="n"/>
-      <c r="I35" s="33" t="n"/>
+      <c r="G35" s="34" t="n"/>
+      <c r="I35" s="34" t="n"/>
+      <c r="K35" s="35" t="n"/>
     </row>
     <row r="36">
-      <c r="G36" s="33" t="n"/>
-      <c r="I36" s="33" t="n"/>
+      <c r="G36" s="34" t="n"/>
+      <c r="I36" s="34" t="n"/>
+      <c r="K36" s="35" t="n"/>
     </row>
     <row r="37">
-      <c r="G37" s="33">
-        <f>SUM(G6:G34)</f>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>Février</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>LAM2503</t>
+        </is>
+      </c>
+      <c r="G37" s="31" t="n">
+        <v>5145</v>
+      </c>
+      <c r="H37" s="28" t="inlineStr">
+        <is>
+          <t>Achat vêtements sport - PVH Maasmechelen</t>
+        </is>
+      </c>
+      <c r="I37" s="36" t="n">
+        <v>210.49</v>
+      </c>
+      <c r="J37" s="28" t="n"/>
+      <c r="K37" s="33" t="n"/>
+    </row>
+    <row r="38">
+      <c r="E38" s="16" t="n"/>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>Remboursement Electrabel</t>
+        </is>
+      </c>
+      <c r="G38" s="31" t="n">
+        <v>256.99</v>
+      </c>
+      <c r="H38" s="13" t="inlineStr">
+        <is>
+          <t>Achat vêtements sport - NIKE Maasmechelen</t>
+        </is>
+      </c>
+      <c r="I38" s="32" t="n">
+        <v>141.47</v>
+      </c>
+      <c r="J38" s="28" t="n"/>
+      <c r="K38" s="33" t="n"/>
+    </row>
+    <row r="39">
+      <c r="E39" s="16" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="31" t="n"/>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I39" s="32" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J39" s="28" t="n"/>
+      <c r="K39" s="33" t="inlineStr">
+        <is>
+          <t>Indigo Park Docks</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" s="16" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="31" t="n"/>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I40" s="32" t="n">
+        <v>256.99</v>
+      </c>
+      <c r="J40" s="28" t="n"/>
+      <c r="K40" s="33" t="inlineStr">
+        <is>
+          <t>Facture 468/9192/57548 payée 2× (16-01 et 04-02) — remboursée le 10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" s="16" t="n"/>
+      <c r="F41" s="17" t="n"/>
+      <c r="G41" s="31" t="n"/>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>Telenet</t>
+        </is>
+      </c>
+      <c r="I41" s="32" t="n">
+        <v>149.1</v>
+      </c>
+      <c r="J41" s="28" t="n"/>
+      <c r="K41" s="33" t="n"/>
+    </row>
+    <row r="42">
+      <c r="E42" s="16" t="n"/>
+      <c r="F42" s="17" t="n"/>
+      <c r="G42" s="31" t="n"/>
+      <c r="H42" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I42" s="32" t="n">
+        <v>65</v>
+      </c>
+      <c r="J42" s="28" t="n"/>
+      <c r="K42" s="33" t="inlineStr">
+        <is>
+          <t>Dats 24 Nossegem</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="E43" s="16" t="n"/>
+      <c r="F43" s="17" t="n"/>
+      <c r="G43" s="31" t="n"/>
+      <c r="H43" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I43" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J43" s="28" t="n"/>
+      <c r="K43" s="33" t="n"/>
+    </row>
+    <row r="44">
+      <c r="E44" s="16" t="n"/>
+      <c r="F44" s="17" t="n"/>
+      <c r="G44" s="31" t="n"/>
+      <c r="H44" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I44" s="32" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J44" s="28" t="n"/>
+      <c r="K44" s="33" t="inlineStr">
+        <is>
+          <t>Schaerbeek</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="E45" s="16" t="n"/>
+      <c r="F45" s="17" t="n"/>
+      <c r="G45" s="31" t="n"/>
+      <c r="H45" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I45" s="32" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="J45" s="28" t="n"/>
+      <c r="K45" s="33" t="inlineStr">
+        <is>
+          <t>Administration communale Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="E46" s="16" t="n"/>
+      <c r="F46" s="17" t="n"/>
+      <c r="G46" s="31" t="n"/>
+      <c r="H46" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I46" s="32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J46" s="28" t="n"/>
+      <c r="K46" s="33" t="inlineStr">
+        <is>
+          <t>Parking Ixelles - Gand</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="E47" s="16" t="n"/>
+      <c r="F47" s="17" t="n"/>
+      <c r="G47" s="31" t="n"/>
+      <c r="H47" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I47" s="32" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="J47" s="28" t="n"/>
+      <c r="K47" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Heilig Hart Louvain</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="E48" s="16" t="n"/>
+      <c r="F48" s="17" t="n"/>
+      <c r="G48" s="31" t="n"/>
+      <c r="H48" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I48" s="32" t="n">
+        <v>69.47</v>
+      </c>
+      <c r="J48" s="28" t="n"/>
+      <c r="K48" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="E49" s="16" t="n"/>
+      <c r="F49" s="17" t="n"/>
+      <c r="G49" s="31" t="n"/>
+      <c r="H49" s="13" t="inlineStr">
+        <is>
+          <t>Transport - STIB</t>
+        </is>
+      </c>
+      <c r="I49" s="32" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J49" s="28" t="n"/>
+      <c r="K49" s="33" t="n"/>
+    </row>
+    <row r="50">
+      <c r="E50" s="16" t="n"/>
+      <c r="F50" s="17" t="n"/>
+      <c r="G50" s="31" t="n"/>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>Transport - De Lijn</t>
+        </is>
+      </c>
+      <c r="I50" s="32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J50" s="28" t="n"/>
+      <c r="K50" s="33" t="n"/>
+    </row>
+    <row r="51">
+      <c r="E51" s="16" t="n"/>
+      <c r="F51" s="17" t="n"/>
+      <c r="G51" s="31" t="n"/>
+      <c r="H51" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I51" s="32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="J51" s="28" t="n"/>
+      <c r="K51" s="33" t="inlineStr">
+        <is>
+          <t>Parkeren Louvain</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="E52" s="16" t="n"/>
+      <c r="F52" s="17" t="n"/>
+      <c r="G52" s="31" t="n"/>
+      <c r="H52" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I52" s="32" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J52" s="28" t="n"/>
+      <c r="K52" s="33" t="inlineStr">
+        <is>
+          <t>Commune Saint-Josse</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="E53" s="16" t="n"/>
+      <c r="F53" s="17" t="n"/>
+      <c r="G53" s="31" t="n"/>
+      <c r="H53" s="13" t="inlineStr">
+        <is>
+          <t>Partena</t>
+        </is>
+      </c>
+      <c r="I53" s="32" t="n">
+        <v>1441.87</v>
+      </c>
+      <c r="J53" s="28" t="n"/>
+      <c r="K53" s="33" t="n"/>
+    </row>
+    <row r="54">
+      <c r="E54" s="16" t="n"/>
+      <c r="F54" s="17" t="n"/>
+      <c r="G54" s="31" t="n"/>
+      <c r="H54" s="13" t="inlineStr">
+        <is>
+          <t>Farys (eau)</t>
+        </is>
+      </c>
+      <c r="I54" s="32" t="n">
+        <v>290</v>
+      </c>
+      <c r="J54" s="28" t="n"/>
+      <c r="K54" s="33" t="n"/>
+    </row>
+    <row r="55">
+      <c r="E55" s="16" t="n"/>
+      <c r="F55" s="17" t="n"/>
+      <c r="G55" s="31" t="n"/>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I55" s="32" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="J55" s="28" t="n"/>
+      <c r="K55" s="33" t="inlineStr">
+        <is>
+          <t>Parking Ixelles - Gand</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="E56" s="16" t="n"/>
+      <c r="F56" s="17" t="n"/>
+      <c r="G56" s="31" t="n"/>
+      <c r="H56" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I56" s="32" t="n">
+        <v>68.61</v>
+      </c>
+      <c r="J56" s="28" t="n"/>
+      <c r="K56" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="E57" s="16" t="n"/>
+      <c r="F57" s="17" t="n"/>
+      <c r="G57" s="31" t="n"/>
+      <c r="H57" s="13" t="inlineStr">
+        <is>
+          <t>Repas Lunch Garden</t>
+        </is>
+      </c>
+      <c r="I57" s="32" t="n">
+        <v>39.47</v>
+      </c>
+      <c r="J57" s="28" t="n"/>
+      <c r="K57" s="33" t="inlineStr">
+        <is>
+          <t>LG Auderghem</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="E58" s="16" t="n"/>
+      <c r="F58" s="17" t="n"/>
+      <c r="G58" s="31" t="n"/>
+      <c r="H58" s="13" t="inlineStr">
+        <is>
+          <t>Achat matériel sportif - DECATHLON</t>
+        </is>
+      </c>
+      <c r="I58" s="32" t="n">
+        <v>140</v>
+      </c>
+      <c r="J58" s="28" t="n"/>
+      <c r="K58" s="33" t="inlineStr">
+        <is>
+          <t>Decathlon Evere</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="E59" s="16" t="n"/>
+      <c r="F59" s="17" t="n"/>
+      <c r="G59" s="31" t="n"/>
+      <c r="H59" s="13" t="inlineStr">
+        <is>
+          <t>Précompte salarial février 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I59" s="32" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J59" s="28" t="n"/>
+      <c r="K59" s="33" t="n"/>
+    </row>
+    <row r="60">
+      <c r="E60" s="16" t="n"/>
+      <c r="F60" s="17" t="n"/>
+      <c r="G60" s="31" t="n"/>
+      <c r="H60" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I60" s="32" t="n">
+        <v>331.52</v>
+      </c>
+      <c r="J60" s="28" t="n"/>
+      <c r="K60" s="33" t="n"/>
+    </row>
+    <row r="61">
+      <c r="E61" s="16" t="n"/>
+      <c r="F61" s="17" t="n"/>
+      <c r="G61" s="31" t="n"/>
+      <c r="H61" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I61" s="32" t="n">
+        <v>66.06999999999999</v>
+      </c>
+      <c r="J61" s="28" t="n"/>
+      <c r="K61" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="E62" s="16" t="n"/>
+      <c r="F62" s="17" t="n"/>
+      <c r="G62" s="31" t="n"/>
+      <c r="H62" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I62" s="32" t="n">
+        <v>49.98</v>
+      </c>
+      <c r="J62" s="28" t="n"/>
+      <c r="K62" s="33" t="n"/>
+    </row>
+    <row r="63">
+      <c r="G63" s="34" t="n"/>
+      <c r="I63" s="34" t="n"/>
+      <c r="K63" s="35" t="n"/>
+    </row>
+    <row r="64">
+      <c r="G64" s="34" t="n"/>
+      <c r="I64" s="34" t="n"/>
+      <c r="K64" s="35" t="n"/>
+    </row>
+    <row r="65">
+      <c r="G65" s="34">
+        <f>SUM(G6:G62)</f>
         <v/>
       </c>
-      <c r="I37" s="33">
-        <f>SUM(I6:I34)</f>
+      <c r="I65" s="34">
+        <f>SUM(I6:I62)</f>
         <v/>
       </c>
-    </row>
-    <row r="309" ht="15.75" customHeight="1" thickBot="1"/>
+      <c r="K65" s="35" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Bilan 2025 : ajout de mars
Extrait BNP Paribas Fortis n 2025-003 (operations 0067 a 0093, remises en
ordre chronologique).
2 entrees = 9.888,80 / 25 depenses = 8.750,37.
Rapprochement exact : 2.468,17 + 9.888,80 - 8.750,37 = 3.606,60.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K65"/>
+  <dimension ref="D1:K92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -1831,15 +1831,488 @@
       <c r="K64" s="35" t="n"/>
     </row>
     <row r="65">
-      <c r="G65" s="34">
-        <f>SUM(G6:G62)</f>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
+          <t>Mars</t>
+        </is>
+      </c>
+      <c r="F65" s="17" t="inlineStr">
+        <is>
+          <t>LAM2504</t>
+        </is>
+      </c>
+      <c r="G65" s="31" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H65" s="28" t="inlineStr">
+        <is>
+          <t>Achat - NEW BS SPRL</t>
+        </is>
+      </c>
+      <c r="I65" s="36" t="n">
+        <v>290.5</v>
+      </c>
+      <c r="J65" s="28" t="n"/>
+      <c r="K65" s="33" t="inlineStr">
+        <is>
+          <t>Bruxelles — commerçant à identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="E66" s="16" t="n"/>
+      <c r="F66" s="17" t="inlineStr">
+        <is>
+          <t>LAM2505</t>
+        </is>
+      </c>
+      <c r="G66" s="31" t="n">
+        <v>4888.8</v>
+      </c>
+      <c r="H66" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I66" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J66" s="28" t="n"/>
+      <c r="K66" s="33" t="n"/>
+    </row>
+    <row r="67">
+      <c r="E67" s="16" t="n"/>
+      <c r="F67" s="17" t="n"/>
+      <c r="G67" s="31" t="n"/>
+      <c r="H67" s="13" t="inlineStr">
+        <is>
+          <t>Repas Topogigio</t>
+        </is>
+      </c>
+      <c r="I67" s="32" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="J67" s="28" t="n"/>
+      <c r="K67" s="33" t="n"/>
+    </row>
+    <row r="68">
+      <c r="E68" s="16" t="n"/>
+      <c r="F68" s="17" t="n"/>
+      <c r="G68" s="31" t="n"/>
+      <c r="H68" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I68" s="32" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="J68" s="28" t="n"/>
+      <c r="K68" s="33" t="inlineStr">
+        <is>
+          <t>Brucity - Ville de Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="E69" s="16" t="n"/>
+      <c r="F69" s="17" t="n"/>
+      <c r="G69" s="31" t="n"/>
+      <c r="H69" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I69" s="32" t="n">
+        <v>67.55</v>
+      </c>
+      <c r="J69" s="28" t="n"/>
+      <c r="K69" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Limal</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="E70" s="16" t="n"/>
+      <c r="F70" s="17" t="n"/>
+      <c r="G70" s="31" t="n"/>
+      <c r="H70" s="13" t="inlineStr">
+        <is>
+          <t>Paiement carte VISA</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="J70" s="28" t="n"/>
+      <c r="K70" s="33" t="inlineStr">
+        <is>
+          <t>Décompte n° 060</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="E71" s="16" t="n"/>
+      <c r="F71" s="17" t="n"/>
+      <c r="G71" s="31" t="n"/>
+      <c r="H71" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I71" s="32" t="n">
+        <v>256.99</v>
+      </c>
+      <c r="J71" s="28" t="n"/>
+      <c r="K71" s="33" t="inlineStr">
+        <is>
+          <t>Facture 470/3433/24753</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="E72" s="16" t="n"/>
+      <c r="F72" s="17" t="n"/>
+      <c r="G72" s="31" t="n"/>
+      <c r="H72" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I72" s="32" t="n">
+        <v>256.99</v>
+      </c>
+      <c r="J72" s="28" t="n"/>
+      <c r="K72" s="33" t="inlineStr">
+        <is>
+          <t>Facture 440/7222/59244</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="E73" s="16" t="n"/>
+      <c r="F73" s="17" t="n"/>
+      <c r="G73" s="31" t="n"/>
+      <c r="H73" s="13" t="inlineStr">
+        <is>
+          <t>Telenet</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="n">
+        <v>149.4</v>
+      </c>
+      <c r="J73" s="28" t="n"/>
+      <c r="K73" s="33" t="n"/>
+    </row>
+    <row r="74">
+      <c r="E74" s="16" t="n"/>
+      <c r="F74" s="17" t="n"/>
+      <c r="G74" s="31" t="n"/>
+      <c r="H74" s="13" t="inlineStr">
+        <is>
+          <t>Redevance de stationnement - Ville de Louvain</t>
+        </is>
+      </c>
+      <c r="I74" s="32" t="n">
+        <v>58</v>
+      </c>
+      <c r="J74" s="28" t="n"/>
+      <c r="K74" s="33" t="inlineStr">
+        <is>
+          <t>Comm. 194/3769/90294 — à confirmer (redevance ou amende)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="E75" s="16" t="n"/>
+      <c r="F75" s="17" t="n"/>
+      <c r="G75" s="31" t="n"/>
+      <c r="H75" s="13" t="inlineStr">
+        <is>
+          <t>Redevance de stationnement - Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+      <c r="I75" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="J75" s="28" t="n"/>
+      <c r="K75" s="33" t="inlineStr">
+        <is>
+          <t>Comm. 602/2505/46621 — à confirmer (redevance ou amende)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="E76" s="16" t="n"/>
+      <c r="F76" s="17" t="n"/>
+      <c r="G76" s="31" t="n"/>
+      <c r="H76" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I76" s="32" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J76" s="28" t="n"/>
+      <c r="K76" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="E77" s="16" t="n"/>
+      <c r="F77" s="17" t="n"/>
+      <c r="G77" s="31" t="n"/>
+      <c r="H77" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I77" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="J77" s="28" t="n"/>
+      <c r="K77" s="33" t="inlineStr">
+        <is>
+          <t>T and T Parking Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="E78" s="16" t="n"/>
+      <c r="F78" s="17" t="n"/>
+      <c r="G78" s="31" t="n"/>
+      <c r="H78" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I78" s="32" t="n">
+        <v>60.74</v>
+      </c>
+      <c r="J78" s="28" t="n"/>
+      <c r="K78" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="E79" s="16" t="n"/>
+      <c r="F79" s="17" t="n"/>
+      <c r="G79" s="31" t="n"/>
+      <c r="H79" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I79" s="32" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="J79" s="28" t="n"/>
+      <c r="K79" s="33" t="inlineStr">
+        <is>
+          <t>Commune Saint-Josse</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="E80" s="16" t="n"/>
+      <c r="F80" s="17" t="n"/>
+      <c r="G80" s="31" t="n"/>
+      <c r="H80" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I80" s="32" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="J80" s="28" t="n"/>
+      <c r="K80" s="33" t="inlineStr">
+        <is>
+          <t>Station 15 Zemst</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="E81" s="16" t="n"/>
+      <c r="F81" s="17" t="n"/>
+      <c r="G81" s="31" t="n"/>
+      <c r="H81" s="13" t="inlineStr">
+        <is>
+          <t>Partena</t>
+        </is>
+      </c>
+      <c r="I81" s="32" t="n">
+        <v>3014</v>
+      </c>
+      <c r="J81" s="28" t="n"/>
+      <c r="K81" s="33" t="n"/>
+    </row>
+    <row r="82">
+      <c r="E82" s="16" t="n"/>
+      <c r="F82" s="17" t="n"/>
+      <c r="G82" s="31" t="n"/>
+      <c r="H82" s="13" t="inlineStr">
+        <is>
+          <t>Entretien voiture - Monsieur Pneus</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="n">
+        <v>919.17</v>
+      </c>
+      <c r="J82" s="28" t="n"/>
+      <c r="K82" s="33" t="n"/>
+    </row>
+    <row r="83">
+      <c r="E83" s="16" t="n"/>
+      <c r="F83" s="17" t="n"/>
+      <c r="G83" s="31" t="n"/>
+      <c r="H83" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I83" s="32" t="n">
+        <v>70.68000000000001</v>
+      </c>
+      <c r="J83" s="28" t="n"/>
+      <c r="K83" s="33" t="inlineStr">
+        <is>
+          <t>Shell Kraainem</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="E84" s="16" t="n"/>
+      <c r="F84" s="17" t="n"/>
+      <c r="G84" s="31" t="n"/>
+      <c r="H84" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I84" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="J84" s="28" t="n"/>
+      <c r="K84" s="33" t="inlineStr">
+        <is>
+          <t>Station 15 Zemst</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="E85" s="16" t="n"/>
+      <c r="F85" s="17" t="n"/>
+      <c r="G85" s="31" t="n"/>
+      <c r="H85" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I85" s="32" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="J85" s="28" t="n"/>
+      <c r="K85" s="33" t="inlineStr">
+        <is>
+          <t>Parking Rogier</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="E86" s="16" t="n"/>
+      <c r="F86" s="17" t="n"/>
+      <c r="G86" s="31" t="n"/>
+      <c r="H86" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I86" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J86" s="28" t="n"/>
+      <c r="K86" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="E87" s="16" t="n"/>
+      <c r="F87" s="17" t="n"/>
+      <c r="G87" s="31" t="n"/>
+      <c r="H87" s="13" t="inlineStr">
+        <is>
+          <t>Précompte salarial mars 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I87" s="32" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J87" s="28" t="n"/>
+      <c r="K87" s="33" t="n"/>
+    </row>
+    <row r="88">
+      <c r="E88" s="16" t="n"/>
+      <c r="F88" s="17" t="n"/>
+      <c r="G88" s="31" t="n"/>
+      <c r="H88" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I88" s="32" t="n">
+        <v>331.52</v>
+      </c>
+      <c r="J88" s="28" t="n"/>
+      <c r="K88" s="33" t="n"/>
+    </row>
+    <row r="89">
+      <c r="E89" s="16" t="n"/>
+      <c r="F89" s="17" t="n"/>
+      <c r="G89" s="31" t="n"/>
+      <c r="H89" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I89" s="32" t="n">
+        <v>70.48999999999999</v>
+      </c>
+      <c r="J89" s="28" t="n"/>
+      <c r="K89" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="G90" s="34" t="n"/>
+      <c r="I90" s="34" t="n"/>
+      <c r="K90" s="35" t="n"/>
+    </row>
+    <row r="91">
+      <c r="G91" s="34" t="n"/>
+      <c r="I91" s="34" t="n"/>
+      <c r="K91" s="35" t="n"/>
+    </row>
+    <row r="92">
+      <c r="G92" s="34">
+        <f>SUM(G6:G89)</f>
         <v/>
       </c>
-      <c r="I65" s="34">
-        <f>SUM(I6:I62)</f>
+      <c r="I92" s="34">
+        <f>SUM(I6:I89)</f>
         <v/>
       </c>
-      <c r="K65" s="35" t="n"/>
+      <c r="K92" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout d'avril
Extrait BNP Paribas Fortis n 2025-004 (operations 0094 a 0123), arrete au
26-04 : les operations de fin de mois basculent sur l'extrait de mai.
1 entree = 1.683,78 / 29 depenses = 3.041,93.
Rapprochement exact : 3.606,60 + 1.683,78 - 3.041,93 = 2.248,45.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K92"/>
+  <dimension ref="D1:K123"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -2304,15 +2304,566 @@
       <c r="K91" s="35" t="n"/>
     </row>
     <row r="92">
-      <c r="G92" s="34">
-        <f>SUM(G6:G89)</f>
+      <c r="E92" s="16" t="inlineStr">
+        <is>
+          <t>Avril</t>
+        </is>
+      </c>
+      <c r="F92" s="17" t="inlineStr">
+        <is>
+          <t>Remboursement billet d'avion Lima-Bruxelles</t>
+        </is>
+      </c>
+      <c r="G92" s="31" t="n">
+        <v>1683.78</v>
+      </c>
+      <c r="H92" s="28" t="inlineStr">
+        <is>
+          <t>Repas Exki</t>
+        </is>
+      </c>
+      <c r="I92" s="36" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="J92" s="28" t="n"/>
+      <c r="K92" s="33" t="inlineStr">
+        <is>
+          <t>Exki Woluwe</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="E93" s="16" t="n"/>
+      <c r="F93" s="17" t="n"/>
+      <c r="G93" s="31" t="n"/>
+      <c r="H93" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I93" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J93" s="28" t="n"/>
+      <c r="K93" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="E94" s="16" t="n"/>
+      <c r="F94" s="17" t="n"/>
+      <c r="G94" s="31" t="n"/>
+      <c r="H94" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I94" s="32" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="J94" s="28" t="n"/>
+      <c r="K94" s="33" t="inlineStr">
+        <is>
+          <t>Delft (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="E95" s="16" t="n"/>
+      <c r="F95" s="17" t="n"/>
+      <c r="G95" s="31" t="n"/>
+      <c r="H95" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I95" s="32" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="J95" s="28" t="n"/>
+      <c r="K95" s="33" t="inlineStr">
+        <is>
+          <t>Markthof La Haye (Pays-Bas) — à confirmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="E96" s="16" t="n"/>
+      <c r="F96" s="17" t="n"/>
+      <c r="G96" s="31" t="n"/>
+      <c r="H96" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I96" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J96" s="28" t="n"/>
+      <c r="K96" s="33" t="n"/>
+    </row>
+    <row r="97">
+      <c r="E97" s="16" t="n"/>
+      <c r="F97" s="17" t="n"/>
+      <c r="G97" s="31" t="n"/>
+      <c r="H97" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I97" s="32" t="n">
+        <v>23</v>
+      </c>
+      <c r="J97" s="28" t="n"/>
+      <c r="K97" s="33" t="inlineStr">
+        <is>
+          <t>Stadparkeerplan Leyde (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="E98" s="16" t="n"/>
+      <c r="F98" s="17" t="n"/>
+      <c r="G98" s="31" t="n"/>
+      <c r="H98" s="13" t="inlineStr">
+        <is>
+          <t>Frais bancaires trimestriels</t>
+        </is>
+      </c>
+      <c r="I98" s="32" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="J98" s="28" t="n"/>
+      <c r="K98" s="33" t="n"/>
+    </row>
+    <row r="99">
+      <c r="E99" s="16" t="n"/>
+      <c r="F99" s="17" t="n"/>
+      <c r="G99" s="31" t="n"/>
+      <c r="H99" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I99" s="32" t="n">
+        <v>87</v>
+      </c>
+      <c r="J99" s="28" t="n"/>
+      <c r="K99" s="33" t="inlineStr">
+        <is>
+          <t>Total Leyde (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="E100" s="16" t="n"/>
+      <c r="F100" s="17" t="n"/>
+      <c r="G100" s="31" t="n"/>
+      <c r="H100" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I100" s="32" t="n">
+        <v>10.46</v>
+      </c>
+      <c r="J100" s="28" t="n"/>
+      <c r="K100" s="33" t="inlineStr">
+        <is>
+          <t>Commune d'Utrecht (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="E101" s="16" t="n"/>
+      <c r="F101" s="17" t="n"/>
+      <c r="G101" s="31" t="n"/>
+      <c r="H101" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I101" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="J101" s="28" t="n"/>
+      <c r="K101" s="33" t="inlineStr">
+        <is>
+          <t>Parking De Vooruitgang, Volendam (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="E102" s="16" t="n"/>
+      <c r="F102" s="17" t="n"/>
+      <c r="G102" s="31" t="n"/>
+      <c r="H102" s="13" t="inlineStr">
+        <is>
+          <t>Achat - NZA Utrecht BV</t>
+        </is>
+      </c>
+      <c r="I102" s="32" t="n">
+        <v>289.97</v>
+      </c>
+      <c r="J102" s="28" t="n"/>
+      <c r="K102" s="33" t="inlineStr">
+        <is>
+          <t>Amsterdam (Pays-Bas) — commerçant à identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="E103" s="16" t="n"/>
+      <c r="F103" s="17" t="n"/>
+      <c r="G103" s="31" t="n"/>
+      <c r="H103" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I103" s="32" t="n">
+        <v>141.5</v>
+      </c>
+      <c r="J103" s="28" t="n"/>
+      <c r="K103" s="33" t="n"/>
+    </row>
+    <row r="104">
+      <c r="E104" s="16" t="n"/>
+      <c r="F104" s="17" t="n"/>
+      <c r="G104" s="31" t="n"/>
+      <c r="H104" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I104" s="32" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="J104" s="28" t="n"/>
+      <c r="K104" s="33" t="inlineStr">
+        <is>
+          <t>Commune d'Utrecht (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="E105" s="16" t="n"/>
+      <c r="F105" s="17" t="n"/>
+      <c r="G105" s="31" t="n"/>
+      <c r="H105" s="13" t="inlineStr">
+        <is>
+          <t>Telenet</t>
+        </is>
+      </c>
+      <c r="I105" s="32" t="n">
+        <v>149.1</v>
+      </c>
+      <c r="J105" s="28" t="n"/>
+      <c r="K105" s="33" t="n"/>
+    </row>
+    <row r="106">
+      <c r="E106" s="16" t="n"/>
+      <c r="F106" s="17" t="n"/>
+      <c r="G106" s="31" t="n"/>
+      <c r="H106" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I106" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="J106" s="28" t="n"/>
+      <c r="K106" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Sint Jorisplein, Amersfoort (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="E107" s="16" t="n"/>
+      <c r="F107" s="17" t="n"/>
+      <c r="G107" s="31" t="n"/>
+      <c r="H107" s="13" t="inlineStr">
+        <is>
+          <t>Paiement carte VISA</t>
+        </is>
+      </c>
+      <c r="I107" s="32" t="n">
+        <v>433.78</v>
+      </c>
+      <c r="J107" s="28" t="n"/>
+      <c r="K107" s="33" t="inlineStr">
+        <is>
+          <t>Décompte n° 091</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="E108" s="16" t="n"/>
+      <c r="F108" s="17" t="n"/>
+      <c r="G108" s="31" t="n"/>
+      <c r="H108" s="13" t="inlineStr">
+        <is>
+          <t>Assurance voiture</t>
+        </is>
+      </c>
+      <c r="I108" s="32" t="n">
+        <v>431.25</v>
+      </c>
+      <c r="J108" s="28" t="n"/>
+      <c r="K108" s="33" t="inlineStr">
+        <is>
+          <t>Paiement par domiciliation (AG Insurance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="E109" s="16" t="n"/>
+      <c r="F109" s="17" t="n"/>
+      <c r="G109" s="31" t="n"/>
+      <c r="H109" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I109" s="32" t="n">
+        <v>72.18000000000001</v>
+      </c>
+      <c r="J109" s="28" t="n"/>
+      <c r="K109" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="E110" s="16" t="n"/>
+      <c r="F110" s="17" t="n"/>
+      <c r="G110" s="31" t="n"/>
+      <c r="H110" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I110" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="J110" s="28" t="n"/>
+      <c r="K110" s="33" t="inlineStr">
+        <is>
+          <t>T and T Parking Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="E111" s="16" t="n"/>
+      <c r="F111" s="17" t="n"/>
+      <c r="G111" s="31" t="n"/>
+      <c r="H111" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I111" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="J111" s="28" t="n"/>
+      <c r="K111" s="33" t="inlineStr">
+        <is>
+          <t>Parking Casino Middelkerke</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="E112" s="16" t="n"/>
+      <c r="F112" s="17" t="n"/>
+      <c r="G112" s="31" t="n"/>
+      <c r="H112" s="13" t="inlineStr">
+        <is>
+          <t>Divers - sanitaires autoroute</t>
+        </is>
+      </c>
+      <c r="I112" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J112" s="28" t="n"/>
+      <c r="K112" s="33" t="inlineStr">
+        <is>
+          <t>2theloo, aire E40 Jabbeke</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="E113" s="16" t="n"/>
+      <c r="F113" s="17" t="n"/>
+      <c r="G113" s="31" t="n"/>
+      <c r="H113" s="13" t="inlineStr">
+        <is>
+          <t>Divers - sanitaires autoroute</t>
+        </is>
+      </c>
+      <c r="I113" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J113" s="28" t="n"/>
+      <c r="K113" s="33" t="inlineStr">
+        <is>
+          <t>2theloo, aire E40 Jabbeke</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="E114" s="16" t="n"/>
+      <c r="F114" s="17" t="n"/>
+      <c r="G114" s="31" t="n"/>
+      <c r="H114" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I114" s="32" t="n">
+        <v>64.06999999999999</v>
+      </c>
+      <c r="J114" s="28" t="n"/>
+      <c r="K114" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="E115" s="16" t="n"/>
+      <c r="F115" s="17" t="n"/>
+      <c r="G115" s="31" t="n"/>
+      <c r="H115" s="13" t="inlineStr">
+        <is>
+          <t>Collation</t>
+        </is>
+      </c>
+      <c r="I115" s="32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J115" s="28" t="n"/>
+      <c r="K115" s="33" t="inlineStr">
+        <is>
+          <t>AC Restaurants Wanlin</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="E116" s="16" t="n"/>
+      <c r="F116" s="17" t="n"/>
+      <c r="G116" s="31" t="n"/>
+      <c r="H116" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I116" s="32" t="n">
+        <v>256.99</v>
+      </c>
+      <c r="J116" s="28" t="n"/>
+      <c r="K116" s="33" t="inlineStr">
+        <is>
+          <t>Facture 439/4769/34444</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="E117" s="16" t="n"/>
+      <c r="F117" s="17" t="n"/>
+      <c r="G117" s="31" t="n"/>
+      <c r="H117" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I117" s="32" t="n">
+        <v>60.37</v>
+      </c>
+      <c r="J117" s="28" t="n"/>
+      <c r="K117" s="33" t="inlineStr">
+        <is>
+          <t>Lukoil Wezembeek</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="E118" s="16" t="n"/>
+      <c r="F118" s="17" t="n"/>
+      <c r="G118" s="31" t="n"/>
+      <c r="H118" s="13" t="inlineStr">
+        <is>
+          <t>Repas Topogigio</t>
+        </is>
+      </c>
+      <c r="I118" s="32" t="n">
+        <v>26</v>
+      </c>
+      <c r="J118" s="28" t="n"/>
+      <c r="K118" s="33" t="n"/>
+    </row>
+    <row r="119">
+      <c r="E119" s="16" t="n"/>
+      <c r="F119" s="17" t="n"/>
+      <c r="G119" s="31" t="n"/>
+      <c r="H119" s="13" t="inlineStr">
+        <is>
+          <t>Achat matériel sportif - DECATHLON</t>
+        </is>
+      </c>
+      <c r="I119" s="32" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="J119" s="28" t="n"/>
+      <c r="K119" s="33" t="inlineStr">
+        <is>
+          <t>Decathlon Evere</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="E120" s="16" t="n"/>
+      <c r="F120" s="17" t="n"/>
+      <c r="G120" s="31" t="n"/>
+      <c r="H120" s="13" t="inlineStr">
+        <is>
+          <t>Achat Delhaize</t>
+        </is>
+      </c>
+      <c r="I120" s="32" t="n">
+        <v>43.43</v>
+      </c>
+      <c r="J120" s="28" t="n"/>
+      <c r="K120" s="33" t="inlineStr">
+        <is>
+          <t>Delhaize Sterrebeek - payé avec la carte 5255 (autre carte)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="G121" s="34" t="n"/>
+      <c r="I121" s="34" t="n"/>
+      <c r="K121" s="35" t="n"/>
+    </row>
+    <row r="122">
+      <c r="G122" s="34" t="n"/>
+      <c r="I122" s="34" t="n"/>
+      <c r="K122" s="35" t="n"/>
+    </row>
+    <row r="123">
+      <c r="G123" s="34">
+        <f>SUM(G6:G120)</f>
         <v/>
       </c>
-      <c r="I92" s="34">
-        <f>SUM(I6:I89)</f>
+      <c r="I123" s="34">
+        <f>SUM(I6:I120)</f>
         <v/>
       </c>
-      <c r="K92" s="35" t="n"/>
+      <c r="K123" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout de mai
Extrait BNP Paribas Fortis n 2025-005 (operations 0124 a 0145, periode du
26-04 au 29-05).
2 entrees = 9.631,71 / 20 depenses = 6.522,06.
Rapprochement exact : 2.248,45 + 9.631,71 - 6.522,06 = 5.358,10.

Precision de la remarque d'avril sur la carte 5255, qui remplace la 4871.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K123"/>
+  <dimension ref="D1:K145"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -2840,7 +2840,7 @@
       <c r="J120" s="28" t="n"/>
       <c r="K120" s="33" t="inlineStr">
         <is>
-          <t>Delhaize Sterrebeek - payé avec la carte 5255 (autre carte)</t>
+          <t>Delhaize Sterrebeek - 1er paiement avec la nouvelle carte 5255</t>
         </is>
       </c>
     </row>
@@ -2855,15 +2855,397 @@
       <c r="K122" s="35" t="n"/>
     </row>
     <row r="123">
-      <c r="G123" s="34">
-        <f>SUM(G6:G120)</f>
+      <c r="E123" s="16" t="inlineStr">
+        <is>
+          <t>Mai</t>
+        </is>
+      </c>
+      <c r="F123" s="17" t="inlineStr">
+        <is>
+          <t>LAM2506</t>
+        </is>
+      </c>
+      <c r="G123" s="31" t="n">
+        <v>4554.6</v>
+      </c>
+      <c r="H123" s="28" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I123" s="36" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J123" s="28" t="n"/>
+      <c r="K123" s="33" t="n"/>
+    </row>
+    <row r="124">
+      <c r="E124" s="16" t="n"/>
+      <c r="F124" s="17" t="inlineStr">
+        <is>
+          <t>LAM2507</t>
+        </is>
+      </c>
+      <c r="G124" s="31" t="n">
+        <v>5077.11</v>
+      </c>
+      <c r="H124" s="13" t="inlineStr">
+        <is>
+          <t>Précompte salarial avril 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I124" s="32" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J124" s="28" t="n"/>
+      <c r="K124" s="33" t="n"/>
+    </row>
+    <row r="125">
+      <c r="E125" s="16" t="n"/>
+      <c r="F125" s="17" t="n"/>
+      <c r="G125" s="31" t="n"/>
+      <c r="H125" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I125" s="32" t="n">
+        <v>331.99</v>
+      </c>
+      <c r="J125" s="28" t="n"/>
+      <c r="K125" s="33" t="n"/>
+    </row>
+    <row r="126">
+      <c r="E126" s="16" t="n"/>
+      <c r="F126" s="17" t="n"/>
+      <c r="G126" s="31" t="n"/>
+      <c r="H126" s="13" t="inlineStr">
+        <is>
+          <t>Farys (eau)</t>
+        </is>
+      </c>
+      <c r="I126" s="32" t="n">
+        <v>290</v>
+      </c>
+      <c r="J126" s="28" t="n"/>
+      <c r="K126" s="33" t="n"/>
+    </row>
+    <row r="127">
+      <c r="E127" s="16" t="n"/>
+      <c r="F127" s="17" t="n"/>
+      <c r="G127" s="31" t="n"/>
+      <c r="H127" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I127" s="32" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="J127" s="28" t="n"/>
+      <c r="K127" s="33" t="n"/>
+    </row>
+    <row r="128">
+      <c r="E128" s="16" t="n"/>
+      <c r="F128" s="17" t="n"/>
+      <c r="G128" s="31" t="n"/>
+      <c r="H128" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I128" s="32" t="n">
+        <v>59.49</v>
+      </c>
+      <c r="J128" s="28" t="n"/>
+      <c r="K128" s="33" t="inlineStr">
+        <is>
+          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="E129" s="16" t="n"/>
+      <c r="F129" s="17" t="n"/>
+      <c r="G129" s="31" t="n"/>
+      <c r="H129" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I129" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J129" s="28" t="n"/>
+      <c r="K129" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="E130" s="16" t="n"/>
+      <c r="F130" s="17" t="n"/>
+      <c r="G130" s="31" t="n"/>
+      <c r="H130" s="13" t="inlineStr">
+        <is>
+          <t>Paiement carte VISA</t>
+        </is>
+      </c>
+      <c r="I130" s="32" t="n">
+        <v>2116.19</v>
+      </c>
+      <c r="J130" s="28" t="n"/>
+      <c r="K130" s="33" t="inlineStr">
+        <is>
+          <t>Décompte n° 121</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="E131" s="16" t="n"/>
+      <c r="F131" s="17" t="n"/>
+      <c r="G131" s="31" t="n"/>
+      <c r="H131" s="13" t="inlineStr">
+        <is>
+          <t>Achat matériel sportif - DECATHLON</t>
+        </is>
+      </c>
+      <c r="I131" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="J131" s="28" t="n"/>
+      <c r="K131" s="33" t="inlineStr">
+        <is>
+          <t>Decathlon Evere</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="E132" s="16" t="n"/>
+      <c r="F132" s="17" t="n"/>
+      <c r="G132" s="31" t="n"/>
+      <c r="H132" s="13" t="inlineStr">
+        <is>
+          <t>Telenet</t>
+        </is>
+      </c>
+      <c r="I132" s="32" t="n">
+        <v>149.1</v>
+      </c>
+      <c r="J132" s="28" t="n"/>
+      <c r="K132" s="33" t="n"/>
+    </row>
+    <row r="133">
+      <c r="E133" s="16" t="n"/>
+      <c r="F133" s="17" t="n"/>
+      <c r="G133" s="31" t="n"/>
+      <c r="H133" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I133" s="32" t="n">
+        <v>66.09</v>
+      </c>
+      <c r="J133" s="28" t="n"/>
+      <c r="K133" s="33" t="inlineStr">
+        <is>
+          <t>Lukoil Tervuren</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="E134" s="16" t="n"/>
+      <c r="F134" s="17" t="n"/>
+      <c r="G134" s="31" t="n"/>
+      <c r="H134" s="13" t="inlineStr">
+        <is>
+          <t>Divers - sanitaires autoroute</t>
+        </is>
+      </c>
+      <c r="I134" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J134" s="28" t="n"/>
+      <c r="K134" s="33" t="inlineStr">
+        <is>
+          <t>Tank und Rastanlage, Frechen (Allemagne)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="E135" s="16" t="n"/>
+      <c r="F135" s="17" t="n"/>
+      <c r="G135" s="31" t="n"/>
+      <c r="H135" s="13" t="inlineStr">
+        <is>
+          <t>Divers - sanitaires autoroute</t>
+        </is>
+      </c>
+      <c r="I135" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J135" s="28" t="n"/>
+      <c r="K135" s="33" t="inlineStr">
+        <is>
+          <t>Tank und Rastanlage, Frechen (Allemagne)</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="E136" s="16" t="n"/>
+      <c r="F136" s="17" t="n"/>
+      <c r="G136" s="31" t="n"/>
+      <c r="H136" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I136" s="32" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="J136" s="28" t="n"/>
+      <c r="K136" s="33" t="inlineStr">
+        <is>
+          <t>Bonner City Parkraum, Bonn (Allemagne)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="E137" s="16" t="n"/>
+      <c r="F137" s="17" t="n"/>
+      <c r="G137" s="31" t="n"/>
+      <c r="H137" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I137" s="32" t="n">
+        <v>58.83</v>
+      </c>
+      <c r="J137" s="28" t="n"/>
+      <c r="K137" s="33" t="inlineStr">
+        <is>
+          <t>Shell Kraainem</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="E138" s="16" t="n"/>
+      <c r="F138" s="17" t="n"/>
+      <c r="G138" s="31" t="n"/>
+      <c r="H138" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I138" s="32" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J138" s="28" t="n"/>
+      <c r="K138" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="E139" s="16" t="n"/>
+      <c r="F139" s="17" t="n"/>
+      <c r="G139" s="31" t="n"/>
+      <c r="H139" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I139" s="32" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J139" s="28" t="n"/>
+      <c r="K139" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="E140" s="16" t="n"/>
+      <c r="F140" s="17" t="n"/>
+      <c r="G140" s="31" t="n"/>
+      <c r="H140" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I140" s="32" t="n">
+        <v>256.99</v>
+      </c>
+      <c r="J140" s="28" t="n"/>
+      <c r="K140" s="33" t="inlineStr">
+        <is>
+          <t>Facture 493/0415/84633</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="E141" s="16" t="n"/>
+      <c r="F141" s="17" t="n"/>
+      <c r="G141" s="31" t="n"/>
+      <c r="H141" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I141" s="32" t="n">
+        <v>72.42</v>
+      </c>
+      <c r="J141" s="28" t="n"/>
+      <c r="K141" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Tervuren</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="E142" s="16" t="n"/>
+      <c r="F142" s="17" t="n"/>
+      <c r="G142" s="31" t="n"/>
+      <c r="H142" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I142" s="32" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J142" s="28" t="n"/>
+      <c r="K142" s="33" t="inlineStr">
+        <is>
+          <t>Ville de Dinant</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="G143" s="34" t="n"/>
+      <c r="I143" s="34" t="n"/>
+      <c r="K143" s="35" t="n"/>
+    </row>
+    <row r="144">
+      <c r="G144" s="34" t="n"/>
+      <c r="I144" s="34" t="n"/>
+      <c r="K144" s="35" t="n"/>
+    </row>
+    <row r="145">
+      <c r="G145" s="34">
+        <f>SUM(G6:G142)</f>
         <v/>
       </c>
-      <c r="I123" s="34">
-        <f>SUM(I6:I120)</f>
+      <c r="I145" s="34">
+        <f>SUM(I6:I142)</f>
         <v/>
       </c>
-      <c r="K123" s="35" t="n"/>
+      <c r="K145" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout de juin
Extrait BNP Paribas Fortis n 2025-006 (operations 0146 a 0173, periode du
29-05 au 29-06).
2 entrees = 5.960,00 / 26 depenses = 6.387,98.
Rapprochement exact : 5.358,10 + 5.960,00 - 6.387,98 = 4.930,12.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K145"/>
+  <dimension ref="D1:K173"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -3237,15 +3237,511 @@
       <c r="K144" s="35" t="n"/>
     </row>
     <row r="145">
-      <c r="G145" s="34">
-        <f>SUM(G6:G142)</f>
+      <c r="E145" s="16" t="inlineStr">
+        <is>
+          <t>Juin</t>
+        </is>
+      </c>
+      <c r="F145" s="17" t="inlineStr">
+        <is>
+          <t>LAM2508</t>
+        </is>
+      </c>
+      <c r="G145" s="31" t="n">
+        <v>4460</v>
+      </c>
+      <c r="H145" s="28" t="inlineStr">
+        <is>
+          <t>Achat matériel sportif - DECATHLON</t>
+        </is>
+      </c>
+      <c r="I145" s="36" t="n">
+        <v>200</v>
+      </c>
+      <c r="J145" s="28" t="n"/>
+      <c r="K145" s="33" t="inlineStr">
+        <is>
+          <t>Decathlon Evere</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="E146" s="16" t="n"/>
+      <c r="F146" s="17" t="inlineStr">
+        <is>
+          <t>Approvisionnement compte - Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="G146" s="31" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H146" s="13" t="inlineStr">
+        <is>
+          <t>Précompte salarial mai 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I146" s="32" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J146" s="28" t="n"/>
+      <c r="K146" s="33" t="n"/>
+    </row>
+    <row r="147">
+      <c r="E147" s="16" t="n"/>
+      <c r="F147" s="17" t="n"/>
+      <c r="G147" s="31" t="n"/>
+      <c r="H147" s="13" t="inlineStr">
+        <is>
+          <t>Partena</t>
+        </is>
+      </c>
+      <c r="I147" s="32" t="n">
+        <v>1441.87</v>
+      </c>
+      <c r="J147" s="28" t="n"/>
+      <c r="K147" s="33" t="n"/>
+    </row>
+    <row r="148">
+      <c r="E148" s="16" t="n"/>
+      <c r="F148" s="17" t="n"/>
+      <c r="G148" s="31" t="n"/>
+      <c r="H148" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I148" s="32" t="n">
+        <v>331.99</v>
+      </c>
+      <c r="J148" s="28" t="n"/>
+      <c r="K148" s="33" t="n"/>
+    </row>
+    <row r="149">
+      <c r="E149" s="16" t="n"/>
+      <c r="F149" s="17" t="n"/>
+      <c r="G149" s="31" t="n"/>
+      <c r="H149" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I149" s="32" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="J149" s="28" t="n"/>
+      <c r="K149" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="E150" s="16" t="n"/>
+      <c r="F150" s="17" t="n"/>
+      <c r="G150" s="31" t="n"/>
+      <c r="H150" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I150" s="32" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J150" s="28" t="n"/>
+      <c r="K150" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="E151" s="16" t="n"/>
+      <c r="F151" s="17" t="n"/>
+      <c r="G151" s="31" t="n"/>
+      <c r="H151" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I151" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J151" s="28" t="n"/>
+      <c r="K151" s="33" t="n"/>
+    </row>
+    <row r="152">
+      <c r="E152" s="16" t="n"/>
+      <c r="F152" s="17" t="n"/>
+      <c r="G152" s="31" t="n"/>
+      <c r="H152" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I152" s="32" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="J152" s="28" t="n"/>
+      <c r="K152" s="33" t="inlineStr">
+        <is>
+          <t>RG Public, Paris (France) — à confirmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="E153" s="16" t="n"/>
+      <c r="F153" s="17" t="n"/>
+      <c r="G153" s="31" t="n"/>
+      <c r="H153" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I153" s="32" t="n">
+        <v>75.87</v>
+      </c>
+      <c r="J153" s="28" t="n"/>
+      <c r="K153" s="33" t="inlineStr">
+        <is>
+          <t>Station Avia, Havrincourt (France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="E154" s="16" t="n"/>
+      <c r="F154" s="17" t="n"/>
+      <c r="G154" s="31" t="n"/>
+      <c r="H154" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I154" s="32" t="n">
+        <v>31.05</v>
+      </c>
+      <c r="J154" s="28" t="n"/>
+      <c r="K154" s="33" t="inlineStr">
+        <is>
+          <t>Indigo, Paris (France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="E155" s="16" t="n"/>
+      <c r="F155" s="17" t="n"/>
+      <c r="G155" s="31" t="n"/>
+      <c r="H155" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I155" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="J155" s="28" t="n"/>
+      <c r="K155" s="33" t="inlineStr">
+        <is>
+          <t>Brussels Expo — à confirmer (parking ou entrée)</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="E156" s="16" t="n"/>
+      <c r="F156" s="17" t="n"/>
+      <c r="G156" s="31" t="n"/>
+      <c r="H156" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I156" s="32" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="J156" s="28" t="n"/>
+      <c r="K156" s="33" t="inlineStr">
+        <is>
+          <t>Parking Ladeuze, Louvain</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="E157" s="16" t="n"/>
+      <c r="F157" s="17" t="n"/>
+      <c r="G157" s="31" t="n"/>
+      <c r="H157" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I157" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="J157" s="28" t="n"/>
+      <c r="K157" s="33" t="inlineStr">
+        <is>
+          <t>Province du Brabant flamand, Kessel-Lo</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="E158" s="16" t="n"/>
+      <c r="F158" s="17" t="n"/>
+      <c r="G158" s="31" t="n"/>
+      <c r="H158" s="13" t="inlineStr">
+        <is>
+          <t>Paiement carte VISA</t>
+        </is>
+      </c>
+      <c r="I158" s="32" t="n">
+        <v>543.41</v>
+      </c>
+      <c r="J158" s="28" t="n"/>
+      <c r="K158" s="33" t="inlineStr">
+        <is>
+          <t>Décompte n° 152</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="E159" s="16" t="n"/>
+      <c r="F159" s="17" t="n"/>
+      <c r="G159" s="31" t="n"/>
+      <c r="H159" s="13" t="inlineStr">
+        <is>
+          <t>Telenet</t>
+        </is>
+      </c>
+      <c r="I159" s="32" t="n">
+        <v>155.52</v>
+      </c>
+      <c r="J159" s="28" t="n"/>
+      <c r="K159" s="33" t="n"/>
+    </row>
+    <row r="160">
+      <c r="E160" s="16" t="n"/>
+      <c r="F160" s="17" t="n"/>
+      <c r="G160" s="31" t="n"/>
+      <c r="H160" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I160" s="32" t="n">
+        <v>64.94</v>
+      </c>
+      <c r="J160" s="28" t="n"/>
+      <c r="K160" s="33" t="n"/>
+    </row>
+    <row r="161">
+      <c r="E161" s="16" t="n"/>
+      <c r="F161" s="17" t="n"/>
+      <c r="G161" s="31" t="n"/>
+      <c r="H161" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I161" s="32" t="n">
+        <v>68.06</v>
+      </c>
+      <c r="J161" s="28" t="n"/>
+      <c r="K161" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="E162" s="16" t="n"/>
+      <c r="F162" s="17" t="n"/>
+      <c r="G162" s="31" t="n"/>
+      <c r="H162" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I162" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="J162" s="28" t="n"/>
+      <c r="K162" s="33" t="inlineStr">
+        <is>
+          <t>Parking Grand-Place, Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="E163" s="16" t="n"/>
+      <c r="F163" s="17" t="n"/>
+      <c r="G163" s="31" t="n"/>
+      <c r="H163" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I163" s="32" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J163" s="28" t="n"/>
+      <c r="K163" s="33" t="inlineStr">
+        <is>
+          <t>Parkeren Sint-Gillis, Gand</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="E164" s="16" t="n"/>
+      <c r="F164" s="17" t="n"/>
+      <c r="G164" s="31" t="n"/>
+      <c r="H164" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I164" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="J164" s="28" t="n"/>
+      <c r="K164" s="33" t="inlineStr">
+        <is>
+          <t>Parking FP1, Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="E165" s="16" t="n"/>
+      <c r="F165" s="17" t="n"/>
+      <c r="G165" s="31" t="n"/>
+      <c r="H165" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I165" s="32" t="n">
+        <v>64.97</v>
+      </c>
+      <c r="J165" s="28" t="n"/>
+      <c r="K165" s="33" t="inlineStr">
+        <is>
+          <t>Lukoil Tournai</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="E166" s="16" t="n"/>
+      <c r="F166" s="17" t="n"/>
+      <c r="G166" s="31" t="n"/>
+      <c r="H166" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I166" s="32" t="n">
+        <v>256.99</v>
+      </c>
+      <c r="J166" s="28" t="n"/>
+      <c r="K166" s="33" t="inlineStr">
+        <is>
+          <t>Facture 450/5974/91764</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="E167" s="16" t="n"/>
+      <c r="F167" s="17" t="n"/>
+      <c r="G167" s="31" t="n"/>
+      <c r="H167" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I167" s="32" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J167" s="28" t="n"/>
+      <c r="K167" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="E168" s="16" t="n"/>
+      <c r="F168" s="17" t="n"/>
+      <c r="G168" s="31" t="n"/>
+      <c r="H168" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I168" s="32" t="n">
+        <v>54.33</v>
+      </c>
+      <c r="J168" s="28" t="n"/>
+      <c r="K168" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="E169" s="16" t="n"/>
+      <c r="F169" s="17" t="n"/>
+      <c r="G169" s="31" t="n"/>
+      <c r="H169" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I169" s="32" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J169" s="28" t="n"/>
+      <c r="K169" s="33" t="inlineStr">
+        <is>
+          <t>Parking Sint-Pieters, Gand</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="E170" s="16" t="n"/>
+      <c r="F170" s="17" t="n"/>
+      <c r="G170" s="31" t="n"/>
+      <c r="H170" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I170" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J170" s="28" t="n"/>
+      <c r="K170" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="G171" s="34" t="n"/>
+      <c r="I171" s="34" t="n"/>
+      <c r="K171" s="35" t="n"/>
+    </row>
+    <row r="172">
+      <c r="G172" s="34" t="n"/>
+      <c r="I172" s="34" t="n"/>
+      <c r="K172" s="35" t="n"/>
+    </row>
+    <row r="173">
+      <c r="G173" s="34">
+        <f>SUM(G6:G170)</f>
         <v/>
       </c>
-      <c r="I145" s="34">
-        <f>SUM(I6:I142)</f>
+      <c r="I173" s="34">
+        <f>SUM(I6:I170)</f>
         <v/>
       </c>
-      <c r="K145" s="35" t="n"/>
+      <c r="K173" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout de juillet
Extrait BNP Paribas Fortis n 2025-007 (operations 0174 a 0198, periode du
29-06 au 29-07).
2 entrees = 8.905,40 / 23 depenses = 5.266,63.
Rapprochement exact : 4.930,12 + 8.905,40 - 5.266,63 = 8.568,89.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K173"/>
+  <dimension ref="D1:K198"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -3733,15 +3733,450 @@
       <c r="K172" s="35" t="n"/>
     </row>
     <row r="173">
-      <c r="G173" s="34">
-        <f>SUM(G6:G170)</f>
+      <c r="E173" s="16" t="inlineStr">
+        <is>
+          <t>Juillet</t>
+        </is>
+      </c>
+      <c r="F173" s="17" t="inlineStr">
+        <is>
+          <t>Remboursement paiement à Sandaya</t>
+        </is>
+      </c>
+      <c r="G173" s="31" t="n">
+        <v>1775.4</v>
+      </c>
+      <c r="H173" s="28" t="inlineStr">
+        <is>
+          <t>Précompte salarial juin 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I173" s="36" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J173" s="28" t="n"/>
+      <c r="K173" s="33" t="n"/>
+    </row>
+    <row r="174">
+      <c r="E174" s="16" t="n"/>
+      <c r="F174" s="17" t="inlineStr">
+        <is>
+          <t>Prestations juillet 2025 - RTC Lambermont</t>
+        </is>
+      </c>
+      <c r="G174" s="31" t="n">
+        <v>7130</v>
+      </c>
+      <c r="H174" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I174" s="32" t="n">
+        <v>331.99</v>
+      </c>
+      <c r="J174" s="28" t="n"/>
+      <c r="K174" s="33" t="n"/>
+    </row>
+    <row r="175">
+      <c r="E175" s="16" t="n"/>
+      <c r="F175" s="17" t="n"/>
+      <c r="G175" s="31" t="n"/>
+      <c r="H175" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I175" s="32" t="n">
+        <v>84.91</v>
+      </c>
+      <c r="J175" s="28" t="n"/>
+      <c r="K175" s="33" t="n"/>
+    </row>
+    <row r="176">
+      <c r="E176" s="16" t="n"/>
+      <c r="F176" s="17" t="n"/>
+      <c r="G176" s="31" t="n"/>
+      <c r="H176" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I176" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J176" s="28" t="n"/>
+      <c r="K176" s="33" t="n"/>
+    </row>
+    <row r="177">
+      <c r="E177" s="16" t="n"/>
+      <c r="F177" s="17" t="n"/>
+      <c r="G177" s="31" t="n"/>
+      <c r="H177" s="13" t="inlineStr">
+        <is>
+          <t>Frais bancaires trimestriels</t>
+        </is>
+      </c>
+      <c r="I177" s="32" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="J177" s="28" t="n"/>
+      <c r="K177" s="33" t="n"/>
+    </row>
+    <row r="178">
+      <c r="E178" s="16" t="n"/>
+      <c r="F178" s="17" t="n"/>
+      <c r="G178" s="31" t="n"/>
+      <c r="H178" s="13" t="inlineStr">
+        <is>
+          <t>Intérêt crédit</t>
+        </is>
+      </c>
+      <c r="I178" s="32" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J178" s="28" t="n"/>
+      <c r="K178" s="33" t="inlineStr">
+        <is>
+          <t>Intérêts nets au 01-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="E179" s="16" t="n"/>
+      <c r="F179" s="17" t="n"/>
+      <c r="G179" s="31" t="n"/>
+      <c r="H179" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I179" s="32" t="n">
+        <v>60.86</v>
+      </c>
+      <c r="J179" s="28" t="n"/>
+      <c r="K179" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="E180" s="16" t="n"/>
+      <c r="F180" s="17" t="n"/>
+      <c r="G180" s="31" t="n"/>
+      <c r="H180" s="13" t="inlineStr">
+        <is>
+          <t>Assurance voiture</t>
+        </is>
+      </c>
+      <c r="I180" s="32" t="n">
+        <v>458.66</v>
+      </c>
+      <c r="J180" s="28" t="n"/>
+      <c r="K180" s="33" t="inlineStr">
+        <is>
+          <t>Domiciliation AG Insurance — prime passée de 431,25 à 458,66</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="E181" s="16" t="n"/>
+      <c r="F181" s="17" t="n"/>
+      <c r="G181" s="31" t="n"/>
+      <c r="H181" s="13" t="inlineStr">
+        <is>
+          <t>Paiement carte VISA</t>
+        </is>
+      </c>
+      <c r="I181" s="32" t="n">
+        <v>228.86</v>
+      </c>
+      <c r="J181" s="28" t="n"/>
+      <c r="K181" s="33" t="inlineStr">
+        <is>
+          <t>Décompte n° 182</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="E182" s="16" t="n"/>
+      <c r="F182" s="17" t="n"/>
+      <c r="G182" s="31" t="n"/>
+      <c r="H182" s="13" t="inlineStr">
+        <is>
+          <t>Terrain de tennis - Orée ASBL</t>
+        </is>
+      </c>
+      <c r="I182" s="32" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="J182" s="28" t="n"/>
+      <c r="K182" s="33" t="inlineStr">
+        <is>
+          <t>À confirmer (terrain ou consommation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="E183" s="16" t="n"/>
+      <c r="F183" s="17" t="n"/>
+      <c r="G183" s="31" t="n"/>
+      <c r="H183" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I183" s="32" t="n">
+        <v>56.98</v>
+      </c>
+      <c r="J183" s="28" t="n"/>
+      <c r="K183" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="E184" s="16" t="n"/>
+      <c r="F184" s="17" t="n"/>
+      <c r="G184" s="31" t="n"/>
+      <c r="H184" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I184" s="32" t="n">
+        <v>62.27</v>
+      </c>
+      <c r="J184" s="28" t="n"/>
+      <c r="K184" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="E185" s="16" t="n"/>
+      <c r="F185" s="17" t="n"/>
+      <c r="G185" s="31" t="n"/>
+      <c r="H185" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I185" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J185" s="28" t="n"/>
+      <c r="K185" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="E186" s="16" t="n"/>
+      <c r="F186" s="17" t="n"/>
+      <c r="G186" s="31" t="n"/>
+      <c r="H186" s="13" t="inlineStr">
+        <is>
+          <t>Péage autoroute France</t>
+        </is>
+      </c>
+      <c r="I186" s="32" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="J186" s="28" t="n"/>
+      <c r="K186" s="33" t="inlineStr">
+        <is>
+          <t>Domiciliation Autoroutes du Sud de la France</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="E187" s="16" t="n"/>
+      <c r="F187" s="17" t="n"/>
+      <c r="G187" s="31" t="n"/>
+      <c r="H187" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I187" s="32" t="n">
+        <v>356.79</v>
+      </c>
+      <c r="J187" s="28" t="n"/>
+      <c r="K187" s="33" t="inlineStr">
+        <is>
+          <t>Facture 455/1399/88731 — montant en hausse (256,99 les mois précédents)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="E188" s="16" t="n"/>
+      <c r="F188" s="17" t="n"/>
+      <c r="G188" s="31" t="n"/>
+      <c r="H188" s="13" t="inlineStr">
+        <is>
+          <t>Telenet</t>
+        </is>
+      </c>
+      <c r="I188" s="32" t="n">
+        <v>153.42</v>
+      </c>
+      <c r="J188" s="28" t="n"/>
+      <c r="K188" s="33" t="n"/>
+    </row>
+    <row r="189">
+      <c r="E189" s="16" t="n"/>
+      <c r="F189" s="17" t="n"/>
+      <c r="G189" s="31" t="n"/>
+      <c r="H189" s="13" t="inlineStr">
+        <is>
+          <t>Redevance de stationnement - Saint-Josse</t>
+        </is>
+      </c>
+      <c r="I189" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J189" s="28" t="n"/>
+      <c r="K189" s="33" t="inlineStr">
+        <is>
+          <t>Comm. 500/2300/37391 — à confirmer (redevance ou amende)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="E190" s="16" t="n"/>
+      <c r="F190" s="17" t="n"/>
+      <c r="G190" s="31" t="n"/>
+      <c r="H190" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I190" s="32" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="J190" s="28" t="n"/>
+      <c r="K190" s="33" t="inlineStr">
+        <is>
+          <t>Maes Schaerbeek</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="E191" s="16" t="n"/>
+      <c r="F191" s="17" t="n"/>
+      <c r="G191" s="31" t="n"/>
+      <c r="H191" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I191" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J191" s="28" t="n"/>
+      <c r="K191" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="E192" s="16" t="n"/>
+      <c r="F192" s="17" t="n"/>
+      <c r="G192" s="31" t="n"/>
+      <c r="H192" s="13" t="inlineStr">
+        <is>
+          <t>Repas Topogigio</t>
+        </is>
+      </c>
+      <c r="I192" s="32" t="n">
+        <v>231.5</v>
+      </c>
+      <c r="J192" s="28" t="n"/>
+      <c r="K192" s="33" t="n"/>
+    </row>
+    <row r="193">
+      <c r="E193" s="16" t="n"/>
+      <c r="F193" s="17" t="n"/>
+      <c r="G193" s="31" t="n"/>
+      <c r="H193" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I193" s="32" t="n">
+        <v>43.01</v>
+      </c>
+      <c r="J193" s="28" t="n"/>
+      <c r="K193" s="33" t="inlineStr">
+        <is>
+          <t>Esso Rumst</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="E194" s="16" t="n"/>
+      <c r="F194" s="17" t="n"/>
+      <c r="G194" s="31" t="n"/>
+      <c r="H194" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I194" s="32" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J194" s="28" t="n"/>
+      <c r="K194" s="33" t="inlineStr">
+        <is>
+          <t>Indigo, Tours (France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="E195" s="16" t="n"/>
+      <c r="F195" s="17" t="n"/>
+      <c r="G195" s="31" t="n"/>
+      <c r="H195" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I195" s="32" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J195" s="28" t="n"/>
+      <c r="K195" s="33" t="inlineStr">
+        <is>
+          <t>Commune de Soulac-sur-Mer (France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="G196" s="34" t="n"/>
+      <c r="I196" s="34" t="n"/>
+      <c r="K196" s="35" t="n"/>
+    </row>
+    <row r="197">
+      <c r="G197" s="34" t="n"/>
+      <c r="I197" s="34" t="n"/>
+      <c r="K197" s="35" t="n"/>
+    </row>
+    <row r="198">
+      <c r="G198" s="34">
+        <f>SUM(G6:G195)</f>
         <v/>
       </c>
-      <c r="I173" s="34">
-        <f>SUM(I6:I170)</f>
+      <c r="I198" s="34">
+        <f>SUM(I6:I195)</f>
         <v/>
       </c>
-      <c r="K173" s="35" t="n"/>
+      <c r="K198" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout d'aout
Extrait BNP Paribas Fortis n 2025-008 (operations 0199 a 0220, periode du
29-07 au 31-08).
1 entree = 123,00 / 21 depenses = 6.131,58.
Rapprochement exact : 8.568,89 + 123,00 - 6.131,58 = 2.560,31.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K198"/>
+  <dimension ref="D1:K221"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -4168,15 +4168,422 @@
       <c r="K197" s="35" t="n"/>
     </row>
     <row r="198">
-      <c r="G198" s="34">
-        <f>SUM(G6:G195)</f>
+      <c r="E198" s="16" t="inlineStr">
+        <is>
+          <t>Août</t>
+        </is>
+      </c>
+      <c r="F198" s="17" t="inlineStr">
+        <is>
+          <t>Remboursement achat Decathlon - RTC Lambermont</t>
+        </is>
+      </c>
+      <c r="G198" s="31" t="n">
+        <v>123</v>
+      </c>
+      <c r="H198" s="28" t="inlineStr">
+        <is>
+          <t>Précompte salarial juillet 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I198" s="36" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J198" s="28" t="n"/>
+      <c r="K198" s="33" t="n"/>
+    </row>
+    <row r="199">
+      <c r="E199" s="16" t="n"/>
+      <c r="F199" s="17" t="n"/>
+      <c r="G199" s="31" t="n"/>
+      <c r="H199" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I199" s="32" t="n">
+        <v>331.79</v>
+      </c>
+      <c r="J199" s="28" t="n"/>
+      <c r="K199" s="33" t="n"/>
+    </row>
+    <row r="200">
+      <c r="E200" s="16" t="n"/>
+      <c r="F200" s="17" t="n"/>
+      <c r="G200" s="31" t="n"/>
+      <c r="H200" s="13" t="inlineStr">
+        <is>
+          <t>Entretien voiture - Garage Gobinau</t>
+        </is>
+      </c>
+      <c r="I200" s="32" t="n">
+        <v>87.43000000000001</v>
+      </c>
+      <c r="J200" s="28" t="n"/>
+      <c r="K200" s="33" t="inlineStr">
+        <is>
+          <t>Soulac-sur-Mer (France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="E201" s="16" t="n"/>
+      <c r="F201" s="17" t="n"/>
+      <c r="G201" s="31" t="n"/>
+      <c r="H201" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I201" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J201" s="28" t="n"/>
+      <c r="K201" s="33" t="n"/>
+    </row>
+    <row r="202">
+      <c r="E202" s="16" t="n"/>
+      <c r="F202" s="17" t="n"/>
+      <c r="G202" s="31" t="n"/>
+      <c r="H202" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I202" s="32" t="n">
+        <v>72.01000000000001</v>
+      </c>
+      <c r="J202" s="28" t="n"/>
+      <c r="K202" s="33" t="inlineStr">
+        <is>
+          <t>BP Esso Saint-Léger (France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="E203" s="16" t="n"/>
+      <c r="F203" s="17" t="n"/>
+      <c r="G203" s="31" t="n"/>
+      <c r="H203" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I203" s="32" t="n">
+        <v>77.28</v>
+      </c>
+      <c r="J203" s="28" t="n"/>
+      <c r="K203" s="33" t="inlineStr">
+        <is>
+          <t>Shell Vémars (France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="E204" s="16" t="n"/>
+      <c r="F204" s="17" t="n"/>
+      <c r="G204" s="31" t="n"/>
+      <c r="H204" s="13" t="inlineStr">
+        <is>
+          <t>Achat matériel sportif - DECATHLON</t>
+        </is>
+      </c>
+      <c r="I204" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="J204" s="28" t="n"/>
+      <c r="K204" s="33" t="inlineStr">
+        <is>
+          <t>Decathlon Evere</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="E205" s="16" t="n"/>
+      <c r="F205" s="17" t="n"/>
+      <c r="G205" s="31" t="n"/>
+      <c r="H205" s="13" t="inlineStr">
+        <is>
+          <t>Paiement carte VISA</t>
+        </is>
+      </c>
+      <c r="I205" s="32" t="n">
+        <v>2134.71</v>
+      </c>
+      <c r="J205" s="28" t="n"/>
+      <c r="K205" s="33" t="inlineStr">
+        <is>
+          <t>Décompte n° 213</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="E206" s="16" t="n"/>
+      <c r="F206" s="17" t="n"/>
+      <c r="G206" s="31" t="n"/>
+      <c r="H206" s="13" t="inlineStr">
+        <is>
+          <t>Paiement carte MASTERCARD</t>
+        </is>
+      </c>
+      <c r="I206" s="32" t="n">
+        <v>66.73999999999999</v>
+      </c>
+      <c r="J206" s="28" t="n"/>
+      <c r="K206" s="33" t="inlineStr">
+        <is>
+          <t>Décompte n° 216 - nouveau compte carte 80845055</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="E207" s="16" t="n"/>
+      <c r="F207" s="17" t="n"/>
+      <c r="G207" s="31" t="n"/>
+      <c r="H207" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I207" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J207" s="28" t="n"/>
+      <c r="K207" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="E208" s="16" t="n"/>
+      <c r="F208" s="17" t="n"/>
+      <c r="G208" s="31" t="n"/>
+      <c r="H208" s="13" t="inlineStr">
+        <is>
+          <t>Achat matériel sportif - DECATHLON</t>
+        </is>
+      </c>
+      <c r="I208" s="32" t="n">
+        <v>123</v>
+      </c>
+      <c r="J208" s="28" t="n"/>
+      <c r="K208" s="33" t="inlineStr">
+        <is>
+          <t>Decathlon Evere - remboursé par le RTC Lambermont le même jour</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="E209" s="16" t="n"/>
+      <c r="F209" s="17" t="n"/>
+      <c r="G209" s="31" t="n"/>
+      <c r="H209" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I209" s="32" t="n">
+        <v>62.86</v>
+      </c>
+      <c r="J209" s="28" t="n"/>
+      <c r="K209" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="E210" s="16" t="n"/>
+      <c r="F210" s="17" t="n"/>
+      <c r="G210" s="31" t="n"/>
+      <c r="H210" s="13" t="inlineStr">
+        <is>
+          <t>Péage autoroute France</t>
+        </is>
+      </c>
+      <c r="I210" s="32" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="J210" s="28" t="n"/>
+      <c r="K210" s="33" t="inlineStr">
+        <is>
+          <t>Domiciliation Autoroutes du Sud de la France</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="E211" s="16" t="n"/>
+      <c r="F211" s="17" t="n"/>
+      <c r="G211" s="31" t="n"/>
+      <c r="H211" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I211" s="32" t="n">
+        <v>72.59</v>
+      </c>
+      <c r="J211" s="28" t="n"/>
+      <c r="K211" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="E212" s="16" t="n"/>
+      <c r="F212" s="17" t="n"/>
+      <c r="G212" s="31" t="n"/>
+      <c r="H212" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I212" s="32" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="J212" s="28" t="n"/>
+      <c r="K212" s="33" t="inlineStr">
+        <is>
+          <t>Parking Parkpoort, Heverlee</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="E213" s="16" t="n"/>
+      <c r="F213" s="17" t="n"/>
+      <c r="G213" s="31" t="n"/>
+      <c r="H213" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I213" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J213" s="28" t="n"/>
+      <c r="K213" s="33" t="inlineStr">
+        <is>
+          <t>Parking Ladeuze, Louvain</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="E214" s="16" t="n"/>
+      <c r="F214" s="17" t="n"/>
+      <c r="G214" s="31" t="n"/>
+      <c r="H214" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I214" s="32" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J214" s="28" t="n"/>
+      <c r="K214" s="33" t="inlineStr">
+        <is>
+          <t>Indigo Park Docks, Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="E215" s="16" t="n"/>
+      <c r="F215" s="17" t="n"/>
+      <c r="G215" s="31" t="n"/>
+      <c r="H215" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I215" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="J215" s="28" t="n"/>
+      <c r="K215" s="33" t="inlineStr">
+        <is>
+          <t>Parking Bokrijk, Genk</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="E216" s="16" t="n"/>
+      <c r="F216" s="17" t="n"/>
+      <c r="G216" s="31" t="n"/>
+      <c r="H216" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I216" s="32" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="J216" s="28" t="n"/>
+      <c r="K216" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="E217" s="16" t="n"/>
+      <c r="F217" s="17" t="n"/>
+      <c r="G217" s="31" t="n"/>
+      <c r="H217" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I217" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="J217" s="28" t="n"/>
+      <c r="K217" s="33" t="inlineStr">
+        <is>
+          <t>Brussels Expo — à confirmer (parking ou entrée)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="E218" s="16" t="n"/>
+      <c r="F218" s="17" t="n"/>
+      <c r="G218" s="31" t="n"/>
+      <c r="H218" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I218" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J218" s="28" t="n"/>
+      <c r="K218" s="33" t="inlineStr">
+        <is>
+          <t>Parking Grand-Place, Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="G219" s="34" t="n"/>
+      <c r="I219" s="34" t="n"/>
+      <c r="K219" s="35" t="n"/>
+    </row>
+    <row r="220">
+      <c r="G220" s="34" t="n"/>
+      <c r="I220" s="34" t="n"/>
+      <c r="K220" s="35" t="n"/>
+    </row>
+    <row r="221">
+      <c r="G221" s="34">
+        <f>SUM(G6:G218)</f>
         <v/>
       </c>
-      <c r="I198" s="34">
-        <f>SUM(I6:I195)</f>
+      <c r="I221" s="34">
+        <f>SUM(I6:I218)</f>
         <v/>
       </c>
-      <c r="K198" s="35" t="n"/>
+      <c r="K221" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout de septembre
Extrait BNP Paribas Fortis n 2025-009 (operations 0221 a 0247, periode du
31-08 au 27-09).
1 entree = 5.501,95 / 26 depenses = 7.031,16.
Rapprochement exact : 2.560,31 + 5.501,95 - 7.031,16 = 1.031,10.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K221"/>
+  <dimension ref="D1:K249"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -4575,15 +4575,501 @@
       <c r="K220" s="35" t="n"/>
     </row>
     <row r="221">
-      <c r="G221" s="34">
-        <f>SUM(G6:G218)</f>
+      <c r="E221" s="16" t="inlineStr">
+        <is>
+          <t>Septembre</t>
+        </is>
+      </c>
+      <c r="F221" s="17" t="inlineStr">
+        <is>
+          <t>LAM2510</t>
+        </is>
+      </c>
+      <c r="G221" s="31" t="n">
+        <v>5501.95</v>
+      </c>
+      <c r="H221" s="28" t="inlineStr">
+        <is>
+          <t>Partena</t>
+        </is>
+      </c>
+      <c r="I221" s="36" t="n">
+        <v>1441.87</v>
+      </c>
+      <c r="J221" s="28" t="n"/>
+      <c r="K221" s="33" t="n"/>
+    </row>
+    <row r="222">
+      <c r="E222" s="16" t="n"/>
+      <c r="F222" s="17" t="n"/>
+      <c r="G222" s="31" t="n"/>
+      <c r="H222" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I222" s="32" t="n">
+        <v>263.44</v>
+      </c>
+      <c r="J222" s="28" t="n"/>
+      <c r="K222" s="33" t="inlineStr">
+        <is>
+          <t>Facture 412/3802/96359</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="E223" s="16" t="n"/>
+      <c r="F223" s="17" t="n"/>
+      <c r="G223" s="31" t="n"/>
+      <c r="H223" s="13" t="inlineStr">
+        <is>
+          <t>Telenet</t>
+        </is>
+      </c>
+      <c r="I223" s="32" t="n">
+        <v>153.42</v>
+      </c>
+      <c r="J223" s="28" t="n"/>
+      <c r="K223" s="33" t="n"/>
+    </row>
+    <row r="224">
+      <c r="E224" s="16" t="n"/>
+      <c r="F224" s="17" t="n"/>
+      <c r="G224" s="31" t="n"/>
+      <c r="H224" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I224" s="32" t="n">
+        <v>65.14</v>
+      </c>
+      <c r="J224" s="28" t="n"/>
+      <c r="K224" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Tervuren</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="E225" s="16" t="n"/>
+      <c r="F225" s="17" t="n"/>
+      <c r="G225" s="31" t="n"/>
+      <c r="H225" s="13" t="inlineStr">
+        <is>
+          <t>Précompte salarial août 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I225" s="32" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J225" s="28" t="n"/>
+      <c r="K225" s="33" t="n"/>
+    </row>
+    <row r="226">
+      <c r="E226" s="16" t="n"/>
+      <c r="F226" s="17" t="n"/>
+      <c r="G226" s="31" t="n"/>
+      <c r="H226" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I226" s="32" t="n">
+        <v>331.79</v>
+      </c>
+      <c r="J226" s="28" t="n"/>
+      <c r="K226" s="33" t="n"/>
+    </row>
+    <row r="227">
+      <c r="E227" s="16" t="n"/>
+      <c r="F227" s="17" t="n"/>
+      <c r="G227" s="31" t="n"/>
+      <c r="H227" s="13" t="inlineStr">
+        <is>
+          <t>Farys (eau)</t>
+        </is>
+      </c>
+      <c r="I227" s="32" t="n">
+        <v>300</v>
+      </c>
+      <c r="J227" s="28" t="n"/>
+      <c r="K227" s="33" t="n"/>
+    </row>
+    <row r="228">
+      <c r="E228" s="16" t="n"/>
+      <c r="F228" s="17" t="n"/>
+      <c r="G228" s="31" t="n"/>
+      <c r="H228" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I228" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J228" s="28" t="n"/>
+      <c r="K228" s="33" t="n"/>
+    </row>
+    <row r="229">
+      <c r="E229" s="16" t="n"/>
+      <c r="F229" s="17" t="n"/>
+      <c r="G229" s="31" t="n"/>
+      <c r="H229" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I229" s="32" t="n">
+        <v>70.62</v>
+      </c>
+      <c r="J229" s="28" t="n"/>
+      <c r="K229" s="33" t="n"/>
+    </row>
+    <row r="230">
+      <c r="E230" s="16" t="n"/>
+      <c r="F230" s="17" t="n"/>
+      <c r="G230" s="31" t="n"/>
+      <c r="H230" s="13" t="inlineStr">
+        <is>
+          <t>Vlaamse Belastingsdienst - taxe de circulation</t>
+        </is>
+      </c>
+      <c r="I230" s="32" t="n">
+        <v>161.02</v>
+      </c>
+      <c r="J230" s="28" t="n"/>
+      <c r="K230" s="33" t="inlineStr">
+        <is>
+          <t>Comm. 255/2756/05470</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="E231" s="16" t="n"/>
+      <c r="F231" s="17" t="n"/>
+      <c r="G231" s="31" t="n"/>
+      <c r="H231" s="13" t="inlineStr">
+        <is>
+          <t>Paiement carte VISA</t>
+        </is>
+      </c>
+      <c r="I231" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J231" s="28" t="n"/>
+      <c r="K231" s="33" t="inlineStr">
+        <is>
+          <t>Décompte n° 244</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="E232" s="16" t="n"/>
+      <c r="F232" s="17" t="n"/>
+      <c r="G232" s="31" t="n"/>
+      <c r="H232" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I232" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J232" s="28" t="n"/>
+      <c r="K232" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="E233" s="16" t="n"/>
+      <c r="F233" s="17" t="n"/>
+      <c r="G233" s="31" t="n"/>
+      <c r="H233" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I233" s="32" t="n">
+        <v>66.73999999999999</v>
+      </c>
+      <c r="J233" s="28" t="n"/>
+      <c r="K233" s="33" t="inlineStr">
+        <is>
+          <t>Shell Kraainem</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="E234" s="16" t="n"/>
+      <c r="F234" s="17" t="n"/>
+      <c r="G234" s="31" t="n"/>
+      <c r="H234" s="13" t="inlineStr">
+        <is>
+          <t>Repas Lunch Garden</t>
+        </is>
+      </c>
+      <c r="I234" s="32" t="n">
+        <v>45.77</v>
+      </c>
+      <c r="J234" s="28" t="n"/>
+      <c r="K234" s="33" t="inlineStr">
+        <is>
+          <t>Lunch Garden Kraainem</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="E235" s="16" t="n"/>
+      <c r="F235" s="17" t="n"/>
+      <c r="G235" s="31" t="n"/>
+      <c r="H235" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I235" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J235" s="28" t="n"/>
+      <c r="K235" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="E236" s="16" t="n"/>
+      <c r="F236" s="17" t="n"/>
+      <c r="G236" s="31" t="n"/>
+      <c r="H236" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I236" s="32" t="n">
+        <v>161.83</v>
+      </c>
+      <c r="J236" s="28" t="n"/>
+      <c r="K236" s="33" t="inlineStr">
+        <is>
+          <t>2e facture du mois</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="E237" s="16" t="n"/>
+      <c r="F237" s="17" t="n"/>
+      <c r="G237" s="31" t="n"/>
+      <c r="H237" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I237" s="32" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J237" s="28" t="n"/>
+      <c r="K237" s="33" t="inlineStr">
+        <is>
+          <t>Schaerbeek</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="E238" s="16" t="n"/>
+      <c r="F238" s="17" t="n"/>
+      <c r="G238" s="31" t="n"/>
+      <c r="H238" s="13" t="inlineStr">
+        <is>
+          <t>Péage autoroute France</t>
+        </is>
+      </c>
+      <c r="I238" s="32" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="J238" s="28" t="n"/>
+      <c r="K238" s="33" t="inlineStr">
+        <is>
+          <t>Domiciliation Autoroutes du Sud de la France</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="E239" s="16" t="n"/>
+      <c r="F239" s="17" t="n"/>
+      <c r="G239" s="31" t="n"/>
+      <c r="H239" s="13" t="inlineStr">
+        <is>
+          <t>Repas Exki</t>
+        </is>
+      </c>
+      <c r="I239" s="32" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="J239" s="28" t="n"/>
+      <c r="K239" s="33" t="inlineStr">
+        <is>
+          <t>Exki Woluwe</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="E240" s="16" t="n"/>
+      <c r="F240" s="17" t="n"/>
+      <c r="G240" s="31" t="n"/>
+      <c r="H240" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I240" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J240" s="28" t="n"/>
+      <c r="K240" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="E241" s="16" t="n"/>
+      <c r="F241" s="17" t="n"/>
+      <c r="G241" s="31" t="n"/>
+      <c r="H241" s="13" t="inlineStr">
+        <is>
+          <t>Formation Indigo Nails Lab Belgium</t>
+        </is>
+      </c>
+      <c r="I241" s="32" t="n">
+        <v>630</v>
+      </c>
+      <c r="J241" s="28" t="n"/>
+      <c r="K241" s="33" t="inlineStr">
+        <is>
+          <t>Facture FA002548 avancée par T. Duchène et remboursée par la société</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="E242" s="16" t="n"/>
+      <c r="F242" s="17" t="n"/>
+      <c r="G242" s="31" t="n"/>
+      <c r="H242" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I242" s="32" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="J242" s="28" t="n"/>
+      <c r="K242" s="33" t="inlineStr">
+        <is>
+          <t>Shell Kraainem</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="E243" s="16" t="n"/>
+      <c r="F243" s="17" t="n"/>
+      <c r="G243" s="31" t="n"/>
+      <c r="H243" s="13" t="inlineStr">
+        <is>
+          <t>Repas - Chez Ji SPRL</t>
+        </is>
+      </c>
+      <c r="I243" s="32" t="n">
+        <v>47</v>
+      </c>
+      <c r="J243" s="28" t="n"/>
+      <c r="K243" s="33" t="inlineStr">
+        <is>
+          <t>Péruwelz</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="E244" s="16" t="n"/>
+      <c r="F244" s="17" t="n"/>
+      <c r="G244" s="31" t="n"/>
+      <c r="H244" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I244" s="32" t="n">
+        <v>58.45</v>
+      </c>
+      <c r="J244" s="28" t="n"/>
+      <c r="K244" s="33" t="inlineStr">
+        <is>
+          <t>Esso Péruwelz</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="E245" s="16" t="n"/>
+      <c r="F245" s="17" t="n"/>
+      <c r="G245" s="31" t="n"/>
+      <c r="H245" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I245" s="32" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="J245" s="28" t="n"/>
+      <c r="K245" s="33" t="inlineStr">
+        <is>
+          <t>Total Nivelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="E246" s="16" t="n"/>
+      <c r="F246" s="17" t="n"/>
+      <c r="G246" s="31" t="n"/>
+      <c r="H246" s="13" t="inlineStr">
+        <is>
+          <t>Achat - NEW BS SPRL</t>
+        </is>
+      </c>
+      <c r="I246" s="32" t="n">
+        <v>40</v>
+      </c>
+      <c r="J246" s="28" t="n"/>
+      <c r="K246" s="33" t="inlineStr">
+        <is>
+          <t>Bruxelles — même commerçant qu'en mars (290,50) à identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="G247" s="34" t="n"/>
+      <c r="I247" s="34" t="n"/>
+      <c r="K247" s="35" t="n"/>
+    </row>
+    <row r="248">
+      <c r="G248" s="34" t="n"/>
+      <c r="I248" s="34" t="n"/>
+      <c r="K248" s="35" t="n"/>
+    </row>
+    <row r="249">
+      <c r="G249" s="34">
+        <f>SUM(G6:G246)</f>
         <v/>
       </c>
-      <c r="I221" s="34">
-        <f>SUM(I6:I218)</f>
+      <c r="I249" s="34">
+        <f>SUM(I6:I246)</f>
         <v/>
       </c>
-      <c r="K221" s="35" t="n"/>
+      <c r="K249" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout d'octobre
Extrait BNP Paribas Fortis n 2025-010 (operations 0248 a 0280, periode du
27-09 au 29-10).
3 entrees = 22.377,81 / 30 depenses = 12.450,12.
Rapprochement exact : 1.031,10 + 22.377,81 - 12.450,12 = 10.958,79.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K249"/>
+  <dimension ref="D1:K281"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -5061,15 +5061,585 @@
       <c r="K248" s="35" t="n"/>
     </row>
     <row r="249">
-      <c r="G249" s="34">
-        <f>SUM(G6:G246)</f>
+      <c r="E249" s="16" t="inlineStr">
+        <is>
+          <t>Octobre</t>
+        </is>
+      </c>
+      <c r="F249" s="17" t="inlineStr">
+        <is>
+          <t>LAM2511</t>
+        </is>
+      </c>
+      <c r="G249" s="31" t="n">
+        <v>3858.09</v>
+      </c>
+      <c r="H249" s="28" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I249" s="36" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J249" s="28" t="n"/>
+      <c r="K249" s="33" t="n"/>
+    </row>
+    <row r="250">
+      <c r="E250" s="16" t="n"/>
+      <c r="F250" s="17" t="inlineStr">
+        <is>
+          <t>LAM2512</t>
+        </is>
+      </c>
+      <c r="G250" s="31" t="n">
+        <v>13994</v>
+      </c>
+      <c r="H250" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I250" s="32" t="n">
+        <v>68.23</v>
+      </c>
+      <c r="J250" s="28" t="n"/>
+      <c r="K250" s="33" t="inlineStr">
+        <is>
+          <t>Total Hoegaarden</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="E251" s="16" t="n"/>
+      <c r="F251" s="17" t="inlineStr">
+        <is>
+          <t>Prestations octobre 2025 - RTC Lambermont</t>
+        </is>
+      </c>
+      <c r="G251" s="31" t="n">
+        <v>4525.72</v>
+      </c>
+      <c r="H251" s="13" t="inlineStr">
+        <is>
+          <t>Précompte salarial septembre 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I251" s="32" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J251" s="28" t="n"/>
+      <c r="K251" s="33" t="n"/>
+    </row>
+    <row r="252">
+      <c r="E252" s="16" t="n"/>
+      <c r="F252" s="17" t="n"/>
+      <c r="G252" s="31" t="n"/>
+      <c r="H252" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I252" s="32" t="n">
+        <v>331.79</v>
+      </c>
+      <c r="J252" s="28" t="n"/>
+      <c r="K252" s="33" t="n"/>
+    </row>
+    <row r="253">
+      <c r="E253" s="16" t="n"/>
+      <c r="F253" s="17" t="n"/>
+      <c r="G253" s="31" t="n"/>
+      <c r="H253" s="13" t="inlineStr">
+        <is>
+          <t>Farys (eau)</t>
+        </is>
+      </c>
+      <c r="I253" s="32" t="n">
+        <v>172.14</v>
+      </c>
+      <c r="J253" s="28" t="n"/>
+      <c r="K253" s="33" t="n"/>
+    </row>
+    <row r="254">
+      <c r="E254" s="16" t="n"/>
+      <c r="F254" s="17" t="n"/>
+      <c r="G254" s="31" t="n"/>
+      <c r="H254" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I254" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="J254" s="28" t="n"/>
+      <c r="K254" s="33" t="inlineStr">
+        <is>
+          <t>Parking 't Centrum, Valkenburg (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="E255" s="16" t="n"/>
+      <c r="F255" s="17" t="n"/>
+      <c r="G255" s="31" t="n"/>
+      <c r="H255" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I255" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="J255" s="28" t="n"/>
+      <c r="K255" s="33" t="inlineStr">
+        <is>
+          <t>Valkenburg (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="E256" s="16" t="n"/>
+      <c r="F256" s="17" t="n"/>
+      <c r="G256" s="31" t="n"/>
+      <c r="H256" s="13" t="inlineStr">
+        <is>
+          <t>Frais bancaires trimestriels</t>
+        </is>
+      </c>
+      <c r="I256" s="32" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="J256" s="28" t="n"/>
+      <c r="K256" s="33" t="n"/>
+    </row>
+    <row r="257">
+      <c r="E257" s="16" t="n"/>
+      <c r="F257" s="17" t="n"/>
+      <c r="G257" s="31" t="n"/>
+      <c r="H257" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I257" s="32" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J257" s="28" t="n"/>
+      <c r="K257" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="E258" s="16" t="n"/>
+      <c r="F258" s="17" t="n"/>
+      <c r="G258" s="31" t="n"/>
+      <c r="H258" s="13" t="inlineStr">
+        <is>
+          <t>Assurance voiture</t>
+        </is>
+      </c>
+      <c r="I258" s="32" t="n">
+        <v>458.66</v>
+      </c>
+      <c r="J258" s="28" t="n"/>
+      <c r="K258" s="33" t="inlineStr">
+        <is>
+          <t>Paiement par domiciliation (AG Insurance)</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="E259" s="16" t="n"/>
+      <c r="F259" s="17" t="n"/>
+      <c r="G259" s="31" t="n"/>
+      <c r="H259" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I259" s="32" t="n">
+        <v>263.44</v>
+      </c>
+      <c r="J259" s="28" t="n"/>
+      <c r="K259" s="33" t="inlineStr">
+        <is>
+          <t>Facture 495/0336/32914</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="E260" s="16" t="n"/>
+      <c r="F260" s="17" t="n"/>
+      <c r="G260" s="31" t="n"/>
+      <c r="H260" s="13" t="inlineStr">
+        <is>
+          <t>Réception marchandise - FEDEX</t>
+        </is>
+      </c>
+      <c r="I260" s="32" t="n">
+        <v>17.37</v>
+      </c>
+      <c r="J260" s="28" t="n"/>
+      <c r="K260" s="33" t="n"/>
+    </row>
+    <row r="261">
+      <c r="E261" s="16" t="n"/>
+      <c r="F261" s="17" t="n"/>
+      <c r="G261" s="31" t="n"/>
+      <c r="H261" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I261" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="J261" s="28" t="n"/>
+      <c r="K261" s="33" t="inlineStr">
+        <is>
+          <t>Parking FP1, Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="E262" s="16" t="n"/>
+      <c r="F262" s="17" t="n"/>
+      <c r="G262" s="31" t="n"/>
+      <c r="H262" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I262" s="32" t="n">
+        <v>64.26000000000001</v>
+      </c>
+      <c r="J262" s="28" t="n"/>
+      <c r="K262" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="E263" s="16" t="n"/>
+      <c r="F263" s="17" t="n"/>
+      <c r="G263" s="31" t="n"/>
+      <c r="H263" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I263" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J263" s="28" t="n"/>
+      <c r="K263" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="E264" s="16" t="n"/>
+      <c r="F264" s="17" t="n"/>
+      <c r="G264" s="31" t="n"/>
+      <c r="H264" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I264" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="J264" s="28" t="n"/>
+      <c r="K264" s="33" t="inlineStr">
+        <is>
+          <t>Brussels Expo — à confirmer (parking ou entrée)</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="E265" s="16" t="n"/>
+      <c r="F265" s="17" t="n"/>
+      <c r="G265" s="31" t="n"/>
+      <c r="H265" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I265" s="32" t="n">
+        <v>67.14</v>
+      </c>
+      <c r="J265" s="28" t="n"/>
+      <c r="K265" s="33" t="inlineStr">
+        <is>
+          <t>Total Rumst</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="E266" s="16" t="n"/>
+      <c r="F266" s="17" t="n"/>
+      <c r="G266" s="31" t="n"/>
+      <c r="H266" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I266" s="32" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="J266" s="28" t="n"/>
+      <c r="K266" s="33" t="inlineStr">
+        <is>
+          <t>Parking De Vooruitgang, Volendam (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="E267" s="16" t="n"/>
+      <c r="F267" s="17" t="n"/>
+      <c r="G267" s="31" t="n"/>
+      <c r="H267" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I267" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J267" s="28" t="n"/>
+      <c r="K267" s="33" t="inlineStr">
+        <is>
+          <t>Zaanstad (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="E268" s="16" t="n"/>
+      <c r="F268" s="17" t="n"/>
+      <c r="G268" s="31" t="n"/>
+      <c r="H268" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I268" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J268" s="28" t="n"/>
+      <c r="K268" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Rozenhof, Zaandam (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="E269" s="16" t="n"/>
+      <c r="F269" s="17" t="n"/>
+      <c r="G269" s="31" t="n"/>
+      <c r="H269" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I269" s="32" t="n">
+        <v>81.39</v>
+      </c>
+      <c r="J269" s="28" t="n"/>
+      <c r="K269" s="33" t="inlineStr">
+        <is>
+          <t>Esso Dorst (Pays-Bas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="E270" s="16" t="n"/>
+      <c r="F270" s="17" t="n"/>
+      <c r="G270" s="31" t="n"/>
+      <c r="H270" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I270" s="32" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="J270" s="28" t="n"/>
+      <c r="K270" s="33" t="inlineStr">
+        <is>
+          <t>Parking Ladeuze, Louvain</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="E271" s="16" t="n"/>
+      <c r="F271" s="17" t="n"/>
+      <c r="G271" s="31" t="n"/>
+      <c r="H271" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I271" s="32" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J271" s="28" t="n"/>
+      <c r="K271" s="33" t="inlineStr">
+        <is>
+          <t>Commune Saint-Josse</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="E272" s="16" t="n"/>
+      <c r="F272" s="17" t="n"/>
+      <c r="G272" s="31" t="n"/>
+      <c r="H272" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I272" s="32" t="n">
+        <v>70.66</v>
+      </c>
+      <c r="J272" s="28" t="n"/>
+      <c r="K272" s="33" t="inlineStr">
+        <is>
+          <t>Shell Kraainem</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="E273" s="16" t="n"/>
+      <c r="F273" s="17" t="n"/>
+      <c r="G273" s="31" t="n"/>
+      <c r="H273" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I273" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="J273" s="28" t="n"/>
+      <c r="K273" s="33" t="inlineStr">
+        <is>
+          <t>Parking Bokrijk, Genk</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="E274" s="16" t="n"/>
+      <c r="F274" s="17" t="n"/>
+      <c r="G274" s="31" t="n"/>
+      <c r="H274" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I274" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J274" s="28" t="n"/>
+      <c r="K274" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="E275" s="16" t="n"/>
+      <c r="F275" s="17" t="n"/>
+      <c r="G275" s="31" t="n"/>
+      <c r="H275" s="13" t="inlineStr">
+        <is>
+          <t>Versement impôts anticipé</t>
+        </is>
+      </c>
+      <c r="I275" s="32" t="n">
+        <v>5500</v>
+      </c>
+      <c r="J275" s="28" t="n"/>
+      <c r="K275" s="33" t="inlineStr">
+        <is>
+          <t>Comm. 073/4616/33527</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="E276" s="16" t="n"/>
+      <c r="F276" s="17" t="n"/>
+      <c r="G276" s="31" t="n"/>
+      <c r="H276" s="13" t="inlineStr">
+        <is>
+          <t>Précompte mobilier</t>
+        </is>
+      </c>
+      <c r="I276" s="32" t="n">
+        <v>2100</v>
+      </c>
+      <c r="J276" s="28" t="n"/>
+      <c r="K276" s="33" t="inlineStr">
+        <is>
+          <t>Comm. 204/0596/50233 — lié à une distribution de dividendes ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="E277" s="16" t="n"/>
+      <c r="F277" s="17" t="n"/>
+      <c r="G277" s="31" t="n"/>
+      <c r="H277" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I277" s="32" t="n">
+        <v>148.72</v>
+      </c>
+      <c r="J277" s="28" t="n"/>
+      <c r="K277" s="33" t="n"/>
+    </row>
+    <row r="278">
+      <c r="E278" s="16" t="n"/>
+      <c r="F278" s="17" t="n"/>
+      <c r="G278" s="31" t="n"/>
+      <c r="H278" s="13" t="inlineStr">
+        <is>
+          <t>Consommation Lambermont</t>
+        </is>
+      </c>
+      <c r="I278" s="32" t="n">
+        <v>58</v>
+      </c>
+      <c r="J278" s="28" t="n"/>
+      <c r="K278" s="33" t="n"/>
+    </row>
+    <row r="279">
+      <c r="G279" s="34" t="n"/>
+      <c r="I279" s="34" t="n"/>
+      <c r="K279" s="35" t="n"/>
+    </row>
+    <row r="280">
+      <c r="G280" s="34" t="n"/>
+      <c r="I280" s="34" t="n"/>
+      <c r="K280" s="35" t="n"/>
+    </row>
+    <row r="281">
+      <c r="G281" s="34">
+        <f>SUM(G6:G278)</f>
         <v/>
       </c>
-      <c r="I249" s="34">
-        <f>SUM(I6:I246)</f>
+      <c r="I281" s="34">
+        <f>SUM(I6:I278)</f>
         <v/>
       </c>
-      <c r="K249" s="35" t="n"/>
+      <c r="K281" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout de novembre
Extrait BNP Paribas Fortis n 2025-011 (operations 0281 a 0306, periode du
29-10 au 30-11). Aucun encaissement ce mois-ci.
0 entree / 26 depenses = 6.986,96.
Rapprochement exact : 10.958,79 - 6.986,96 = 3.971,83.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K281"/>
+  <dimension ref="D1:K309"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -5631,15 +5631,503 @@
       <c r="K280" s="35" t="n"/>
     </row>
     <row r="281">
-      <c r="G281" s="34">
-        <f>SUM(G6:G278)</f>
+      <c r="E281" s="16" t="inlineStr">
+        <is>
+          <t>Novembre</t>
+        </is>
+      </c>
+      <c r="F281" s="17" t="n"/>
+      <c r="G281" s="31" t="n"/>
+      <c r="H281" s="28" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I281" s="36" t="n">
+        <v>65.29000000000001</v>
+      </c>
+      <c r="J281" s="28" t="n"/>
+      <c r="K281" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="E282" s="16" t="n"/>
+      <c r="F282" s="17" t="n"/>
+      <c r="G282" s="31" t="n"/>
+      <c r="H282" s="13" t="inlineStr">
+        <is>
+          <t>Achat - Media Markt</t>
+        </is>
+      </c>
+      <c r="I282" s="32" t="n">
+        <v>748</v>
+      </c>
+      <c r="J282" s="28" t="n"/>
+      <c r="K282" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert — nature de l'achat à préciser</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="E283" s="16" t="n"/>
+      <c r="F283" s="17" t="n"/>
+      <c r="G283" s="31" t="n"/>
+      <c r="H283" s="13" t="inlineStr">
+        <is>
+          <t>Achat - Media Markt</t>
+        </is>
+      </c>
+      <c r="I283" s="32" t="n">
+        <v>39</v>
+      </c>
+      <c r="J283" s="28" t="n"/>
+      <c r="K283" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert — nature de l'achat à préciser</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="E284" s="16" t="n"/>
+      <c r="F284" s="17" t="n"/>
+      <c r="G284" s="31" t="n"/>
+      <c r="H284" s="13" t="inlineStr">
+        <is>
+          <t>Précompte salarial octobre 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I284" s="32" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J284" s="28" t="n"/>
+      <c r="K284" s="33" t="n"/>
+    </row>
+    <row r="285">
+      <c r="E285" s="16" t="n"/>
+      <c r="F285" s="17" t="n"/>
+      <c r="G285" s="31" t="n"/>
+      <c r="H285" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I285" s="32" t="n">
+        <v>331.85</v>
+      </c>
+      <c r="J285" s="28" t="n"/>
+      <c r="K285" s="33" t="n"/>
+    </row>
+    <row r="286">
+      <c r="E286" s="16" t="n"/>
+      <c r="F286" s="17" t="n"/>
+      <c r="G286" s="31" t="n"/>
+      <c r="H286" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I286" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J286" s="28" t="n"/>
+      <c r="K286" s="33" t="n"/>
+    </row>
+    <row r="287">
+      <c r="E287" s="16" t="n"/>
+      <c r="F287" s="17" t="n"/>
+      <c r="G287" s="31" t="n"/>
+      <c r="H287" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I287" s="32" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="J287" s="28" t="n"/>
+      <c r="K287" s="33" t="inlineStr">
+        <is>
+          <t>Commune Saint-Josse</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="E288" s="16" t="n"/>
+      <c r="F288" s="17" t="n"/>
+      <c r="G288" s="31" t="n"/>
+      <c r="H288" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I288" s="32" t="n">
+        <v>70.44</v>
+      </c>
+      <c r="J288" s="28" t="n"/>
+      <c r="K288" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Tervuren</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="E289" s="16" t="n"/>
+      <c r="F289" s="17" t="n"/>
+      <c r="G289" s="31" t="n"/>
+      <c r="H289" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I289" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J289" s="28" t="n"/>
+      <c r="K289" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="E290" s="16" t="n"/>
+      <c r="F290" s="17" t="n"/>
+      <c r="G290" s="31" t="n"/>
+      <c r="H290" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I290" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J290" s="28" t="n"/>
+      <c r="K290" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="E291" s="16" t="n"/>
+      <c r="F291" s="17" t="n"/>
+      <c r="G291" s="31" t="n"/>
+      <c r="H291" s="13" t="inlineStr">
+        <is>
+          <t>Partena</t>
+        </is>
+      </c>
+      <c r="I291" s="32" t="n">
+        <v>1441.87</v>
+      </c>
+      <c r="J291" s="28" t="n"/>
+      <c r="K291" s="33" t="n"/>
+    </row>
+    <row r="292">
+      <c r="E292" s="16" t="n"/>
+      <c r="F292" s="17" t="n"/>
+      <c r="G292" s="31" t="n"/>
+      <c r="H292" s="13" t="inlineStr">
+        <is>
+          <t>Frais comptable BDH - publication BNB</t>
+        </is>
+      </c>
+      <c r="I292" s="32" t="n">
+        <v>287.7</v>
+      </c>
+      <c r="J292" s="28" t="n"/>
+      <c r="K292" s="33" t="inlineStr">
+        <is>
+          <t>Remboursement des frais BNB avancés par BDH</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="E293" s="16" t="n"/>
+      <c r="F293" s="17" t="n"/>
+      <c r="G293" s="31" t="n"/>
+      <c r="H293" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I293" s="32" t="n">
+        <v>270.94</v>
+      </c>
+      <c r="J293" s="28" t="n"/>
+      <c r="K293" s="33" t="inlineStr">
+        <is>
+          <t>Facture 433/7265/65993</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="E294" s="16" t="n"/>
+      <c r="F294" s="17" t="n"/>
+      <c r="G294" s="31" t="n"/>
+      <c r="H294" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I294" s="32" t="n">
+        <v>263.44</v>
+      </c>
+      <c r="J294" s="28" t="n"/>
+      <c r="K294" s="33" t="inlineStr">
+        <is>
+          <t>Facture 464/6637/65902</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="E295" s="16" t="n"/>
+      <c r="F295" s="17" t="n"/>
+      <c r="G295" s="31" t="n"/>
+      <c r="H295" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I295" s="32" t="n">
+        <v>143.48</v>
+      </c>
+      <c r="J295" s="28" t="n"/>
+      <c r="K295" s="33" t="n"/>
+    </row>
+    <row r="296">
+      <c r="E296" s="16" t="n"/>
+      <c r="F296" s="17" t="n"/>
+      <c r="G296" s="31" t="n"/>
+      <c r="H296" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I296" s="32" t="n">
+        <v>65.52</v>
+      </c>
+      <c r="J296" s="28" t="n"/>
+      <c r="K296" s="33" t="inlineStr">
+        <is>
+          <t>Shell Haine-Saint-Pierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="E297" s="16" t="n"/>
+      <c r="F297" s="17" t="n"/>
+      <c r="G297" s="31" t="n"/>
+      <c r="H297" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I297" s="32" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J297" s="28" t="n"/>
+      <c r="K297" s="33" t="inlineStr">
+        <is>
+          <t>Schaerbeek</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="E298" s="16" t="n"/>
+      <c r="F298" s="17" t="n"/>
+      <c r="G298" s="31" t="n"/>
+      <c r="H298" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I298" s="32" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="J298" s="28" t="n"/>
+      <c r="K298" s="33" t="inlineStr">
+        <is>
+          <t>Louvain</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="E299" s="16" t="n"/>
+      <c r="F299" s="17" t="n"/>
+      <c r="G299" s="31" t="n"/>
+      <c r="H299" s="13" t="inlineStr">
+        <is>
+          <t>Achat matériel sportif - DECATHLON</t>
+        </is>
+      </c>
+      <c r="I299" s="32" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="J299" s="28" t="n"/>
+      <c r="K299" s="33" t="inlineStr">
+        <is>
+          <t>Decathlon Evere</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="E300" s="16" t="n"/>
+      <c r="F300" s="17" t="n"/>
+      <c r="G300" s="31" t="n"/>
+      <c r="H300" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I300" s="32" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="J300" s="28" t="n"/>
+      <c r="K300" s="33" t="inlineStr">
+        <is>
+          <t>Parking Rogier</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="E301" s="16" t="n"/>
+      <c r="F301" s="17" t="n"/>
+      <c r="G301" s="31" t="n"/>
+      <c r="H301" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I301" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J301" s="28" t="n"/>
+      <c r="K301" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="E302" s="16" t="n"/>
+      <c r="F302" s="17" t="n"/>
+      <c r="G302" s="31" t="n"/>
+      <c r="H302" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I302" s="32" t="n">
+        <v>69.11</v>
+      </c>
+      <c r="J302" s="28" t="n"/>
+      <c r="K302" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="E303" s="16" t="n"/>
+      <c r="F303" s="17" t="n"/>
+      <c r="G303" s="31" t="n"/>
+      <c r="H303" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I303" s="32" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J303" s="28" t="n"/>
+      <c r="K303" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="E304" s="16" t="n"/>
+      <c r="F304" s="17" t="n"/>
+      <c r="G304" s="31" t="n"/>
+      <c r="H304" s="13" t="inlineStr">
+        <is>
+          <t>Semelles orthopédiques de travail - Podomed</t>
+        </is>
+      </c>
+      <c r="I304" s="32" t="n">
+        <v>65</v>
+      </c>
+      <c r="J304" s="28" t="n"/>
+      <c r="K304" s="33" t="inlineStr">
+        <is>
+          <t>Consultation</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="E305" s="16" t="n"/>
+      <c r="F305" s="17" t="n"/>
+      <c r="G305" s="31" t="n"/>
+      <c r="H305" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I305" s="32" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="J305" s="28" t="n"/>
+      <c r="K305" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="E306" s="16" t="n"/>
+      <c r="F306" s="17" t="n"/>
+      <c r="G306" s="31" t="n"/>
+      <c r="H306" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I306" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J306" s="28" t="n"/>
+      <c r="K306" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="G307" s="34" t="n"/>
+      <c r="I307" s="34" t="n"/>
+      <c r="K307" s="35" t="n"/>
+    </row>
+    <row r="308">
+      <c r="G308" s="34" t="n"/>
+      <c r="I308" s="34" t="n"/>
+      <c r="K308" s="35" t="n"/>
+    </row>
+    <row r="309" ht="15.75" customHeight="1" thickBot="1">
+      <c r="G309" s="34">
+        <f>SUM(G6:G306)</f>
         <v/>
       </c>
-      <c r="I281" s="34">
-        <f>SUM(I6:I278)</f>
+      <c r="I309" s="34">
+        <f>SUM(I6:I306)</f>
         <v/>
       </c>
-      <c r="K281" s="35" t="n"/>
+      <c r="K309" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : ajout de decembre - annee complete
Extrait BNP Paribas Fortis n 2025-012 (operations 0307 a 0330, periode du
30-11 au 31-12).
2 entrees = 9.544,95 / 22 depenses = 4.993,89.
Rapprochement exact : 3.971,83 + 9.544,95 - 4.993,89 = 8.522,89.

Annee 2025 complete : 91.347,59 d'entrees, 85.849,93 de depenses,
resultat +5.497,66 sur 303 lignes de depenses.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K309"/>
+  <dimension ref="D1:K333"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -6119,15 +6119,443 @@
       <c r="K308" s="35" t="n"/>
     </row>
     <row r="309" ht="15.75" customHeight="1" thickBot="1">
-      <c r="G309" s="34">
-        <f>SUM(G6:G306)</f>
+      <c r="E309" s="16" t="inlineStr">
+        <is>
+          <t>Décembre</t>
+        </is>
+      </c>
+      <c r="F309" s="17" t="inlineStr">
+        <is>
+          <t>LAM2514</t>
+        </is>
+      </c>
+      <c r="G309" s="31" t="n">
+        <v>4162.5</v>
+      </c>
+      <c r="H309" s="28" t="inlineStr">
+        <is>
+          <t>Précompte salarial novembre 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I309" s="36" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J309" s="28" t="n"/>
+      <c r="K309" s="33" t="n"/>
+    </row>
+    <row r="310">
+      <c r="E310" s="16" t="n"/>
+      <c r="F310" s="17" t="inlineStr">
+        <is>
+          <t>LAM2515</t>
+        </is>
+      </c>
+      <c r="G310" s="31" t="n">
+        <v>5382.45</v>
+      </c>
+      <c r="H310" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I310" s="32" t="n">
+        <v>331.85</v>
+      </c>
+      <c r="J310" s="28" t="n"/>
+      <c r="K310" s="33" t="n"/>
+    </row>
+    <row r="311">
+      <c r="E311" s="16" t="n"/>
+      <c r="F311" s="17" t="n"/>
+      <c r="G311" s="31" t="n"/>
+      <c r="H311" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I311" s="32" t="n">
+        <v>63.61</v>
+      </c>
+      <c r="J311" s="28" t="n"/>
+      <c r="K311" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="E312" s="16" t="n"/>
+      <c r="F312" s="17" t="n"/>
+      <c r="G312" s="31" t="n"/>
+      <c r="H312" s="13" t="inlineStr">
+        <is>
+          <t>Crédit voiture</t>
+        </is>
+      </c>
+      <c r="I312" s="32" t="n">
+        <v>724.12</v>
+      </c>
+      <c r="J312" s="28" t="n"/>
+      <c r="K312" s="33" t="n"/>
+    </row>
+    <row r="313">
+      <c r="E313" s="16" t="n"/>
+      <c r="F313" s="17" t="n"/>
+      <c r="G313" s="31" t="n"/>
+      <c r="H313" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I313" s="32" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J313" s="28" t="n"/>
+      <c r="K313" s="33" t="inlineStr">
+        <is>
+          <t>Indigo Park Docks, Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="E314" s="16" t="n"/>
+      <c r="F314" s="17" t="n"/>
+      <c r="G314" s="31" t="n"/>
+      <c r="H314" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I314" s="32" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J314" s="28" t="n"/>
+      <c r="K314" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="E315" s="16" t="n"/>
+      <c r="F315" s="17" t="n"/>
+      <c r="G315" s="31" t="n"/>
+      <c r="H315" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I315" s="32" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="J315" s="28" t="n"/>
+      <c r="K315" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="E316" s="16" t="n"/>
+      <c r="F316" s="17" t="n"/>
+      <c r="G316" s="31" t="n"/>
+      <c r="H316" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I316" s="32" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="J316" s="28" t="n"/>
+      <c r="K316" s="33" t="inlineStr">
+        <is>
+          <t>Parcbrux Ixelles, Gand</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="E317" s="16" t="n"/>
+      <c r="F317" s="17" t="n"/>
+      <c r="G317" s="31" t="n"/>
+      <c r="H317" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I317" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="J317" s="28" t="n"/>
+      <c r="K317" s="33" t="inlineStr">
+        <is>
+          <t>Parking Station, Bruges</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="E318" s="16" t="n"/>
+      <c r="F318" s="17" t="n"/>
+      <c r="G318" s="31" t="n"/>
+      <c r="H318" s="13" t="inlineStr">
+        <is>
+          <t>Xerius</t>
+        </is>
+      </c>
+      <c r="I318" s="32" t="n">
+        <v>399.73</v>
+      </c>
+      <c r="J318" s="28" t="n"/>
+      <c r="K318" s="33" t="inlineStr">
+        <is>
+          <t>Cotisations sociales indépendant</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="E319" s="16" t="n"/>
+      <c r="F319" s="17" t="n"/>
+      <c r="G319" s="31" t="n"/>
+      <c r="H319" s="13" t="inlineStr">
+        <is>
+          <t>Electrabel</t>
+        </is>
+      </c>
+      <c r="I319" s="32" t="n">
+        <v>263.44</v>
+      </c>
+      <c r="J319" s="28" t="n"/>
+      <c r="K319" s="33" t="inlineStr">
+        <is>
+          <t>Facture 435/0584/57839</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="E320" s="16" t="n"/>
+      <c r="F320" s="17" t="n"/>
+      <c r="G320" s="31" t="n"/>
+      <c r="H320" s="13" t="inlineStr">
+        <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="I320" s="32" t="n">
+        <v>153.79</v>
+      </c>
+      <c r="J320" s="28" t="n"/>
+      <c r="K320" s="33" t="n"/>
+    </row>
+    <row r="321">
+      <c r="E321" s="16" t="n"/>
+      <c r="F321" s="17" t="n"/>
+      <c r="G321" s="31" t="n"/>
+      <c r="H321" s="13" t="inlineStr">
+        <is>
+          <t>Assurance RC - LRS Insurance</t>
+        </is>
+      </c>
+      <c r="I321" s="32" t="n">
+        <v>55.04</v>
+      </c>
+      <c r="J321" s="28" t="n"/>
+      <c r="K321" s="33" t="inlineStr">
+        <is>
+          <t>Même montant qu'en 2024 (Liantis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="E322" s="16" t="n"/>
+      <c r="F322" s="17" t="n"/>
+      <c r="G322" s="31" t="n"/>
+      <c r="H322" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I322" s="32" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J322" s="28" t="n"/>
+      <c r="K322" s="33" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="E323" s="16" t="n"/>
+      <c r="F323" s="17" t="n"/>
+      <c r="G323" s="31" t="n"/>
+      <c r="H323" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I323" s="32" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J323" s="28" t="n"/>
+      <c r="K323" s="33" t="inlineStr">
+        <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="E324" s="16" t="n"/>
+      <c r="F324" s="17" t="n"/>
+      <c r="G324" s="31" t="n"/>
+      <c r="H324" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I324" s="32" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J324" s="28" t="n"/>
+      <c r="K324" s="33" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="E325" s="16" t="n"/>
+      <c r="F325" s="17" t="n"/>
+      <c r="G325" s="31" t="n"/>
+      <c r="H325" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I325" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="J325" s="28" t="n"/>
+      <c r="K325" s="33" t="inlineStr">
+        <is>
+          <t>Parking Grand-Place, Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="E326" s="16" t="n"/>
+      <c r="F326" s="17" t="n"/>
+      <c r="G326" s="31" t="n"/>
+      <c r="H326" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I326" s="32" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J326" s="28" t="n"/>
+      <c r="K326" s="33" t="inlineStr">
+        <is>
+          <t>Parking Kinepolis, Louvain</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="E327" s="16" t="n"/>
+      <c r="F327" s="17" t="n"/>
+      <c r="G327" s="31" t="n"/>
+      <c r="H327" s="13" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="I327" s="32" t="n">
+        <v>63.32</v>
+      </c>
+      <c r="J327" s="28" t="n"/>
+      <c r="K327" s="33" t="inlineStr">
+        <is>
+          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="E328" s="16" t="n"/>
+      <c r="F328" s="17" t="n"/>
+      <c r="G328" s="31" t="n"/>
+      <c r="H328" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="I328" s="32" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J328" s="28" t="n"/>
+      <c r="K328" s="33" t="inlineStr">
+        <is>
+          <t>Indigo Park Docks, Bruxelles</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="E329" s="16" t="n"/>
+      <c r="F329" s="17" t="n"/>
+      <c r="G329" s="31" t="n"/>
+      <c r="H329" s="13" t="inlineStr">
+        <is>
+          <t>Semelles orthopédiques de travail - Podomed</t>
+        </is>
+      </c>
+      <c r="I329" s="32" t="n">
+        <v>210</v>
+      </c>
+      <c r="J329" s="28" t="n"/>
+      <c r="K329" s="33" t="inlineStr">
+        <is>
+          <t>Solde après la consultation du 27-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="E330" s="16" t="n"/>
+      <c r="F330" s="17" t="n"/>
+      <c r="G330" s="31" t="n"/>
+      <c r="H330" s="13" t="inlineStr">
+        <is>
+          <t>Frais comptable BDH</t>
+        </is>
+      </c>
+      <c r="I330" s="32" t="n">
+        <v>304.92</v>
+      </c>
+      <c r="J330" s="28" t="n"/>
+      <c r="K330" s="33" t="inlineStr">
+        <is>
+          <t>Facture 20250644</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="G331" s="34" t="n"/>
+      <c r="I331" s="34" t="n"/>
+      <c r="K331" s="35" t="n"/>
+    </row>
+    <row r="332">
+      <c r="G332" s="34" t="n"/>
+      <c r="I332" s="34" t="n"/>
+      <c r="K332" s="35" t="n"/>
+    </row>
+    <row r="333">
+      <c r="G333" s="34">
+        <f>SUM(G6:G330)</f>
         <v/>
       </c>
-      <c r="I309" s="34">
-        <f>SUM(I6:I306)</f>
+      <c r="I333" s="34">
+        <f>SUM(I6:I330)</f>
         <v/>
       </c>
-      <c r="K309" s="35" t="n"/>
+      <c r="K333" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : rattachement des charges de decembre payees en janvier 2026
D'apres l'extrait 2026-001, le precompte salarial de decembre 2025 (2.250,00,
paye le 05-01-2026) et le SD Worx correspondant (331,85, le 04-01-2026) sont
rattaches a decembre 2025, par symetrie avec les lignes de decembre 2024
laissees dans le bilan 2024.

Annee 2025 : 91.347,59 d'entrees, 88.431,78 de depenses, resultat +2.915,81.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:K333"/>
+  <dimension ref="D1:K335"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -6537,25 +6537,63 @@
       </c>
     </row>
     <row r="331">
-      <c r="G331" s="34" t="n"/>
-      <c r="I331" s="34" t="n"/>
-      <c r="K331" s="35" t="n"/>
+      <c r="E331" s="16" t="n"/>
+      <c r="F331" s="17" t="n"/>
+      <c r="G331" s="31" t="n"/>
+      <c r="H331" s="13" t="inlineStr">
+        <is>
+          <t>Précompte salarial décembre 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="I331" s="32" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J331" s="28" t="n"/>
+      <c r="K331" s="33" t="inlineStr">
+        <is>
+          <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024)</t>
+        </is>
+      </c>
     </row>
     <row r="332">
-      <c r="G332" s="34" t="n"/>
-      <c r="I332" s="34" t="n"/>
-      <c r="K332" s="35" t="n"/>
+      <c r="E332" s="16" t="n"/>
+      <c r="F332" s="17" t="n"/>
+      <c r="G332" s="31" t="n"/>
+      <c r="H332" s="13" t="inlineStr">
+        <is>
+          <t>SD Worx</t>
+        </is>
+      </c>
+      <c r="I332" s="32" t="n">
+        <v>331.85</v>
+      </c>
+      <c r="J332" s="28" t="n"/>
+      <c r="K332" s="33" t="inlineStr">
+        <is>
+          <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024)</t>
+        </is>
+      </c>
     </row>
     <row r="333">
-      <c r="G333" s="34">
-        <f>SUM(G6:G330)</f>
+      <c r="G333" s="34" t="n"/>
+      <c r="I333" s="34" t="n"/>
+      <c r="K333" s="35" t="n"/>
+    </row>
+    <row r="334">
+      <c r="G334" s="34" t="n"/>
+      <c r="I334" s="34" t="n"/>
+      <c r="K334" s="35" t="n"/>
+    </row>
+    <row r="335">
+      <c r="G335" s="34">
+        <f>SUM(G6:G332)</f>
         <v/>
       </c>
-      <c r="I333" s="34">
-        <f>SUM(I6:I330)</f>
+      <c r="I335" s="34">
+        <f>SUM(I6:I332)</f>
         <v/>
       </c>
-      <c r="K333" s="35" t="n"/>
+      <c r="K335" s="35" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : detail du decompte Mastercard n 216
Une seule transaction : Total Gidy (France), 66,74 le 26-07.
Toutes les depenses par carte de credit de 2025 sont desormais detaillees,
plus aucune ligne globale.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -6869,7 +6869,7 @@
       <c r="G340" s="31" t="n"/>
       <c r="H340" s="13" t="inlineStr">
         <is>
-          <t>Paiement carte MASTERCARD</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="I340" s="32" t="n">
@@ -6878,7 +6878,7 @@
       <c r="J340" s="28" t="n"/>
       <c r="K340" s="33" t="inlineStr">
         <is>
-          <t>Décompte n° 216 - nouveau compte carte 80845055</t>
+          <t>Carte Mastercard 26-07 — décompte n° 216 du 13-08 — Total Gidy (France)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : integration des corrections de Thibault
Reprise des 27 valeurs modifiees et des 20 lignes de-surlignees dans le fichier
corrige : Cora = carburant, NEW BS = Bellissimo, Markthof / RG Public /
Brussels Expo = parkings, Garage Gobinau = carburant, Oree = consommation,
avances Translatina remboursees plus tard.

Deux numeros de facture retrouves : le virement de juillet est LAM2509 et
celui d'octobre LAM2513, ce qui complete la serie.

Les trois redevances de stationnement sont des amendes (203,00) : le libelle
et la remarque le disent maintenant, avec la mention depense non admise.

Ajout d'une liste FORCER_JAUNE pour garder en jaune les lignes que Thibault
veut suivre meme sans marqueur dans la remarque.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -318,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -365,8 +365,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -940,18 +938,18 @@
       <c r="F10" s="17" t="n"/>
       <c r="G10" s="31" t="n"/>
       <c r="H10" s="32" t="n"/>
-      <c r="I10" s="34" t="inlineStr">
+      <c r="I10" s="13" t="inlineStr">
         <is>
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J10" s="35" t="n">
+      <c r="J10" s="33" t="n">
         <v>62.79</v>
       </c>
       <c r="K10" s="28" t="n"/>
-      <c r="L10" s="36" t="inlineStr">
-        <is>
-          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
+      <c r="L10" s="32" t="inlineStr">
+        <is>
+          <t>Cora Woluwe Carburant</t>
         </is>
       </c>
     </row>
@@ -1140,18 +1138,18 @@
       <c r="F21" s="17" t="n"/>
       <c r="G21" s="31" t="n"/>
       <c r="H21" s="32" t="n"/>
-      <c r="I21" s="34" t="inlineStr">
+      <c r="I21" s="13" t="inlineStr">
         <is>
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J21" s="35" t="n">
+      <c r="J21" s="33" t="n">
         <v>71.13</v>
       </c>
       <c r="K21" s="28" t="n"/>
-      <c r="L21" s="36" t="inlineStr">
-        <is>
-          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
+      <c r="L21" s="32" t="inlineStr">
+        <is>
+          <t>Cora Woluwe Carburant</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1225,7 @@
       <c r="K25" s="28" t="n"/>
       <c r="L25" s="36" t="inlineStr">
         <is>
-          <t>Facture de l'agence à joindre</t>
+          <t>Avance - remboursé plus tard</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1261,7 @@
       <c r="K27" s="28" t="n"/>
       <c r="L27" s="36" t="inlineStr">
         <is>
-          <t>Complément — facture à joindre</t>
+          <t>Avance - remboursé plus tard</t>
         </is>
       </c>
     </row>
@@ -1934,18 +1932,18 @@
         <v>5000</v>
       </c>
       <c r="H65" s="32" t="n"/>
-      <c r="I65" s="40" t="inlineStr">
+      <c r="I65" s="28" t="inlineStr">
         <is>
           <t>Achat - NEW BS SPRL</t>
         </is>
       </c>
-      <c r="J65" s="41" t="n">
+      <c r="J65" s="39" t="n">
         <v>290.5</v>
       </c>
       <c r="K65" s="28" t="n"/>
-      <c r="L65" s="36" t="inlineStr">
-        <is>
-          <t>Bruxelles — commerçant à identifier</t>
+      <c r="L65" s="32" t="inlineStr">
+        <is>
+          <t>Bellissimo - Achat vêtements de tennis</t>
         </is>
       </c>
     </row>
@@ -2148,18 +2146,18 @@
       <c r="F76" s="17" t="n"/>
       <c r="G76" s="31" t="n"/>
       <c r="H76" s="32" t="n"/>
-      <c r="I76" s="34" t="inlineStr">
-        <is>
-          <t>Redevance de stationnement - Ville de Louvain</t>
-        </is>
-      </c>
-      <c r="J76" s="35" t="n">
+      <c r="I76" s="13" t="inlineStr">
+        <is>
+          <t>Amende de stationnement - Ville de Louvain</t>
+        </is>
+      </c>
+      <c r="J76" s="33" t="n">
         <v>58</v>
       </c>
       <c r="K76" s="28" t="n"/>
-      <c r="L76" s="36" t="inlineStr">
-        <is>
-          <t>Comm. 194/3769/90294 — à confirmer (redevance ou amende)</t>
+      <c r="L76" s="32" t="inlineStr">
+        <is>
+          <t>Amende — dépense non admise, comm. 194/3769/90294</t>
         </is>
       </c>
     </row>
@@ -2168,18 +2166,18 @@
       <c r="F77" s="17" t="n"/>
       <c r="G77" s="31" t="n"/>
       <c r="H77" s="32" t="n"/>
-      <c r="I77" s="34" t="inlineStr">
-        <is>
-          <t>Redevance de stationnement - Woluwe-Saint-Lambert</t>
-        </is>
-      </c>
-      <c r="J77" s="35" t="n">
+      <c r="I77" s="13" t="inlineStr">
+        <is>
+          <t>Amende de stationnement - Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
+      <c r="J77" s="33" t="n">
         <v>45</v>
       </c>
       <c r="K77" s="28" t="n"/>
-      <c r="L77" s="36" t="inlineStr">
-        <is>
-          <t>Comm. 602/2505/46621 — à confirmer (redevance ou amende)</t>
+      <c r="L77" s="32" t="inlineStr">
+        <is>
+          <t>Amende — dépense non admise, comm. 602/2505/46621</t>
         </is>
       </c>
     </row>
@@ -2465,12 +2463,12 @@
           <t>Avril</t>
         </is>
       </c>
-      <c r="F94" s="42" t="inlineStr">
+      <c r="F94" s="40" t="inlineStr">
         <is>
           <t>Remboursement billet d'avion Lima-Bruxelles</t>
         </is>
       </c>
-      <c r="G94" s="43" t="n">
+      <c r="G94" s="41" t="n">
         <v>1683.78</v>
       </c>
       <c r="H94" s="36" t="inlineStr">
@@ -2538,18 +2536,18 @@
       <c r="F97" s="17" t="n"/>
       <c r="G97" s="31" t="n"/>
       <c r="H97" s="32" t="n"/>
-      <c r="I97" s="34" t="inlineStr">
+      <c r="I97" s="13" t="inlineStr">
         <is>
           <t>Parking</t>
         </is>
       </c>
-      <c r="J97" s="35" t="n">
+      <c r="J97" s="33" t="n">
         <v>10.4</v>
       </c>
       <c r="K97" s="28" t="n"/>
-      <c r="L97" s="36" t="inlineStr">
-        <is>
-          <t>Markthof La Haye (Pays-Bas) — à confirmer</t>
+      <c r="L97" s="32" t="inlineStr">
+        <is>
+          <t>Markthof La Haye (Pays-Bas)</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3667,7 @@
       <c r="K154" s="28" t="n"/>
       <c r="L154" s="32" t="inlineStr">
         <is>
-          <t>Delhaize Sterrebeek - 1er paiement avec la nouvelle carte 5255</t>
+          <t>Delhaize Sterrebeek</t>
         </is>
       </c>
     </row>
@@ -3786,18 +3784,18 @@
       <c r="F162" s="17" t="n"/>
       <c r="G162" s="31" t="n"/>
       <c r="H162" s="32" t="n"/>
-      <c r="I162" s="34" t="inlineStr">
+      <c r="I162" s="13" t="inlineStr">
         <is>
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J162" s="35" t="n">
+      <c r="J162" s="33" t="n">
         <v>59.49</v>
       </c>
       <c r="K162" s="28" t="n"/>
-      <c r="L162" s="36" t="inlineStr">
-        <is>
-          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
+      <c r="L162" s="32" t="inlineStr">
+        <is>
+          <t>Cora Woluwe Carburant</t>
         </is>
       </c>
     </row>
@@ -4761,12 +4759,12 @@
     </row>
     <row r="212">
       <c r="E212" s="16" t="n"/>
-      <c r="F212" s="42" t="inlineStr">
+      <c r="F212" s="40" t="inlineStr">
         <is>
           <t>Approvisionnement compte - Thibault Duchène</t>
         </is>
       </c>
-      <c r="G212" s="43" t="n">
+      <c r="G212" s="41" t="n">
         <v>1500</v>
       </c>
       <c r="H212" s="36" t="inlineStr">
@@ -4878,18 +4876,18 @@
       <c r="F218" s="17" t="n"/>
       <c r="G218" s="31" t="n"/>
       <c r="H218" s="32" t="n"/>
-      <c r="I218" s="34" t="inlineStr">
+      <c r="I218" s="13" t="inlineStr">
         <is>
           <t>Parking</t>
         </is>
       </c>
-      <c r="J218" s="35" t="n">
+      <c r="J218" s="33" t="n">
         <v>15.8</v>
       </c>
       <c r="K218" s="28" t="n"/>
-      <c r="L218" s="36" t="inlineStr">
-        <is>
-          <t>RG Public, Paris (France) — à confirmer</t>
+      <c r="L218" s="32" t="inlineStr">
+        <is>
+          <t>RG Public, Paris (France)</t>
         </is>
       </c>
     </row>
@@ -4938,18 +4936,18 @@
       <c r="F221" s="17" t="n"/>
       <c r="G221" s="31" t="n"/>
       <c r="H221" s="32" t="n"/>
-      <c r="I221" s="34" t="inlineStr">
+      <c r="I221" s="13" t="inlineStr">
         <is>
           <t>Parking</t>
         </is>
       </c>
-      <c r="J221" s="35" t="n">
+      <c r="J221" s="33" t="n">
         <v>12</v>
       </c>
       <c r="K221" s="28" t="n"/>
-      <c r="L221" s="36" t="inlineStr">
-        <is>
-          <t>Brussels Expo — à confirmer (parking ou entrée)</t>
+      <c r="L221" s="32" t="inlineStr">
+        <is>
+          <t>Brussels Expo Parking</t>
         </is>
       </c>
     </row>
@@ -5943,12 +5941,12 @@
           <t>Juillet</t>
         </is>
       </c>
-      <c r="F273" s="42" t="inlineStr">
+      <c r="F273" s="40" t="inlineStr">
         <is>
           <t>Remboursement paiement à Sandaya</t>
         </is>
       </c>
-      <c r="G273" s="43" t="n">
+      <c r="G273" s="41" t="n">
         <v>1775.4</v>
       </c>
       <c r="H273" s="36" t="inlineStr">
@@ -5969,17 +5967,17 @@
     </row>
     <row r="274">
       <c r="E274" s="16" t="n"/>
-      <c r="F274" s="42" t="inlineStr">
-        <is>
-          <t>Prestations juillet 2025 - RTC Lambermont</t>
-        </is>
-      </c>
-      <c r="G274" s="43" t="n">
+      <c r="F274" s="17" t="inlineStr">
+        <is>
+          <t>LAM2509</t>
+        </is>
+      </c>
+      <c r="G274" s="31" t="n">
         <v>7130</v>
       </c>
-      <c r="H274" s="36" t="inlineStr">
-        <is>
-          <t>Communication sans numéro de facture LAM</t>
+      <c r="H274" s="32" t="inlineStr">
+        <is>
+          <t>Virement du 24-07, communication « Prestations juillet 2025 »</t>
         </is>
       </c>
       <c r="I274" s="13" t="inlineStr">
@@ -6606,20 +6604,16 @@
       <c r="F306" s="17" t="n"/>
       <c r="G306" s="31" t="n"/>
       <c r="H306" s="32" t="n"/>
-      <c r="I306" s="34" t="inlineStr">
-        <is>
-          <t>Terrain de tennis - Orée ASBL</t>
-        </is>
-      </c>
-      <c r="J306" s="35" t="n">
+      <c r="I306" s="13" t="inlineStr">
+        <is>
+          <t>Consommation club de tennis Orée</t>
+        </is>
+      </c>
+      <c r="J306" s="33" t="n">
         <v>8.5</v>
       </c>
       <c r="K306" s="28" t="n"/>
-      <c r="L306" s="36" t="inlineStr">
-        <is>
-          <t>À confirmer (terrain ou consommation)</t>
-        </is>
-      </c>
+      <c r="L306" s="32" t="n"/>
     </row>
     <row r="307">
       <c r="E307" s="16" t="n"/>
@@ -6742,18 +6736,18 @@
       <c r="F313" s="17" t="n"/>
       <c r="G313" s="31" t="n"/>
       <c r="H313" s="32" t="n"/>
-      <c r="I313" s="34" t="inlineStr">
-        <is>
-          <t>Redevance de stationnement - Saint-Josse</t>
-        </is>
-      </c>
-      <c r="J313" s="35" t="n">
+      <c r="I313" s="13" t="inlineStr">
+        <is>
+          <t>Amende de stationnement - Saint-Josse</t>
+        </is>
+      </c>
+      <c r="J313" s="33" t="n">
         <v>100</v>
       </c>
       <c r="K313" s="28" t="n"/>
-      <c r="L313" s="36" t="inlineStr">
-        <is>
-          <t>Comm. 500/2300/37391 — à confirmer (redevance ou amende)</t>
+      <c r="L313" s="32" t="inlineStr">
+        <is>
+          <t>Amende — dépense non admise, comm. 500/2300/37391</t>
         </is>
       </c>
     </row>
@@ -6938,7 +6932,7 @@
       <c r="H324" s="32" t="n"/>
       <c r="I324" s="13" t="inlineStr">
         <is>
-          <t>Entretien voiture - Garage Gobinau</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J324" s="33" t="n">
@@ -7472,18 +7466,18 @@
       <c r="F351" s="17" t="n"/>
       <c r="G351" s="31" t="n"/>
       <c r="H351" s="32" t="n"/>
-      <c r="I351" s="34" t="inlineStr">
+      <c r="I351" s="13" t="inlineStr">
         <is>
           <t>Parking</t>
         </is>
       </c>
-      <c r="J351" s="35" t="n">
+      <c r="J351" s="33" t="n">
         <v>12</v>
       </c>
       <c r="K351" s="28" t="n"/>
-      <c r="L351" s="36" t="inlineStr">
-        <is>
-          <t>Brussels Expo — à confirmer (parking ou entrée)</t>
+      <c r="L351" s="32" t="inlineStr">
+        <is>
+          <t>Brussels Expo Parking</t>
         </is>
       </c>
     </row>
@@ -7525,19 +7519,15 @@
           <t>Septembre</t>
         </is>
       </c>
-      <c r="F355" s="42" t="inlineStr">
+      <c r="F355" s="17" t="inlineStr">
         <is>
           <t>LAM2510</t>
         </is>
       </c>
-      <c r="G355" s="43" t="n">
+      <c r="G355" s="31" t="n">
         <v>5501.95</v>
       </c>
-      <c r="H355" s="36" t="inlineStr">
-        <is>
-          <t>Pas de LAM2509 encaissé — correspond peut-être au virement de juillet sans numéro</t>
-        </is>
-      </c>
+      <c r="H355" s="32" t="n"/>
       <c r="I355" s="28" t="inlineStr">
         <is>
           <t>Partena</t>
@@ -8010,18 +8000,18 @@
       <c r="F380" s="17" t="n"/>
       <c r="G380" s="31" t="n"/>
       <c r="H380" s="32" t="n"/>
-      <c r="I380" s="34" t="inlineStr">
+      <c r="I380" s="13" t="inlineStr">
         <is>
           <t>Achat - NEW BS SPRL</t>
         </is>
       </c>
-      <c r="J380" s="35" t="n">
+      <c r="J380" s="33" t="n">
         <v>40</v>
       </c>
       <c r="K380" s="28" t="n"/>
-      <c r="L380" s="36" t="inlineStr">
-        <is>
-          <t>Bruxelles — même commerçant qu'en mars (290,50) à identifier</t>
+      <c r="L380" s="32" t="inlineStr">
+        <is>
+          <t>Bellissimo - Achat article de sport</t>
         </is>
       </c>
     </row>
@@ -8065,19 +8055,15 @@
     </row>
     <row r="384">
       <c r="E384" s="16" t="n"/>
-      <c r="F384" s="42" t="inlineStr">
+      <c r="F384" s="17" t="inlineStr">
         <is>
           <t>LAM2512</t>
         </is>
       </c>
-      <c r="G384" s="43" t="n">
+      <c r="G384" s="31" t="n">
         <v>13994</v>
       </c>
-      <c r="H384" s="36" t="inlineStr">
-        <is>
-          <t>Montant inhabituel — facture assujettie à la TVA comme LAM2412 en 2024 ?</t>
-        </is>
-      </c>
+      <c r="H384" s="32" t="n"/>
       <c r="I384" s="13" t="inlineStr">
         <is>
           <t>Carburant</t>
@@ -8095,19 +8081,15 @@
     </row>
     <row r="385">
       <c r="E385" s="16" t="n"/>
-      <c r="F385" s="42" t="inlineStr">
-        <is>
-          <t>Prestations octobre 2025 - RTC Lambermont</t>
-        </is>
-      </c>
-      <c r="G385" s="43" t="n">
+      <c r="F385" s="17" t="inlineStr">
+        <is>
+          <t>LAM2513</t>
+        </is>
+      </c>
+      <c r="G385" s="31" t="n">
         <v>4525.72</v>
       </c>
-      <c r="H385" s="36" t="inlineStr">
-        <is>
-          <t>Communication sans numéro de facture LAM</t>
-        </is>
-      </c>
+      <c r="H385" s="32" t="n"/>
       <c r="I385" s="13" t="inlineStr">
         <is>
           <t>Précompte salarial septembre 2025 Thibault Duchène</t>
@@ -8348,18 +8330,18 @@
       <c r="F398" s="17" t="n"/>
       <c r="G398" s="31" t="n"/>
       <c r="H398" s="32" t="n"/>
-      <c r="I398" s="34" t="inlineStr">
+      <c r="I398" s="13" t="inlineStr">
         <is>
           <t>Parking</t>
         </is>
       </c>
-      <c r="J398" s="35" t="n">
+      <c r="J398" s="33" t="n">
         <v>12</v>
       </c>
       <c r="K398" s="28" t="n"/>
-      <c r="L398" s="36" t="inlineStr">
-        <is>
-          <t>Brussels Expo — à confirmer (parking ou entrée)</t>
+      <c r="L398" s="32" t="inlineStr">
+        <is>
+          <t>Brussels Expo Parking</t>
         </is>
       </c>
     </row>
@@ -9169,19 +9151,15 @@
           <t>Décembre</t>
         </is>
       </c>
-      <c r="F443" s="42" t="inlineStr">
+      <c r="F443" s="17" t="inlineStr">
         <is>
           <t>LAM2514</t>
         </is>
       </c>
-      <c r="G443" s="43" t="n">
+      <c r="G443" s="31" t="n">
         <v>4162.5</v>
       </c>
-      <c r="H443" s="36" t="inlineStr">
-        <is>
-          <t>Pas de LAM2513 encaissé — correspond peut-être au virement du 29-10 sans numéro</t>
-        </is>
-      </c>
+      <c r="H443" s="32" t="n"/>
       <c r="I443" s="28" t="inlineStr">
         <is>
           <t>Précompte salarial novembre 2025 Thibault Duchène</t>
@@ -9532,18 +9510,18 @@
       <c r="F461" s="17" t="n"/>
       <c r="G461" s="31" t="n"/>
       <c r="H461" s="32" t="n"/>
-      <c r="I461" s="34" t="inlineStr">
+      <c r="I461" s="13" t="inlineStr">
         <is>
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J461" s="35" t="n">
+      <c r="J461" s="33" t="n">
         <v>63.32</v>
       </c>
       <c r="K461" s="28" t="n"/>
-      <c r="L461" s="36" t="inlineStr">
-        <is>
-          <t>Cora Woluwe — à confirmer (carburant ou achats ?)</t>
+      <c r="L461" s="32" t="inlineStr">
+        <is>
+          <t>Cora Woluwe Carburant</t>
         </is>
       </c>
     </row>
@@ -9661,12 +9639,12 @@
     </row>
     <row r="469">
       <c r="G469" s="37">
-        <f>SUM(G6:G466)</f>
+        <f>SUM(G6:G468)</f>
         <v/>
       </c>
       <c r="H469" s="38" t="n"/>
       <c r="J469" s="37">
-        <f>SUM(J6:J466)</f>
+        <f>SUM(J6:J468)</f>
         <v/>
       </c>
       <c r="L469" s="38" t="n"/>

</xml_diff>

<commit_message>
Justificatifs : premier ticket rattache au bilan
Ajout de ticket2pdf.py, qui transforme la photo d'un ticket en PDF A4 :
recadrage, redressement, fond blanchi, contraste releve.

Premier ticket : RTCL Lambermont du 10-01-2025, 22,00. La ligne « Repas
Topogigio » de janvier passe a V dans la colonne Facture et porte le nom du
justificatif en remarque (mecanisme dans justificatifs.py).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1018,8 +1018,16 @@
       <c r="J14" s="33" t="n">
         <v>22</v>
       </c>
-      <c r="K14" s="28" t="n"/>
-      <c r="L14" s="32" t="n"/>
+      <c r="K14" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L14" s="32" t="inlineStr">
+        <is>
+          <t>Justificatif : 2025-01-10_RTCL-Lambermont_22.00.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="E15" s="16" t="n"/>

</xml_diff>

<commit_message>
Justificatifs : 28 tickets convertis en PDF et rattaches au bilan
25 tickets correspondent a une ligne du bilan : colonne Facture a V et nom du
PDF en remarque. 3 tickets restent sans correspondance (Lambermont 29,00 du
23-04, Lambermont 251,50 du 25-07, FedEx 11,84 de fin decembre).

Commercants identifies grace aux tickets :
- PVH Maasmechelen = Tommy Hilfiger
- NZA Utrecht = achat de vetements (3 articles)
- NEW BS SRL = Bellissimo Sport (les deux lignes)
- Total Nivelles 13,65 = restauration sur l'aire d'Orival, pas du carburant
- Lunch Garden = Kraainem et non Auderghem
- Decathlon 140,00 = une veste, ligne reclassee en vetement de sport

ticket2pdf.py : detection du ticket par quantiles (robuste au fond clair),
redressement, fond blanchi, mise en colonnes des tickets tres allonges.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1434,14 +1434,22 @@
       <c r="H37" s="32" t="n"/>
       <c r="I37" s="28" t="inlineStr">
         <is>
-          <t>Achat vêtements sport - PVH Maasmechelen</t>
+          <t>Achat vêtements sport - Tommy Hilfiger Maasmechelen</t>
         </is>
       </c>
       <c r="J37" s="39" t="n">
         <v>210.49</v>
       </c>
-      <c r="K37" s="28" t="n"/>
-      <c r="L37" s="32" t="n"/>
+      <c r="K37" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L37" s="32" t="inlineStr">
+        <is>
+          <t>Outlet Maasmechelen — « PVH » sur l'extrait — Justificatif : 2025-02-01_TommyHilfiger-Maasmechelen_210.49.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="E38" s="16" t="n"/>
@@ -1466,8 +1474,16 @@
       <c r="J38" s="33" t="n">
         <v>141.47</v>
       </c>
-      <c r="K38" s="28" t="n"/>
-      <c r="L38" s="32" t="n"/>
+      <c r="K38" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L38" s="32" t="inlineStr">
+        <is>
+          <t>Justificatif : 2025-02-01_Nike-Maasmechelen_141.47.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="E39" s="16" t="n"/>
@@ -1818,10 +1834,14 @@
       <c r="J57" s="33" t="n">
         <v>39.47</v>
       </c>
-      <c r="K57" s="28" t="n"/>
+      <c r="K57" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L57" s="32" t="inlineStr">
         <is>
-          <t>LG Auderghem</t>
+          <t>Lunch Garden Kraainem — Justificatif : 2025-02-22_LunchGarden-Kraainem_39.47.pdf</t>
         </is>
       </c>
     </row>
@@ -1832,16 +1852,20 @@
       <c r="H58" s="32" t="n"/>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>Achat matériel sportif - DECATHLON</t>
+          <t>Achat vêtement sport - DECATHLON</t>
         </is>
       </c>
       <c r="J58" s="33" t="n">
         <v>140</v>
       </c>
-      <c r="K58" s="28" t="n"/>
+      <c r="K58" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L58" s="32" t="inlineStr">
         <is>
-          <t>Decathlon Evere</t>
+          <t>Decathlon Evere — veste JKT MAN 900 — Justificatif : 2025-02-25_Decathlon-Evere_140.00.pdf</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1966,7 @@
       <c r="H65" s="32" t="n"/>
       <c r="I65" s="28" t="inlineStr">
         <is>
-          <t>Achat - NEW BS SPRL</t>
+          <t>Achat vêtements de tennis - Bellissimo Sport</t>
         </is>
       </c>
       <c r="J65" s="39" t="n">
@@ -1951,7 +1975,7 @@
       <c r="K65" s="28" t="n"/>
       <c r="L65" s="32" t="inlineStr">
         <is>
-          <t>Bellissimo - Achat vêtements de tennis</t>
+          <t>New Bs SRL, Bruxelles</t>
         </is>
       </c>
     </row>
@@ -1990,8 +2014,16 @@
       <c r="J67" s="33" t="n">
         <v>75.5</v>
       </c>
-      <c r="K67" s="28" t="n"/>
-      <c r="L67" s="32" t="n"/>
+      <c r="K67" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L67" s="32" t="inlineStr">
+        <is>
+          <t>Ticket pro forma de 79,50 corrigé à la main à 75,50 — Justificatif : 2025-03-05_RTCL-Lambermont_75.50.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="E68" s="16" t="n"/>
@@ -2282,10 +2314,14 @@
       <c r="J82" s="33" t="n">
         <v>50.2</v>
       </c>
-      <c r="K82" s="28" t="n"/>
+      <c r="K82" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L82" s="32" t="inlineStr">
         <is>
-          <t>Station 15 Zemst</t>
+          <t>Station 15 Zemst — Justificatif : 2025-03-20_Station15-Zemst_50.20.pdf</t>
         </is>
       </c>
     </row>
@@ -2318,8 +2354,16 @@
       <c r="J84" s="33" t="n">
         <v>919.17</v>
       </c>
-      <c r="K84" s="28" t="n"/>
-      <c r="L84" s="32" t="n"/>
+      <c r="K84" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L84" s="32" t="inlineStr">
+        <is>
+          <t>4 pneus Uniroyal + géométrie, VW Tiguan — facture 22501184 — Justificatif : 2025-03-25_MonsieurPneus_919.17.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="E85" s="16" t="n"/>
@@ -2354,10 +2398,14 @@
       <c r="J86" s="33" t="n">
         <v>16</v>
       </c>
-      <c r="K86" s="28" t="n"/>
+      <c r="K86" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L86" s="32" t="inlineStr">
         <is>
-          <t>Station 15 Zemst</t>
+          <t>Station 15 Zemst — Justificatif : 2025-03-27_Station15-Zemst_16.00.pdf</t>
         </is>
       </c>
     </row>
@@ -2492,10 +2540,14 @@
       <c r="J94" s="39" t="n">
         <v>30.3</v>
       </c>
-      <c r="K94" s="28" t="n"/>
+      <c r="K94" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L94" s="32" t="inlineStr">
         <is>
-          <t>Exki Woluwe</t>
+          <t>Exki Woluwe — Justificatif : 2025-04-01_EXKi-Woluwe_30.30.pdf</t>
         </is>
       </c>
     </row>
@@ -2676,18 +2728,22 @@
       <c r="F104" s="17" t="n"/>
       <c r="G104" s="31" t="n"/>
       <c r="H104" s="32" t="n"/>
-      <c r="I104" s="34" t="inlineStr">
-        <is>
-          <t>Achat - NZA Utrecht BV</t>
-        </is>
-      </c>
-      <c r="J104" s="35" t="n">
+      <c r="I104" s="13" t="inlineStr">
+        <is>
+          <t>Achat vêtements - N.Z.A. Utrecht</t>
+        </is>
+      </c>
+      <c r="J104" s="33" t="n">
         <v>289.97</v>
       </c>
-      <c r="K104" s="28" t="n"/>
-      <c r="L104" s="36" t="inlineStr">
-        <is>
-          <t>Amsterdam (Pays-Bas) — commerçant à identifier</t>
+      <c r="K104" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L104" s="32" t="inlineStr">
+        <is>
+          <t>3 articles, Utrecht (Pays-Bas) — Justificatif : 2025-04-06_NZA-Utrecht_289.97.pdf</t>
         </is>
       </c>
     </row>
@@ -3652,10 +3708,14 @@
       <c r="J153" s="33" t="n">
         <v>84.2</v>
       </c>
-      <c r="K153" s="28" t="n"/>
+      <c r="K153" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L153" s="32" t="inlineStr">
         <is>
-          <t>Decathlon Evere</t>
+          <t>Decathlon Evere — Justificatif : 2025-04-26_Decathlon-Evere_84.20.pdf</t>
         </is>
       </c>
     </row>
@@ -4500,10 +4560,14 @@
       <c r="J197" s="33" t="n">
         <v>50</v>
       </c>
-      <c r="K197" s="28" t="n"/>
+      <c r="K197" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L197" s="32" t="inlineStr">
         <is>
-          <t>Decathlon Evere</t>
+          <t>Decathlon Evere — Justificatif : 2025-05-12_Decathlon-Evere_50.00.pdf</t>
         </is>
       </c>
     </row>
@@ -4758,10 +4822,14 @@
       <c r="J211" s="39" t="n">
         <v>200</v>
       </c>
-      <c r="K211" s="28" t="n"/>
+      <c r="K211" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L211" s="32" t="inlineStr">
         <is>
-          <t>Decathlon Evere</t>
+          <t>Decathlon Evere — Justificatif : 2025-06-02_Decathlon-Evere_200.00.pdf</t>
         </is>
       </c>
     </row>
@@ -6620,8 +6688,16 @@
       <c r="J306" s="33" t="n">
         <v>8.5</v>
       </c>
-      <c r="K306" s="28" t="n"/>
-      <c r="L306" s="32" t="n"/>
+      <c r="K306" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L306" s="32" t="inlineStr">
+        <is>
+          <t>Justificatif : 2025-07-10_Oree-ASBL_8.50.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="E307" s="16" t="n"/>
@@ -7022,10 +7098,14 @@
       <c r="J328" s="33" t="n">
         <v>18</v>
       </c>
-      <c r="K328" s="28" t="n"/>
+      <c r="K328" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L328" s="32" t="inlineStr">
         <is>
-          <t>Decathlon Evere</t>
+          <t>Decathlon Evere — Justificatif : 2025-08-08_Decathlon-Evere_18.00.pdf</t>
         </is>
       </c>
     </row>
@@ -7302,10 +7382,14 @@
       <c r="J342" s="33" t="n">
         <v>123</v>
       </c>
-      <c r="K342" s="28" t="n"/>
+      <c r="K342" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L342" s="32" t="inlineStr">
         <is>
-          <t>Decathlon Evere - remboursé par le RTC Lambermont le même jour</t>
+          <t>Decathlon Evere — 28 balles de tennis, remboursé par le RTC Lambermont le même jour — Justificatif : 2025-08-14_Decathlon-Evere_123.00.pdf</t>
         </is>
       </c>
     </row>
@@ -7776,10 +7860,14 @@
       <c r="J368" s="33" t="n">
         <v>45.77</v>
       </c>
-      <c r="K368" s="28" t="n"/>
+      <c r="K368" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L368" s="32" t="inlineStr">
         <is>
-          <t>Lunch Garden Kraainem</t>
+          <t>Lunch Garden Kraainem — Justificatif : 2025-09-13_LunchGarden-Kraainem_45.77.pdf</t>
         </is>
       </c>
     </row>
@@ -7876,10 +7964,14 @@
       <c r="J373" s="33" t="n">
         <v>35.4</v>
       </c>
-      <c r="K373" s="28" t="n"/>
+      <c r="K373" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L373" s="32" t="inlineStr">
         <is>
-          <t>Exki Woluwe</t>
+          <t>Exki Woluwe — Justificatif : 2025-09-19_EXKi-Woluwe_35.40.pdf</t>
         </is>
       </c>
     </row>
@@ -7956,10 +8048,14 @@
       <c r="J377" s="33" t="n">
         <v>47</v>
       </c>
-      <c r="K377" s="28" t="n"/>
+      <c r="K377" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L377" s="32" t="inlineStr">
         <is>
-          <t>Péruwelz</t>
+          <t>Péruwelz — Justificatif : 2025-09-23_ChezJi-Peruwelz_47.00.pdf</t>
         </is>
       </c>
     </row>
@@ -7990,16 +8086,20 @@
       <c r="H379" s="32" t="n"/>
       <c r="I379" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Repas - TotalEnergies Nivelles</t>
         </is>
       </c>
       <c r="J379" s="33" t="n">
         <v>13.65</v>
       </c>
-      <c r="K379" s="28" t="n"/>
+      <c r="K379" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L379" s="32" t="inlineStr">
         <is>
-          <t>Total Nivelles</t>
+          <t>Aire d'Orival E19 — restauration, pas du carburant — Justificatif : 2025-09-26_TotalEnergies-Nivelles_13.65.pdf</t>
         </is>
       </c>
     </row>
@@ -8010,16 +8110,20 @@
       <c r="H380" s="32" t="n"/>
       <c r="I380" s="13" t="inlineStr">
         <is>
-          <t>Achat - NEW BS SPRL</t>
+          <t>Achat matériel sportif - Bellissimo Sport</t>
         </is>
       </c>
       <c r="J380" s="33" t="n">
         <v>40</v>
       </c>
-      <c r="K380" s="28" t="n"/>
+      <c r="K380" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L380" s="32" t="inlineStr">
         <is>
-          <t>Bellissimo - Achat article de sport</t>
+          <t>Chaussures Babolat Pulsion Kid (enfants, pointure 29) — Justificatif : 2025-09-27_Bellissimo-Sport_40.00.pdf</t>
         </is>
       </c>
     </row>
@@ -8270,8 +8374,16 @@
       <c r="J394" s="33" t="n">
         <v>17.37</v>
       </c>
-      <c r="K394" s="28" t="n"/>
-      <c r="L394" s="32" t="n"/>
+      <c r="K394" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L394" s="32" t="inlineStr">
+        <is>
+          <t>Justificatif : 2025-09-25_FedEx_17.37.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="E395" s="16" t="n"/>
@@ -8622,8 +8734,16 @@
       <c r="J412" s="33" t="n">
         <v>58</v>
       </c>
-      <c r="K412" s="28" t="n"/>
-      <c r="L412" s="32" t="n"/>
+      <c r="K412" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L412" s="32" t="inlineStr">
+        <is>
+          <t>Justificatif : 2025-10-29_RTCL-Lambermont_58.00.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="413">
       <c r="G413" s="37" t="n"/>
@@ -8986,18 +9106,22 @@
       <c r="F433" s="17" t="n"/>
       <c r="G433" s="31" t="n"/>
       <c r="H433" s="32" t="n"/>
-      <c r="I433" s="13" t="inlineStr">
+      <c r="I433" s="34" t="inlineStr">
         <is>
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J433" s="33" t="n">
+      <c r="J433" s="35" t="n">
         <v>118.5</v>
       </c>
-      <c r="K433" s="28" t="n"/>
-      <c r="L433" s="32" t="inlineStr">
-        <is>
-          <t>Decathlon Evere</t>
+      <c r="K433" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L433" s="36" t="inlineStr">
+        <is>
+          <t>Decathlon Evere — 10 articles dont masque de ski, luge et vêtements enfant : usage professionnel à confirmer — Justificatif : 2025-11-22_Decathlon-Evere_118.50.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : communications structurees de janvier pour Electrabel et Telenet
Les deux lignes de janvier n'avaient pas leur reference de facture en
remarque, ce qui genait le pointage avec l'espace client.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1103,7 +1103,11 @@
         <v>256.99</v>
       </c>
       <c r="K18" s="28" t="n"/>
-      <c r="L18" s="32" t="n"/>
+      <c r="L18" s="32" t="inlineStr">
+        <is>
+          <t>Facture 468/9192/57548</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="E19" s="16" t="n"/>
@@ -1119,7 +1123,11 @@
         <v>159.1</v>
       </c>
       <c r="K19" s="28" t="n"/>
-      <c r="L19" s="32" t="n"/>
+      <c r="L19" s="32" t="inlineStr">
+        <is>
+          <t>Facture 308/8521/00268</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="E20" s="16" t="n"/>

</xml_diff>

<commit_message>
Bilan 2025 : Electrabel de juillet identifie comme decompte annuel
Thibault confirme que les 356,79 du 19-07 sont l'afrekening et non un
voorschot. La remarque le dit, et note le relevement de l'acompte de 256,99
a 263,44 qui suit. La double facture de novembre est signalee a verifier.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -6803,7 +6803,7 @@
       <c r="K311" s="28" t="n"/>
       <c r="L311" s="32" t="inlineStr">
         <is>
-          <t>Facture 455/1399/88731 — montant en hausse (256,99 les mois précédents)</t>
+          <t>Décompte annuel (afrekening) — facture 455/1399/88731 ; l'acompte passe ensuite de 256,99 à 263,44</t>
         </is>
       </c>
     </row>
@@ -8998,18 +8998,18 @@
       <c r="F427" s="17" t="n"/>
       <c r="G427" s="31" t="n"/>
       <c r="H427" s="32" t="n"/>
-      <c r="I427" s="13" t="inlineStr">
+      <c r="I427" s="34" t="inlineStr">
         <is>
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J427" s="33" t="n">
+      <c r="J427" s="35" t="n">
         <v>270.94</v>
       </c>
       <c r="K427" s="28" t="n"/>
-      <c r="L427" s="32" t="inlineStr">
-        <is>
-          <t>Facture 433/7265/65993</t>
+      <c r="L427" s="36" t="inlineStr">
+        <is>
+          <t>Facture 433/7265/65993 — 2e facture du mois, acompte ou décompte à vérifier</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : la 2e facture Electrabel de novembre est l'acompte d'aout
270,94 = 263,44 d'acompte + 7,50 de frais de rappel. Aucun paiement
Electrabel en aout, et cinq paiements couvrent bien aout a decembre.
La ligne n'est plus signalee en jaune.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -8998,18 +8998,18 @@
       <c r="F427" s="17" t="n"/>
       <c r="G427" s="31" t="n"/>
       <c r="H427" s="32" t="n"/>
-      <c r="I427" s="34" t="inlineStr">
+      <c r="I427" s="13" t="inlineStr">
         <is>
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J427" s="35" t="n">
+      <c r="J427" s="33" t="n">
         <v>270.94</v>
       </c>
       <c r="K427" s="28" t="n"/>
-      <c r="L427" s="36" t="inlineStr">
-        <is>
-          <t>Facture 433/7265/65993 — 2e facture du mois, acompte ou décompte à vérifier</t>
+      <c r="L427" s="32" t="inlineStr">
+        <is>
+          <t>Acompte d'août payé en retard le 18-11 : 263,44 + 7,50 de frais de rappel — facture 433/7265/65993</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : les 13 lignes Electrabel passent a V
Thibault a recupere les 12 pieces ENGIE (11 acomptes + le decompte annuel
de juillet). Les lignes de janvier et de fevrier renvoient a la meme facture,
payee deux fois et remboursee.

build.py : une entree de justificatifs qui n'est pas un PDF est reprise telle
quelle en remarque, pour cocher une piece detenue sans fichier transmis.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1102,10 +1102,14 @@
       <c r="J18" s="33" t="n">
         <v>256.99</v>
       </c>
-      <c r="K18" s="28" t="n"/>
+      <c r="K18" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L18" s="32" t="inlineStr">
         <is>
-          <t>Facture 468/9192/57548</t>
+          <t>Facture 468/9192/57548 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -1526,10 +1530,14 @@
       <c r="J40" s="33" t="n">
         <v>256.99</v>
       </c>
-      <c r="K40" s="28" t="n"/>
+      <c r="K40" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L40" s="32" t="inlineStr">
         <is>
-          <t>Facture 468/9192/57548 payée 2× (16-01 et 04-02) — remboursée le 10-02</t>
+          <t>Facture 468/9192/57548 payée 2× (16-01 et 04-02) — remboursée le 10-02 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -2146,10 +2154,14 @@
       <c r="J73" s="33" t="n">
         <v>256.99</v>
       </c>
-      <c r="K73" s="28" t="n"/>
+      <c r="K73" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L73" s="32" t="inlineStr">
         <is>
-          <t>Facture 470/3433/24753</t>
+          <t>Facture 470/3433/24753 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -2166,10 +2178,14 @@
       <c r="J74" s="33" t="n">
         <v>256.99</v>
       </c>
-      <c r="K74" s="28" t="n"/>
+      <c r="K74" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L74" s="32" t="inlineStr">
         <is>
-          <t>Facture 440/7222/59244</t>
+          <t>Facture 440/7222/59244 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -3660,10 +3676,14 @@
       <c r="J150" s="33" t="n">
         <v>256.99</v>
       </c>
-      <c r="K150" s="28" t="n"/>
+      <c r="K150" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L150" s="32" t="inlineStr">
         <is>
-          <t>Facture 439/4769/34444</t>
+          <t>Facture 439/4769/34444 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -4748,10 +4768,14 @@
       <c r="J206" s="33" t="n">
         <v>256.99</v>
       </c>
-      <c r="K206" s="28" t="n"/>
+      <c r="K206" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L206" s="32" t="inlineStr">
         <is>
-          <t>Facture 493/0415/84633</t>
+          <t>Facture 493/0415/84633 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -5920,10 +5944,14 @@
       <c r="J266" s="33" t="n">
         <v>256.99</v>
       </c>
-      <c r="K266" s="28" t="n"/>
+      <c r="K266" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L266" s="32" t="inlineStr">
         <is>
-          <t>Facture 450/5974/91764</t>
+          <t>Facture 450/5974/91764 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -6800,10 +6828,14 @@
       <c r="J311" s="33" t="n">
         <v>356.79</v>
       </c>
-      <c r="K311" s="28" t="n"/>
+      <c r="K311" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L311" s="32" t="inlineStr">
         <is>
-          <t>Décompte annuel (afrekening) — facture 455/1399/88731 ; l'acompte passe ensuite de 256,99 à 263,44</t>
+          <t>Décompte annuel (afrekening) — facture 455/1399/88731 ; l'acompte passe ensuite de 256,99 à 263,44 — Décompte annuel ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -7652,10 +7684,14 @@
       <c r="J356" s="33" t="n">
         <v>263.44</v>
       </c>
-      <c r="K356" s="28" t="n"/>
+      <c r="K356" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L356" s="32" t="inlineStr">
         <is>
-          <t>Facture 412/3802/96359</t>
+          <t>Facture 412/3802/96359 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -8362,10 +8398,14 @@
       <c r="J393" s="33" t="n">
         <v>263.44</v>
       </c>
-      <c r="K393" s="28" t="n"/>
+      <c r="K393" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L393" s="32" t="inlineStr">
         <is>
-          <t>Facture 495/0336/32914</t>
+          <t>Facture 495/0336/32914 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -9006,10 +9046,14 @@
       <c r="J427" s="33" t="n">
         <v>270.94</v>
       </c>
-      <c r="K427" s="28" t="n"/>
+      <c r="K427" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L427" s="32" t="inlineStr">
         <is>
-          <t>Acompte d'août payé en retard le 18-11 : 263,44 + 7,50 de frais de rappel — facture 433/7265/65993</t>
+          <t>Acompte d'août payé en retard le 18-11 : 263,44 + 7,50 de frais de rappel — facture 433/7265/65993 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -9026,10 +9070,14 @@
       <c r="J428" s="33" t="n">
         <v>263.44</v>
       </c>
-      <c r="K428" s="28" t="n"/>
+      <c r="K428" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L428" s="32" t="inlineStr">
         <is>
-          <t>Facture 464/6637/65902</t>
+          <t>Facture 464/6637/65902 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -9502,10 +9550,14 @@
       <c r="J453" s="33" t="n">
         <v>263.44</v>
       </c>
-      <c r="K453" s="28" t="n"/>
+      <c r="K453" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L453" s="32" t="inlineStr">
         <is>
-          <t>Facture 435/0584/57839</t>
+          <t>Facture 435/0584/57839 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : communications structurees des 5 paiements Partena
Quatre cotisations trimestrielles de 1.441,87 et une regularisation de
3.014,00, chacune avec sa reference, pour permettre le pointage avec
l'espace client.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1779,7 +1779,11 @@
         <v>1441.87</v>
       </c>
       <c r="K53" s="28" t="n"/>
-      <c r="L53" s="32" t="n"/>
+      <c r="L53" s="32" t="inlineStr">
+        <is>
+          <t>Cotisation trimestrielle — facture 425/0507/35746</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="E54" s="16" t="n"/>
@@ -2363,7 +2367,11 @@
         <v>3014</v>
       </c>
       <c r="K83" s="28" t="n"/>
-      <c r="L83" s="32" t="n"/>
+      <c r="L83" s="32" t="inlineStr">
+        <is>
+          <t>Régularisation — facture 425/0248/37251</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="E84" s="16" t="n"/>
@@ -4905,7 +4913,11 @@
         <v>1441.87</v>
       </c>
       <c r="K213" s="28" t="n"/>
-      <c r="L213" s="32" t="n"/>
+      <c r="L213" s="32" t="inlineStr">
+        <is>
+          <t>Cotisation trimestrielle — facture 425/0719/16405</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="E214" s="16" t="n"/>
@@ -7669,7 +7681,11 @@
         <v>1441.87</v>
       </c>
       <c r="K355" s="28" t="n"/>
-      <c r="L355" s="32" t="n"/>
+      <c r="L355" s="32" t="inlineStr">
+        <is>
+          <t>Cotisation trimestrielle — facture 425/0896/51742</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="E356" s="16" t="n"/>
@@ -9011,7 +9027,11 @@
         <v>1441.87</v>
       </c>
       <c r="K425" s="28" t="n"/>
-      <c r="L425" s="32" t="n"/>
+      <c r="L425" s="32" t="inlineStr">
+        <is>
+          <t>Cotisation trimestrielle — facture 425/1102/67272</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="E426" s="16" t="n"/>

</xml_diff>

<commit_message>
Bilan 2025 : les 5 lignes Partena passent a V
8.781,48 couverts : quatre cotisations trimestrielles et la regularisation
de mars. Couverture globale : 43 lignes, 15.055,86 sur 88.431,78 (17 %).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1778,10 +1778,14 @@
       <c r="J53" s="33" t="n">
         <v>1441.87</v>
       </c>
-      <c r="K53" s="28" t="n"/>
+      <c r="K53" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L53" s="32" t="inlineStr">
         <is>
-          <t>Cotisation trimestrielle — facture 425/0507/35746</t>
+          <t>Cotisation trimestrielle — facture 425/0507/35746 — Décompte Partena en main</t>
         </is>
       </c>
     </row>
@@ -2366,10 +2370,14 @@
       <c r="J83" s="33" t="n">
         <v>3014</v>
       </c>
-      <c r="K83" s="28" t="n"/>
+      <c r="K83" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L83" s="32" t="inlineStr">
         <is>
-          <t>Régularisation — facture 425/0248/37251</t>
+          <t>Régularisation — facture 425/0248/37251 — Décompte Partena en main</t>
         </is>
       </c>
     </row>
@@ -4912,10 +4920,14 @@
       <c r="J213" s="33" t="n">
         <v>1441.87</v>
       </c>
-      <c r="K213" s="28" t="n"/>
+      <c r="K213" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L213" s="32" t="inlineStr">
         <is>
-          <t>Cotisation trimestrielle — facture 425/0719/16405</t>
+          <t>Cotisation trimestrielle — facture 425/0719/16405 — Décompte Partena en main</t>
         </is>
       </c>
     </row>
@@ -7680,10 +7692,14 @@
       <c r="J355" s="39" t="n">
         <v>1441.87</v>
       </c>
-      <c r="K355" s="28" t="n"/>
+      <c r="K355" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L355" s="32" t="inlineStr">
         <is>
-          <t>Cotisation trimestrielle — facture 425/0896/51742</t>
+          <t>Cotisation trimestrielle — facture 425/0896/51742 — Décompte Partena en main</t>
         </is>
       </c>
     </row>
@@ -9026,10 +9042,14 @@
       <c r="J425" s="33" t="n">
         <v>1441.87</v>
       </c>
-      <c r="K425" s="28" t="n"/>
+      <c r="K425" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L425" s="32" t="inlineStr">
         <is>
-          <t>Cotisation trimestrielle — facture 425/1102/67272</t>
+          <t>Cotisation trimestrielle — facture 425/1102/67272 — Décompte Partena en main</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : SD Worx et precompte salarial coches
24 lignes (12 decomptes SD Worx, 12 fiches de precompte), deja chargees
dans Billtobox. Couverture : 67 lignes, 46.037,31 sur 88.431,78 (52 %).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1262,8 +1262,16 @@
       <c r="J26" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K26" s="28" t="n"/>
-      <c r="L26" s="32" t="n"/>
+      <c r="K26" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L26" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="E27" s="16" t="n"/>
@@ -1358,8 +1366,16 @@
       <c r="J31" s="33" t="n">
         <v>331.52</v>
       </c>
-      <c r="K31" s="28" t="n"/>
-      <c r="L31" s="32" t="n"/>
+      <c r="K31" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L31" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="E32" s="16" t="n"/>
@@ -1906,8 +1922,16 @@
       <c r="J59" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K59" s="28" t="n"/>
-      <c r="L59" s="32" t="n"/>
+      <c r="K59" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L59" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="E60" s="16" t="n"/>
@@ -1922,8 +1946,16 @@
       <c r="J60" s="33" t="n">
         <v>331.52</v>
       </c>
-      <c r="K60" s="28" t="n"/>
-      <c r="L60" s="32" t="n"/>
+      <c r="K60" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L60" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="E61" s="16" t="n"/>
@@ -2502,8 +2534,16 @@
       <c r="J89" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K89" s="28" t="n"/>
-      <c r="L89" s="32" t="n"/>
+      <c r="K89" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L89" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="E90" s="16" t="n"/>
@@ -2518,8 +2558,16 @@
       <c r="J90" s="33" t="n">
         <v>331.52</v>
       </c>
-      <c r="K90" s="28" t="n"/>
-      <c r="L90" s="32" t="n"/>
+      <c r="K90" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L90" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="E91" s="16" t="n"/>
@@ -3840,8 +3888,16 @@
       <c r="J158" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K158" s="28" t="n"/>
-      <c r="L158" s="32" t="n"/>
+      <c r="K158" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L158" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="E159" s="16" t="n"/>
@@ -3856,8 +3912,16 @@
       <c r="J159" s="33" t="n">
         <v>331.99</v>
       </c>
-      <c r="K159" s="28" t="n"/>
-      <c r="L159" s="32" t="n"/>
+      <c r="K159" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L159" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="E160" s="16" t="n"/>
@@ -4904,8 +4968,16 @@
       <c r="J212" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K212" s="28" t="n"/>
-      <c r="L212" s="32" t="n"/>
+      <c r="K212" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L212" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="E213" s="16" t="n"/>
@@ -4944,8 +5016,16 @@
       <c r="J214" s="33" t="n">
         <v>331.99</v>
       </c>
-      <c r="K214" s="28" t="n"/>
-      <c r="L214" s="32" t="n"/>
+      <c r="K214" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L214" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="E215" s="16" t="n"/>
@@ -6098,8 +6178,16 @@
       <c r="J273" s="39" t="n">
         <v>2250</v>
       </c>
-      <c r="K273" s="28" t="n"/>
-      <c r="L273" s="32" t="n"/>
+      <c r="K273" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L273" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="E274" s="16" t="n"/>
@@ -6124,8 +6212,16 @@
       <c r="J274" s="33" t="n">
         <v>331.99</v>
       </c>
-      <c r="K274" s="28" t="n"/>
-      <c r="L274" s="32" t="n"/>
+      <c r="K274" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L274" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="E275" s="16" t="n"/>
@@ -7054,8 +7150,16 @@
       <c r="J322" s="39" t="n">
         <v>2250</v>
       </c>
-      <c r="K322" s="28" t="n"/>
-      <c r="L322" s="32" t="n"/>
+      <c r="K322" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L322" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="E323" s="16" t="n"/>
@@ -7070,8 +7174,16 @@
       <c r="J323" s="33" t="n">
         <v>331.79</v>
       </c>
-      <c r="K323" s="28" t="n"/>
-      <c r="L323" s="32" t="n"/>
+      <c r="K323" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L323" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="E324" s="16" t="n"/>
@@ -7776,8 +7888,16 @@
       <c r="J359" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K359" s="28" t="n"/>
-      <c r="L359" s="32" t="n"/>
+      <c r="K359" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L359" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="E360" s="16" t="n"/>
@@ -7792,8 +7912,16 @@
       <c r="J360" s="33" t="n">
         <v>331.79</v>
       </c>
-      <c r="K360" s="28" t="n"/>
-      <c r="L360" s="32" t="n"/>
+      <c r="K360" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L360" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="E361" s="16" t="n"/>
@@ -8286,8 +8414,16 @@
       <c r="J385" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K385" s="28" t="n"/>
-      <c r="L385" s="32" t="n"/>
+      <c r="K385" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L385" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="E386" s="16" t="n"/>
@@ -8302,8 +8438,16 @@
       <c r="J386" s="33" t="n">
         <v>331.79</v>
       </c>
-      <c r="K386" s="28" t="n"/>
-      <c r="L386" s="32" t="n"/>
+      <c r="K386" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L386" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="E387" s="16" t="n"/>
@@ -8914,8 +9058,16 @@
       <c r="J418" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K418" s="28" t="n"/>
-      <c r="L418" s="32" t="n"/>
+      <c r="K418" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L418" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="E419" s="16" t="n"/>
@@ -8930,8 +9082,16 @@
       <c r="J419" s="33" t="n">
         <v>331.85</v>
       </c>
-      <c r="K419" s="28" t="n"/>
-      <c r="L419" s="32" t="n"/>
+      <c r="K419" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L419" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="420">
       <c r="E420" s="16" t="n"/>
@@ -9396,8 +9556,16 @@
       <c r="J443" s="39" t="n">
         <v>2250</v>
       </c>
-      <c r="K443" s="28" t="n"/>
-      <c r="L443" s="32" t="n"/>
+      <c r="K443" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L443" s="32" t="inlineStr">
+        <is>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="E444" s="16" t="n"/>
@@ -9418,8 +9586,16 @@
       <c r="J444" s="33" t="n">
         <v>331.85</v>
       </c>
-      <c r="K444" s="28" t="n"/>
-      <c r="L444" s="32" t="n"/>
+      <c r="K444" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L444" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="E445" s="16" t="n"/>
@@ -9830,10 +10006,14 @@
       <c r="J465" s="33" t="n">
         <v>2250</v>
       </c>
-      <c r="K465" s="28" t="n"/>
+      <c r="K465" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L465" s="32" t="inlineStr">
         <is>
-          <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024)</t>
+          <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024) — Fiche de précompte — déjà chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -9850,10 +10030,14 @@
       <c r="J466" s="33" t="n">
         <v>331.85</v>
       </c>
-      <c r="K466" s="28" t="n"/>
+      <c r="K466" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L466" s="32" t="inlineStr">
         <is>
-          <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024)</t>
+          <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024) — Décompte SD Worx — déjà chargé dans Billtobox</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : communications structurees des 8 paiements Telenet
Relevees extrait par extrait : trois paiements partagent le montant de
149,10, un rapprochement par montant les intervertissait.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1571,7 +1571,11 @@
         <v>149.1</v>
       </c>
       <c r="K41" s="28" t="n"/>
-      <c r="L41" s="32" t="n"/>
+      <c r="L41" s="32" t="inlineStr">
+        <is>
+          <t>Facture 309/1274/44771</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="E42" s="16" t="n"/>
@@ -2243,7 +2247,11 @@
         <v>149.4</v>
       </c>
       <c r="K75" s="28" t="n"/>
-      <c r="L75" s="32" t="n"/>
+      <c r="L75" s="32" t="inlineStr">
+        <is>
+          <t>Facture 309/3944/58489</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="E76" s="16" t="n"/>
@@ -2885,7 +2893,11 @@
         <v>149.1</v>
       </c>
       <c r="K107" s="28" t="n"/>
-      <c r="L107" s="32" t="n"/>
+      <c r="L107" s="32" t="inlineStr">
+        <is>
+          <t>Facture 309/6596/00616</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="E108" s="16" t="n"/>
@@ -4693,7 +4705,11 @@
         <v>149.1</v>
       </c>
       <c r="K198" s="28" t="n"/>
-      <c r="L198" s="32" t="n"/>
+      <c r="L198" s="32" t="inlineStr">
+        <is>
+          <t>Facture 309/9292/68801</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="E199" s="16" t="n"/>
@@ -5917,7 +5933,11 @@
         <v>155.52</v>
       </c>
       <c r="K259" s="28" t="n"/>
-      <c r="L259" s="32" t="n"/>
+      <c r="L259" s="32" t="inlineStr">
+        <is>
+          <t>Facture 310/1956/94152</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="E260" s="16" t="n"/>
@@ -6973,7 +6993,11 @@
         <v>153.42</v>
       </c>
       <c r="K312" s="28" t="n"/>
-      <c r="L312" s="32" t="n"/>
+      <c r="L312" s="32" t="inlineStr">
+        <is>
+          <t>Facture 310/4609/85819</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="E313" s="16" t="n"/>
@@ -7853,7 +7877,11 @@
         <v>153.42</v>
       </c>
       <c r="K357" s="28" t="n"/>
-      <c r="L357" s="32" t="n"/>
+      <c r="L357" s="32" t="inlineStr">
+        <is>
+          <t>Facture 310/7313/00668</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="E358" s="16" t="n"/>

</xml_diff>

<commit_message>
Bilan 2025 : les 8 lignes Telenet passent a V
Couverture : 75 lignes, 47.255,47 sur 88.431,78 (53 %).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1126,10 +1126,14 @@
       <c r="J19" s="33" t="n">
         <v>159.1</v>
       </c>
-      <c r="K19" s="28" t="n"/>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L19" s="32" t="inlineStr">
         <is>
-          <t>Facture 308/8521/00268</t>
+          <t>Facture 308/8521/00268 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -1570,10 +1574,14 @@
       <c r="J41" s="33" t="n">
         <v>149.1</v>
       </c>
-      <c r="K41" s="28" t="n"/>
+      <c r="K41" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L41" s="32" t="inlineStr">
         <is>
-          <t>Facture 309/1274/44771</t>
+          <t>Facture 309/1274/44771 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -2246,10 +2254,14 @@
       <c r="J75" s="33" t="n">
         <v>149.4</v>
       </c>
-      <c r="K75" s="28" t="n"/>
+      <c r="K75" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L75" s="32" t="inlineStr">
         <is>
-          <t>Facture 309/3944/58489</t>
+          <t>Facture 309/3944/58489 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -2892,10 +2904,14 @@
       <c r="J107" s="33" t="n">
         <v>149.1</v>
       </c>
-      <c r="K107" s="28" t="n"/>
+      <c r="K107" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L107" s="32" t="inlineStr">
         <is>
-          <t>Facture 309/6596/00616</t>
+          <t>Facture 309/6596/00616 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -4704,10 +4720,14 @@
       <c r="J198" s="33" t="n">
         <v>149.1</v>
       </c>
-      <c r="K198" s="28" t="n"/>
+      <c r="K198" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L198" s="32" t="inlineStr">
         <is>
-          <t>Facture 309/9292/68801</t>
+          <t>Facture 309/9292/68801 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -5932,10 +5952,14 @@
       <c r="J259" s="33" t="n">
         <v>155.52</v>
       </c>
-      <c r="K259" s="28" t="n"/>
+      <c r="K259" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L259" s="32" t="inlineStr">
         <is>
-          <t>Facture 310/1956/94152</t>
+          <t>Facture 310/1956/94152 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -6992,10 +7016,14 @@
       <c r="J312" s="33" t="n">
         <v>153.42</v>
       </c>
-      <c r="K312" s="28" t="n"/>
+      <c r="K312" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L312" s="32" t="inlineStr">
         <is>
-          <t>Facture 310/4609/85819</t>
+          <t>Facture 310/4609/85819 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -7876,10 +7904,14 @@
       <c r="J357" s="33" t="n">
         <v>153.42</v>
       </c>
-      <c r="K357" s="28" t="n"/>
+      <c r="K357" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L357" s="32" t="inlineStr">
         <is>
-          <t>Facture 310/7313/00668</t>
+          <t>Facture 310/7313/00668 — Facture Telenet en main</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : communications structurees des 11 paiements Proximus
Relevees extrait par extrait. Un 12e paiement figure sur l'extrait de
janvier (82,99, comm 740/7360/50629) mais appartient au bilan 2024.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1435,7 +1435,11 @@
         <v>70.18000000000001</v>
       </c>
       <c r="K34" s="28" t="n"/>
-      <c r="L34" s="32" t="n"/>
+      <c r="L34" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/1364/96037</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="G35" s="37" t="n"/>
@@ -2003,7 +2007,11 @@
         <v>49.98</v>
       </c>
       <c r="K62" s="28" t="n"/>
-      <c r="L62" s="32" t="n"/>
+      <c r="L62" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/1903/98331</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="G63" s="37" t="n"/>
@@ -2869,7 +2877,11 @@
         <v>141.5</v>
       </c>
       <c r="K105" s="28" t="n"/>
-      <c r="L105" s="32" t="n"/>
+      <c r="L105" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/2441/84528</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="E106" s="16" t="n"/>
@@ -3981,7 +3993,11 @@
         <v>71.54000000000001</v>
       </c>
       <c r="K161" s="28" t="n"/>
-      <c r="L161" s="32" t="n"/>
+      <c r="L161" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/2981/21578</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="E162" s="16" t="n"/>
@@ -5977,7 +5993,11 @@
         <v>64.94</v>
       </c>
       <c r="K260" s="28" t="n"/>
-      <c r="L260" s="32" t="n"/>
+      <c r="L260" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/3518/42505</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="E261" s="16" t="n"/>
@@ -6281,7 +6301,11 @@
         <v>84.91</v>
       </c>
       <c r="K275" s="28" t="n"/>
-      <c r="L275" s="32" t="n"/>
+      <c r="L275" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/4054/27527</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="E276" s="16" t="n"/>
@@ -8029,7 +8053,11 @@
         <v>70.62</v>
       </c>
       <c r="K363" s="28" t="n"/>
-      <c r="L363" s="32" t="n"/>
+      <c r="L363" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/5179/27218</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="E364" s="16" t="n"/>
@@ -8171,7 +8199,7 @@
       <c r="K370" s="28" t="n"/>
       <c r="L370" s="32" t="inlineStr">
         <is>
-          <t>2e facture du mois</t>
+          <t>Facture 750/5709/83285 — 2e facture du mois</t>
         </is>
       </c>
     </row>
@@ -9003,7 +9031,11 @@
         <v>148.72</v>
       </c>
       <c r="K411" s="28" t="n"/>
-      <c r="L411" s="32" t="n"/>
+      <c r="L411" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/6239/84691</t>
+        </is>
+      </c>
     </row>
     <row r="412">
       <c r="E412" s="16" t="n"/>
@@ -9355,7 +9387,11 @@
         <v>143.48</v>
       </c>
       <c r="K429" s="28" t="n"/>
-      <c r="L429" s="32" t="n"/>
+      <c r="L429" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/6769/40530</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="E430" s="16" t="n"/>
@@ -9851,7 +9887,11 @@
         <v>153.79</v>
       </c>
       <c r="K454" s="28" t="n"/>
-      <c r="L454" s="32" t="n"/>
+      <c r="L454" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/7299/18694</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="E455" s="16" t="n"/>

</xml_diff>

<commit_message>
Bilan 2025 : facture Proximus payee a titre prive inscrite en juillet
La facture 7504645054 de 109,59 n'est sortie d'aucun compte de la societe :
elle est inscrite en charge, avec en contrepartie une entree « prise en
charge par T. Duchene ». Les deux se compensent, le mois se rapproche
toujours du solde bancaire et le resultat de l'annee ne bouge pas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -764,7 +764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D1:L469"/>
+  <dimension ref="D1:L470"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="37.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
@@ -6223,15 +6223,15 @@
       </c>
       <c r="F273" s="40" t="inlineStr">
         <is>
-          <t>Remboursement paiement à Sandaya</t>
+          <t>Prise en charge par T. Duchène - facture Proximus 7504645054</t>
         </is>
       </c>
       <c r="G273" s="41" t="n">
-        <v>1775.4</v>
+        <v>109.59</v>
       </c>
       <c r="H273" s="36" t="inlineStr">
         <is>
-          <t>Versement de Thibault Duchène — dépense privée payée par la société ?</t>
+          <t>Contrepartie de la facture payée à titre privé — à traiter en compte courant</t>
         </is>
       </c>
       <c r="I273" s="28" t="inlineStr">
@@ -6255,17 +6255,17 @@
     </row>
     <row r="274">
       <c r="E274" s="16" t="n"/>
-      <c r="F274" s="17" t="inlineStr">
-        <is>
-          <t>LAM2509</t>
-        </is>
-      </c>
-      <c r="G274" s="31" t="n">
-        <v>7130</v>
-      </c>
-      <c r="H274" s="32" t="inlineStr">
-        <is>
-          <t>Virement du 24-07, communication « Prestations juillet 2025 »</t>
+      <c r="F274" s="40" t="inlineStr">
+        <is>
+          <t>Remboursement paiement à Sandaya</t>
+        </is>
+      </c>
+      <c r="G274" s="41" t="n">
+        <v>1775.4</v>
+      </c>
+      <c r="H274" s="36" t="inlineStr">
+        <is>
+          <t>Versement de Thibault Duchène — dépense privée payée par la société ?</t>
         </is>
       </c>
       <c r="I274" s="13" t="inlineStr">
@@ -6289,9 +6289,19 @@
     </row>
     <row r="275">
       <c r="E275" s="16" t="n"/>
-      <c r="F275" s="17" t="n"/>
-      <c r="G275" s="31" t="n"/>
-      <c r="H275" s="32" t="n"/>
+      <c r="F275" s="17" t="inlineStr">
+        <is>
+          <t>LAM2509</t>
+        </is>
+      </c>
+      <c r="G275" s="31" t="n">
+        <v>7130</v>
+      </c>
+      <c r="H275" s="32" t="inlineStr">
+        <is>
+          <t>Virement du 24-07, communication « Prestations juillet 2025 »</t>
+        </is>
+      </c>
       <c r="I275" s="13" t="inlineStr">
         <is>
           <t>Proximus</t>
@@ -6314,14 +6324,18 @@
       <c r="H276" s="32" t="n"/>
       <c r="I276" s="13" t="inlineStr">
         <is>
-          <t>Crédit voiture</t>
+          <t>Proximus</t>
         </is>
       </c>
       <c r="J276" s="33" t="n">
-        <v>724.12</v>
+        <v>109.59</v>
       </c>
       <c r="K276" s="28" t="n"/>
-      <c r="L276" s="32" t="n"/>
+      <c r="L276" s="32" t="inlineStr">
+        <is>
+          <t>Facture 7504645054 payée par QR code depuis le compte privé de T. Duchène — hors extrait bancaire</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="E277" s="16" t="n"/>
@@ -6330,11 +6344,11 @@
       <c r="H277" s="32" t="n"/>
       <c r="I277" s="13" t="inlineStr">
         <is>
-          <t>Frais bancaires trimestriels</t>
+          <t>Crédit voiture</t>
         </is>
       </c>
       <c r="J277" s="33" t="n">
-        <v>11.25</v>
+        <v>724.12</v>
       </c>
       <c r="K277" s="28" t="n"/>
       <c r="L277" s="32" t="n"/>
@@ -6346,18 +6360,14 @@
       <c r="H278" s="32" t="n"/>
       <c r="I278" s="13" t="inlineStr">
         <is>
-          <t>Intérêt crédit</t>
+          <t>Frais bancaires trimestriels</t>
         </is>
       </c>
       <c r="J278" s="33" t="n">
-        <v>0.51</v>
+        <v>11.25</v>
       </c>
       <c r="K278" s="28" t="n"/>
-      <c r="L278" s="32" t="inlineStr">
-        <is>
-          <t>Intérêts nets au 01-07</t>
-        </is>
-      </c>
+      <c r="L278" s="32" t="n"/>
     </row>
     <row r="279">
       <c r="E279" s="16" t="n"/>
@@ -6366,16 +6376,16 @@
       <c r="H279" s="32" t="n"/>
       <c r="I279" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Intérêt crédit</t>
         </is>
       </c>
       <c r="J279" s="33" t="n">
-        <v>60.86</v>
+        <v>0.51</v>
       </c>
       <c r="K279" s="28" t="n"/>
       <c r="L279" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Intérêts nets au 01-07</t>
         </is>
       </c>
     </row>
@@ -6386,16 +6396,16 @@
       <c r="H280" s="32" t="n"/>
       <c r="I280" s="13" t="inlineStr">
         <is>
-          <t>Assurance voiture</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J280" s="33" t="n">
-        <v>458.66</v>
+        <v>60.86</v>
       </c>
       <c r="K280" s="28" t="n"/>
       <c r="L280" s="32" t="inlineStr">
         <is>
-          <t>Domiciliation AG Insurance — prime passée de 431,25 à 458,66</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -6406,16 +6416,16 @@
       <c r="H281" s="32" t="n"/>
       <c r="I281" s="13" t="inlineStr">
         <is>
-          <t>Publicité Facebook</t>
+          <t>Assurance voiture</t>
         </is>
       </c>
       <c r="J281" s="33" t="n">
-        <v>20.78</v>
+        <v>458.66</v>
       </c>
       <c r="K281" s="28" t="n"/>
       <c r="L281" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 01-06 — décompte n° 182 du 10-07</t>
+          <t>Domiciliation AG Insurance — prime passée de 431,25 à 458,66</t>
         </is>
       </c>
     </row>
@@ -6426,16 +6436,16 @@
       <c r="H282" s="32" t="n"/>
       <c r="I282" s="13" t="inlineStr">
         <is>
-          <t>Achat Delhaize Wezembeek</t>
+          <t>Publicité Facebook</t>
         </is>
       </c>
       <c r="J282" s="33" t="n">
-        <v>5.67</v>
+        <v>20.78</v>
       </c>
       <c r="K282" s="28" t="n"/>
       <c r="L282" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 03-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 01-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6450,7 +6460,7 @@
         </is>
       </c>
       <c r="J283" s="33" t="n">
-        <v>0.92</v>
+        <v>5.67</v>
       </c>
       <c r="K283" s="28" t="n"/>
       <c r="L283" s="32" t="inlineStr">
@@ -6466,11 +6476,11 @@
       <c r="H284" s="32" t="n"/>
       <c r="I284" s="13" t="inlineStr">
         <is>
-          <t>Transport - De Lijn</t>
+          <t>Achat Delhaize Wezembeek</t>
         </is>
       </c>
       <c r="J284" s="33" t="n">
-        <v>6</v>
+        <v>0.92</v>
       </c>
       <c r="K284" s="28" t="n"/>
       <c r="L284" s="32" t="inlineStr">
@@ -6490,12 +6500,12 @@
         </is>
       </c>
       <c r="J285" s="33" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K285" s="28" t="n"/>
       <c r="L285" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 04-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 03-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6506,11 +6516,11 @@
       <c r="H286" s="32" t="n"/>
       <c r="I286" s="13" t="inlineStr">
         <is>
-          <t>Transport - STIB</t>
+          <t>Transport - De Lijn</t>
         </is>
       </c>
       <c r="J286" s="33" t="n">
-        <v>2.3</v>
+        <v>9</v>
       </c>
       <c r="K286" s="28" t="n"/>
       <c r="L286" s="32" t="inlineStr">
@@ -6526,16 +6536,16 @@
       <c r="H287" s="32" t="n"/>
       <c r="I287" s="13" t="inlineStr">
         <is>
-          <t>Transport - De Lijn</t>
+          <t>Transport - STIB</t>
         </is>
       </c>
       <c r="J287" s="33" t="n">
-        <v>12</v>
+        <v>2.3</v>
       </c>
       <c r="K287" s="28" t="n"/>
       <c r="L287" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 05-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 04-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6550,12 +6560,12 @@
         </is>
       </c>
       <c r="J288" s="33" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K288" s="28" t="n"/>
       <c r="L288" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 06-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 05-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6566,16 +6576,16 @@
       <c r="H289" s="32" t="n"/>
       <c r="I289" s="13" t="inlineStr">
         <is>
-          <t>Abonnement Shopify</t>
+          <t>Transport - De Lijn</t>
         </is>
       </c>
       <c r="J289" s="33" t="n">
-        <v>27.96</v>
+        <v>6</v>
       </c>
       <c r="K289" s="28" t="n"/>
       <c r="L289" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 06-06 — décompte n° 182 du 10-07 — 31,38 USD - facture 375321628</t>
+          <t>Carte Visa 06-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6586,16 +6596,16 @@
       <c r="H290" s="32" t="n"/>
       <c r="I290" s="13" t="inlineStr">
         <is>
-          <t>Transport - STIB</t>
+          <t>Abonnement Shopify</t>
         </is>
       </c>
       <c r="J290" s="33" t="n">
-        <v>6.9</v>
+        <v>27.96</v>
       </c>
       <c r="K290" s="28" t="n"/>
       <c r="L290" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 06-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 06-06 — décompte n° 182 du 10-07 — 31,38 USD - facture 375321628</t>
         </is>
       </c>
     </row>
@@ -6606,16 +6616,16 @@
       <c r="H291" s="32" t="n"/>
       <c r="I291" s="13" t="inlineStr">
         <is>
-          <t>Transport - De Lijn</t>
+          <t>Transport - STIB</t>
         </is>
       </c>
       <c r="J291" s="33" t="n">
-        <v>18</v>
+        <v>6.9</v>
       </c>
       <c r="K291" s="28" t="n"/>
       <c r="L291" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 07-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 06-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6626,16 +6636,16 @@
       <c r="H292" s="32" t="n"/>
       <c r="I292" s="13" t="inlineStr">
         <is>
-          <t>Achat - Carrefour Bruxelles</t>
+          <t>Transport - De Lijn</t>
         </is>
       </c>
       <c r="J292" s="33" t="n">
-        <v>4.79</v>
+        <v>18</v>
       </c>
       <c r="K292" s="28" t="n"/>
       <c r="L292" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 08-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 07-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6646,11 +6656,11 @@
       <c r="H293" s="32" t="n"/>
       <c r="I293" s="13" t="inlineStr">
         <is>
-          <t>Repas - Dal Long Yi, Bruxelles</t>
+          <t>Achat - Carrefour Bruxelles</t>
         </is>
       </c>
       <c r="J293" s="33" t="n">
-        <v>9.4</v>
+        <v>4.79</v>
       </c>
       <c r="K293" s="28" t="n"/>
       <c r="L293" s="32" t="inlineStr">
@@ -6664,18 +6674,18 @@
       <c r="F294" s="17" t="n"/>
       <c r="G294" s="31" t="n"/>
       <c r="H294" s="32" t="n"/>
-      <c r="I294" s="34" t="inlineStr">
-        <is>
-          <t>Achat - Proxy Meiser, Schaerbeek</t>
-        </is>
-      </c>
-      <c r="J294" s="35" t="n">
-        <v>33.84</v>
+      <c r="I294" s="13" t="inlineStr">
+        <is>
+          <t>Repas - Dal Long Yi, Bruxelles</t>
+        </is>
+      </c>
+      <c r="J294" s="33" t="n">
+        <v>9.4</v>
       </c>
       <c r="K294" s="28" t="n"/>
-      <c r="L294" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 09-06 — décompte n° 182 du 10-07 — nature de l'achat à préciser</t>
+      <c r="L294" s="32" t="inlineStr">
+        <is>
+          <t>Carte Visa 08-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6684,18 +6694,18 @@
       <c r="F295" s="17" t="n"/>
       <c r="G295" s="31" t="n"/>
       <c r="H295" s="32" t="n"/>
-      <c r="I295" s="13" t="inlineStr">
-        <is>
-          <t>Transport - De Lijn</t>
-        </is>
-      </c>
-      <c r="J295" s="33" t="n">
-        <v>3</v>
+      <c r="I295" s="34" t="inlineStr">
+        <is>
+          <t>Achat - Proxy Meiser, Schaerbeek</t>
+        </is>
+      </c>
+      <c r="J295" s="35" t="n">
+        <v>33.84</v>
       </c>
       <c r="K295" s="28" t="n"/>
-      <c r="L295" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 10-06 — décompte n° 182 du 10-07</t>
+      <c r="L295" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 09-06 — décompte n° 182 du 10-07 — nature de l'achat à préciser</t>
         </is>
       </c>
     </row>
@@ -6710,12 +6720,12 @@
         </is>
       </c>
       <c r="J296" s="33" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K296" s="28" t="n"/>
       <c r="L296" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 11-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 10-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6730,12 +6740,12 @@
         </is>
       </c>
       <c r="J297" s="33" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="K297" s="28" t="n"/>
       <c r="L297" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 12-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 11-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6750,12 +6760,12 @@
         </is>
       </c>
       <c r="J298" s="33" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K298" s="28" t="n"/>
       <c r="L298" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 17-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 12-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6785,7 @@
       <c r="K299" s="28" t="n"/>
       <c r="L299" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 18-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 17-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6795,7 +6805,7 @@
       <c r="K300" s="28" t="n"/>
       <c r="L300" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 19-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 18-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6806,16 +6816,16 @@
       <c r="H301" s="32" t="n"/>
       <c r="I301" s="13" t="inlineStr">
         <is>
-          <t>Transport - STIB</t>
+          <t>Transport - De Lijn</t>
         </is>
       </c>
       <c r="J301" s="33" t="n">
-        <v>2.3</v>
+        <v>6</v>
       </c>
       <c r="K301" s="28" t="n"/>
       <c r="L301" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 20-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 19-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6826,16 +6836,16 @@
       <c r="H302" s="32" t="n"/>
       <c r="I302" s="13" t="inlineStr">
         <is>
-          <t>Transport - De Lijn</t>
+          <t>Transport - STIB</t>
         </is>
       </c>
       <c r="J302" s="33" t="n">
-        <v>6</v>
+        <v>2.3</v>
       </c>
       <c r="K302" s="28" t="n"/>
       <c r="L302" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 21-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 20-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6850,12 +6860,12 @@
         </is>
       </c>
       <c r="J303" s="33" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K303" s="28" t="n"/>
       <c r="L303" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 23-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 21-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6870,12 +6880,12 @@
         </is>
       </c>
       <c r="J304" s="33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K304" s="28" t="n"/>
       <c r="L304" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 25-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 23-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6890,12 +6900,12 @@
         </is>
       </c>
       <c r="J305" s="33" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K305" s="28" t="n"/>
       <c r="L305" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 27-06 — décompte n° 182 du 10-07</t>
+          <t>Carte Visa 25-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6906,20 +6916,16 @@
       <c r="H306" s="32" t="n"/>
       <c r="I306" s="13" t="inlineStr">
         <is>
-          <t>Consommation club de tennis Orée</t>
+          <t>Transport - De Lijn</t>
         </is>
       </c>
       <c r="J306" s="33" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="K306" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K306" s="28" t="n"/>
       <c r="L306" s="32" t="inlineStr">
         <is>
-          <t>Justificatif : 2025-07-10_Oree-ASBL_8.50.pdf</t>
+          <t>Carte Visa 27-06 — décompte n° 182 du 10-07</t>
         </is>
       </c>
     </row>
@@ -6930,16 +6936,20 @@
       <c r="H307" s="32" t="n"/>
       <c r="I307" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Consommation club de tennis Orée</t>
         </is>
       </c>
       <c r="J307" s="33" t="n">
-        <v>56.98</v>
-      </c>
-      <c r="K307" s="28" t="n"/>
+        <v>8.5</v>
+      </c>
+      <c r="K307" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L307" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Justificatif : 2025-07-10_Oree-ASBL_8.50.pdf</t>
         </is>
       </c>
     </row>
@@ -6954,7 +6964,7 @@
         </is>
       </c>
       <c r="J308" s="33" t="n">
-        <v>62.27</v>
+        <v>56.98</v>
       </c>
       <c r="K308" s="28" t="n"/>
       <c r="L308" s="32" t="inlineStr">
@@ -6970,16 +6980,16 @@
       <c r="H309" s="32" t="n"/>
       <c r="I309" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J309" s="33" t="n">
-        <v>1.6</v>
+        <v>62.27</v>
       </c>
       <c r="K309" s="28" t="n"/>
       <c r="L309" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -6990,16 +7000,16 @@
       <c r="H310" s="32" t="n"/>
       <c r="I310" s="13" t="inlineStr">
         <is>
-          <t>Péage autoroute France</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J310" s="33" t="n">
-        <v>34.4</v>
+        <v>1.6</v>
       </c>
       <c r="K310" s="28" t="n"/>
       <c r="L310" s="32" t="inlineStr">
         <is>
-          <t>Domiciliation Autoroutes du Sud de la France</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -7010,20 +7020,16 @@
       <c r="H311" s="32" t="n"/>
       <c r="I311" s="13" t="inlineStr">
         <is>
-          <t>Electrabel</t>
+          <t>Péage autoroute France</t>
         </is>
       </c>
       <c r="J311" s="33" t="n">
-        <v>356.79</v>
-      </c>
-      <c r="K311" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>34.4</v>
+      </c>
+      <c r="K311" s="28" t="n"/>
       <c r="L311" s="32" t="inlineStr">
         <is>
-          <t>Décompte annuel (afrekening) — facture 455/1399/88731 ; l'acompte passe ensuite de 256,99 à 263,44 — Décompte annuel ENGIE en main</t>
+          <t>Domiciliation Autoroutes du Sud de la France</t>
         </is>
       </c>
     </row>
@@ -7034,11 +7040,11 @@
       <c r="H312" s="32" t="n"/>
       <c r="I312" s="13" t="inlineStr">
         <is>
-          <t>Telenet</t>
+          <t>Electrabel</t>
         </is>
       </c>
       <c r="J312" s="33" t="n">
-        <v>153.42</v>
+        <v>356.79</v>
       </c>
       <c r="K312" s="28" t="inlineStr">
         <is>
@@ -7047,7 +7053,7 @@
       </c>
       <c r="L312" s="32" t="inlineStr">
         <is>
-          <t>Facture 310/4609/85819 — Facture Telenet en main</t>
+          <t>Décompte annuel (afrekening) — facture 455/1399/88731 ; l'acompte passe ensuite de 256,99 à 263,44 — Décompte annuel ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -7058,16 +7064,20 @@
       <c r="H313" s="32" t="n"/>
       <c r="I313" s="13" t="inlineStr">
         <is>
-          <t>Amende de stationnement - Saint-Josse</t>
+          <t>Telenet</t>
         </is>
       </c>
       <c r="J313" s="33" t="n">
-        <v>100</v>
-      </c>
-      <c r="K313" s="28" t="n"/>
+        <v>153.42</v>
+      </c>
+      <c r="K313" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L313" s="32" t="inlineStr">
         <is>
-          <t>Amende — dépense non admise, comm. 500/2300/37391</t>
+          <t>Facture 310/4609/85819 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -7078,16 +7088,16 @@
       <c r="H314" s="32" t="n"/>
       <c r="I314" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Amende de stationnement - Saint-Josse</t>
         </is>
       </c>
       <c r="J314" s="33" t="n">
-        <v>60.9</v>
+        <v>100</v>
       </c>
       <c r="K314" s="28" t="n"/>
       <c r="L314" s="32" t="inlineStr">
         <is>
-          <t>Maes Schaerbeek</t>
+          <t>Amende — dépense non admise, comm. 500/2300/37391</t>
         </is>
       </c>
     </row>
@@ -7098,16 +7108,16 @@
       <c r="H315" s="32" t="n"/>
       <c r="I315" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J315" s="33" t="n">
-        <v>1.6</v>
+        <v>60.9</v>
       </c>
       <c r="K315" s="28" t="n"/>
       <c r="L315" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Maes Schaerbeek</t>
         </is>
       </c>
     </row>
@@ -7118,14 +7128,18 @@
       <c r="H316" s="32" t="n"/>
       <c r="I316" s="13" t="inlineStr">
         <is>
-          <t>Repas Topogigio</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J316" s="33" t="n">
-        <v>231.5</v>
+        <v>1.6</v>
       </c>
       <c r="K316" s="28" t="n"/>
-      <c r="L316" s="32" t="n"/>
+      <c r="L316" s="32" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="E317" s="16" t="n"/>
@@ -7134,18 +7148,14 @@
       <c r="H317" s="32" t="n"/>
       <c r="I317" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Repas Topogigio</t>
         </is>
       </c>
       <c r="J317" s="33" t="n">
-        <v>43.01</v>
+        <v>231.5</v>
       </c>
       <c r="K317" s="28" t="n"/>
-      <c r="L317" s="32" t="inlineStr">
-        <is>
-          <t>Esso Rumst</t>
-        </is>
-      </c>
+      <c r="L317" s="32" t="n"/>
     </row>
     <row r="318">
       <c r="E318" s="16" t="n"/>
@@ -7154,16 +7164,16 @@
       <c r="H318" s="32" t="n"/>
       <c r="I318" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J318" s="33" t="n">
-        <v>1.7</v>
+        <v>43.01</v>
       </c>
       <c r="K318" s="28" t="n"/>
       <c r="L318" s="32" t="inlineStr">
         <is>
-          <t>Indigo, Tours (France)</t>
+          <t>Esso Rumst</t>
         </is>
       </c>
     </row>
@@ -7178,20 +7188,34 @@
         </is>
       </c>
       <c r="J319" s="33" t="n">
-        <v>2.8</v>
+        <v>1.7</v>
       </c>
       <c r="K319" s="28" t="n"/>
       <c r="L319" s="32" t="inlineStr">
         <is>
+          <t>Indigo, Tours (France)</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="E320" s="16" t="n"/>
+      <c r="F320" s="17" t="n"/>
+      <c r="G320" s="31" t="n"/>
+      <c r="H320" s="32" t="n"/>
+      <c r="I320" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="J320" s="33" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K320" s="28" t="n"/>
+      <c r="L320" s="32" t="inlineStr">
+        <is>
           <t>Commune de Soulac-sur-Mer (France)</t>
         </is>
       </c>
-    </row>
-    <row r="320">
-      <c r="G320" s="37" t="n"/>
-      <c r="H320" s="38" t="n"/>
-      <c r="J320" s="37" t="n"/>
-      <c r="L320" s="38" t="n"/>
     </row>
     <row r="321">
       <c r="G321" s="37" t="n"/>
@@ -7200,64 +7224,46 @@
       <c r="L321" s="38" t="n"/>
     </row>
     <row r="322">
-      <c r="E322" s="16" t="inlineStr">
+      <c r="G322" s="37" t="n"/>
+      <c r="H322" s="38" t="n"/>
+      <c r="J322" s="37" t="n"/>
+      <c r="L322" s="38" t="n"/>
+    </row>
+    <row r="323">
+      <c r="E323" s="16" t="inlineStr">
         <is>
           <t>Août</t>
         </is>
       </c>
-      <c r="F322" s="17" t="inlineStr">
+      <c r="F323" s="17" t="inlineStr">
         <is>
           <t>Remboursement achat Decathlon - RTC Lambermont</t>
         </is>
       </c>
-      <c r="G322" s="31" t="n">
+      <c r="G323" s="31" t="n">
         <v>123</v>
       </c>
-      <c r="H322" s="32" t="inlineStr">
+      <c r="H323" s="32" t="inlineStr">
         <is>
           <t>Contrepartie de l'achat Decathlon du 14-08</t>
         </is>
       </c>
-      <c r="I322" s="28" t="inlineStr">
+      <c r="I323" s="28" t="inlineStr">
         <is>
           <t>Précompte salarial juillet 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J322" s="39" t="n">
+      <c r="J323" s="39" t="n">
         <v>2250</v>
       </c>
-      <c r="K322" s="28" t="inlineStr">
+      <c r="K323" s="28" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L322" s="32" t="inlineStr">
+      <c r="L323" s="32" t="inlineStr">
         <is>
           <t>Fiche de précompte — déjà chargée dans Billtobox</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="E323" s="16" t="n"/>
-      <c r="F323" s="17" t="n"/>
-      <c r="G323" s="31" t="n"/>
-      <c r="H323" s="32" t="n"/>
-      <c r="I323" s="13" t="inlineStr">
-        <is>
-          <t>SD Worx</t>
-        </is>
-      </c>
-      <c r="J323" s="33" t="n">
-        <v>331.79</v>
-      </c>
-      <c r="K323" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L323" s="32" t="inlineStr">
-        <is>
-          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -7268,16 +7274,20 @@
       <c r="H324" s="32" t="n"/>
       <c r="I324" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>SD Worx</t>
         </is>
       </c>
       <c r="J324" s="33" t="n">
-        <v>87.43000000000001</v>
-      </c>
-      <c r="K324" s="28" t="n"/>
+        <v>331.79</v>
+      </c>
+      <c r="K324" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L324" s="32" t="inlineStr">
         <is>
-          <t>Soulac-sur-Mer (France)</t>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -7288,14 +7298,18 @@
       <c r="H325" s="32" t="n"/>
       <c r="I325" s="13" t="inlineStr">
         <is>
-          <t>Crédit voiture</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J325" s="33" t="n">
-        <v>724.12</v>
+        <v>87.43000000000001</v>
       </c>
       <c r="K325" s="28" t="n"/>
-      <c r="L325" s="32" t="n"/>
+      <c r="L325" s="32" t="inlineStr">
+        <is>
+          <t>Soulac-sur-Mer (France)</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="E326" s="16" t="n"/>
@@ -7304,18 +7318,14 @@
       <c r="H326" s="32" t="n"/>
       <c r="I326" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Crédit voiture</t>
         </is>
       </c>
       <c r="J326" s="33" t="n">
-        <v>72.01000000000001</v>
+        <v>724.12</v>
       </c>
       <c r="K326" s="28" t="n"/>
-      <c r="L326" s="32" t="inlineStr">
-        <is>
-          <t>BP Esso Saint-Léger (France)</t>
-        </is>
-      </c>
+      <c r="L326" s="32" t="n"/>
     </row>
     <row r="327">
       <c r="E327" s="16" t="n"/>
@@ -7328,12 +7338,12 @@
         </is>
       </c>
       <c r="J327" s="33" t="n">
-        <v>77.28</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="K327" s="28" t="n"/>
       <c r="L327" s="32" t="inlineStr">
         <is>
-          <t>Shell Vémars (France)</t>
+          <t>BP Esso Saint-Léger (France)</t>
         </is>
       </c>
     </row>
@@ -7344,20 +7354,16 @@
       <c r="H328" s="32" t="n"/>
       <c r="I328" s="13" t="inlineStr">
         <is>
-          <t>Achat matériel sportif - DECATHLON</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J328" s="33" t="n">
-        <v>18</v>
-      </c>
-      <c r="K328" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>77.28</v>
+      </c>
+      <c r="K328" s="28" t="n"/>
       <c r="L328" s="32" t="inlineStr">
         <is>
-          <t>Decathlon Evere — Justificatif : 2025-08-08_Decathlon-Evere_18.00.pdf</t>
+          <t>Shell Vémars (France)</t>
         </is>
       </c>
     </row>
@@ -7368,16 +7374,20 @@
       <c r="H329" s="32" t="n"/>
       <c r="I329" s="13" t="inlineStr">
         <is>
-          <t>Publicité Facebook</t>
+          <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
       <c r="J329" s="33" t="n">
-        <v>26.47</v>
-      </c>
-      <c r="K329" s="28" t="n"/>
+        <v>18</v>
+      </c>
+      <c r="K329" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L329" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 01-07 — décompte n° 213 du 11-08</t>
+          <t>Decathlon Evere — Justificatif : 2025-08-08_Decathlon-Evere_18.00.pdf</t>
         </is>
       </c>
     </row>
@@ -7388,16 +7398,16 @@
       <c r="H330" s="32" t="n"/>
       <c r="I330" s="13" t="inlineStr">
         <is>
-          <t>Réception marchandise - FEDEX</t>
+          <t>Publicité Facebook</t>
         </is>
       </c>
       <c r="J330" s="33" t="n">
-        <v>5.51</v>
+        <v>26.47</v>
       </c>
       <c r="K330" s="28" t="n"/>
       <c r="L330" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 04-07 — décompte n° 213 du 11-08 — Envoi 798875231</t>
+          <t>Carte Visa 01-07 — décompte n° 213 du 11-08</t>
         </is>
       </c>
     </row>
@@ -7408,16 +7418,16 @@
       <c r="H331" s="32" t="n"/>
       <c r="I331" s="13" t="inlineStr">
         <is>
-          <t>Abonnement Shopify</t>
+          <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
       <c r="J331" s="33" t="n">
-        <v>22.48</v>
+        <v>5.51</v>
       </c>
       <c r="K331" s="28" t="n"/>
       <c r="L331" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 06-07 — décompte n° 213 du 11-08 — 26,00 USD - facture 387615031</t>
+          <t>Carte Visa 04-07 — décompte n° 213 du 11-08 — Envoi 798875231</t>
         </is>
       </c>
     </row>
@@ -7428,16 +7438,16 @@
       <c r="H332" s="32" t="n"/>
       <c r="I332" s="13" t="inlineStr">
         <is>
-          <t>Transport - De Lijn</t>
+          <t>Abonnement Shopify</t>
         </is>
       </c>
       <c r="J332" s="33" t="n">
-        <v>6</v>
+        <v>22.48</v>
       </c>
       <c r="K332" s="28" t="n"/>
       <c r="L332" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 10-07 — décompte n° 213 du 11-08</t>
+          <t>Carte Visa 06-07 — décompte n° 213 du 11-08 — 26,00 USD - facture 387615031</t>
         </is>
       </c>
     </row>
@@ -7448,16 +7458,16 @@
       <c r="H333" s="32" t="n"/>
       <c r="I333" s="13" t="inlineStr">
         <is>
-          <t>Séjour Sandaya Lyon</t>
+          <t>Transport - De Lijn</t>
         </is>
       </c>
       <c r="J333" s="33" t="n">
-        <v>1775.4</v>
+        <v>6</v>
       </c>
       <c r="K333" s="28" t="n"/>
       <c r="L333" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 11-07 — décompte n° 213 du 11-08 — Remboursé par T. Duchène le 22-07 (entrée de juillet)</t>
+          <t>Carte Visa 10-07 — décompte n° 213 du 11-08</t>
         </is>
       </c>
     </row>
@@ -7468,16 +7478,16 @@
       <c r="H334" s="32" t="n"/>
       <c r="I334" s="13" t="inlineStr">
         <is>
-          <t>Transport - Uber</t>
+          <t>Séjour Sandaya Lyon</t>
         </is>
       </c>
       <c r="J334" s="33" t="n">
-        <v>42.66</v>
+        <v>1775.4</v>
       </c>
       <c r="K334" s="28" t="n"/>
       <c r="L334" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 14-07 — décompte n° 213 du 11-08</t>
+          <t>Carte Visa 11-07 — décompte n° 213 du 11-08 — Remboursé par T. Duchène le 22-07 (entrée de juillet)</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7502,7 @@
         </is>
       </c>
       <c r="J335" s="33" t="n">
-        <v>48.18</v>
+        <v>42.66</v>
       </c>
       <c r="K335" s="28" t="n"/>
       <c r="L335" s="32" t="inlineStr">
@@ -7512,12 +7522,12 @@
         </is>
       </c>
       <c r="J336" s="33" t="n">
-        <v>111.19</v>
+        <v>48.18</v>
       </c>
       <c r="K336" s="28" t="n"/>
       <c r="L336" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 15-07 — décompte n° 213 du 11-08</t>
+          <t>Carte Visa 14-07 — décompte n° 213 du 11-08</t>
         </is>
       </c>
     </row>
@@ -7532,7 +7542,7 @@
         </is>
       </c>
       <c r="J337" s="33" t="n">
-        <v>91.52</v>
+        <v>111.19</v>
       </c>
       <c r="K337" s="28" t="n"/>
       <c r="L337" s="32" t="inlineStr">
@@ -7548,16 +7558,16 @@
       <c r="H338" s="32" t="n"/>
       <c r="I338" s="13" t="inlineStr">
         <is>
-          <t>Transport - STIB</t>
+          <t>Transport - Uber</t>
         </is>
       </c>
       <c r="J338" s="33" t="n">
-        <v>2.3</v>
+        <v>91.52</v>
       </c>
       <c r="K338" s="28" t="n"/>
       <c r="L338" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 17-07 — décompte n° 213 du 11-08</t>
+          <t>Carte Visa 15-07 — décompte n° 213 du 11-08</t>
         </is>
       </c>
     </row>
@@ -7568,16 +7578,16 @@
       <c r="H339" s="32" t="n"/>
       <c r="I339" s="13" t="inlineStr">
         <is>
-          <t>Transport - De Lijn</t>
+          <t>Transport - STIB</t>
         </is>
       </c>
       <c r="J339" s="33" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="K339" s="28" t="n"/>
       <c r="L339" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 19-07 — décompte n° 213 du 11-08</t>
+          <t>Carte Visa 17-07 — décompte n° 213 du 11-08</t>
         </is>
       </c>
     </row>
@@ -7588,16 +7598,16 @@
       <c r="H340" s="32" t="n"/>
       <c r="I340" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Transport - De Lijn</t>
         </is>
       </c>
       <c r="J340" s="33" t="n">
-        <v>66.73999999999999</v>
+        <v>3</v>
       </c>
       <c r="K340" s="28" t="n"/>
       <c r="L340" s="32" t="inlineStr">
         <is>
-          <t>Carte Mastercard 26-07 — décompte n° 216 du 13-08 — Total Gidy (France)</t>
+          <t>Carte Visa 19-07 — décompte n° 213 du 11-08</t>
         </is>
       </c>
     </row>
@@ -7608,16 +7618,16 @@
       <c r="H341" s="32" t="n"/>
       <c r="I341" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J341" s="33" t="n">
-        <v>1.6</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="K341" s="28" t="n"/>
       <c r="L341" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Carte Mastercard 26-07 — décompte n° 216 du 13-08 — Total Gidy (France)</t>
         </is>
       </c>
     </row>
@@ -7628,20 +7638,16 @@
       <c r="H342" s="32" t="n"/>
       <c r="I342" s="13" t="inlineStr">
         <is>
-          <t>Achat matériel sportif - DECATHLON</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J342" s="33" t="n">
-        <v>123</v>
-      </c>
-      <c r="K342" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>1.6</v>
+      </c>
+      <c r="K342" s="28" t="n"/>
       <c r="L342" s="32" t="inlineStr">
         <is>
-          <t>Decathlon Evere — 28 balles de tennis, remboursé par le RTC Lambermont le même jour — Justificatif : 2025-08-14_Decathlon-Evere_123.00.pdf</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -7652,16 +7658,20 @@
       <c r="H343" s="32" t="n"/>
       <c r="I343" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
       <c r="J343" s="33" t="n">
-        <v>62.86</v>
-      </c>
-      <c r="K343" s="28" t="n"/>
+        <v>123</v>
+      </c>
+      <c r="K343" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L343" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Decathlon Evere — 28 balles de tennis, remboursé par le RTC Lambermont le même jour — Justificatif : 2025-08-14_Decathlon-Evere_123.00.pdf</t>
         </is>
       </c>
     </row>
@@ -7672,16 +7682,16 @@
       <c r="H344" s="32" t="n"/>
       <c r="I344" s="13" t="inlineStr">
         <is>
-          <t>Péage autoroute France</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J344" s="33" t="n">
-        <v>73.90000000000001</v>
+        <v>62.86</v>
       </c>
       <c r="K344" s="28" t="n"/>
       <c r="L344" s="32" t="inlineStr">
         <is>
-          <t>Domiciliation Autoroutes du Sud de la France</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -7692,16 +7702,16 @@
       <c r="H345" s="32" t="n"/>
       <c r="I345" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Péage autoroute France</t>
         </is>
       </c>
       <c r="J345" s="33" t="n">
-        <v>72.59</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="K345" s="28" t="n"/>
       <c r="L345" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Domiciliation Autoroutes du Sud de la France</t>
         </is>
       </c>
     </row>
@@ -7712,16 +7722,16 @@
       <c r="H346" s="32" t="n"/>
       <c r="I346" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J346" s="33" t="n">
-        <v>4.2</v>
+        <v>72.59</v>
       </c>
       <c r="K346" s="28" t="n"/>
       <c r="L346" s="32" t="inlineStr">
         <is>
-          <t>Parking Parkpoort, Heverlee</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -7736,12 +7746,12 @@
         </is>
       </c>
       <c r="J347" s="33" t="n">
-        <v>3</v>
+        <v>4.2</v>
       </c>
       <c r="K347" s="28" t="n"/>
       <c r="L347" s="32" t="inlineStr">
         <is>
-          <t>Parking Ladeuze, Louvain</t>
+          <t>Parking Parkpoort, Heverlee</t>
         </is>
       </c>
     </row>
@@ -7756,12 +7766,12 @@
         </is>
       </c>
       <c r="J348" s="33" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="K348" s="28" t="n"/>
       <c r="L348" s="32" t="inlineStr">
         <is>
-          <t>Indigo Park Docks, Bruxelles</t>
+          <t>Parking Ladeuze, Louvain</t>
         </is>
       </c>
     </row>
@@ -7776,12 +7786,12 @@
         </is>
       </c>
       <c r="J349" s="33" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
       <c r="K349" s="28" t="n"/>
       <c r="L349" s="32" t="inlineStr">
         <is>
-          <t>Parking Bokrijk, Genk</t>
+          <t>Indigo Park Docks, Bruxelles</t>
         </is>
       </c>
     </row>
@@ -7796,12 +7806,12 @@
         </is>
       </c>
       <c r="J350" s="33" t="n">
-        <v>5.55</v>
+        <v>5</v>
       </c>
       <c r="K350" s="28" t="n"/>
       <c r="L350" s="32" t="inlineStr">
         <is>
-          <t>Q-Park Woluwe Esplanade</t>
+          <t>Parking Bokrijk, Genk</t>
         </is>
       </c>
     </row>
@@ -7816,12 +7826,12 @@
         </is>
       </c>
       <c r="J351" s="33" t="n">
-        <v>12</v>
+        <v>5.55</v>
       </c>
       <c r="K351" s="28" t="n"/>
       <c r="L351" s="32" t="inlineStr">
         <is>
-          <t>Brussels Expo Parking</t>
+          <t>Q-Park Woluwe Esplanade</t>
         </is>
       </c>
     </row>
@@ -7836,20 +7846,34 @@
         </is>
       </c>
       <c r="J352" s="33" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K352" s="28" t="n"/>
       <c r="L352" s="32" t="inlineStr">
         <is>
+          <t>Brussels Expo Parking</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="E353" s="16" t="n"/>
+      <c r="F353" s="17" t="n"/>
+      <c r="G353" s="31" t="n"/>
+      <c r="H353" s="32" t="n"/>
+      <c r="I353" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="J353" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="K353" s="28" t="n"/>
+      <c r="L353" s="32" t="inlineStr">
+        <is>
           <t>Parking Grand-Place, Bruxelles</t>
         </is>
       </c>
-    </row>
-    <row r="353">
-      <c r="G353" s="37" t="n"/>
-      <c r="H353" s="38" t="n"/>
-      <c r="J353" s="37" t="n"/>
-      <c r="L353" s="38" t="n"/>
     </row>
     <row r="354">
       <c r="G354" s="37" t="n"/>
@@ -7858,60 +7882,42 @@
       <c r="L354" s="38" t="n"/>
     </row>
     <row r="355">
-      <c r="E355" s="16" t="inlineStr">
+      <c r="G355" s="37" t="n"/>
+      <c r="H355" s="38" t="n"/>
+      <c r="J355" s="37" t="n"/>
+      <c r="L355" s="38" t="n"/>
+    </row>
+    <row r="356">
+      <c r="E356" s="16" t="inlineStr">
         <is>
           <t>Septembre</t>
         </is>
       </c>
-      <c r="F355" s="17" t="inlineStr">
+      <c r="F356" s="17" t="inlineStr">
         <is>
           <t>LAM2510</t>
         </is>
       </c>
-      <c r="G355" s="31" t="n">
+      <c r="G356" s="31" t="n">
         <v>5501.95</v>
       </c>
-      <c r="H355" s="32" t="n"/>
-      <c r="I355" s="28" t="inlineStr">
+      <c r="H356" s="32" t="n"/>
+      <c r="I356" s="28" t="inlineStr">
         <is>
           <t>Partena</t>
         </is>
       </c>
-      <c r="J355" s="39" t="n">
+      <c r="J356" s="39" t="n">
         <v>1441.87</v>
       </c>
-      <c r="K355" s="28" t="inlineStr">
+      <c r="K356" s="28" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L355" s="32" t="inlineStr">
+      <c r="L356" s="32" t="inlineStr">
         <is>
           <t>Cotisation trimestrielle — facture 425/0896/51742 — Décompte Partena en main</t>
-        </is>
-      </c>
-    </row>
-    <row r="356">
-      <c r="E356" s="16" t="n"/>
-      <c r="F356" s="17" t="n"/>
-      <c r="G356" s="31" t="n"/>
-      <c r="H356" s="32" t="n"/>
-      <c r="I356" s="13" t="inlineStr">
-        <is>
-          <t>Electrabel</t>
-        </is>
-      </c>
-      <c r="J356" s="33" t="n">
-        <v>263.44</v>
-      </c>
-      <c r="K356" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L356" s="32" t="inlineStr">
-        <is>
-          <t>Facture 412/3802/96359 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -7922,11 +7928,11 @@
       <c r="H357" s="32" t="n"/>
       <c r="I357" s="13" t="inlineStr">
         <is>
-          <t>Telenet</t>
+          <t>Electrabel</t>
         </is>
       </c>
       <c r="J357" s="33" t="n">
-        <v>153.42</v>
+        <v>263.44</v>
       </c>
       <c r="K357" s="28" t="inlineStr">
         <is>
@@ -7935,7 +7941,7 @@
       </c>
       <c r="L357" s="32" t="inlineStr">
         <is>
-          <t>Facture 310/7313/00668 — Facture Telenet en main</t>
+          <t>Facture 412/3802/96359 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -7946,16 +7952,20 @@
       <c r="H358" s="32" t="n"/>
       <c r="I358" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Telenet</t>
         </is>
       </c>
       <c r="J358" s="33" t="n">
-        <v>65.14</v>
-      </c>
-      <c r="K358" s="28" t="n"/>
+        <v>153.42</v>
+      </c>
+      <c r="K358" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L358" s="32" t="inlineStr">
         <is>
-          <t>Q8 Tervuren</t>
+          <t>Facture 310/7313/00668 — Facture Telenet en main</t>
         </is>
       </c>
     </row>
@@ -7966,20 +7976,16 @@
       <c r="H359" s="32" t="n"/>
       <c r="I359" s="13" t="inlineStr">
         <is>
-          <t>Précompte salarial août 2025 Thibault Duchène</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J359" s="33" t="n">
-        <v>2250</v>
-      </c>
-      <c r="K359" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>65.14</v>
+      </c>
+      <c r="K359" s="28" t="n"/>
       <c r="L359" s="32" t="inlineStr">
         <is>
-          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+          <t>Q8 Tervuren</t>
         </is>
       </c>
     </row>
@@ -7990,11 +7996,11 @@
       <c r="H360" s="32" t="n"/>
       <c r="I360" s="13" t="inlineStr">
         <is>
-          <t>SD Worx</t>
+          <t>Précompte salarial août 2025 Thibault Duchène</t>
         </is>
       </c>
       <c r="J360" s="33" t="n">
-        <v>331.79</v>
+        <v>2250</v>
       </c>
       <c r="K360" s="28" t="inlineStr">
         <is>
@@ -8003,7 +8009,7 @@
       </c>
       <c r="L360" s="32" t="inlineStr">
         <is>
-          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -8014,14 +8020,22 @@
       <c r="H361" s="32" t="n"/>
       <c r="I361" s="13" t="inlineStr">
         <is>
-          <t>Farys (eau)</t>
+          <t>SD Worx</t>
         </is>
       </c>
       <c r="J361" s="33" t="n">
-        <v>300</v>
-      </c>
-      <c r="K361" s="28" t="n"/>
-      <c r="L361" s="32" t="n"/>
+        <v>331.79</v>
+      </c>
+      <c r="K361" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L361" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="E362" s="16" t="n"/>
@@ -8030,11 +8044,11 @@
       <c r="H362" s="32" t="n"/>
       <c r="I362" s="13" t="inlineStr">
         <is>
-          <t>Crédit voiture</t>
+          <t>Farys (eau)</t>
         </is>
       </c>
       <c r="J362" s="33" t="n">
-        <v>724.12</v>
+        <v>300</v>
       </c>
       <c r="K362" s="28" t="n"/>
       <c r="L362" s="32" t="n"/>
@@ -8046,18 +8060,14 @@
       <c r="H363" s="32" t="n"/>
       <c r="I363" s="13" t="inlineStr">
         <is>
-          <t>Proximus</t>
+          <t>Crédit voiture</t>
         </is>
       </c>
       <c r="J363" s="33" t="n">
-        <v>70.62</v>
+        <v>724.12</v>
       </c>
       <c r="K363" s="28" t="n"/>
-      <c r="L363" s="32" t="inlineStr">
-        <is>
-          <t>Facture 750/5179/27218</t>
-        </is>
-      </c>
+      <c r="L363" s="32" t="n"/>
     </row>
     <row r="364">
       <c r="E364" s="16" t="n"/>
@@ -8066,16 +8076,16 @@
       <c r="H364" s="32" t="n"/>
       <c r="I364" s="13" t="inlineStr">
         <is>
-          <t>Vlaamse Belastingsdienst - taxe de circulation</t>
+          <t>Proximus</t>
         </is>
       </c>
       <c r="J364" s="33" t="n">
-        <v>161.02</v>
+        <v>70.62</v>
       </c>
       <c r="K364" s="28" t="n"/>
       <c r="L364" s="32" t="inlineStr">
         <is>
-          <t>Comm. 255/2756/05470</t>
+          <t>Facture 750/5179/27218</t>
         </is>
       </c>
     </row>
@@ -8086,16 +8096,16 @@
       <c r="H365" s="32" t="n"/>
       <c r="I365" s="13" t="inlineStr">
         <is>
-          <t>Transport - De Lijn</t>
+          <t>Vlaamse Belastingsdienst - taxe de circulation</t>
         </is>
       </c>
       <c r="J365" s="33" t="n">
-        <v>3</v>
+        <v>161.02</v>
       </c>
       <c r="K365" s="28" t="n"/>
       <c r="L365" s="32" t="inlineStr">
         <is>
-          <t>Carte Visa 13-08 — décompte n° 244 du 10-09</t>
+          <t>Comm. 255/2756/05470</t>
         </is>
       </c>
     </row>
@@ -8106,16 +8116,16 @@
       <c r="H366" s="32" t="n"/>
       <c r="I366" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Transport - De Lijn</t>
         </is>
       </c>
       <c r="J366" s="33" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="K366" s="28" t="n"/>
       <c r="L366" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Carte Visa 13-08 — décompte n° 244 du 10-09</t>
         </is>
       </c>
     </row>
@@ -8126,16 +8136,16 @@
       <c r="H367" s="32" t="n"/>
       <c r="I367" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J367" s="33" t="n">
-        <v>66.73999999999999</v>
+        <v>3.2</v>
       </c>
       <c r="K367" s="28" t="n"/>
       <c r="L367" s="32" t="inlineStr">
         <is>
-          <t>Shell Kraainem</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -8146,20 +8156,16 @@
       <c r="H368" s="32" t="n"/>
       <c r="I368" s="13" t="inlineStr">
         <is>
-          <t>Repas Lunch Garden</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J368" s="33" t="n">
-        <v>45.77</v>
-      </c>
-      <c r="K368" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>66.73999999999999</v>
+      </c>
+      <c r="K368" s="28" t="n"/>
       <c r="L368" s="32" t="inlineStr">
         <is>
-          <t>Lunch Garden Kraainem — Justificatif : 2025-09-13_LunchGarden-Kraainem_45.77.pdf</t>
+          <t>Shell Kraainem</t>
         </is>
       </c>
     </row>
@@ -8170,16 +8176,20 @@
       <c r="H369" s="32" t="n"/>
       <c r="I369" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Repas Lunch Garden</t>
         </is>
       </c>
       <c r="J369" s="33" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="K369" s="28" t="n"/>
+        <v>45.77</v>
+      </c>
+      <c r="K369" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L369" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Lunch Garden Kraainem — Justificatif : 2025-09-13_LunchGarden-Kraainem_45.77.pdf</t>
         </is>
       </c>
     </row>
@@ -8190,16 +8200,16 @@
       <c r="H370" s="32" t="n"/>
       <c r="I370" s="13" t="inlineStr">
         <is>
-          <t>Proximus</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J370" s="33" t="n">
-        <v>161.83</v>
+        <v>1.6</v>
       </c>
       <c r="K370" s="28" t="n"/>
       <c r="L370" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/5709/83285 — 2e facture du mois</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -8210,16 +8220,16 @@
       <c r="H371" s="32" t="n"/>
       <c r="I371" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Proximus</t>
         </is>
       </c>
       <c r="J371" s="33" t="n">
-        <v>0.9</v>
+        <v>161.83</v>
       </c>
       <c r="K371" s="28" t="n"/>
       <c r="L371" s="32" t="inlineStr">
         <is>
-          <t>Schaerbeek</t>
+          <t>Facture 750/5709/83285 — 2e facture du mois</t>
         </is>
       </c>
     </row>
@@ -8230,16 +8240,16 @@
       <c r="H372" s="32" t="n"/>
       <c r="I372" s="13" t="inlineStr">
         <is>
-          <t>Péage autoroute France</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J372" s="33" t="n">
-        <v>101.2</v>
+        <v>0.9</v>
       </c>
       <c r="K372" s="28" t="n"/>
       <c r="L372" s="32" t="inlineStr">
         <is>
-          <t>Domiciliation Autoroutes du Sud de la France</t>
+          <t>Schaerbeek</t>
         </is>
       </c>
     </row>
@@ -8250,20 +8260,16 @@
       <c r="H373" s="32" t="n"/>
       <c r="I373" s="13" t="inlineStr">
         <is>
-          <t>Repas Exki</t>
+          <t>Péage autoroute France</t>
         </is>
       </c>
       <c r="J373" s="33" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="K373" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>101.2</v>
+      </c>
+      <c r="K373" s="28" t="n"/>
       <c r="L373" s="32" t="inlineStr">
         <is>
-          <t>Exki Woluwe — Justificatif : 2025-09-19_EXKi-Woluwe_35.40.pdf</t>
+          <t>Domiciliation Autoroutes du Sud de la France</t>
         </is>
       </c>
     </row>
@@ -8274,16 +8280,20 @@
       <c r="H374" s="32" t="n"/>
       <c r="I374" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Repas Exki</t>
         </is>
       </c>
       <c r="J374" s="33" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="K374" s="28" t="n"/>
+        <v>35.4</v>
+      </c>
+      <c r="K374" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L374" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Exki Woluwe — Justificatif : 2025-09-19_EXKi-Woluwe_35.40.pdf</t>
         </is>
       </c>
     </row>
@@ -8294,16 +8304,16 @@
       <c r="H375" s="32" t="n"/>
       <c r="I375" s="13" t="inlineStr">
         <is>
-          <t>Formation Indigo Nails Lab Belgium</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J375" s="33" t="n">
-        <v>630</v>
+        <v>1.6</v>
       </c>
       <c r="K375" s="28" t="n"/>
       <c r="L375" s="32" t="inlineStr">
         <is>
-          <t>Facture FA002548 avancée par T. Duchène et remboursée par la société</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -8314,16 +8324,16 @@
       <c r="H376" s="32" t="n"/>
       <c r="I376" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Formation Indigo Nails Lab Belgium</t>
         </is>
       </c>
       <c r="J376" s="33" t="n">
-        <v>59.4</v>
+        <v>630</v>
       </c>
       <c r="K376" s="28" t="n"/>
       <c r="L376" s="32" t="inlineStr">
         <is>
-          <t>Shell Kraainem</t>
+          <t>Facture FA002548 avancée par T. Duchène et remboursée par la société</t>
         </is>
       </c>
     </row>
@@ -8334,20 +8344,16 @@
       <c r="H377" s="32" t="n"/>
       <c r="I377" s="13" t="inlineStr">
         <is>
-          <t>Repas - Chez Ji SPRL</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J377" s="33" t="n">
-        <v>47</v>
-      </c>
-      <c r="K377" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>59.4</v>
+      </c>
+      <c r="K377" s="28" t="n"/>
       <c r="L377" s="32" t="inlineStr">
         <is>
-          <t>Péruwelz — Justificatif : 2025-09-23_ChezJi-Peruwelz_47.00.pdf</t>
+          <t>Shell Kraainem</t>
         </is>
       </c>
     </row>
@@ -8358,16 +8364,20 @@
       <c r="H378" s="32" t="n"/>
       <c r="I378" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Repas - Chez Ji SPRL</t>
         </is>
       </c>
       <c r="J378" s="33" t="n">
-        <v>58.45</v>
-      </c>
-      <c r="K378" s="28" t="n"/>
+        <v>47</v>
+      </c>
+      <c r="K378" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L378" s="32" t="inlineStr">
         <is>
-          <t>Esso Péruwelz</t>
+          <t>Péruwelz — Justificatif : 2025-09-23_ChezJi-Peruwelz_47.00.pdf</t>
         </is>
       </c>
     </row>
@@ -8378,20 +8388,16 @@
       <c r="H379" s="32" t="n"/>
       <c r="I379" s="13" t="inlineStr">
         <is>
-          <t>Repas - TotalEnergies Nivelles</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J379" s="33" t="n">
-        <v>13.65</v>
-      </c>
-      <c r="K379" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>58.45</v>
+      </c>
+      <c r="K379" s="28" t="n"/>
       <c r="L379" s="32" t="inlineStr">
         <is>
-          <t>Aire d'Orival E19 — restauration, pas du carburant — Justificatif : 2025-09-26_TotalEnergies-Nivelles_13.65.pdf</t>
+          <t>Esso Péruwelz</t>
         </is>
       </c>
     </row>
@@ -8402,28 +8408,46 @@
       <c r="H380" s="32" t="n"/>
       <c r="I380" s="13" t="inlineStr">
         <is>
+          <t>Repas - TotalEnergies Nivelles</t>
+        </is>
+      </c>
+      <c r="J380" s="33" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="K380" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L380" s="32" t="inlineStr">
+        <is>
+          <t>Aire d'Orival E19 — restauration, pas du carburant — Justificatif : 2025-09-26_TotalEnergies-Nivelles_13.65.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="E381" s="16" t="n"/>
+      <c r="F381" s="17" t="n"/>
+      <c r="G381" s="31" t="n"/>
+      <c r="H381" s="32" t="n"/>
+      <c r="I381" s="13" t="inlineStr">
+        <is>
           <t>Achat matériel sportif - Bellissimo Sport</t>
         </is>
       </c>
-      <c r="J380" s="33" t="n">
+      <c r="J381" s="33" t="n">
         <v>40</v>
       </c>
-      <c r="K380" s="28" t="inlineStr">
+      <c r="K381" s="28" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L380" s="32" t="inlineStr">
+      <c r="L381" s="32" t="inlineStr">
         <is>
           <t>Chaussures Babolat Pulsion Kid (enfants, pointure 29) — Justificatif : 2025-09-27_Bellissimo-Sport_40.00.pdf</t>
         </is>
       </c>
-    </row>
-    <row r="381">
-      <c r="G381" s="37" t="n"/>
-      <c r="H381" s="38" t="n"/>
-      <c r="J381" s="37" t="n"/>
-      <c r="L381" s="38" t="n"/>
     </row>
     <row r="382">
       <c r="G382" s="37" t="n"/>
@@ -8432,99 +8456,81 @@
       <c r="L382" s="38" t="n"/>
     </row>
     <row r="383">
-      <c r="E383" s="16" t="inlineStr">
+      <c r="G383" s="37" t="n"/>
+      <c r="H383" s="38" t="n"/>
+      <c r="J383" s="37" t="n"/>
+      <c r="L383" s="38" t="n"/>
+    </row>
+    <row r="384">
+      <c r="E384" s="16" t="inlineStr">
         <is>
           <t>Octobre</t>
         </is>
       </c>
-      <c r="F383" s="17" t="inlineStr">
+      <c r="F384" s="17" t="inlineStr">
         <is>
           <t>LAM2511</t>
         </is>
       </c>
-      <c r="G383" s="31" t="n">
+      <c r="G384" s="31" t="n">
         <v>3858.09</v>
       </c>
-      <c r="H383" s="32" t="n"/>
-      <c r="I383" s="28" t="inlineStr">
+      <c r="H384" s="32" t="n"/>
+      <c r="I384" s="28" t="inlineStr">
         <is>
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J383" s="39" t="n">
+      <c r="J384" s="39" t="n">
         <v>724.12</v>
       </c>
-      <c r="K383" s="28" t="n"/>
-      <c r="L383" s="32" t="n"/>
-    </row>
-    <row r="384">
-      <c r="E384" s="16" t="n"/>
-      <c r="F384" s="17" t="inlineStr">
-        <is>
-          <t>LAM2512</t>
-        </is>
-      </c>
-      <c r="G384" s="31" t="n">
-        <v>13994</v>
-      </c>
-      <c r="H384" s="32" t="n"/>
-      <c r="I384" s="13" t="inlineStr">
-        <is>
-          <t>Carburant</t>
-        </is>
-      </c>
-      <c r="J384" s="33" t="n">
-        <v>68.23</v>
-      </c>
       <c r="K384" s="28" t="n"/>
-      <c r="L384" s="32" t="inlineStr">
-        <is>
-          <t>Total Hoegaarden</t>
-        </is>
-      </c>
+      <c r="L384" s="32" t="n"/>
     </row>
     <row r="385">
       <c r="E385" s="16" t="n"/>
       <c r="F385" s="17" t="inlineStr">
         <is>
-          <t>LAM2513</t>
+          <t>LAM2512</t>
         </is>
       </c>
       <c r="G385" s="31" t="n">
-        <v>4525.72</v>
+        <v>13994</v>
       </c>
       <c r="H385" s="32" t="n"/>
       <c r="I385" s="13" t="inlineStr">
         <is>
-          <t>Précompte salarial septembre 2025 Thibault Duchène</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J385" s="33" t="n">
-        <v>2250</v>
-      </c>
-      <c r="K385" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>68.23</v>
+      </c>
+      <c r="K385" s="28" t="n"/>
       <c r="L385" s="32" t="inlineStr">
         <is>
-          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+          <t>Total Hoegaarden</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="E386" s="16" t="n"/>
-      <c r="F386" s="17" t="n"/>
-      <c r="G386" s="31" t="n"/>
+      <c r="F386" s="17" t="inlineStr">
+        <is>
+          <t>LAM2513</t>
+        </is>
+      </c>
+      <c r="G386" s="31" t="n">
+        <v>4525.72</v>
+      </c>
       <c r="H386" s="32" t="n"/>
       <c r="I386" s="13" t="inlineStr">
         <is>
-          <t>SD Worx</t>
+          <t>Précompte salarial septembre 2025 Thibault Duchène</t>
         </is>
       </c>
       <c r="J386" s="33" t="n">
-        <v>331.79</v>
+        <v>2250</v>
       </c>
       <c r="K386" s="28" t="inlineStr">
         <is>
@@ -8533,7 +8539,7 @@
       </c>
       <c r="L386" s="32" t="inlineStr">
         <is>
-          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -8544,14 +8550,22 @@
       <c r="H387" s="32" t="n"/>
       <c r="I387" s="13" t="inlineStr">
         <is>
-          <t>Farys (eau)</t>
+          <t>SD Worx</t>
         </is>
       </c>
       <c r="J387" s="33" t="n">
-        <v>172.14</v>
-      </c>
-      <c r="K387" s="28" t="n"/>
-      <c r="L387" s="32" t="n"/>
+        <v>331.79</v>
+      </c>
+      <c r="K387" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L387" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="E388" s="16" t="n"/>
@@ -8560,18 +8574,14 @@
       <c r="H388" s="32" t="n"/>
       <c r="I388" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Farys (eau)</t>
         </is>
       </c>
       <c r="J388" s="33" t="n">
-        <v>10</v>
+        <v>172.14</v>
       </c>
       <c r="K388" s="28" t="n"/>
-      <c r="L388" s="32" t="inlineStr">
-        <is>
-          <t>Parking 't Centrum, Valkenburg (Pays-Bas)</t>
-        </is>
-      </c>
+      <c r="L388" s="32" t="n"/>
     </row>
     <row r="389">
       <c r="E389" s="16" t="n"/>
@@ -8584,12 +8594,12 @@
         </is>
       </c>
       <c r="J389" s="33" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K389" s="28" t="n"/>
       <c r="L389" s="32" t="inlineStr">
         <is>
-          <t>Valkenburg (Pays-Bas)</t>
+          <t>Parking 't Centrum, Valkenburg (Pays-Bas)</t>
         </is>
       </c>
     </row>
@@ -8600,14 +8610,18 @@
       <c r="H390" s="32" t="n"/>
       <c r="I390" s="13" t="inlineStr">
         <is>
-          <t>Frais bancaires trimestriels</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J390" s="33" t="n">
-        <v>11.25</v>
+        <v>1</v>
       </c>
       <c r="K390" s="28" t="n"/>
-      <c r="L390" s="32" t="n"/>
+      <c r="L390" s="32" t="inlineStr">
+        <is>
+          <t>Valkenburg (Pays-Bas)</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="E391" s="16" t="n"/>
@@ -8616,18 +8630,14 @@
       <c r="H391" s="32" t="n"/>
       <c r="I391" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Frais bancaires trimestriels</t>
         </is>
       </c>
       <c r="J391" s="33" t="n">
-        <v>1.85</v>
+        <v>11.25</v>
       </c>
       <c r="K391" s="28" t="n"/>
-      <c r="L391" s="32" t="inlineStr">
-        <is>
-          <t>Q-Park Woluwe Esplanade</t>
-        </is>
-      </c>
+      <c r="L391" s="32" t="n"/>
     </row>
     <row r="392">
       <c r="E392" s="16" t="n"/>
@@ -8636,16 +8646,16 @@
       <c r="H392" s="32" t="n"/>
       <c r="I392" s="13" t="inlineStr">
         <is>
-          <t>Assurance voiture</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J392" s="33" t="n">
-        <v>458.66</v>
+        <v>1.85</v>
       </c>
       <c r="K392" s="28" t="n"/>
       <c r="L392" s="32" t="inlineStr">
         <is>
-          <t>Paiement par domiciliation (AG Insurance)</t>
+          <t>Q-Park Woluwe Esplanade</t>
         </is>
       </c>
     </row>
@@ -8656,20 +8666,16 @@
       <c r="H393" s="32" t="n"/>
       <c r="I393" s="13" t="inlineStr">
         <is>
-          <t>Electrabel</t>
+          <t>Assurance voiture</t>
         </is>
       </c>
       <c r="J393" s="33" t="n">
-        <v>263.44</v>
-      </c>
-      <c r="K393" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>458.66</v>
+      </c>
+      <c r="K393" s="28" t="n"/>
       <c r="L393" s="32" t="inlineStr">
         <is>
-          <t>Facture 495/0336/32914 — Facture ENGIE en main</t>
+          <t>Paiement par domiciliation (AG Insurance)</t>
         </is>
       </c>
     </row>
@@ -8680,11 +8686,11 @@
       <c r="H394" s="32" t="n"/>
       <c r="I394" s="13" t="inlineStr">
         <is>
-          <t>Réception marchandise - FEDEX</t>
+          <t>Electrabel</t>
         </is>
       </c>
       <c r="J394" s="33" t="n">
-        <v>17.37</v>
+        <v>263.44</v>
       </c>
       <c r="K394" s="28" t="inlineStr">
         <is>
@@ -8693,7 +8699,7 @@
       </c>
       <c r="L394" s="32" t="inlineStr">
         <is>
-          <t>Justificatif : 2025-09-25_FedEx_17.37.pdf</t>
+          <t>Facture 495/0336/32914 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -8704,16 +8710,20 @@
       <c r="H395" s="32" t="n"/>
       <c r="I395" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
       <c r="J395" s="33" t="n">
-        <v>5</v>
-      </c>
-      <c r="K395" s="28" t="n"/>
+        <v>17.37</v>
+      </c>
+      <c r="K395" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L395" s="32" t="inlineStr">
         <is>
-          <t>Parking FP1, Zaventem</t>
+          <t>Justificatif : 2025-09-25_FedEx_17.37.pdf</t>
         </is>
       </c>
     </row>
@@ -8724,16 +8734,16 @@
       <c r="H396" s="32" t="n"/>
       <c r="I396" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J396" s="33" t="n">
-        <v>64.26000000000001</v>
+        <v>5</v>
       </c>
       <c r="K396" s="28" t="n"/>
       <c r="L396" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Parking FP1, Zaventem</t>
         </is>
       </c>
     </row>
@@ -8744,16 +8754,16 @@
       <c r="H397" s="32" t="n"/>
       <c r="I397" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J397" s="33" t="n">
-        <v>1.6</v>
+        <v>64.26000000000001</v>
       </c>
       <c r="K397" s="28" t="n"/>
       <c r="L397" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -8768,12 +8778,12 @@
         </is>
       </c>
       <c r="J398" s="33" t="n">
-        <v>12</v>
+        <v>1.6</v>
       </c>
       <c r="K398" s="28" t="n"/>
       <c r="L398" s="32" t="inlineStr">
         <is>
-          <t>Brussels Expo Parking</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -8784,16 +8794,16 @@
       <c r="H399" s="32" t="n"/>
       <c r="I399" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J399" s="33" t="n">
-        <v>67.14</v>
+        <v>12</v>
       </c>
       <c r="K399" s="28" t="n"/>
       <c r="L399" s="32" t="inlineStr">
         <is>
-          <t>Total Rumst</t>
+          <t>Brussels Expo Parking</t>
         </is>
       </c>
     </row>
@@ -8804,16 +8814,16 @@
       <c r="H400" s="32" t="n"/>
       <c r="I400" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J400" s="33" t="n">
-        <v>7.7</v>
+        <v>67.14</v>
       </c>
       <c r="K400" s="28" t="n"/>
       <c r="L400" s="32" t="inlineStr">
         <is>
-          <t>Parking De Vooruitgang, Volendam (Pays-Bas)</t>
+          <t>Total Rumst</t>
         </is>
       </c>
     </row>
@@ -8828,12 +8838,12 @@
         </is>
       </c>
       <c r="J401" s="33" t="n">
-        <v>3.2</v>
+        <v>7.7</v>
       </c>
       <c r="K401" s="28" t="n"/>
       <c r="L401" s="32" t="inlineStr">
         <is>
-          <t>Zaanstad (Pays-Bas)</t>
+          <t>Parking De Vooruitgang, Volendam (Pays-Bas)</t>
         </is>
       </c>
     </row>
@@ -8848,12 +8858,12 @@
         </is>
       </c>
       <c r="J402" s="33" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="K402" s="28" t="n"/>
       <c r="L402" s="32" t="inlineStr">
         <is>
-          <t>Q-Park Rozenhof, Zaandam (Pays-Bas)</t>
+          <t>Zaanstad (Pays-Bas)</t>
         </is>
       </c>
     </row>
@@ -8864,16 +8874,16 @@
       <c r="H403" s="32" t="n"/>
       <c r="I403" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J403" s="33" t="n">
-        <v>81.39</v>
+        <v>3</v>
       </c>
       <c r="K403" s="28" t="n"/>
       <c r="L403" s="32" t="inlineStr">
         <is>
-          <t>Esso Dorst (Pays-Bas)</t>
+          <t>Q-Park Rozenhof, Zaandam (Pays-Bas)</t>
         </is>
       </c>
     </row>
@@ -8884,16 +8894,16 @@
       <c r="H404" s="32" t="n"/>
       <c r="I404" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J404" s="33" t="n">
-        <v>9.199999999999999</v>
+        <v>81.39</v>
       </c>
       <c r="K404" s="28" t="n"/>
       <c r="L404" s="32" t="inlineStr">
         <is>
-          <t>Parking Ladeuze, Louvain</t>
+          <t>Esso Dorst (Pays-Bas)</t>
         </is>
       </c>
     </row>
@@ -8908,12 +8918,12 @@
         </is>
       </c>
       <c r="J405" s="33" t="n">
-        <v>1.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K405" s="28" t="n"/>
       <c r="L405" s="32" t="inlineStr">
         <is>
-          <t>Commune Saint-Josse</t>
+          <t>Parking Ladeuze, Louvain</t>
         </is>
       </c>
     </row>
@@ -8924,16 +8934,16 @@
       <c r="H406" s="32" t="n"/>
       <c r="I406" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J406" s="33" t="n">
-        <v>70.66</v>
+        <v>1.8</v>
       </c>
       <c r="K406" s="28" t="n"/>
       <c r="L406" s="32" t="inlineStr">
         <is>
-          <t>Shell Kraainem</t>
+          <t>Commune Saint-Josse</t>
         </is>
       </c>
     </row>
@@ -8944,16 +8954,16 @@
       <c r="H407" s="32" t="n"/>
       <c r="I407" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J407" s="33" t="n">
-        <v>5</v>
+        <v>70.66</v>
       </c>
       <c r="K407" s="28" t="n"/>
       <c r="L407" s="32" t="inlineStr">
         <is>
-          <t>Parking Bokrijk, Genk</t>
+          <t>Shell Kraainem</t>
         </is>
       </c>
     </row>
@@ -8968,12 +8978,12 @@
         </is>
       </c>
       <c r="J408" s="33" t="n">
-        <v>1.6</v>
+        <v>5</v>
       </c>
       <c r="K408" s="28" t="n"/>
       <c r="L408" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Parking Bokrijk, Genk</t>
         </is>
       </c>
     </row>
@@ -8984,16 +8994,16 @@
       <c r="H409" s="32" t="n"/>
       <c r="I409" s="13" t="inlineStr">
         <is>
-          <t>Versement impôts anticipé</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J409" s="33" t="n">
-        <v>5500</v>
+        <v>1.6</v>
       </c>
       <c r="K409" s="28" t="n"/>
       <c r="L409" s="32" t="inlineStr">
         <is>
-          <t>Comm. 073/4616/33527</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -9002,18 +9012,18 @@
       <c r="F410" s="17" t="n"/>
       <c r="G410" s="31" t="n"/>
       <c r="H410" s="32" t="n"/>
-      <c r="I410" s="34" t="inlineStr">
-        <is>
-          <t>Précompte mobilier</t>
-        </is>
-      </c>
-      <c r="J410" s="35" t="n">
-        <v>2100</v>
+      <c r="I410" s="13" t="inlineStr">
+        <is>
+          <t>Versement impôts anticipé</t>
+        </is>
+      </c>
+      <c r="J410" s="33" t="n">
+        <v>5500</v>
       </c>
       <c r="K410" s="28" t="n"/>
-      <c r="L410" s="36" t="inlineStr">
-        <is>
-          <t>Comm. 204/0596/50233 — lié à une distribution de dividendes ?</t>
+      <c r="L410" s="32" t="inlineStr">
+        <is>
+          <t>Comm. 073/4616/33527</t>
         </is>
       </c>
     </row>
@@ -9022,18 +9032,18 @@
       <c r="F411" s="17" t="n"/>
       <c r="G411" s="31" t="n"/>
       <c r="H411" s="32" t="n"/>
-      <c r="I411" s="13" t="inlineStr">
-        <is>
-          <t>Proximus</t>
-        </is>
-      </c>
-      <c r="J411" s="33" t="n">
-        <v>148.72</v>
+      <c r="I411" s="34" t="inlineStr">
+        <is>
+          <t>Précompte mobilier</t>
+        </is>
+      </c>
+      <c r="J411" s="35" t="n">
+        <v>2100</v>
       </c>
       <c r="K411" s="28" t="n"/>
-      <c r="L411" s="32" t="inlineStr">
-        <is>
-          <t>Facture 750/6239/84691</t>
+      <c r="L411" s="36" t="inlineStr">
+        <is>
+          <t>Comm. 204/0596/50233 — lié à une distribution de dividendes ?</t>
         </is>
       </c>
     </row>
@@ -9044,28 +9054,42 @@
       <c r="H412" s="32" t="n"/>
       <c r="I412" s="13" t="inlineStr">
         <is>
+          <t>Proximus</t>
+        </is>
+      </c>
+      <c r="J412" s="33" t="n">
+        <v>148.72</v>
+      </c>
+      <c r="K412" s="28" t="n"/>
+      <c r="L412" s="32" t="inlineStr">
+        <is>
+          <t>Facture 750/6239/84691</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="E413" s="16" t="n"/>
+      <c r="F413" s="17" t="n"/>
+      <c r="G413" s="31" t="n"/>
+      <c r="H413" s="32" t="n"/>
+      <c r="I413" s="13" t="inlineStr">
+        <is>
           <t>Consommation Lambermont</t>
         </is>
       </c>
-      <c r="J412" s="33" t="n">
+      <c r="J413" s="33" t="n">
         <v>58</v>
       </c>
-      <c r="K412" s="28" t="inlineStr">
+      <c r="K413" s="28" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L412" s="32" t="inlineStr">
+      <c r="L413" s="32" t="inlineStr">
         <is>
           <t>Justificatif : 2025-10-29_RTCL-Lambermont_58.00.pdf</t>
         </is>
       </c>
-    </row>
-    <row r="413">
-      <c r="G413" s="37" t="n"/>
-      <c r="H413" s="38" t="n"/>
-      <c r="J413" s="37" t="n"/>
-      <c r="L413" s="38" t="n"/>
     </row>
     <row r="414">
       <c r="G414" s="37" t="n"/>
@@ -9074,46 +9098,32 @@
       <c r="L414" s="38" t="n"/>
     </row>
     <row r="415">
-      <c r="E415" s="16" t="inlineStr">
+      <c r="G415" s="37" t="n"/>
+      <c r="H415" s="38" t="n"/>
+      <c r="J415" s="37" t="n"/>
+      <c r="L415" s="38" t="n"/>
+    </row>
+    <row r="416">
+      <c r="E416" s="16" t="inlineStr">
         <is>
           <t>Novembre</t>
         </is>
       </c>
-      <c r="F415" s="17" t="n"/>
-      <c r="G415" s="31" t="n"/>
-      <c r="H415" s="32" t="n"/>
-      <c r="I415" s="28" t="inlineStr">
-        <is>
-          <t>Carburant</t>
-        </is>
-      </c>
-      <c r="J415" s="39" t="n">
-        <v>65.29000000000001</v>
-      </c>
-      <c r="K415" s="28" t="n"/>
-      <c r="L415" s="32" t="inlineStr">
-        <is>
-          <t>Q8 Easy Zaventem</t>
-        </is>
-      </c>
-    </row>
-    <row r="416">
-      <c r="E416" s="16" t="n"/>
       <c r="F416" s="17" t="n"/>
       <c r="G416" s="31" t="n"/>
       <c r="H416" s="32" t="n"/>
-      <c r="I416" s="34" t="inlineStr">
-        <is>
-          <t>Achat - Media Markt</t>
-        </is>
-      </c>
-      <c r="J416" s="35" t="n">
-        <v>748</v>
+      <c r="I416" s="28" t="inlineStr">
+        <is>
+          <t>Carburant</t>
+        </is>
+      </c>
+      <c r="J416" s="39" t="n">
+        <v>65.29000000000001</v>
       </c>
       <c r="K416" s="28" t="n"/>
-      <c r="L416" s="36" t="inlineStr">
-        <is>
-          <t>Woluwe-Saint-Lambert — nature de l'achat à préciser</t>
+      <c r="L416" s="32" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -9128,7 +9138,7 @@
         </is>
       </c>
       <c r="J417" s="35" t="n">
-        <v>39</v>
+        <v>748</v>
       </c>
       <c r="K417" s="28" t="n"/>
       <c r="L417" s="36" t="inlineStr">
@@ -9142,22 +9152,18 @@
       <c r="F418" s="17" t="n"/>
       <c r="G418" s="31" t="n"/>
       <c r="H418" s="32" t="n"/>
-      <c r="I418" s="13" t="inlineStr">
-        <is>
-          <t>Précompte salarial octobre 2025 Thibault Duchène</t>
-        </is>
-      </c>
-      <c r="J418" s="33" t="n">
-        <v>2250</v>
-      </c>
-      <c r="K418" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L418" s="32" t="inlineStr">
-        <is>
-          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
+      <c r="I418" s="34" t="inlineStr">
+        <is>
+          <t>Achat - Media Markt</t>
+        </is>
+      </c>
+      <c r="J418" s="35" t="n">
+        <v>39</v>
+      </c>
+      <c r="K418" s="28" t="n"/>
+      <c r="L418" s="36" t="inlineStr">
+        <is>
+          <t>Woluwe-Saint-Lambert — nature de l'achat à préciser</t>
         </is>
       </c>
     </row>
@@ -9168,11 +9174,11 @@
       <c r="H419" s="32" t="n"/>
       <c r="I419" s="13" t="inlineStr">
         <is>
-          <t>SD Worx</t>
+          <t>Précompte salarial octobre 2025 Thibault Duchène</t>
         </is>
       </c>
       <c r="J419" s="33" t="n">
-        <v>331.85</v>
+        <v>2250</v>
       </c>
       <c r="K419" s="28" t="inlineStr">
         <is>
@@ -9181,7 +9187,7 @@
       </c>
       <c r="L419" s="32" t="inlineStr">
         <is>
-          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+          <t>Fiche de précompte — déjà chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -9192,14 +9198,22 @@
       <c r="H420" s="32" t="n"/>
       <c r="I420" s="13" t="inlineStr">
         <is>
-          <t>Crédit voiture</t>
+          <t>SD Worx</t>
         </is>
       </c>
       <c r="J420" s="33" t="n">
-        <v>724.12</v>
-      </c>
-      <c r="K420" s="28" t="n"/>
-      <c r="L420" s="32" t="n"/>
+        <v>331.85</v>
+      </c>
+      <c r="K420" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L420" s="32" t="inlineStr">
+        <is>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="E421" s="16" t="n"/>
@@ -9208,18 +9222,14 @@
       <c r="H421" s="32" t="n"/>
       <c r="I421" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Crédit voiture</t>
         </is>
       </c>
       <c r="J421" s="33" t="n">
-        <v>2.72</v>
+        <v>724.12</v>
       </c>
       <c r="K421" s="28" t="n"/>
-      <c r="L421" s="32" t="inlineStr">
-        <is>
-          <t>Commune Saint-Josse</t>
-        </is>
-      </c>
+      <c r="L421" s="32" t="n"/>
     </row>
     <row r="422">
       <c r="E422" s="16" t="n"/>
@@ -9228,16 +9238,16 @@
       <c r="H422" s="32" t="n"/>
       <c r="I422" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J422" s="33" t="n">
-        <v>70.44</v>
+        <v>2.72</v>
       </c>
       <c r="K422" s="28" t="n"/>
       <c r="L422" s="32" t="inlineStr">
         <is>
-          <t>Q8 Tervuren</t>
+          <t>Commune Saint-Josse</t>
         </is>
       </c>
     </row>
@@ -9248,16 +9258,16 @@
       <c r="H423" s="32" t="n"/>
       <c r="I423" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J423" s="33" t="n">
-        <v>1.6</v>
+        <v>70.44</v>
       </c>
       <c r="K423" s="28" t="n"/>
       <c r="L423" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Q8 Tervuren</t>
         </is>
       </c>
     </row>
@@ -9288,20 +9298,16 @@
       <c r="H425" s="32" t="n"/>
       <c r="I425" s="13" t="inlineStr">
         <is>
-          <t>Partena</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J425" s="33" t="n">
-        <v>1441.87</v>
-      </c>
-      <c r="K425" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>1.6</v>
+      </c>
+      <c r="K425" s="28" t="n"/>
       <c r="L425" s="32" t="inlineStr">
         <is>
-          <t>Cotisation trimestrielle — facture 425/1102/67272 — Décompte Partena en main</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -9312,16 +9318,20 @@
       <c r="H426" s="32" t="n"/>
       <c r="I426" s="13" t="inlineStr">
         <is>
-          <t>Frais comptable BDH - publication BNB</t>
+          <t>Partena</t>
         </is>
       </c>
       <c r="J426" s="33" t="n">
-        <v>287.7</v>
-      </c>
-      <c r="K426" s="28" t="n"/>
+        <v>1441.87</v>
+      </c>
+      <c r="K426" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L426" s="32" t="inlineStr">
         <is>
-          <t>Remboursement des frais BNB avancés par BDH</t>
+          <t>Cotisation trimestrielle — facture 425/1102/67272 — Décompte Partena en main</t>
         </is>
       </c>
     </row>
@@ -9332,20 +9342,16 @@
       <c r="H427" s="32" t="n"/>
       <c r="I427" s="13" t="inlineStr">
         <is>
-          <t>Electrabel</t>
+          <t>Frais comptable BDH - publication BNB</t>
         </is>
       </c>
       <c r="J427" s="33" t="n">
-        <v>270.94</v>
-      </c>
-      <c r="K427" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>287.7</v>
+      </c>
+      <c r="K427" s="28" t="n"/>
       <c r="L427" s="32" t="inlineStr">
         <is>
-          <t>Acompte d'août payé en retard le 18-11 : 263,44 + 7,50 de frais de rappel — facture 433/7265/65993 — Facture ENGIE en main</t>
+          <t>Remboursement des frais BNB avancés par BDH</t>
         </is>
       </c>
     </row>
@@ -9360,7 +9366,7 @@
         </is>
       </c>
       <c r="J428" s="33" t="n">
-        <v>263.44</v>
+        <v>270.94</v>
       </c>
       <c r="K428" s="28" t="inlineStr">
         <is>
@@ -9369,7 +9375,7 @@
       </c>
       <c r="L428" s="32" t="inlineStr">
         <is>
-          <t>Facture 464/6637/65902 — Facture ENGIE en main</t>
+          <t>Acompte d'août payé en retard le 18-11 : 263,44 + 7,50 de frais de rappel — facture 433/7265/65993 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -9380,16 +9386,20 @@
       <c r="H429" s="32" t="n"/>
       <c r="I429" s="13" t="inlineStr">
         <is>
-          <t>Proximus</t>
+          <t>Electrabel</t>
         </is>
       </c>
       <c r="J429" s="33" t="n">
-        <v>143.48</v>
-      </c>
-      <c r="K429" s="28" t="n"/>
+        <v>263.44</v>
+      </c>
+      <c r="K429" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L429" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/6769/40530</t>
+          <t>Facture 464/6637/65902 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -9400,16 +9410,16 @@
       <c r="H430" s="32" t="n"/>
       <c r="I430" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Proximus</t>
         </is>
       </c>
       <c r="J430" s="33" t="n">
-        <v>65.52</v>
+        <v>143.48</v>
       </c>
       <c r="K430" s="28" t="n"/>
       <c r="L430" s="32" t="inlineStr">
         <is>
-          <t>Shell Haine-Saint-Pierre</t>
+          <t>Facture 750/6769/40530</t>
         </is>
       </c>
     </row>
@@ -9420,16 +9430,16 @@
       <c r="H431" s="32" t="n"/>
       <c r="I431" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J431" s="33" t="n">
-        <v>0.9</v>
+        <v>65.52</v>
       </c>
       <c r="K431" s="28" t="n"/>
       <c r="L431" s="32" t="inlineStr">
         <is>
-          <t>Schaerbeek</t>
+          <t>Shell Haine-Saint-Pierre</t>
         </is>
       </c>
     </row>
@@ -9444,12 +9454,12 @@
         </is>
       </c>
       <c r="J432" s="33" t="n">
-        <v>2.68</v>
+        <v>0.9</v>
       </c>
       <c r="K432" s="28" t="n"/>
       <c r="L432" s="32" t="inlineStr">
         <is>
-          <t>Louvain</t>
+          <t>Schaerbeek</t>
         </is>
       </c>
     </row>
@@ -9458,22 +9468,18 @@
       <c r="F433" s="17" t="n"/>
       <c r="G433" s="31" t="n"/>
       <c r="H433" s="32" t="n"/>
-      <c r="I433" s="34" t="inlineStr">
-        <is>
-          <t>Achat matériel sportif - DECATHLON</t>
-        </is>
-      </c>
-      <c r="J433" s="35" t="n">
-        <v>118.5</v>
-      </c>
-      <c r="K433" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L433" s="36" t="inlineStr">
-        <is>
-          <t>Decathlon Evere — 10 articles dont masque de ski, luge et vêtements enfant : usage professionnel à confirmer — Justificatif : 2025-11-22_Decathlon-Evere_118.50.pdf</t>
+      <c r="I433" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="J433" s="33" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="K433" s="28" t="n"/>
+      <c r="L433" s="32" t="inlineStr">
+        <is>
+          <t>Louvain</t>
         </is>
       </c>
     </row>
@@ -9482,18 +9488,22 @@
       <c r="F434" s="17" t="n"/>
       <c r="G434" s="31" t="n"/>
       <c r="H434" s="32" t="n"/>
-      <c r="I434" s="13" t="inlineStr">
-        <is>
-          <t>Parking</t>
-        </is>
-      </c>
-      <c r="J434" s="33" t="n">
-        <v>12.6</v>
-      </c>
-      <c r="K434" s="28" t="n"/>
-      <c r="L434" s="32" t="inlineStr">
-        <is>
-          <t>Parking Rogier</t>
+      <c r="I434" s="34" t="inlineStr">
+        <is>
+          <t>Achat matériel sportif - DECATHLON</t>
+        </is>
+      </c>
+      <c r="J434" s="35" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="K434" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L434" s="36" t="inlineStr">
+        <is>
+          <t>Decathlon Evere — 10 articles dont masque de ski, luge et vêtements enfant : usage professionnel à confirmer — Justificatif : 2025-11-22_Decathlon-Evere_118.50.pdf</t>
         </is>
       </c>
     </row>
@@ -9508,12 +9518,12 @@
         </is>
       </c>
       <c r="J435" s="33" t="n">
-        <v>1.6</v>
+        <v>12.6</v>
       </c>
       <c r="K435" s="28" t="n"/>
       <c r="L435" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Parking Rogier</t>
         </is>
       </c>
     </row>
@@ -9524,16 +9534,16 @@
       <c r="H436" s="32" t="n"/>
       <c r="I436" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J436" s="33" t="n">
-        <v>69.11</v>
+        <v>1.6</v>
       </c>
       <c r="K436" s="28" t="n"/>
       <c r="L436" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -9544,16 +9554,16 @@
       <c r="H437" s="32" t="n"/>
       <c r="I437" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J437" s="33" t="n">
-        <v>1.85</v>
+        <v>69.11</v>
       </c>
       <c r="K437" s="28" t="n"/>
       <c r="L437" s="32" t="inlineStr">
         <is>
-          <t>Q-Park Woluwe Esplanade</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -9564,16 +9574,16 @@
       <c r="H438" s="32" t="n"/>
       <c r="I438" s="13" t="inlineStr">
         <is>
-          <t>Semelles orthopédiques de travail - Podomed</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J438" s="33" t="n">
-        <v>65</v>
+        <v>1.85</v>
       </c>
       <c r="K438" s="28" t="n"/>
       <c r="L438" s="32" t="inlineStr">
         <is>
-          <t>Consultation</t>
+          <t>Q-Park Woluwe Esplanade</t>
         </is>
       </c>
     </row>
@@ -9584,16 +9594,16 @@
       <c r="H439" s="32" t="n"/>
       <c r="I439" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Semelles orthopédiques de travail - Podomed</t>
         </is>
       </c>
       <c r="J439" s="33" t="n">
-        <v>5.55</v>
+        <v>65</v>
       </c>
       <c r="K439" s="28" t="n"/>
       <c r="L439" s="32" t="inlineStr">
         <is>
-          <t>Q-Park Woluwe Esplanade</t>
+          <t>Consultation</t>
         </is>
       </c>
     </row>
@@ -9608,20 +9618,34 @@
         </is>
       </c>
       <c r="J440" s="33" t="n">
-        <v>1.6</v>
+        <v>5.55</v>
       </c>
       <c r="K440" s="28" t="n"/>
       <c r="L440" s="32" t="inlineStr">
         <is>
+          <t>Q-Park Woluwe Esplanade</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="E441" s="16" t="n"/>
+      <c r="F441" s="17" t="n"/>
+      <c r="G441" s="31" t="n"/>
+      <c r="H441" s="32" t="n"/>
+      <c r="I441" s="13" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="J441" s="33" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K441" s="28" t="n"/>
+      <c r="L441" s="32" t="inlineStr">
+        <is>
           <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
-    </row>
-    <row r="441">
-      <c r="G441" s="37" t="n"/>
-      <c r="H441" s="38" t="n"/>
-      <c r="J441" s="37" t="n"/>
-      <c r="L441" s="38" t="n"/>
     </row>
     <row r="442">
       <c r="G442" s="37" t="n"/>
@@ -9630,86 +9654,72 @@
       <c r="L442" s="38" t="n"/>
     </row>
     <row r="443">
-      <c r="E443" s="16" t="inlineStr">
+      <c r="G443" s="37" t="n"/>
+      <c r="H443" s="38" t="n"/>
+      <c r="J443" s="37" t="n"/>
+      <c r="L443" s="38" t="n"/>
+    </row>
+    <row r="444">
+      <c r="E444" s="16" t="inlineStr">
         <is>
           <t>Décembre</t>
         </is>
       </c>
-      <c r="F443" s="17" t="inlineStr">
+      <c r="F444" s="17" t="inlineStr">
         <is>
           <t>LAM2514</t>
         </is>
       </c>
-      <c r="G443" s="31" t="n">
+      <c r="G444" s="31" t="n">
         <v>4162.5</v>
       </c>
-      <c r="H443" s="32" t="n"/>
-      <c r="I443" s="28" t="inlineStr">
+      <c r="H444" s="32" t="n"/>
+      <c r="I444" s="28" t="inlineStr">
         <is>
           <t>Précompte salarial novembre 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J443" s="39" t="n">
+      <c r="J444" s="39" t="n">
         <v>2250</v>
       </c>
-      <c r="K443" s="28" t="inlineStr">
+      <c r="K444" s="28" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L443" s="32" t="inlineStr">
+      <c r="L444" s="32" t="inlineStr">
         <is>
           <t>Fiche de précompte — déjà chargée dans Billtobox</t>
-        </is>
-      </c>
-    </row>
-    <row r="444">
-      <c r="E444" s="16" t="n"/>
-      <c r="F444" s="17" t="inlineStr">
-        <is>
-          <t>LAM2515</t>
-        </is>
-      </c>
-      <c r="G444" s="31" t="n">
-        <v>5382.45</v>
-      </c>
-      <c r="H444" s="32" t="n"/>
-      <c r="I444" s="13" t="inlineStr">
-        <is>
-          <t>SD Worx</t>
-        </is>
-      </c>
-      <c r="J444" s="33" t="n">
-        <v>331.85</v>
-      </c>
-      <c r="K444" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="L444" s="32" t="inlineStr">
-        <is>
-          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="E445" s="16" t="n"/>
-      <c r="F445" s="17" t="n"/>
-      <c r="G445" s="31" t="n"/>
+      <c r="F445" s="17" t="inlineStr">
+        <is>
+          <t>LAM2515</t>
+        </is>
+      </c>
+      <c r="G445" s="31" t="n">
+        <v>5382.45</v>
+      </c>
       <c r="H445" s="32" t="n"/>
       <c r="I445" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>SD Worx</t>
         </is>
       </c>
       <c r="J445" s="33" t="n">
-        <v>63.61</v>
-      </c>
-      <c r="K445" s="28" t="n"/>
+        <v>331.85</v>
+      </c>
+      <c r="K445" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L445" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Décompte SD Worx — déjà chargé dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -9720,14 +9730,18 @@
       <c r="H446" s="32" t="n"/>
       <c r="I446" s="13" t="inlineStr">
         <is>
-          <t>Crédit voiture</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J446" s="33" t="n">
-        <v>724.12</v>
+        <v>63.61</v>
       </c>
       <c r="K446" s="28" t="n"/>
-      <c r="L446" s="32" t="n"/>
+      <c r="L446" s="32" t="inlineStr">
+        <is>
+          <t>Q8 Easy Zaventem</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="E447" s="16" t="n"/>
@@ -9736,18 +9750,14 @@
       <c r="H447" s="32" t="n"/>
       <c r="I447" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Crédit voiture</t>
         </is>
       </c>
       <c r="J447" s="33" t="n">
-        <v>4.6</v>
+        <v>724.12</v>
       </c>
       <c r="K447" s="28" t="n"/>
-      <c r="L447" s="32" t="inlineStr">
-        <is>
-          <t>Indigo Park Docks, Bruxelles</t>
-        </is>
-      </c>
+      <c r="L447" s="32" t="n"/>
     </row>
     <row r="448">
       <c r="E448" s="16" t="n"/>
@@ -9760,12 +9770,12 @@
         </is>
       </c>
       <c r="J448" s="33" t="n">
-        <v>3.2</v>
+        <v>4.6</v>
       </c>
       <c r="K448" s="28" t="n"/>
       <c r="L448" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Indigo Park Docks, Bruxelles</t>
         </is>
       </c>
     </row>
@@ -9776,16 +9786,16 @@
       <c r="H449" s="32" t="n"/>
       <c r="I449" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J449" s="33" t="n">
-        <v>63.8</v>
+        <v>3.2</v>
       </c>
       <c r="K449" s="28" t="n"/>
       <c r="L449" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -9796,16 +9806,16 @@
       <c r="H450" s="32" t="n"/>
       <c r="I450" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J450" s="33" t="n">
-        <v>6.97</v>
+        <v>63.8</v>
       </c>
       <c r="K450" s="28" t="n"/>
       <c r="L450" s="32" t="inlineStr">
         <is>
-          <t>Parcbrux Ixelles, Gand</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -9820,12 +9830,12 @@
         </is>
       </c>
       <c r="J451" s="33" t="n">
-        <v>7</v>
+        <v>6.97</v>
       </c>
       <c r="K451" s="28" t="n"/>
       <c r="L451" s="32" t="inlineStr">
         <is>
-          <t>Parking Station, Bruges</t>
+          <t>Parcbrux Ixelles, Gand</t>
         </is>
       </c>
     </row>
@@ -9836,16 +9846,16 @@
       <c r="H452" s="32" t="n"/>
       <c r="I452" s="13" t="inlineStr">
         <is>
-          <t>Xerius</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J452" s="33" t="n">
-        <v>399.73</v>
+        <v>7</v>
       </c>
       <c r="K452" s="28" t="n"/>
       <c r="L452" s="32" t="inlineStr">
         <is>
-          <t>Cotisations sociales indépendant</t>
+          <t>Parking Station, Bruges</t>
         </is>
       </c>
     </row>
@@ -9856,20 +9866,16 @@
       <c r="H453" s="32" t="n"/>
       <c r="I453" s="13" t="inlineStr">
         <is>
-          <t>Electrabel</t>
+          <t>Xerius</t>
         </is>
       </c>
       <c r="J453" s="33" t="n">
-        <v>263.44</v>
-      </c>
-      <c r="K453" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>399.73</v>
+      </c>
+      <c r="K453" s="28" t="n"/>
       <c r="L453" s="32" t="inlineStr">
         <is>
-          <t>Facture 435/0584/57839 — Facture ENGIE en main</t>
+          <t>Cotisations sociales indépendant</t>
         </is>
       </c>
     </row>
@@ -9880,16 +9886,20 @@
       <c r="H454" s="32" t="n"/>
       <c r="I454" s="13" t="inlineStr">
         <is>
-          <t>Proximus</t>
+          <t>Electrabel</t>
         </is>
       </c>
       <c r="J454" s="33" t="n">
-        <v>153.79</v>
-      </c>
-      <c r="K454" s="28" t="n"/>
+        <v>263.44</v>
+      </c>
+      <c r="K454" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L454" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/7299/18694</t>
+          <t>Facture 435/0584/57839 — Facture ENGIE en main</t>
         </is>
       </c>
     </row>
@@ -9900,16 +9910,16 @@
       <c r="H455" s="32" t="n"/>
       <c r="I455" s="13" t="inlineStr">
         <is>
-          <t>Assurance RC - LRS Insurance</t>
+          <t>Proximus</t>
         </is>
       </c>
       <c r="J455" s="33" t="n">
-        <v>55.04</v>
+        <v>153.79</v>
       </c>
       <c r="K455" s="28" t="n"/>
       <c r="L455" s="32" t="inlineStr">
         <is>
-          <t>Même montant qu'en 2024 (Liantis)</t>
+          <t>Facture 750/7299/18694</t>
         </is>
       </c>
     </row>
@@ -9920,16 +9930,16 @@
       <c r="H456" s="32" t="n"/>
       <c r="I456" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Assurance RC - LRS Insurance</t>
         </is>
       </c>
       <c r="J456" s="33" t="n">
-        <v>63.2</v>
+        <v>55.04</v>
       </c>
       <c r="K456" s="28" t="n"/>
       <c r="L456" s="32" t="inlineStr">
         <is>
-          <t>Q8 Easy Zaventem</t>
+          <t>Même montant qu'en 2024 (Liantis)</t>
         </is>
       </c>
     </row>
@@ -9940,16 +9950,16 @@
       <c r="H457" s="32" t="n"/>
       <c r="I457" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J457" s="33" t="n">
-        <v>3.7</v>
+        <v>63.2</v>
       </c>
       <c r="K457" s="28" t="n"/>
       <c r="L457" s="32" t="inlineStr">
         <is>
-          <t>Q-Park Woluwe Esplanade</t>
+          <t>Q8 Easy Zaventem</t>
         </is>
       </c>
     </row>
@@ -9964,12 +9974,12 @@
         </is>
       </c>
       <c r="J458" s="33" t="n">
-        <v>1.6</v>
+        <v>3.7</v>
       </c>
       <c r="K458" s="28" t="n"/>
       <c r="L458" s="32" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert</t>
+          <t>Q-Park Woluwe Esplanade</t>
         </is>
       </c>
     </row>
@@ -9984,12 +9994,12 @@
         </is>
       </c>
       <c r="J459" s="33" t="n">
-        <v>14</v>
+        <v>1.6</v>
       </c>
       <c r="K459" s="28" t="n"/>
       <c r="L459" s="32" t="inlineStr">
         <is>
-          <t>Parking Grand-Place, Bruxelles</t>
+          <t>Woluwe-Saint-Lambert</t>
         </is>
       </c>
     </row>
@@ -10004,12 +10014,12 @@
         </is>
       </c>
       <c r="J460" s="33" t="n">
-        <v>2.6</v>
+        <v>14</v>
       </c>
       <c r="K460" s="28" t="n"/>
       <c r="L460" s="32" t="inlineStr">
         <is>
-          <t>Parking Kinepolis, Louvain</t>
+          <t>Parking Grand-Place, Bruxelles</t>
         </is>
       </c>
     </row>
@@ -10020,16 +10030,16 @@
       <c r="H461" s="32" t="n"/>
       <c r="I461" s="13" t="inlineStr">
         <is>
-          <t>Carburant</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J461" s="33" t="n">
-        <v>63.32</v>
+        <v>2.6</v>
       </c>
       <c r="K461" s="28" t="n"/>
       <c r="L461" s="32" t="inlineStr">
         <is>
-          <t>Cora Woluwe Carburant</t>
+          <t>Parking Kinepolis, Louvain</t>
         </is>
       </c>
     </row>
@@ -10040,16 +10050,16 @@
       <c r="H462" s="32" t="n"/>
       <c r="I462" s="13" t="inlineStr">
         <is>
-          <t>Parking</t>
+          <t>Carburant</t>
         </is>
       </c>
       <c r="J462" s="33" t="n">
-        <v>3.4</v>
+        <v>63.32</v>
       </c>
       <c r="K462" s="28" t="n"/>
       <c r="L462" s="32" t="inlineStr">
         <is>
-          <t>Indigo Park Docks, Bruxelles</t>
+          <t>Cora Woluwe Carburant</t>
         </is>
       </c>
     </row>
@@ -10060,16 +10070,16 @@
       <c r="H463" s="32" t="n"/>
       <c r="I463" s="13" t="inlineStr">
         <is>
-          <t>Semelles orthopédiques de travail - Podomed</t>
+          <t>Parking</t>
         </is>
       </c>
       <c r="J463" s="33" t="n">
-        <v>210</v>
+        <v>3.4</v>
       </c>
       <c r="K463" s="28" t="n"/>
       <c r="L463" s="32" t="inlineStr">
         <is>
-          <t>Solde après la consultation du 27-11</t>
+          <t>Indigo Park Docks, Bruxelles</t>
         </is>
       </c>
     </row>
@@ -10080,16 +10090,16 @@
       <c r="H464" s="32" t="n"/>
       <c r="I464" s="13" t="inlineStr">
         <is>
-          <t>Frais comptable BDH</t>
+          <t>Semelles orthopédiques de travail - Podomed</t>
         </is>
       </c>
       <c r="J464" s="33" t="n">
-        <v>304.92</v>
+        <v>210</v>
       </c>
       <c r="K464" s="28" t="n"/>
       <c r="L464" s="32" t="inlineStr">
         <is>
-          <t>Facture 20250644</t>
+          <t>Solde après la consultation du 27-11</t>
         </is>
       </c>
     </row>
@@ -10100,20 +10110,16 @@
       <c r="H465" s="32" t="n"/>
       <c r="I465" s="13" t="inlineStr">
         <is>
-          <t>Précompte salarial décembre 2025 Thibault Duchène</t>
+          <t>Frais comptable BDH</t>
         </is>
       </c>
       <c r="J465" s="33" t="n">
-        <v>2250</v>
-      </c>
-      <c r="K465" s="28" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
+        <v>304.92</v>
+      </c>
+      <c r="K465" s="28" t="n"/>
       <c r="L465" s="32" t="inlineStr">
         <is>
-          <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024) — Fiche de précompte — déjà chargée dans Billtobox</t>
+          <t>Facture 20250644</t>
         </is>
       </c>
     </row>
@@ -10124,28 +10130,46 @@
       <c r="H466" s="32" t="n"/>
       <c r="I466" s="13" t="inlineStr">
         <is>
+          <t>Précompte salarial décembre 2025 Thibault Duchène</t>
+        </is>
+      </c>
+      <c r="J466" s="33" t="n">
+        <v>2250</v>
+      </c>
+      <c r="K466" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L466" s="32" t="inlineStr">
+        <is>
+          <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024) — Fiche de précompte — déjà chargée dans Billtobox</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="E467" s="16" t="n"/>
+      <c r="F467" s="17" t="n"/>
+      <c r="G467" s="31" t="n"/>
+      <c r="H467" s="32" t="n"/>
+      <c r="I467" s="13" t="inlineStr">
+        <is>
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J466" s="33" t="n">
+      <c r="J467" s="33" t="n">
         <v>331.85</v>
       </c>
-      <c r="K466" s="28" t="inlineStr">
+      <c r="K467" s="28" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L466" s="32" t="inlineStr">
+      <c r="L467" s="32" t="inlineStr">
         <is>
           <t>Payé le 04/05-01-2026 mais rattaché à décembre 2025 (même règle qu'en 2024) — Décompte SD Worx — déjà chargé dans Billtobox</t>
         </is>
       </c>
-    </row>
-    <row r="467">
-      <c r="G467" s="37" t="n"/>
-      <c r="H467" s="38" t="n"/>
-      <c r="J467" s="37" t="n"/>
-      <c r="L467" s="38" t="n"/>
     </row>
     <row r="468">
       <c r="G468" s="37" t="n"/>
@@ -10154,16 +10178,22 @@
       <c r="L468" s="38" t="n"/>
     </row>
     <row r="469">
-      <c r="G469" s="37">
-        <f>SUM(G6:G468)</f>
+      <c r="G469" s="37" t="n"/>
+      <c r="H469" s="38" t="n"/>
+      <c r="J469" s="37" t="n"/>
+      <c r="L469" s="38" t="n"/>
+    </row>
+    <row r="470">
+      <c r="G470" s="37">
+        <f>SUM(G6:G469)</f>
         <v/>
       </c>
-      <c r="H469" s="38" t="n"/>
-      <c r="J469" s="37">
-        <f>SUM(J6:J468)</f>
+      <c r="H470" s="38" t="n"/>
+      <c r="J470" s="37">
+        <f>SUM(J6:J469)</f>
         <v/>
       </c>
-      <c r="L469" s="38" t="n"/>
+      <c r="L470" s="38" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : six factures Proximus coches, six en attente
Coches les factures accessibles sur le portail (juillet a decembre), dont
celle payee a titre prive et les deux nettes d'une note de credit. Les six
paiements de janvier a juillet (483,05) attendent l'envoi par mail.

Couverture : 81 lignes, 48.043,50 sur 88.541,37 (54 %).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -6330,10 +6330,14 @@
       <c r="J276" s="33" t="n">
         <v>109.59</v>
       </c>
-      <c r="K276" s="28" t="n"/>
+      <c r="K276" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L276" s="32" t="inlineStr">
         <is>
-          <t>Facture 7504645054 payée par QR code depuis le compte privé de T. Duchène — hors extrait bancaire</t>
+          <t>Facture 7504645054 payée par QR code depuis le compte privé de T. Duchène — hors extrait bancaire — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -8082,10 +8086,14 @@
       <c r="J364" s="33" t="n">
         <v>70.62</v>
       </c>
-      <c r="K364" s="28" t="n"/>
+      <c r="K364" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L364" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/5179/27218</t>
+          <t>Facture 750/5179/27218 — Facture Proximus en main, chargée dans Billtobox avec sa note de crédit</t>
         </is>
       </c>
     </row>
@@ -8226,10 +8234,14 @@
       <c r="J371" s="33" t="n">
         <v>161.83</v>
       </c>
-      <c r="K371" s="28" t="n"/>
+      <c r="K371" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L371" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/5709/83285 — 2e facture du mois</t>
+          <t>Facture 750/5709/83285 — 2e facture du mois — Facture Proximus en main, chargée dans Billtobox avec sa note de crédit</t>
         </is>
       </c>
     </row>
@@ -9060,10 +9072,14 @@
       <c r="J412" s="33" t="n">
         <v>148.72</v>
       </c>
-      <c r="K412" s="28" t="n"/>
+      <c r="K412" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L412" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/6239/84691</t>
+          <t>Facture 750/6239/84691 — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -9416,10 +9432,14 @@
       <c r="J430" s="33" t="n">
         <v>143.48</v>
       </c>
-      <c r="K430" s="28" t="n"/>
+      <c r="K430" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L430" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/6769/40530</t>
+          <t>Facture 750/6769/40530 — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -9916,10 +9936,14 @@
       <c r="J455" s="33" t="n">
         <v>153.79</v>
       </c>
-      <c r="K455" s="28" t="n"/>
+      <c r="K455" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L455" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/7299/18694</t>
+          <t>Facture 750/7299/18694 — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilans 2025 et 2026 : deux factures BDH cochees
20250644 (304,92) sur le bilan 2025 en decembre, 20250542 (1.179,75) sur le
bilan 2026 en janvier. Creation de justificatifs_2026.py.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -10140,10 +10140,14 @@
       <c r="J465" s="33" t="n">
         <v>304.92</v>
       </c>
-      <c r="K465" s="28" t="n"/>
+      <c r="K465" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L465" s="32" t="inlineStr">
         <is>
-          <t>Facture 20250644</t>
+          <t>Facture 20250644 — Facture BDH en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : refacturation des frais BNB cochee
Piece BDH du 18-11 (287,70), chargee dans Billtobox.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -9364,10 +9364,14 @@
       <c r="J427" s="33" t="n">
         <v>287.7</v>
       </c>
-      <c r="K427" s="28" t="n"/>
+      <c r="K427" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L427" s="32" t="inlineStr">
         <is>
-          <t>Remboursement des frais BNB avancés par BDH</t>
+          <t>Remboursement des frais BNB avancés par BDH — Pièce BDH en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : les trois dernieres factures BDH cochees
Question de rattachement d'exercice posee au comptable, consignee dans
POINTS_OUVERTS.md avec son impact chiffre (477,95 sur le resultat 2025).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1350,10 +1350,14 @@
       <c r="J30" s="33" t="n">
         <v>1125.3</v>
       </c>
-      <c r="K30" s="28" t="n"/>
+      <c r="K30" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L30" s="32" t="inlineStr">
         <is>
-          <t>Facture 20240512</t>
+          <t>Facture 20240512 — Facture BDH en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -1394,10 +1398,14 @@
       <c r="J32" s="33" t="n">
         <v>290.4</v>
       </c>
-      <c r="K32" s="28" t="n"/>
+      <c r="K32" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L32" s="32" t="inlineStr">
         <is>
-          <t>Facture 20240616</t>
+          <t>Facture 20240616 — Facture BDH en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -1414,10 +1422,14 @@
       <c r="J33" s="33" t="n">
         <v>242</v>
       </c>
-      <c r="K33" s="28" t="n"/>
+      <c r="K33" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L33" s="32" t="inlineStr">
         <is>
-          <t>Facture 20240705</t>
+          <t>Facture 20240705 — Facture BDH en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilans 2025 et 2026 : carburant marque X
Le comptable ne demande pas de justificatif pour le carburant. 54 lignes en
2025 et 40 en 2026 recoivent un X ; les deux tickets Station 15 Zemst gardent
leur V puisque la piece existe.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -894,7 +894,11 @@
       <c r="J7" s="33" t="n">
         <v>22.9</v>
       </c>
-      <c r="K7" s="28" t="n"/>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L7" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -946,7 +950,11 @@
       <c r="J10" s="33" t="n">
         <v>62.79</v>
       </c>
-      <c r="K10" s="28" t="n"/>
+      <c r="K10" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L10" s="32" t="inlineStr">
         <is>
           <t>Cora Woluwe Carburant</t>
@@ -1042,7 +1050,11 @@
       <c r="J15" s="33" t="n">
         <v>66.72</v>
       </c>
-      <c r="K15" s="28" t="n"/>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L15" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -1170,7 +1182,11 @@
       <c r="J21" s="33" t="n">
         <v>71.13</v>
       </c>
-      <c r="K21" s="28" t="n"/>
+      <c r="K21" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L21" s="32" t="inlineStr">
         <is>
           <t>Cora Woluwe Carburant</t>
@@ -1310,7 +1326,11 @@
       <c r="J28" s="33" t="n">
         <v>69.44</v>
       </c>
-      <c r="K28" s="28" t="n"/>
+      <c r="K28" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L28" s="32" t="inlineStr">
         <is>
           <t>Lukoil Wezembeek</t>
@@ -1614,7 +1634,11 @@
       <c r="J42" s="33" t="n">
         <v>65</v>
       </c>
-      <c r="K42" s="28" t="n"/>
+      <c r="K42" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L42" s="32" t="inlineStr">
         <is>
           <t>Dats 24 Nossegem</t>
@@ -1730,7 +1754,11 @@
       <c r="J48" s="33" t="n">
         <v>69.47</v>
       </c>
-      <c r="K48" s="28" t="n"/>
+      <c r="K48" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L48" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -1882,7 +1910,11 @@
       <c r="J56" s="33" t="n">
         <v>68.61</v>
       </c>
-      <c r="K56" s="28" t="n"/>
+      <c r="K56" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L56" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -1998,7 +2030,11 @@
       <c r="J61" s="33" t="n">
         <v>66.06999999999999</v>
       </c>
-      <c r="K61" s="28" t="n"/>
+      <c r="K61" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L61" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -2146,7 +2182,11 @@
       <c r="J69" s="33" t="n">
         <v>67.55</v>
       </c>
-      <c r="K69" s="28" t="n"/>
+      <c r="K69" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L69" s="32" t="inlineStr">
         <is>
           <t>Q8 Limal</t>
@@ -2378,7 +2418,11 @@
       <c r="J80" s="33" t="n">
         <v>60.74</v>
       </c>
-      <c r="K80" s="28" t="n"/>
+      <c r="K80" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L80" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -2490,7 +2534,11 @@
       <c r="J85" s="33" t="n">
         <v>70.68000000000001</v>
       </c>
-      <c r="K85" s="28" t="n"/>
+      <c r="K85" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L85" s="32" t="inlineStr">
         <is>
           <t>Shell Kraainem</t>
@@ -2622,7 +2670,11 @@
       <c r="J91" s="33" t="n">
         <v>70.48999999999999</v>
       </c>
-      <c r="K91" s="28" t="n"/>
+      <c r="K91" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L91" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -2804,7 +2856,11 @@
       <c r="J101" s="33" t="n">
         <v>87</v>
       </c>
-      <c r="K101" s="28" t="n"/>
+      <c r="K101" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L101" s="32" t="inlineStr">
         <is>
           <t>Total Leyde (Pays-Bas)</t>
@@ -3652,7 +3708,11 @@
       <c r="J143" s="33" t="n">
         <v>72.18000000000001</v>
       </c>
-      <c r="K143" s="28" t="n"/>
+      <c r="K143" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L143" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -3752,7 +3812,11 @@
       <c r="J148" s="33" t="n">
         <v>64.06999999999999</v>
       </c>
-      <c r="K148" s="28" t="n"/>
+      <c r="K148" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L148" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -3816,7 +3880,11 @@
       <c r="J151" s="33" t="n">
         <v>60.37</v>
       </c>
-      <c r="K151" s="28" t="n"/>
+      <c r="K151" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L151" s="32" t="inlineStr">
         <is>
           <t>Lukoil Wezembeek</t>
@@ -4024,7 +4092,11 @@
       <c r="J162" s="33" t="n">
         <v>59.49</v>
       </c>
-      <c r="K162" s="28" t="n"/>
+      <c r="K162" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L162" s="32" t="inlineStr">
         <is>
           <t>Cora Woluwe Carburant</t>
@@ -4772,7 +4844,11 @@
       <c r="J199" s="33" t="n">
         <v>66.09</v>
       </c>
-      <c r="K199" s="28" t="n"/>
+      <c r="K199" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L199" s="32" t="inlineStr">
         <is>
           <t>Lukoil Tervuren</t>
@@ -4852,7 +4928,11 @@
       <c r="J203" s="33" t="n">
         <v>58.83</v>
       </c>
-      <c r="K203" s="28" t="n"/>
+      <c r="K203" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L203" s="32" t="inlineStr">
         <is>
           <t>Shell Kraainem</t>
@@ -4936,7 +5016,11 @@
       <c r="J207" s="33" t="n">
         <v>72.42</v>
       </c>
-      <c r="K207" s="28" t="n"/>
+      <c r="K207" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L207" s="32" t="inlineStr">
         <is>
           <t>Q8 Tervuren</t>
@@ -5104,7 +5188,11 @@
       <c r="J215" s="33" t="n">
         <v>55.61</v>
       </c>
-      <c r="K215" s="28" t="n"/>
+      <c r="K215" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L215" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -5180,7 +5268,11 @@
       <c r="J219" s="33" t="n">
         <v>75.87</v>
       </c>
-      <c r="K219" s="28" t="n"/>
+      <c r="K219" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L219" s="32" t="inlineStr">
         <is>
           <t>Station Avia, Havrincourt (France)</t>
@@ -6024,7 +6116,11 @@
       <c r="J261" s="33" t="n">
         <v>68.06</v>
       </c>
-      <c r="K261" s="28" t="n"/>
+      <c r="K261" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L261" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -6104,7 +6200,11 @@
       <c r="J265" s="33" t="n">
         <v>64.97</v>
       </c>
-      <c r="K265" s="28" t="n"/>
+      <c r="K265" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L265" s="32" t="inlineStr">
         <is>
           <t>Lukoil Tournai</t>
@@ -6168,7 +6268,11 @@
       <c r="J268" s="33" t="n">
         <v>54.33</v>
       </c>
-      <c r="K268" s="28" t="n"/>
+      <c r="K268" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L268" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -6418,7 +6522,11 @@
       <c r="J280" s="33" t="n">
         <v>60.86</v>
       </c>
-      <c r="K280" s="28" t="n"/>
+      <c r="K280" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L280" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -6982,7 +7090,11 @@
       <c r="J308" s="33" t="n">
         <v>56.98</v>
       </c>
-      <c r="K308" s="28" t="n"/>
+      <c r="K308" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L308" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -7002,7 +7114,11 @@
       <c r="J309" s="33" t="n">
         <v>62.27</v>
       </c>
-      <c r="K309" s="28" t="n"/>
+      <c r="K309" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L309" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -7130,7 +7246,11 @@
       <c r="J315" s="33" t="n">
         <v>60.9</v>
       </c>
-      <c r="K315" s="28" t="n"/>
+      <c r="K315" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L315" s="32" t="inlineStr">
         <is>
           <t>Maes Schaerbeek</t>
@@ -7186,7 +7306,11 @@
       <c r="J318" s="33" t="n">
         <v>43.01</v>
       </c>
-      <c r="K318" s="28" t="n"/>
+      <c r="K318" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L318" s="32" t="inlineStr">
         <is>
           <t>Esso Rumst</t>
@@ -7320,7 +7444,11 @@
       <c r="J325" s="33" t="n">
         <v>87.43000000000001</v>
       </c>
-      <c r="K325" s="28" t="n"/>
+      <c r="K325" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L325" s="32" t="inlineStr">
         <is>
           <t>Soulac-sur-Mer (France)</t>
@@ -7356,7 +7484,11 @@
       <c r="J327" s="33" t="n">
         <v>72.01000000000001</v>
       </c>
-      <c r="K327" s="28" t="n"/>
+      <c r="K327" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L327" s="32" t="inlineStr">
         <is>
           <t>BP Esso Saint-Léger (France)</t>
@@ -7376,7 +7508,11 @@
       <c r="J328" s="33" t="n">
         <v>77.28</v>
       </c>
-      <c r="K328" s="28" t="n"/>
+      <c r="K328" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L328" s="32" t="inlineStr">
         <is>
           <t>Shell Vémars (France)</t>
@@ -7640,7 +7776,11 @@
       <c r="J341" s="33" t="n">
         <v>66.73999999999999</v>
       </c>
-      <c r="K341" s="28" t="n"/>
+      <c r="K341" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L341" s="32" t="inlineStr">
         <is>
           <t>Carte Mastercard 26-07 — décompte n° 216 du 13-08 — Total Gidy (France)</t>
@@ -7704,7 +7844,11 @@
       <c r="J344" s="33" t="n">
         <v>62.86</v>
       </c>
-      <c r="K344" s="28" t="n"/>
+      <c r="K344" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L344" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -7744,7 +7888,11 @@
       <c r="J346" s="33" t="n">
         <v>72.59</v>
       </c>
-      <c r="K346" s="28" t="n"/>
+      <c r="K346" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L346" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -7998,7 +8146,11 @@
       <c r="J359" s="33" t="n">
         <v>65.14</v>
       </c>
-      <c r="K359" s="28" t="n"/>
+      <c r="K359" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L359" s="32" t="inlineStr">
         <is>
           <t>Q8 Tervuren</t>
@@ -8182,7 +8334,11 @@
       <c r="J368" s="33" t="n">
         <v>66.73999999999999</v>
       </c>
-      <c r="K368" s="28" t="n"/>
+      <c r="K368" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L368" s="32" t="inlineStr">
         <is>
           <t>Shell Kraainem</t>
@@ -8374,7 +8530,11 @@
       <c r="J377" s="33" t="n">
         <v>59.4</v>
       </c>
-      <c r="K377" s="28" t="n"/>
+      <c r="K377" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L377" s="32" t="inlineStr">
         <is>
           <t>Shell Kraainem</t>
@@ -8418,7 +8578,11 @@
       <c r="J379" s="33" t="n">
         <v>58.45</v>
       </c>
-      <c r="K379" s="28" t="n"/>
+      <c r="K379" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L379" s="32" t="inlineStr">
         <is>
           <t>Esso Péruwelz</t>
@@ -8530,7 +8694,11 @@
       <c r="J385" s="33" t="n">
         <v>68.23</v>
       </c>
-      <c r="K385" s="28" t="n"/>
+      <c r="K385" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L385" s="32" t="inlineStr">
         <is>
           <t>Total Hoegaarden</t>
@@ -8784,7 +8952,11 @@
       <c r="J397" s="33" t="n">
         <v>64.26000000000001</v>
       </c>
-      <c r="K397" s="28" t="n"/>
+      <c r="K397" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L397" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -8844,7 +9016,11 @@
       <c r="J400" s="33" t="n">
         <v>67.14</v>
       </c>
-      <c r="K400" s="28" t="n"/>
+      <c r="K400" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L400" s="32" t="inlineStr">
         <is>
           <t>Total Rumst</t>
@@ -8924,7 +9100,11 @@
       <c r="J404" s="33" t="n">
         <v>81.39</v>
       </c>
-      <c r="K404" s="28" t="n"/>
+      <c r="K404" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L404" s="32" t="inlineStr">
         <is>
           <t>Esso Dorst (Pays-Bas)</t>
@@ -8984,7 +9164,11 @@
       <c r="J407" s="33" t="n">
         <v>70.66</v>
       </c>
-      <c r="K407" s="28" t="n"/>
+      <c r="K407" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L407" s="32" t="inlineStr">
         <is>
           <t>Shell Kraainem</t>
@@ -9148,7 +9332,11 @@
       <c r="J416" s="39" t="n">
         <v>65.29000000000001</v>
       </c>
-      <c r="K416" s="28" t="n"/>
+      <c r="K416" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L416" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -9292,7 +9480,11 @@
       <c r="J423" s="33" t="n">
         <v>70.44</v>
       </c>
-      <c r="K423" s="28" t="n"/>
+      <c r="K423" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L423" s="32" t="inlineStr">
         <is>
           <t>Q8 Tervuren</t>
@@ -9472,7 +9664,11 @@
       <c r="J431" s="33" t="n">
         <v>65.52</v>
       </c>
-      <c r="K431" s="28" t="n"/>
+      <c r="K431" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L431" s="32" t="inlineStr">
         <is>
           <t>Shell Haine-Saint-Pierre</t>
@@ -9596,7 +9792,11 @@
       <c r="J437" s="33" t="n">
         <v>69.11</v>
       </c>
-      <c r="K437" s="28" t="n"/>
+      <c r="K437" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L437" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -9772,7 +9972,11 @@
       <c r="J446" s="33" t="n">
         <v>63.61</v>
       </c>
-      <c r="K446" s="28" t="n"/>
+      <c r="K446" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L446" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -9848,7 +10052,11 @@
       <c r="J450" s="33" t="n">
         <v>63.8</v>
       </c>
-      <c r="K450" s="28" t="n"/>
+      <c r="K450" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L450" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -9996,7 +10204,11 @@
       <c r="J457" s="33" t="n">
         <v>63.2</v>
       </c>
-      <c r="K457" s="28" t="n"/>
+      <c r="K457" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L457" s="32" t="inlineStr">
         <is>
           <t>Q8 Easy Zaventem</t>
@@ -10096,7 +10308,11 @@
       <c r="J462" s="33" t="n">
         <v>63.32</v>
       </c>
-      <c r="K462" s="28" t="n"/>
+      <c r="K462" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L462" s="32" t="inlineStr">
         <is>
           <t>Cora Woluwe Carburant</t>

</xml_diff>

<commit_message>
Bilans 2025 et 2026 : parkings, transports, credit voiture et impots marques X
Le comptable ne demande pas de justificatif pour ces postes non plus.
Bilan 2025 : 335 lignes traitees, 76.086,16 sur 88.541,37 (86 %).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -934,7 +934,11 @@
       <c r="J9" s="33" t="n">
         <v>1.35</v>
       </c>
-      <c r="K9" s="28" t="n"/>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L9" s="32" t="n"/>
     </row>
     <row r="10">
@@ -974,7 +978,11 @@
       <c r="J11" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K11" s="28" t="n"/>
+      <c r="K11" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L11" s="32" t="n"/>
     </row>
     <row r="12">
@@ -1074,7 +1082,11 @@
       <c r="J16" s="33" t="n">
         <v>22.5</v>
       </c>
-      <c r="K16" s="28" t="n"/>
+      <c r="K16" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L16" s="32" t="inlineStr">
         <is>
           <t>Parking Centraal Anvers</t>
@@ -1094,7 +1106,11 @@
       <c r="J17" s="33" t="n">
         <v>1.8</v>
       </c>
-      <c r="K17" s="28" t="n"/>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L17" s="32" t="inlineStr">
         <is>
           <t>Commune Saint-Josse</t>
@@ -1162,7 +1178,11 @@
       <c r="J20" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K20" s="28" t="n"/>
+      <c r="K20" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L20" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -1226,7 +1246,11 @@
       <c r="J23" s="33" t="n">
         <v>7.2</v>
       </c>
-      <c r="K23" s="28" t="n"/>
+      <c r="K23" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L23" s="32" t="inlineStr">
         <is>
           <t>Parking Rogier</t>
@@ -1246,7 +1270,11 @@
       <c r="J24" s="33" t="n">
         <v>2.68</v>
       </c>
-      <c r="K24" s="28" t="n"/>
+      <c r="K24" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L24" s="32" t="n"/>
     </row>
     <row r="25">
@@ -1350,7 +1378,11 @@
       <c r="J29" s="33" t="n">
         <v>4517.28</v>
       </c>
-      <c r="K29" s="28" t="n"/>
+      <c r="K29" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L29" s="32" t="inlineStr">
         <is>
           <t>Communication 202/9987/63859</t>
@@ -1566,7 +1598,11 @@
       <c r="J39" s="33" t="n">
         <v>2.1</v>
       </c>
-      <c r="K39" s="28" t="n"/>
+      <c r="K39" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L39" s="32" t="inlineStr">
         <is>
           <t>Indigo Park Docks</t>
@@ -1658,7 +1694,11 @@
       <c r="J43" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K43" s="28" t="n"/>
+      <c r="K43" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L43" s="32" t="n"/>
     </row>
     <row r="44">
@@ -1674,7 +1714,11 @@
       <c r="J44" s="33" t="n">
         <v>1.8</v>
       </c>
-      <c r="K44" s="28" t="n"/>
+      <c r="K44" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L44" s="32" t="inlineStr">
         <is>
           <t>Schaerbeek</t>
@@ -1694,7 +1738,11 @@
       <c r="J45" s="33" t="n">
         <v>6.2</v>
       </c>
-      <c r="K45" s="28" t="n"/>
+      <c r="K45" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L45" s="32" t="inlineStr">
         <is>
           <t>Administration communale Bruxelles</t>
@@ -1714,7 +1762,11 @@
       <c r="J46" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K46" s="28" t="n"/>
+      <c r="K46" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L46" s="32" t="inlineStr">
         <is>
           <t>Parking Ixelles - Gand</t>
@@ -1734,7 +1786,11 @@
       <c r="J47" s="33" t="n">
         <v>17.1</v>
       </c>
-      <c r="K47" s="28" t="n"/>
+      <c r="K47" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L47" s="32" t="inlineStr">
         <is>
           <t>Q-Park Heilig Hart Louvain</t>
@@ -1778,7 +1834,11 @@
       <c r="J49" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K49" s="28" t="n"/>
+      <c r="K49" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L49" s="32" t="n"/>
     </row>
     <row r="50">
@@ -1794,7 +1854,11 @@
       <c r="J50" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K50" s="28" t="n"/>
+      <c r="K50" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L50" s="32" t="n"/>
     </row>
     <row r="51">
@@ -1810,7 +1874,11 @@
       <c r="J51" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K51" s="28" t="n"/>
+      <c r="K51" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L51" s="32" t="inlineStr">
         <is>
           <t>Parkeren Louvain</t>
@@ -1830,7 +1898,11 @@
       <c r="J52" s="33" t="n">
         <v>1.8</v>
       </c>
-      <c r="K52" s="28" t="n"/>
+      <c r="K52" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L52" s="32" t="inlineStr">
         <is>
           <t>Commune Saint-Josse</t>
@@ -1890,7 +1962,11 @@
       <c r="J55" s="33" t="n">
         <v>6.5</v>
       </c>
-      <c r="K55" s="28" t="n"/>
+      <c r="K55" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L55" s="32" t="inlineStr">
         <is>
           <t>Parking Ixelles - Gand</t>
@@ -2122,7 +2198,11 @@
       <c r="J66" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K66" s="28" t="n"/>
+      <c r="K66" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L66" s="32" t="n"/>
     </row>
     <row r="67">
@@ -2162,7 +2242,11 @@
       <c r="J68" s="33" t="n">
         <v>6.3</v>
       </c>
-      <c r="K68" s="28" t="n"/>
+      <c r="K68" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L68" s="32" t="inlineStr">
         <is>
           <t>Brucity - Ville de Bruxelles</t>
@@ -2206,7 +2290,11 @@
       <c r="J70" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K70" s="28" t="n"/>
+      <c r="K70" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L70" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 21-02 — décompte n° 060 du 10-03</t>
@@ -2226,7 +2314,11 @@
       <c r="J71" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K71" s="28" t="n"/>
+      <c r="K71" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L71" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 22-02 — décompte n° 060 du 10-03</t>
@@ -2246,7 +2338,11 @@
       <c r="J72" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K72" s="28" t="n"/>
+      <c r="K72" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L72" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 27-02 — décompte n° 060 du 10-03</t>
@@ -2378,7 +2474,11 @@
       <c r="J78" s="33" t="n">
         <v>1.85</v>
       </c>
-      <c r="K78" s="28" t="n"/>
+      <c r="K78" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L78" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -2398,7 +2498,11 @@
       <c r="J79" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K79" s="28" t="n"/>
+      <c r="K79" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L79" s="32" t="inlineStr">
         <is>
           <t>T and T Parking Bruxelles</t>
@@ -2442,7 +2546,11 @@
       <c r="J81" s="33" t="n">
         <v>2.67</v>
       </c>
-      <c r="K81" s="28" t="n"/>
+      <c r="K81" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L81" s="32" t="inlineStr">
         <is>
           <t>Commune Saint-Josse</t>
@@ -2582,7 +2690,11 @@
       <c r="J87" s="33" t="n">
         <v>16.2</v>
       </c>
-      <c r="K87" s="28" t="n"/>
+      <c r="K87" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L87" s="32" t="inlineStr">
         <is>
           <t>Parking Rogier</t>
@@ -2602,7 +2714,11 @@
       <c r="J88" s="33" t="n">
         <v>3.2</v>
       </c>
-      <c r="K88" s="28" t="n"/>
+      <c r="K88" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L88" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -2744,7 +2860,11 @@
       <c r="J95" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K95" s="28" t="n"/>
+      <c r="K95" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L95" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -2764,7 +2884,11 @@
       <c r="J96" s="33" t="n">
         <v>18.4</v>
       </c>
-      <c r="K96" s="28" t="n"/>
+      <c r="K96" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L96" s="32" t="inlineStr">
         <is>
           <t>Delft (Pays-Bas)</t>
@@ -2784,7 +2908,11 @@
       <c r="J97" s="33" t="n">
         <v>10.4</v>
       </c>
-      <c r="K97" s="28" t="n"/>
+      <c r="K97" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L97" s="32" t="inlineStr">
         <is>
           <t>Markthof La Haye (Pays-Bas)</t>
@@ -2804,7 +2932,11 @@
       <c r="J98" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K98" s="28" t="n"/>
+      <c r="K98" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L98" s="32" t="n"/>
     </row>
     <row r="99">
@@ -2820,7 +2952,11 @@
       <c r="J99" s="33" t="n">
         <v>23</v>
       </c>
-      <c r="K99" s="28" t="n"/>
+      <c r="K99" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L99" s="32" t="inlineStr">
         <is>
           <t>Stadparkeerplan Leyde (Pays-Bas)</t>
@@ -2880,7 +3016,11 @@
       <c r="J102" s="33" t="n">
         <v>10.46</v>
       </c>
-      <c r="K102" s="28" t="n"/>
+      <c r="K102" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L102" s="32" t="inlineStr">
         <is>
           <t>Commune d'Utrecht (Pays-Bas)</t>
@@ -2900,7 +3040,11 @@
       <c r="J103" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="K103" s="28" t="n"/>
+      <c r="K103" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L103" s="32" t="inlineStr">
         <is>
           <t>Parking De Vooruitgang, Volendam (Pays-Bas)</t>
@@ -2964,7 +3108,11 @@
       <c r="J106" s="33" t="n">
         <v>32.76</v>
       </c>
-      <c r="K106" s="28" t="n"/>
+      <c r="K106" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L106" s="32" t="inlineStr">
         <is>
           <t>Commune d'Utrecht (Pays-Bas)</t>
@@ -3008,7 +3156,11 @@
       <c r="J108" s="33" t="n">
         <v>8</v>
       </c>
-      <c r="K108" s="28" t="n"/>
+      <c r="K108" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L108" s="32" t="inlineStr">
         <is>
           <t>Q-Park Sint Jorisplein, Amersfoort (Pays-Bas)</t>
@@ -3048,7 +3200,11 @@
       <c r="J110" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K110" s="28" t="n"/>
+      <c r="K110" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L110" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 01-03 — décompte n° 091 du 10-04</t>
@@ -3148,7 +3304,11 @@
       <c r="J115" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K115" s="28" t="n"/>
+      <c r="K115" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L115" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 10-03 — décompte n° 091 du 10-04</t>
@@ -3168,7 +3328,11 @@
       <c r="J116" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K116" s="28" t="n"/>
+      <c r="K116" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L116" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 11-03 — décompte n° 091 du 10-04</t>
@@ -3188,7 +3352,11 @@
       <c r="J117" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K117" s="28" t="n"/>
+      <c r="K117" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L117" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 11-03 — décompte n° 091 du 10-04</t>
@@ -3228,7 +3396,11 @@
       <c r="J119" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K119" s="28" t="n"/>
+      <c r="K119" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L119" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 12-03 — décompte n° 091 du 10-04</t>
@@ -3248,7 +3420,11 @@
       <c r="J120" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K120" s="28" t="n"/>
+      <c r="K120" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L120" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 12-03 — décompte n° 091 du 10-04</t>
@@ -3268,7 +3444,11 @@
       <c r="J121" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K121" s="28" t="n"/>
+      <c r="K121" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L121" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 13-03 — décompte n° 091 du 10-04</t>
@@ -3288,7 +3468,11 @@
       <c r="J122" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K122" s="28" t="n"/>
+      <c r="K122" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L122" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 14-03 — décompte n° 091 du 10-04</t>
@@ -3308,7 +3492,11 @@
       <c r="J123" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="K123" s="28" t="n"/>
+      <c r="K123" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L123" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 15-03 — décompte n° 091 du 10-04</t>
@@ -3328,7 +3516,11 @@
       <c r="J124" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K124" s="28" t="n"/>
+      <c r="K124" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L124" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 15-03 — décompte n° 091 du 10-04</t>
@@ -3388,7 +3580,11 @@
       <c r="J127" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K127" s="28" t="n"/>
+      <c r="K127" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L127" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 22-03 — décompte n° 091 du 10-04</t>
@@ -3408,7 +3604,11 @@
       <c r="J128" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K128" s="28" t="n"/>
+      <c r="K128" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L128" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 23-03 — décompte n° 091 du 10-04</t>
@@ -3428,7 +3628,11 @@
       <c r="J129" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K129" s="28" t="n"/>
+      <c r="K129" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L129" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 24-03 — décompte n° 091 du 10-04</t>
@@ -3448,7 +3652,11 @@
       <c r="J130" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K130" s="28" t="n"/>
+      <c r="K130" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L130" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 26-03 — décompte n° 091 du 10-04</t>
@@ -3468,7 +3676,11 @@
       <c r="J131" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K131" s="28" t="n"/>
+      <c r="K131" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L131" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 27-03 — décompte n° 091 du 10-04</t>
@@ -3628,7 +3840,11 @@
       <c r="J139" s="33" t="n">
         <v>6.9</v>
       </c>
-      <c r="K139" s="28" t="n"/>
+      <c r="K139" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L139" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 29-03 — décompte n° 091 du 10-04</t>
@@ -3648,7 +3864,11 @@
       <c r="J140" s="33" t="n">
         <v>2.5</v>
       </c>
-      <c r="K140" s="28" t="n"/>
+      <c r="K140" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L140" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 30-03 — décompte n° 091 du 10-04</t>
@@ -3732,7 +3952,11 @@
       <c r="J144" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K144" s="28" t="n"/>
+      <c r="K144" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L144" s="32" t="inlineStr">
         <is>
           <t>T and T Parking Bruxelles</t>
@@ -3752,7 +3976,11 @@
       <c r="J145" s="33" t="n">
         <v>14</v>
       </c>
-      <c r="K145" s="28" t="n"/>
+      <c r="K145" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L145" s="32" t="inlineStr">
         <is>
           <t>Parking Casino Middelkerke</t>
@@ -3986,7 +4214,11 @@
       <c r="J157" s="39" t="n">
         <v>724.12</v>
       </c>
-      <c r="K157" s="28" t="n"/>
+      <c r="K157" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L157" s="32" t="n"/>
     </row>
     <row r="158">
@@ -4116,7 +4348,11 @@
       <c r="J163" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K163" s="28" t="n"/>
+      <c r="K163" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L163" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -4456,7 +4692,11 @@
       <c r="J180" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K180" s="28" t="n"/>
+      <c r="K180" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L180" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 12-04 — décompte n° 121 du 12-05</t>
@@ -4496,7 +4736,11 @@
       <c r="J182" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K182" s="28" t="n"/>
+      <c r="K182" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L182" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 14-04 — décompte n° 121 du 12-05</t>
@@ -4516,7 +4760,11 @@
       <c r="J183" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K183" s="28" t="n"/>
+      <c r="K183" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L183" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 15-04 — décompte n° 121 du 12-05</t>
@@ -4576,7 +4824,11 @@
       <c r="J186" s="33" t="n">
         <v>6.9</v>
       </c>
-      <c r="K186" s="28" t="n"/>
+      <c r="K186" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L186" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 16-04 — décompte n° 121 du 12-05</t>
@@ -4596,7 +4848,11 @@
       <c r="J187" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K187" s="28" t="n"/>
+      <c r="K187" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L187" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 17-04 — décompte n° 121 du 12-05</t>
@@ -4636,7 +4892,11 @@
       <c r="J189" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K189" s="28" t="n"/>
+      <c r="K189" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L189" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 18-04 — décompte n° 121 du 12-05</t>
@@ -4676,7 +4936,11 @@
       <c r="J191" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K191" s="28" t="n"/>
+      <c r="K191" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L191" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 19-04 — décompte n° 121 du 12-05</t>
@@ -4716,7 +4980,11 @@
       <c r="J193" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K193" s="28" t="n"/>
+      <c r="K193" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L193" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 23-04 — décompte n° 121 du 12-05</t>
@@ -4756,7 +5024,11 @@
       <c r="J195" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K195" s="28" t="n"/>
+      <c r="K195" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L195" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 25-04 — décompte n° 121 du 12-05</t>
@@ -4908,7 +5180,11 @@
       <c r="J202" s="33" t="n">
         <v>16.5</v>
       </c>
-      <c r="K202" s="28" t="n"/>
+      <c r="K202" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L202" s="32" t="inlineStr">
         <is>
           <t>Bonner City Parkraum, Bonn (Allemagne)</t>
@@ -4952,7 +5228,11 @@
       <c r="J204" s="33" t="n">
         <v>1.85</v>
       </c>
-      <c r="K204" s="28" t="n"/>
+      <c r="K204" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L204" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -4972,7 +5252,11 @@
       <c r="J205" s="33" t="n">
         <v>1.85</v>
       </c>
-      <c r="K205" s="28" t="n"/>
+      <c r="K205" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L205" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -5040,7 +5324,11 @@
       <c r="J208" s="33" t="n">
         <v>1.5</v>
       </c>
-      <c r="K208" s="28" t="n"/>
+      <c r="K208" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L208" s="32" t="inlineStr">
         <is>
           <t>Ville de Dinant</t>
@@ -5212,7 +5500,11 @@
       <c r="J216" s="33" t="n">
         <v>3.7</v>
       </c>
-      <c r="K216" s="28" t="n"/>
+      <c r="K216" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L216" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -5232,7 +5524,11 @@
       <c r="J217" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K217" s="28" t="n"/>
+      <c r="K217" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L217" s="32" t="n"/>
     </row>
     <row r="218">
@@ -5248,7 +5544,11 @@
       <c r="J218" s="33" t="n">
         <v>15.8</v>
       </c>
-      <c r="K218" s="28" t="n"/>
+      <c r="K218" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L218" s="32" t="inlineStr">
         <is>
           <t>RG Public, Paris (France)</t>
@@ -5292,7 +5592,11 @@
       <c r="J220" s="33" t="n">
         <v>31.05</v>
       </c>
-      <c r="K220" s="28" t="n"/>
+      <c r="K220" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L220" s="32" t="inlineStr">
         <is>
           <t>Indigo, Paris (France)</t>
@@ -5312,7 +5616,11 @@
       <c r="J221" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K221" s="28" t="n"/>
+      <c r="K221" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L221" s="32" t="inlineStr">
         <is>
           <t>Brussels Expo Parking</t>
@@ -5332,7 +5640,11 @@
       <c r="J222" s="33" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K222" s="28" t="n"/>
+      <c r="K222" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L222" s="32" t="inlineStr">
         <is>
           <t>Parking Ladeuze, Louvain</t>
@@ -5352,7 +5664,11 @@
       <c r="J223" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="K223" s="28" t="n"/>
+      <c r="K223" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L223" s="32" t="inlineStr">
         <is>
           <t>Province du Brabant flamand, Kessel-Lo</t>
@@ -5412,7 +5728,11 @@
       <c r="J226" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K226" s="28" t="n"/>
+      <c r="K226" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L226" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 03-05 — décompte n° 152 du 10-06</t>
@@ -5472,7 +5792,11 @@
       <c r="J229" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="K229" s="28" t="n"/>
+      <c r="K229" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L229" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 09-05 — décompte n° 152 du 10-06</t>
@@ -5492,7 +5816,11 @@
       <c r="J230" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K230" s="28" t="n"/>
+      <c r="K230" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L230" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 09-05 — décompte n° 152 du 10-06</t>
@@ -5532,7 +5860,11 @@
       <c r="J232" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="K232" s="28" t="n"/>
+      <c r="K232" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L232" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 10-05 — décompte n° 152 du 10-06</t>
@@ -5552,7 +5884,11 @@
       <c r="J233" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K233" s="28" t="n"/>
+      <c r="K233" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L233" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 11-05 — décompte n° 152 du 10-06</t>
@@ -5572,7 +5908,11 @@
       <c r="J234" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K234" s="28" t="n"/>
+      <c r="K234" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L234" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 12-05 — décompte n° 152 du 10-06</t>
@@ -5592,7 +5932,11 @@
       <c r="J235" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K235" s="28" t="n"/>
+      <c r="K235" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L235" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 13-05 — décompte n° 152 du 10-06</t>
@@ -5632,7 +5976,11 @@
       <c r="J237" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K237" s="28" t="n"/>
+      <c r="K237" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L237" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 14-05 — décompte n° 152 du 10-06</t>
@@ -5652,7 +6000,11 @@
       <c r="J238" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="K238" s="28" t="n"/>
+      <c r="K238" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L238" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 15-05 — décompte n° 152 du 10-06</t>
@@ -5672,7 +6024,11 @@
       <c r="J239" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="K239" s="28" t="n"/>
+      <c r="K239" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L239" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 15-05 — décompte n° 152 du 10-06</t>
@@ -5692,7 +6048,11 @@
       <c r="J240" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K240" s="28" t="n"/>
+      <c r="K240" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L240" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 15-05 — décompte n° 152 du 10-06</t>
@@ -5712,7 +6072,11 @@
       <c r="J241" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="K241" s="28" t="n"/>
+      <c r="K241" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L241" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 16-05 — décompte n° 152 du 10-06</t>
@@ -5732,7 +6096,11 @@
       <c r="J242" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K242" s="28" t="n"/>
+      <c r="K242" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L242" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 17-05 — décompte n° 152 du 10-06</t>
@@ -5752,7 +6120,11 @@
       <c r="J243" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K243" s="28" t="n"/>
+      <c r="K243" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L243" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 19-05 — décompte n° 152 du 10-06</t>
@@ -5772,7 +6144,11 @@
       <c r="J244" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K244" s="28" t="n"/>
+      <c r="K244" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L244" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 20-05 — décompte n° 152 du 10-06</t>
@@ -5812,7 +6188,11 @@
       <c r="J246" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K246" s="28" t="n"/>
+      <c r="K246" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L246" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 21-05 — décompte n° 152 du 10-06</t>
@@ -5832,7 +6212,11 @@
       <c r="J247" s="33" t="n">
         <v>15</v>
       </c>
-      <c r="K247" s="28" t="n"/>
+      <c r="K247" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L247" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 22-05 — décompte n° 152 du 10-06</t>
@@ -5852,7 +6236,11 @@
       <c r="J248" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K248" s="28" t="n"/>
+      <c r="K248" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L248" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 22-05 — décompte n° 152 du 10-06</t>
@@ -5872,7 +6260,11 @@
       <c r="J249" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K249" s="28" t="n"/>
+      <c r="K249" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L249" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 23-05 — décompte n° 152 du 10-06</t>
@@ -5892,7 +6284,11 @@
       <c r="J250" s="33" t="n">
         <v>6.9</v>
       </c>
-      <c r="K250" s="28" t="n"/>
+      <c r="K250" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L250" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 23-05 — décompte n° 152 du 10-06</t>
@@ -5912,7 +6308,11 @@
       <c r="J251" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K251" s="28" t="n"/>
+      <c r="K251" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L251" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 24-05 — décompte n° 152 du 10-06</t>
@@ -5952,7 +6352,11 @@
       <c r="J253" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K253" s="28" t="n"/>
+      <c r="K253" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L253" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 27-05 — décompte n° 152 du 10-06</t>
@@ -5972,7 +6376,11 @@
       <c r="J254" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K254" s="28" t="n"/>
+      <c r="K254" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L254" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 28-05 — décompte n° 152 du 10-06</t>
@@ -5992,7 +6400,11 @@
       <c r="J255" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K255" s="28" t="n"/>
+      <c r="K255" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L255" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 28-05 — décompte n° 152 du 10-06</t>
@@ -6012,7 +6424,11 @@
       <c r="J256" s="33" t="n">
         <v>24</v>
       </c>
-      <c r="K256" s="28" t="n"/>
+      <c r="K256" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L256" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 29-05 — décompte n° 152 du 10-06</t>
@@ -6032,7 +6448,11 @@
       <c r="J257" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K257" s="28" t="n"/>
+      <c r="K257" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L257" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 30-05 — décompte n° 152 du 10-06</t>
@@ -6052,7 +6472,11 @@
       <c r="J258" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K258" s="28" t="n"/>
+      <c r="K258" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L258" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 31-05 — décompte n° 152 du 10-06</t>
@@ -6140,7 +6564,11 @@
       <c r="J262" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="K262" s="28" t="n"/>
+      <c r="K262" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L262" s="32" t="inlineStr">
         <is>
           <t>Parking Grand-Place, Bruxelles</t>
@@ -6160,7 +6588,11 @@
       <c r="J263" s="33" t="n">
         <v>3.6</v>
       </c>
-      <c r="K263" s="28" t="n"/>
+      <c r="K263" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L263" s="32" t="inlineStr">
         <is>
           <t>Parkeren Sint-Gillis, Gand</t>
@@ -6180,7 +6612,11 @@
       <c r="J264" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="K264" s="28" t="n"/>
+      <c r="K264" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L264" s="32" t="inlineStr">
         <is>
           <t>Parking FP1, Zaventem</t>
@@ -6248,7 +6684,11 @@
       <c r="J267" s="33" t="n">
         <v>1.85</v>
       </c>
-      <c r="K267" s="28" t="n"/>
+      <c r="K267" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L267" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -6292,7 +6732,11 @@
       <c r="J269" s="33" t="n">
         <v>3.5</v>
       </c>
-      <c r="K269" s="28" t="n"/>
+      <c r="K269" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L269" s="32" t="inlineStr">
         <is>
           <t>Parking Sint-Pieters, Gand</t>
@@ -6312,7 +6756,11 @@
       <c r="J270" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K270" s="28" t="n"/>
+      <c r="K270" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L270" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -6470,7 +6918,11 @@
       <c r="J277" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K277" s="28" t="n"/>
+      <c r="K277" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L277" s="32" t="n"/>
     </row>
     <row r="278">
@@ -6626,7 +7078,11 @@
       <c r="J285" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K285" s="28" t="n"/>
+      <c r="K285" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L285" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 03-06 — décompte n° 182 du 10-07</t>
@@ -6646,7 +7102,11 @@
       <c r="J286" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="K286" s="28" t="n"/>
+      <c r="K286" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L286" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 04-06 — décompte n° 182 du 10-07</t>
@@ -6666,7 +7126,11 @@
       <c r="J287" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K287" s="28" t="n"/>
+      <c r="K287" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L287" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 04-06 — décompte n° 182 du 10-07</t>
@@ -6686,7 +7150,11 @@
       <c r="J288" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K288" s="28" t="n"/>
+      <c r="K288" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L288" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 05-06 — décompte n° 182 du 10-07</t>
@@ -6706,7 +7174,11 @@
       <c r="J289" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K289" s="28" t="n"/>
+      <c r="K289" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L289" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 06-06 — décompte n° 182 du 10-07</t>
@@ -6746,7 +7218,11 @@
       <c r="J291" s="33" t="n">
         <v>6.9</v>
       </c>
-      <c r="K291" s="28" t="n"/>
+      <c r="K291" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L291" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 06-06 — décompte n° 182 du 10-07</t>
@@ -6766,7 +7242,11 @@
       <c r="J292" s="33" t="n">
         <v>18</v>
       </c>
-      <c r="K292" s="28" t="n"/>
+      <c r="K292" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L292" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 07-06 — décompte n° 182 du 10-07</t>
@@ -6846,7 +7326,11 @@
       <c r="J296" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K296" s="28" t="n"/>
+      <c r="K296" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L296" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 10-06 — décompte n° 182 du 10-07</t>
@@ -6866,7 +7350,11 @@
       <c r="J297" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K297" s="28" t="n"/>
+      <c r="K297" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L297" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 11-06 — décompte n° 182 du 10-07</t>
@@ -6886,7 +7374,11 @@
       <c r="J298" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K298" s="28" t="n"/>
+      <c r="K298" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L298" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 12-06 — décompte n° 182 du 10-07</t>
@@ -6906,7 +7398,11 @@
       <c r="J299" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K299" s="28" t="n"/>
+      <c r="K299" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L299" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 17-06 — décompte n° 182 du 10-07</t>
@@ -6926,7 +7422,11 @@
       <c r="J300" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K300" s="28" t="n"/>
+      <c r="K300" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L300" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 18-06 — décompte n° 182 du 10-07</t>
@@ -6946,7 +7446,11 @@
       <c r="J301" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K301" s="28" t="n"/>
+      <c r="K301" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L301" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 19-06 — décompte n° 182 du 10-07</t>
@@ -6966,7 +7470,11 @@
       <c r="J302" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K302" s="28" t="n"/>
+      <c r="K302" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L302" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 20-06 — décompte n° 182 du 10-07</t>
@@ -6986,7 +7494,11 @@
       <c r="J303" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K303" s="28" t="n"/>
+      <c r="K303" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L303" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 21-06 — décompte n° 182 du 10-07</t>
@@ -7006,7 +7518,11 @@
       <c r="J304" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K304" s="28" t="n"/>
+      <c r="K304" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L304" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 23-06 — décompte n° 182 du 10-07</t>
@@ -7026,7 +7542,11 @@
       <c r="J305" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="K305" s="28" t="n"/>
+      <c r="K305" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L305" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 25-06 — décompte n° 182 du 10-07</t>
@@ -7046,7 +7566,11 @@
       <c r="J306" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K306" s="28" t="n"/>
+      <c r="K306" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L306" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 27-06 — décompte n° 182 du 10-07</t>
@@ -7138,7 +7662,11 @@
       <c r="J310" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K310" s="28" t="n"/>
+      <c r="K310" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L310" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -7270,7 +7798,11 @@
       <c r="J316" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K316" s="28" t="n"/>
+      <c r="K316" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L316" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -7330,7 +7862,11 @@
       <c r="J319" s="33" t="n">
         <v>1.7</v>
       </c>
-      <c r="K319" s="28" t="n"/>
+      <c r="K319" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L319" s="32" t="inlineStr">
         <is>
           <t>Indigo, Tours (France)</t>
@@ -7350,7 +7886,11 @@
       <c r="J320" s="33" t="n">
         <v>2.8</v>
       </c>
-      <c r="K320" s="28" t="n"/>
+      <c r="K320" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L320" s="32" t="inlineStr">
         <is>
           <t>Commune de Soulac-sur-Mer (France)</t>
@@ -7468,7 +8008,11 @@
       <c r="J326" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K326" s="28" t="n"/>
+      <c r="K326" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L326" s="32" t="n"/>
     </row>
     <row r="327">
@@ -7616,7 +8160,11 @@
       <c r="J333" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="K333" s="28" t="n"/>
+      <c r="K333" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L333" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 10-07 — décompte n° 213 du 11-08</t>
@@ -7656,7 +8204,11 @@
       <c r="J335" s="33" t="n">
         <v>42.66</v>
       </c>
-      <c r="K335" s="28" t="n"/>
+      <c r="K335" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L335" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 14-07 — décompte n° 213 du 11-08</t>
@@ -7676,7 +8228,11 @@
       <c r="J336" s="33" t="n">
         <v>48.18</v>
       </c>
-      <c r="K336" s="28" t="n"/>
+      <c r="K336" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L336" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 14-07 — décompte n° 213 du 11-08</t>
@@ -7696,7 +8252,11 @@
       <c r="J337" s="33" t="n">
         <v>111.19</v>
       </c>
-      <c r="K337" s="28" t="n"/>
+      <c r="K337" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L337" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 15-07 — décompte n° 213 du 11-08</t>
@@ -7716,7 +8276,11 @@
       <c r="J338" s="33" t="n">
         <v>91.52</v>
       </c>
-      <c r="K338" s="28" t="n"/>
+      <c r="K338" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L338" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 15-07 — décompte n° 213 du 11-08</t>
@@ -7736,7 +8300,11 @@
       <c r="J339" s="33" t="n">
         <v>2.3</v>
       </c>
-      <c r="K339" s="28" t="n"/>
+      <c r="K339" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L339" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 17-07 — décompte n° 213 du 11-08</t>
@@ -7756,7 +8324,11 @@
       <c r="J340" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K340" s="28" t="n"/>
+      <c r="K340" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L340" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 19-07 — décompte n° 213 du 11-08</t>
@@ -7800,7 +8372,11 @@
       <c r="J342" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K342" s="28" t="n"/>
+      <c r="K342" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L342" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -7912,7 +8488,11 @@
       <c r="J347" s="33" t="n">
         <v>4.2</v>
       </c>
-      <c r="K347" s="28" t="n"/>
+      <c r="K347" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L347" s="32" t="inlineStr">
         <is>
           <t>Parking Parkpoort, Heverlee</t>
@@ -7932,7 +8512,11 @@
       <c r="J348" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K348" s="28" t="n"/>
+      <c r="K348" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L348" s="32" t="inlineStr">
         <is>
           <t>Parking Ladeuze, Louvain</t>
@@ -7952,7 +8536,11 @@
       <c r="J349" s="33" t="n">
         <v>2.8</v>
       </c>
-      <c r="K349" s="28" t="n"/>
+      <c r="K349" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L349" s="32" t="inlineStr">
         <is>
           <t>Indigo Park Docks, Bruxelles</t>
@@ -7972,7 +8560,11 @@
       <c r="J350" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="K350" s="28" t="n"/>
+      <c r="K350" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L350" s="32" t="inlineStr">
         <is>
           <t>Parking Bokrijk, Genk</t>
@@ -7992,7 +8584,11 @@
       <c r="J351" s="33" t="n">
         <v>5.55</v>
       </c>
-      <c r="K351" s="28" t="n"/>
+      <c r="K351" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L351" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -8012,7 +8608,11 @@
       <c r="J352" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K352" s="28" t="n"/>
+      <c r="K352" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L352" s="32" t="inlineStr">
         <is>
           <t>Brussels Expo Parking</t>
@@ -8032,7 +8632,11 @@
       <c r="J353" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K353" s="28" t="n"/>
+      <c r="K353" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L353" s="32" t="inlineStr">
         <is>
           <t>Parking Grand-Place, Bruxelles</t>
@@ -8234,7 +8838,11 @@
       <c r="J363" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K363" s="28" t="n"/>
+      <c r="K363" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L363" s="32" t="n"/>
     </row>
     <row r="364">
@@ -8274,7 +8882,11 @@
       <c r="J365" s="33" t="n">
         <v>161.02</v>
       </c>
-      <c r="K365" s="28" t="n"/>
+      <c r="K365" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L365" s="32" t="inlineStr">
         <is>
           <t>Comm. 255/2756/05470</t>
@@ -8294,7 +8906,11 @@
       <c r="J366" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K366" s="28" t="n"/>
+      <c r="K366" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L366" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 13-08 — décompte n° 244 du 10-09</t>
@@ -8314,7 +8930,11 @@
       <c r="J367" s="33" t="n">
         <v>3.2</v>
       </c>
-      <c r="K367" s="28" t="n"/>
+      <c r="K367" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L367" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -8382,7 +9002,11 @@
       <c r="J370" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K370" s="28" t="n"/>
+      <c r="K370" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L370" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -8426,7 +9050,11 @@
       <c r="J372" s="33" t="n">
         <v>0.9</v>
       </c>
-      <c r="K372" s="28" t="n"/>
+      <c r="K372" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L372" s="32" t="inlineStr">
         <is>
           <t>Schaerbeek</t>
@@ -8490,7 +9118,11 @@
       <c r="J375" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K375" s="28" t="n"/>
+      <c r="K375" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L375" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -8672,7 +9304,11 @@
       <c r="J384" s="39" t="n">
         <v>724.12</v>
       </c>
-      <c r="K384" s="28" t="n"/>
+      <c r="K384" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L384" s="32" t="n"/>
     </row>
     <row r="385">
@@ -8788,7 +9424,11 @@
       <c r="J389" s="33" t="n">
         <v>10</v>
       </c>
-      <c r="K389" s="28" t="n"/>
+      <c r="K389" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L389" s="32" t="inlineStr">
         <is>
           <t>Parking 't Centrum, Valkenburg (Pays-Bas)</t>
@@ -8808,7 +9448,11 @@
       <c r="J390" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="K390" s="28" t="n"/>
+      <c r="K390" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L390" s="32" t="inlineStr">
         <is>
           <t>Valkenburg (Pays-Bas)</t>
@@ -8844,7 +9488,11 @@
       <c r="J392" s="33" t="n">
         <v>1.85</v>
       </c>
-      <c r="K392" s="28" t="n"/>
+      <c r="K392" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L392" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -8932,7 +9580,11 @@
       <c r="J396" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="K396" s="28" t="n"/>
+      <c r="K396" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L396" s="32" t="inlineStr">
         <is>
           <t>Parking FP1, Zaventem</t>
@@ -8976,7 +9628,11 @@
       <c r="J398" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K398" s="28" t="n"/>
+      <c r="K398" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L398" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -8996,7 +9652,11 @@
       <c r="J399" s="33" t="n">
         <v>12</v>
       </c>
-      <c r="K399" s="28" t="n"/>
+      <c r="K399" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L399" s="32" t="inlineStr">
         <is>
           <t>Brussels Expo Parking</t>
@@ -9040,7 +9700,11 @@
       <c r="J401" s="33" t="n">
         <v>7.7</v>
       </c>
-      <c r="K401" s="28" t="n"/>
+      <c r="K401" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L401" s="32" t="inlineStr">
         <is>
           <t>Parking De Vooruitgang, Volendam (Pays-Bas)</t>
@@ -9060,7 +9724,11 @@
       <c r="J402" s="33" t="n">
         <v>3.2</v>
       </c>
-      <c r="K402" s="28" t="n"/>
+      <c r="K402" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L402" s="32" t="inlineStr">
         <is>
           <t>Zaanstad (Pays-Bas)</t>
@@ -9080,7 +9748,11 @@
       <c r="J403" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="K403" s="28" t="n"/>
+      <c r="K403" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L403" s="32" t="inlineStr">
         <is>
           <t>Q-Park Rozenhof, Zaandam (Pays-Bas)</t>
@@ -9124,7 +9796,11 @@
       <c r="J405" s="33" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="K405" s="28" t="n"/>
+      <c r="K405" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L405" s="32" t="inlineStr">
         <is>
           <t>Parking Ladeuze, Louvain</t>
@@ -9144,7 +9820,11 @@
       <c r="J406" s="33" t="n">
         <v>1.8</v>
       </c>
-      <c r="K406" s="28" t="n"/>
+      <c r="K406" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L406" s="32" t="inlineStr">
         <is>
           <t>Commune Saint-Josse</t>
@@ -9188,7 +9868,11 @@
       <c r="J408" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="K408" s="28" t="n"/>
+      <c r="K408" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L408" s="32" t="inlineStr">
         <is>
           <t>Parking Bokrijk, Genk</t>
@@ -9208,7 +9892,11 @@
       <c r="J409" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K409" s="28" t="n"/>
+      <c r="K409" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L409" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -9228,7 +9916,11 @@
       <c r="J410" s="33" t="n">
         <v>5500</v>
       </c>
-      <c r="K410" s="28" t="n"/>
+      <c r="K410" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L410" s="32" t="inlineStr">
         <is>
           <t>Comm. 073/4616/33527</t>
@@ -9248,7 +9940,11 @@
       <c r="J411" s="35" t="n">
         <v>2100</v>
       </c>
-      <c r="K411" s="28" t="n"/>
+      <c r="K411" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L411" s="36" t="inlineStr">
         <is>
           <t>Comm. 204/0596/50233 — lié à une distribution de dividendes ?</t>
@@ -9444,7 +10140,11 @@
       <c r="J421" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K421" s="28" t="n"/>
+      <c r="K421" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L421" s="32" t="n"/>
     </row>
     <row r="422">
@@ -9460,7 +10160,11 @@
       <c r="J422" s="33" t="n">
         <v>2.72</v>
       </c>
-      <c r="K422" s="28" t="n"/>
+      <c r="K422" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L422" s="32" t="inlineStr">
         <is>
           <t>Commune Saint-Josse</t>
@@ -9504,7 +10208,11 @@
       <c r="J424" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K424" s="28" t="n"/>
+      <c r="K424" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L424" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -9524,7 +10232,11 @@
       <c r="J425" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K425" s="28" t="n"/>
+      <c r="K425" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L425" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -9688,7 +10400,11 @@
       <c r="J432" s="33" t="n">
         <v>0.9</v>
       </c>
-      <c r="K432" s="28" t="n"/>
+      <c r="K432" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L432" s="32" t="inlineStr">
         <is>
           <t>Schaerbeek</t>
@@ -9708,7 +10424,11 @@
       <c r="J433" s="33" t="n">
         <v>2.68</v>
       </c>
-      <c r="K433" s="28" t="n"/>
+      <c r="K433" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L433" s="32" t="inlineStr">
         <is>
           <t>Louvain</t>
@@ -9752,7 +10472,11 @@
       <c r="J435" s="33" t="n">
         <v>12.6</v>
       </c>
-      <c r="K435" s="28" t="n"/>
+      <c r="K435" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L435" s="32" t="inlineStr">
         <is>
           <t>Parking Rogier</t>
@@ -9772,7 +10496,11 @@
       <c r="J436" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K436" s="28" t="n"/>
+      <c r="K436" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L436" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -9816,7 +10544,11 @@
       <c r="J438" s="33" t="n">
         <v>1.85</v>
       </c>
-      <c r="K438" s="28" t="n"/>
+      <c r="K438" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L438" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -9856,7 +10588,11 @@
       <c r="J440" s="33" t="n">
         <v>5.55</v>
       </c>
-      <c r="K440" s="28" t="n"/>
+      <c r="K440" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L440" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -9876,7 +10612,11 @@
       <c r="J441" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K441" s="28" t="n"/>
+      <c r="K441" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L441" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -9996,7 +10736,11 @@
       <c r="J447" s="33" t="n">
         <v>724.12</v>
       </c>
-      <c r="K447" s="28" t="n"/>
+      <c r="K447" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L447" s="32" t="n"/>
     </row>
     <row r="448">
@@ -10012,7 +10756,11 @@
       <c r="J448" s="33" t="n">
         <v>4.6</v>
       </c>
-      <c r="K448" s="28" t="n"/>
+      <c r="K448" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L448" s="32" t="inlineStr">
         <is>
           <t>Indigo Park Docks, Bruxelles</t>
@@ -10032,7 +10780,11 @@
       <c r="J449" s="33" t="n">
         <v>3.2</v>
       </c>
-      <c r="K449" s="28" t="n"/>
+      <c r="K449" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L449" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -10076,7 +10828,11 @@
       <c r="J451" s="33" t="n">
         <v>6.97</v>
       </c>
-      <c r="K451" s="28" t="n"/>
+      <c r="K451" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L451" s="32" t="inlineStr">
         <is>
           <t>Parcbrux Ixelles, Gand</t>
@@ -10096,7 +10852,11 @@
       <c r="J452" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="K452" s="28" t="n"/>
+      <c r="K452" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L452" s="32" t="inlineStr">
         <is>
           <t>Parking Station, Bruges</t>
@@ -10228,7 +10988,11 @@
       <c r="J458" s="33" t="n">
         <v>3.7</v>
       </c>
-      <c r="K458" s="28" t="n"/>
+      <c r="K458" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L458" s="32" t="inlineStr">
         <is>
           <t>Q-Park Woluwe Esplanade</t>
@@ -10248,7 +11012,11 @@
       <c r="J459" s="33" t="n">
         <v>1.6</v>
       </c>
-      <c r="K459" s="28" t="n"/>
+      <c r="K459" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L459" s="32" t="inlineStr">
         <is>
           <t>Woluwe-Saint-Lambert</t>
@@ -10268,7 +11036,11 @@
       <c r="J460" s="33" t="n">
         <v>14</v>
       </c>
-      <c r="K460" s="28" t="n"/>
+      <c r="K460" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L460" s="32" t="inlineStr">
         <is>
           <t>Parking Grand-Place, Bruxelles</t>
@@ -10288,7 +11060,11 @@
       <c r="J461" s="33" t="n">
         <v>2.6</v>
       </c>
-      <c r="K461" s="28" t="n"/>
+      <c r="K461" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L461" s="32" t="inlineStr">
         <is>
           <t>Parking Kinepolis, Louvain</t>
@@ -10332,7 +11108,11 @@
       <c r="J463" s="33" t="n">
         <v>3.4</v>
       </c>
-      <c r="K463" s="28" t="n"/>
+      <c r="K463" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L463" s="32" t="inlineStr">
         <is>
           <t>Indigo Park Docks, Bruxelles</t>

</xml_diff>

<commit_message>
Bilan 2025 : les quatre factures Farys sont cochees
Farys (eau) de fevrier, mai, septembre et octobre : 1.052,14 EUR au
total, factures en main et chargees dans Billtobox.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1874,8 +1874,16 @@
       <c r="J51" s="33" t="n">
         <v>290</v>
       </c>
-      <c r="K51" s="28" t="n"/>
-      <c r="L51" s="32" t="n"/>
+      <c r="K51" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L51" s="32" t="inlineStr">
+        <is>
+          <t>Facture Farys en main, chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="E52" s="16" t="n"/>
@@ -4216,8 +4224,16 @@
       <c r="J157" s="33" t="n">
         <v>290</v>
       </c>
-      <c r="K157" s="28" t="n"/>
-      <c r="L157" s="32" t="n"/>
+      <c r="K157" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L157" s="32" t="inlineStr">
+        <is>
+          <t>Facture Farys en main, chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="E158" s="16" t="n"/>
@@ -8750,8 +8766,16 @@
       <c r="J359" s="33" t="n">
         <v>300</v>
       </c>
-      <c r="K359" s="28" t="n"/>
-      <c r="L359" s="32" t="n"/>
+      <c r="K359" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L359" s="32" t="inlineStr">
+        <is>
+          <t>Facture Farys en main, chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="E360" s="16" t="n"/>
@@ -9336,8 +9360,16 @@
       <c r="J385" s="33" t="n">
         <v>172.14</v>
       </c>
-      <c r="K385" s="28" t="n"/>
-      <c r="L385" s="32" t="n"/>
+      <c r="K385" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L385" s="32" t="inlineStr">
+        <is>
+          <t>Facture Farys en main, chargée dans Billtobox</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="E386" s="16" t="n"/>

</xml_diff>

<commit_message>
Bilan 2025 : cinq factures Proximus recues par mail
Fevrier 49,98 / avril 141,50 / mai 71,54 / juin 64,94 / juillet 84,91,
soit 412,87 EUR. Les montants correspondent aux paiements. Reste la
facture de janvier (70,18 EUR, n° 7501364960).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -2066,10 +2066,14 @@
       <c r="J59" s="33" t="n">
         <v>49.98</v>
       </c>
-      <c r="K59" s="28" t="n"/>
+      <c r="K59" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L59" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/1903/98331</t>
+          <t>Facture 750/1903/98331 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -3024,10 +3028,14 @@
       <c r="J102" s="33" t="n">
         <v>141.5</v>
       </c>
-      <c r="K102" s="28" t="n"/>
+      <c r="K102" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L102" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/2441/84528</t>
+          <t>Facture 750/2441/84528 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -4248,10 +4256,14 @@
       <c r="J158" s="33" t="n">
         <v>71.54000000000001</v>
       </c>
-      <c r="K158" s="28" t="n"/>
+      <c r="K158" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L158" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/2981/21578</t>
+          <t>Facture 750/2981/21578 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -6464,10 +6476,14 @@
       <c r="J257" s="33" t="n">
         <v>64.94</v>
       </c>
-      <c r="K257" s="28" t="n"/>
+      <c r="K257" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L257" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/3518/42505</t>
+          <t>Facture 750/3518/42505 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -6818,10 +6834,14 @@
       <c r="J272" s="33" t="n">
         <v>84.91</v>
       </c>
-      <c r="K272" s="28" t="n"/>
+      <c r="K272" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L272" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/4054/27527</t>
+          <t>Facture 750/4054/27527 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : les cinq factures Proximus sont chargees dans Billtobox
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -2073,7 +2073,7 @@
       </c>
       <c r="L59" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/1903/98331 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
+          <t>Facture 750/1903/98331 — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -3035,7 +3035,7 @@
       </c>
       <c r="L102" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/2441/84528 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
+          <t>Facture 750/2441/84528 — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="L158" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/2981/21578 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
+          <t>Facture 750/2981/21578 — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -6483,7 +6483,7 @@
       </c>
       <c r="L257" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/3518/42505 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
+          <t>Facture 750/3518/42505 — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="L272" s="32" t="inlineStr">
         <is>
-          <t>Facture 750/4054/27527 — Facture Proximus reçue par mail, à charger dans Billtobox</t>
+          <t>Facture 750/4054/27527 — Facture Proximus en main, chargée dans Billtobox</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : les quatre factures de peage Ulys/ASF sont cochees
Contrat 0046686176 : janvier 27,90 (consommation 12/2024, facture emise
en 2025) / juillet 34,40 / aout 73,90 / septembre 101,20, soit 237,40 EUR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1226,10 +1226,14 @@
       <c r="J22" s="33" t="n">
         <v>27.9</v>
       </c>
-      <c r="K22" s="28" t="n"/>
+      <c r="K22" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L22" s="32" t="inlineStr">
         <is>
-          <t>Domiciliation Autoroutes du Sud de la France</t>
+          <t>Domiciliation Autoroutes du Sud de la France — Facture Ulys/ASF en main — consommation 12/2024, facture datée 2025</t>
         </is>
       </c>
     </row>
@@ -7650,10 +7654,14 @@
       <c r="J308" s="33" t="n">
         <v>34.4</v>
       </c>
-      <c r="K308" s="28" t="n"/>
+      <c r="K308" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L308" s="32" t="inlineStr">
         <is>
-          <t>Domiciliation Autoroutes du Sud de la France</t>
+          <t>Domiciliation Autoroutes du Sud de la France — Facture Ulys/ASF en main</t>
         </is>
       </c>
     </row>
@@ -8408,10 +8416,14 @@
       <c r="J342" s="33" t="n">
         <v>73.90000000000001</v>
       </c>
-      <c r="K342" s="28" t="n"/>
+      <c r="K342" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L342" s="32" t="inlineStr">
         <is>
-          <t>Domiciliation Autoroutes du Sud de la France</t>
+          <t>Domiciliation Autoroutes du Sud de la France — Facture Ulys/ASF en main</t>
         </is>
       </c>
     </row>
@@ -9046,10 +9058,14 @@
       <c r="J370" s="33" t="n">
         <v>101.2</v>
       </c>
-      <c r="K370" s="28" t="n"/>
+      <c r="K370" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L370" s="32" t="inlineStr">
         <is>
-          <t>Domiciliation Autoroutes du Sud de la France</t>
+          <t>Domiciliation Autoroutes du Sud de la France — Facture Ulys/ASF en main</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : les deux factures Translatina Travel sont cochees
1.100,00 et 42,00 de janvier. Les lignes restent en jaune : la piece est
la, mais la question prive/societe reste ouverte pour BDH.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -1270,10 +1270,14 @@
       <c r="J24" s="35" t="n">
         <v>1100</v>
       </c>
-      <c r="K24" s="28" t="n"/>
+      <c r="K24" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L24" s="36" t="inlineStr">
         <is>
-          <t>Avance - remboursé plus tard</t>
+          <t>Avance - remboursé plus tard — Facture Translatina Travel en main — rattachement privé/société à trancher</t>
         </is>
       </c>
     </row>
@@ -1314,10 +1318,14 @@
       <c r="J26" s="35" t="n">
         <v>42</v>
       </c>
-      <c r="K26" s="28" t="n"/>
+      <c r="K26" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L26" s="36" t="inlineStr">
         <is>
-          <t>Avance - remboursé plus tard</t>
+          <t>Avance - remboursé plus tard — Facture Translatina Travel en main — rattachement privé/société à trancher</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : pas de justificatif pour les avances privees remboursees
Le billet Air Europa (1.683,78) et le sejour Sandaya (1.775,40) ont ete
rembourses au centime par le gerant quelques jours apres : la depense et
l'entree s'annulent, la colonne Facture recoit un X.

Points ouverts : proposer a BDH de passer ces paires par le compte courant
plutot qu'en charge et produit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -4660,7 +4660,11 @@
       <c r="J177" s="33" t="n">
         <v>1683.78</v>
       </c>
-      <c r="K177" s="28" t="n"/>
+      <c r="K177" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L177" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 13-04 — décompte n° 121 du 12-05 — Remboursé par T. Duchène le 23-04 (entrée d'avril)</t>
@@ -8140,7 +8144,11 @@
       <c r="J330" s="33" t="n">
         <v>1775.4</v>
       </c>
-      <c r="K330" s="28" t="n"/>
+      <c r="K330" s="28" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L330" s="32" t="inlineStr">
         <is>
           <t>Carte Visa 11-07 — décompte n° 213 du 11-08 — Remboursé par T. Duchène le 22-07 (entrée de juillet)</t>

</xml_diff>

<commit_message>
Bilan 2025 : la formation Indigo Nails est justifiee
Facture FA002548 du 18-09-2025, au nom de MT Cosmetics Belgium avec son
numero de TVA, chargee dans Billtobox. 520,66 HT + 109,34 de TVA
recuperable.

L'adresse de facturation est Moorselsteenweg 65 a Sterrebeek : c'est donc
aussi l'adresse de la societe, ce qui nuance le point ENGIE.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -9122,10 +9122,14 @@
       <c r="J372" s="33" t="n">
         <v>630</v>
       </c>
-      <c r="K372" s="28" t="n"/>
+      <c r="K372" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L372" s="32" t="inlineStr">
         <is>
-          <t>Facture FA002548 avancée par T. Duchène et remboursée par la société</t>
+          <t>Facture FA002548 avancée par T. Duchène et remboursée par la société — Facture Indigo School FA002548 du 18-09-2025, au nom de MT Cosmetics Belgium (TVA BE0734616335), chargée dans Billtobox — formation onglerie 3 jours, 520,66 HT + 109,34 TVA récupérable</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : Xerius est la cotisation annuelle des societes
Ce n'est pas une cotisation sociale personnelle : la remarque etait fausse
et aurait induit BDH en erreur. Communication 925/3695/86745, payee le
16-12-2025. Le surplus de 52,23 sur la base de 347,50 reste a eclaircir,
la ligne passe en jaune.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -10860,18 +10860,18 @@
       <c r="F449" s="17" t="n"/>
       <c r="G449" s="31" t="n"/>
       <c r="H449" s="32" t="n"/>
-      <c r="I449" s="13" t="inlineStr">
+      <c r="I449" s="34" t="inlineStr">
         <is>
           <t>Xerius</t>
         </is>
       </c>
-      <c r="J449" s="33" t="n">
+      <c r="J449" s="35" t="n">
         <v>399.73</v>
       </c>
       <c r="K449" s="28" t="n"/>
-      <c r="L449" s="32" t="inlineStr">
-        <is>
-          <t>Cotisations sociales indépendant</t>
+      <c r="L449" s="36" t="inlineStr">
+        <is>
+          <t>Cotisation annuelle à charge des sociétés ('taxe société') — communication 925/3695/86745, payée le 16-12-2025. Base 347,50 : le surplus de 52,23 est à vérifier — indexation ou majoration de retard ?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : Media Markt, c'est un ordinateur
Les deux factures du 03-11 sont en main (748,00 a 12:33 et 39,00 a 12:35).
A ce montant le PC releve de l'immobilisation amortie plutot que de la
charge : les lignes restent en jaune et le point part chez BDH.

Le surlignage reconnait desormais aussi "a trancher" et "a amortir".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -10044,10 +10044,14 @@
       <c r="J413" s="35" t="n">
         <v>748</v>
       </c>
-      <c r="K413" s="28" t="n"/>
+      <c r="K413" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L413" s="36" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert — nature de l'achat à préciser</t>
+          <t>Ordinateur acheté le 03-11-2025 à 12:33 — investissement à amortir plutôt que charge de l'exercice, à trancher avec BDH — Facture Media Markt en main (achat du 03-11-2025)</t>
         </is>
       </c>
     </row>
@@ -10064,10 +10068,14 @@
       <c r="J414" s="35" t="n">
         <v>39</v>
       </c>
-      <c r="K414" s="28" t="n"/>
+      <c r="K414" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L414" s="36" t="inlineStr">
         <is>
-          <t>Woluwe-Saint-Lambert — nature de l'achat à préciser</t>
+          <t>Même passage en caisse, à 12:35 — accessoire ou garantie : à trancher avec le PC — intégré à sa valeur ou laissé en charge — Facture Media Markt en main (achat du 03-11-2025)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : les deux lignes Podomed sont couvertes par une seule facture
Facture 2025-30 du 26-12-2025, 275,00 au nom de MT Cosmetics Belgium :
bilan 65,00 paye en novembre et semelles 210,00 payees en decembre. TVA
0 %. Les lignes restent en jaune, la deductibilite d'un soin paramedical
au nom de la societe est a trancher par BDH.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -10560,18 +10560,22 @@
       <c r="F435" s="17" t="n"/>
       <c r="G435" s="31" t="n"/>
       <c r="H435" s="32" t="n"/>
-      <c r="I435" s="13" t="inlineStr">
+      <c r="I435" s="34" t="inlineStr">
         <is>
           <t>Semelles orthopédiques de travail - Podomed</t>
         </is>
       </c>
-      <c r="J435" s="33" t="n">
+      <c r="J435" s="35" t="n">
         <v>65</v>
       </c>
-      <c r="K435" s="28" t="n"/>
-      <c r="L435" s="32" t="inlineStr">
-        <is>
-          <t>Consultation</t>
+      <c r="K435" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L435" s="36" t="inlineStr">
+        <is>
+          <t>Bilan et prise de mesures du 27-11 — soin paramédical facturé à la société : déductibilité à trancher — Facture Podomed 2025-30 du 26-12-2025, au nom de MT Cosmetics Belgium — une seule facture pour les deux paiements (bilan 65,00 + semelles 210,00), TVA 0 %</t>
         </is>
       </c>
     </row>
@@ -11124,18 +11128,22 @@
       <c r="F460" s="17" t="n"/>
       <c r="G460" s="31" t="n"/>
       <c r="H460" s="32" t="n"/>
-      <c r="I460" s="13" t="inlineStr">
+      <c r="I460" s="34" t="inlineStr">
         <is>
           <t>Semelles orthopédiques de travail - Podomed</t>
         </is>
       </c>
-      <c r="J460" s="33" t="n">
+      <c r="J460" s="35" t="n">
         <v>210</v>
       </c>
-      <c r="K460" s="28" t="n"/>
-      <c r="L460" s="32" t="inlineStr">
-        <is>
-          <t>Solde après la consultation du 27-11</t>
+      <c r="K460" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L460" s="36" t="inlineStr">
+        <is>
+          <t>Semelles de travail sur mesure — soin paramédical facturé à la société : déductibilité à trancher — Facture Podomed 2025-30 du 26-12-2025, au nom de MT Cosmetics Belgium — une seule facture pour les deux paiements (bilan 65,00 + semelles 210,00), TVA 0 %</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : les semelles Podomed sont de l'equipement de travail
Thibault Duchene est entraineur de tennis : debout et en deplacement sur
le terrain toute la journee. L'intitule de la facture dit lui-meme
"semelles de travail sur mesure". Les lignes sortent du jaune et passent
en charge deductible ; BDH est informe sans question ouverte.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -10560,12 +10560,12 @@
       <c r="F435" s="17" t="n"/>
       <c r="G435" s="31" t="n"/>
       <c r="H435" s="32" t="n"/>
-      <c r="I435" s="34" t="inlineStr">
+      <c r="I435" s="13" t="inlineStr">
         <is>
           <t>Semelles orthopédiques de travail - Podomed</t>
         </is>
       </c>
-      <c r="J435" s="35" t="n">
+      <c r="J435" s="33" t="n">
         <v>65</v>
       </c>
       <c r="K435" s="28" t="inlineStr">
@@ -10573,9 +10573,9 @@
           <t>V</t>
         </is>
       </c>
-      <c r="L435" s="36" t="inlineStr">
-        <is>
-          <t>Bilan et prise de mesures du 27-11 — soin paramédical facturé à la société : déductibilité à trancher — Facture Podomed 2025-30 du 26-12-2025, au nom de MT Cosmetics Belgium — une seule facture pour les deux paiements (bilan 65,00 + semelles 210,00), TVA 0 %</t>
+      <c r="L435" s="32" t="inlineStr">
+        <is>
+          <t>Bilan et prise de mesures du 27-11 — facture Podomed 2025-30, équipement de travail : Thibault Duchène est entraîneur de tennis, debout et en déplacement toute la journée — Facture Podomed 2025-30 du 26-12-2025, au nom de MT Cosmetics Belgium — une seule facture pour les deux paiements (bilan 65,00 + semelles 210,00), TVA 0 %</t>
         </is>
       </c>
     </row>
@@ -11128,12 +11128,12 @@
       <c r="F460" s="17" t="n"/>
       <c r="G460" s="31" t="n"/>
       <c r="H460" s="32" t="n"/>
-      <c r="I460" s="34" t="inlineStr">
+      <c r="I460" s="13" t="inlineStr">
         <is>
           <t>Semelles orthopédiques de travail - Podomed</t>
         </is>
       </c>
-      <c r="J460" s="35" t="n">
+      <c r="J460" s="33" t="n">
         <v>210</v>
       </c>
       <c r="K460" s="28" t="inlineStr">
@@ -11141,9 +11141,9 @@
           <t>V</t>
         </is>
       </c>
-      <c r="L460" s="36" t="inlineStr">
-        <is>
-          <t>Semelles de travail sur mesure — soin paramédical facturé à la société : déductibilité à trancher — Facture Podomed 2025-30 du 26-12-2025, au nom de MT Cosmetics Belgium — une seule facture pour les deux paiements (bilan 65,00 + semelles 210,00), TVA 0 %</t>
+      <c r="L460" s="32" t="inlineStr">
+        <is>
+          <t>Semelles de travail sur mesure — même facture Podomed 2025-30, liées à l'exercice du métier d'entraîneur de tennis — Facture Podomed 2025-30 du 26-12-2025, au nom de MT Cosmetics Belgium — une seule facture pour les deux paiements (bilan 65,00 + semelles 210,00), TVA 0 %</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : la facture Bellissimo Sport de mars est cochee
Achat du 04-03-2025 chez New BS, 290,50.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -2100,10 +2100,14 @@
       <c r="J61" s="39" t="n">
         <v>290.5</v>
       </c>
-      <c r="K61" s="28" t="n"/>
+      <c r="K61" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
       <c r="L61" s="32" t="inlineStr">
         <is>
-          <t>New Bs SRL, Bruxelles</t>
+          <t>New Bs SRL, Bruxelles — Facture New BS (Bellissimo Sport) du 04-03-2025 en main</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : les deux tickets Topogigio manquants sont rattaches
Ils avaient ete ecartes parce que les totaux imprimes ne collaient pas
avec la banque : 29,00 pour 26,00 debites le 23-04 et 251,50 pour 231,50
le 25-07. Meme ecart qu'en mars, ou le ticket portait une correction a la
main. Les lignes sont cochees, l'ecart est decrit dans les remarques.

Le PDF du 23 avril etait ampute : le masque se laissait piéger par le
reflet sur le bois. Regenere avec la voie fond clair, ticket entier et
lisible.

Topogigio est le bar du RTC Lambermont, pas un restaurant : 85 pieces le
25-07 pour un groupe. La qualification revient a BDH.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -4068,8 +4068,16 @@
       <c r="J148" s="33" t="n">
         <v>26</v>
       </c>
-      <c r="K148" s="28" t="n"/>
-      <c r="L148" s="32" t="n"/>
+      <c r="K148" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L148" s="32" t="inlineStr">
+        <is>
+          <t>Bar du RTCL Lambermont, 23-04 à 16:09 — 12 pièces (sodas et gaufres), ticket de 29,00 pour 26,00 débités — Justificatif : 2025-04-23_RTCL-Lambermont_29.00.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="E149" s="16" t="n"/>
@@ -7786,8 +7794,16 @@
       <c r="J313" s="33" t="n">
         <v>231.5</v>
       </c>
-      <c r="K313" s="28" t="n"/>
-      <c r="L313" s="32" t="n"/>
+      <c r="K313" s="28" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="L313" s="32" t="inlineStr">
+        <is>
+          <t>Bar du RTCL Lambermont, 25-07 à 15:05 — 85 pièces pour un groupe (sodas, gaufres, chips, croque-monsieur), ticket de 251,50 pour 231,50 débités via SumUp — Justificatif : 2025-07-25_RTCL-Lambermont_251.50.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="E314" s="16" t="n"/>

</xml_diff>

<commit_message>
Bilan 2025 : les tickets du bar du club sont des ardoises cumulees
Le gerant du bar notait les consommations sur papier puis les encodait
toutes d'un coup. Un ticket de 85 pieces n'est donc pas une consommation
unique, et cela explique aussi les ecarts avec les montants debites.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -4075,7 +4075,7 @@
       </c>
       <c r="L148" s="32" t="inlineStr">
         <is>
-          <t>Bar du RTCL Lambermont, 23-04 à 16:09 — 12 pièces (sodas et gaufres), ticket de 29,00 pour 26,00 débités — Justificatif : 2025-04-23_RTCL-Lambermont_29.00.pdf</t>
+          <t>Bar du RTCL Lambermont — ardoise encodée en une fois le 23-04 à 16:09 : 12 pièces (sodas et gaufres). Ticket de 29,00 pour 26,00 débités — Justificatif : 2025-04-23_RTCL-Lambermont_29.00.pdf</t>
         </is>
       </c>
     </row>
@@ -7801,7 +7801,7 @@
       </c>
       <c r="L313" s="32" t="inlineStr">
         <is>
-          <t>Bar du RTCL Lambermont, 25-07 à 15:05 — 85 pièces pour un groupe (sodas, gaufres, chips, croque-monsieur), ticket de 251,50 pour 231,50 débités via SumUp — Justificatif : 2025-07-25_RTCL-Lambermont_251.50.pdf</t>
+          <t>Bar du RTCL Lambermont — ardoise tenue sur papier par le gérant du bar puis encodée en une fois le 25-07 à 15:05 : 85 pièces (sodas, gaufres, chips, croque-monsieur). Ticket de 251,50 pour 231,50 débités via SumUp — Justificatif : 2025-07-25_RTCL-Lambermont_251.50.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bilan 2025 : trente petites depenses sans ticket
La carte de societe a ete pretee et les tickets n'ont pas ete conserves.
Ces lignes recoivent un X, mais surligne et assorti de "Ticket non
conserve" : sans quoi il se confondrait avec les postes que le comptable
dispense de justificatif et laisserait croire la question reglee.

build.py gere desormais une liste SANS_TICKET distincte de JUSTIFICATIFS.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -318,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -354,12 +354,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -864,16 +865,24 @@
         <v>5328.2</v>
       </c>
       <c r="H6" s="32" t="n"/>
-      <c r="I6" s="13" t="inlineStr">
+      <c r="I6" s="33" t="inlineStr">
         <is>
           <t>Collation - Plouf et Baballe</t>
         </is>
       </c>
-      <c r="J6" s="33" t="n">
+      <c r="J6" s="34" t="n">
         <v>8.4</v>
       </c>
-      <c r="K6" s="28" t="n"/>
-      <c r="L6" s="32" t="n"/>
+      <c r="K6" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L6" s="36" t="inlineStr">
+        <is>
+          <t>Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="E7" s="16" t="n"/>
@@ -891,7 +900,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J7" s="33" t="n">
+      <c r="J7" s="37" t="n">
         <v>22.9</v>
       </c>
       <c r="K7" s="28" t="inlineStr">
@@ -915,7 +924,7 @@
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J8" s="33" t="n">
+      <c r="J8" s="37" t="n">
         <v>5.69</v>
       </c>
       <c r="K8" s="28" t="n"/>
@@ -931,7 +940,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J9" s="33" t="n">
+      <c r="J9" s="37" t="n">
         <v>1.35</v>
       </c>
       <c r="K9" s="28" t="inlineStr">
@@ -951,7 +960,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J10" s="33" t="n">
+      <c r="J10" s="37" t="n">
         <v>62.79</v>
       </c>
       <c r="K10" s="28" t="inlineStr">
@@ -975,7 +984,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J11" s="33" t="n">
+      <c r="J11" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K11" s="28" t="inlineStr">
@@ -995,7 +1004,7 @@
           <t>Frais bancaires trimestriels</t>
         </is>
       </c>
-      <c r="J12" s="33" t="n">
+      <c r="J12" s="37" t="n">
         <v>11.25</v>
       </c>
       <c r="K12" s="28" t="n"/>
@@ -1011,7 +1020,7 @@
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J13" s="33" t="n">
+      <c r="J13" s="37" t="n">
         <v>431.25</v>
       </c>
       <c r="K13" s="28" t="n"/>
@@ -1031,7 +1040,7 @@
           <t>Repas Topogigio</t>
         </is>
       </c>
-      <c r="J14" s="33" t="n">
+      <c r="J14" s="37" t="n">
         <v>22</v>
       </c>
       <c r="K14" s="28" t="inlineStr">
@@ -1055,7 +1064,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J15" s="33" t="n">
+      <c r="J15" s="37" t="n">
         <v>66.72</v>
       </c>
       <c r="K15" s="28" t="inlineStr">
@@ -1079,7 +1088,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J16" s="33" t="n">
+      <c r="J16" s="37" t="n">
         <v>22.5</v>
       </c>
       <c r="K16" s="28" t="inlineStr">
@@ -1103,7 +1112,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J17" s="33" t="n">
+      <c r="J17" s="37" t="n">
         <v>1.8</v>
       </c>
       <c r="K17" s="28" t="inlineStr">
@@ -1127,7 +1136,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J18" s="33" t="n">
+      <c r="J18" s="37" t="n">
         <v>256.99</v>
       </c>
       <c r="K18" s="28" t="inlineStr">
@@ -1151,7 +1160,7 @@
           <t>Telenet</t>
         </is>
       </c>
-      <c r="J19" s="33" t="n">
+      <c r="J19" s="37" t="n">
         <v>159.1</v>
       </c>
       <c r="K19" s="28" t="inlineStr">
@@ -1175,7 +1184,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J20" s="33" t="n">
+      <c r="J20" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K20" s="28" t="inlineStr">
@@ -1199,7 +1208,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J21" s="33" t="n">
+      <c r="J21" s="37" t="n">
         <v>71.13</v>
       </c>
       <c r="K21" s="28" t="inlineStr">
@@ -1223,7 +1232,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J22" s="33" t="n">
+      <c r="J22" s="37" t="n">
         <v>7.2</v>
       </c>
       <c r="K22" s="28" t="inlineStr">
@@ -1247,7 +1256,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J23" s="33" t="n">
+      <c r="J23" s="37" t="n">
         <v>2.68</v>
       </c>
       <c r="K23" s="28" t="inlineStr">
@@ -1262,12 +1271,12 @@
       <c r="F24" s="17" t="n"/>
       <c r="G24" s="31" t="n"/>
       <c r="H24" s="32" t="n"/>
-      <c r="I24" s="34" t="inlineStr">
+      <c r="I24" s="33" t="inlineStr">
         <is>
           <t>Billets d'avion Pérou - Translatina Travel</t>
         </is>
       </c>
-      <c r="J24" s="35" t="n">
+      <c r="J24" s="34" t="n">
         <v>1100</v>
       </c>
       <c r="K24" s="28" t="inlineStr">
@@ -1291,7 +1300,7 @@
           <t>Précompte salarial janvier 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J25" s="33" t="n">
+      <c r="J25" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K25" s="28" t="inlineStr">
@@ -1310,12 +1319,12 @@
       <c r="F26" s="17" t="n"/>
       <c r="G26" s="31" t="n"/>
       <c r="H26" s="32" t="n"/>
-      <c r="I26" s="34" t="inlineStr">
+      <c r="I26" s="33" t="inlineStr">
         <is>
           <t>Billets d'avion Pérou - Translatina Travel</t>
         </is>
       </c>
-      <c r="J26" s="35" t="n">
+      <c r="J26" s="34" t="n">
         <v>42</v>
       </c>
       <c r="K26" s="28" t="inlineStr">
@@ -1339,7 +1348,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J27" s="33" t="n">
+      <c r="J27" s="37" t="n">
         <v>69.44</v>
       </c>
       <c r="K27" s="28" t="inlineStr">
@@ -1363,7 +1372,7 @@
           <t>Impôt des sociétés</t>
         </is>
       </c>
-      <c r="J28" s="33" t="n">
+      <c r="J28" s="37" t="n">
         <v>4517.28</v>
       </c>
       <c r="K28" s="28" t="inlineStr">
@@ -1387,7 +1396,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J29" s="33" t="n">
+      <c r="J29" s="37" t="n">
         <v>331.52</v>
       </c>
       <c r="K29" s="28" t="inlineStr">
@@ -1411,7 +1420,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J30" s="33" t="n">
+      <c r="J30" s="37" t="n">
         <v>70.18000000000001</v>
       </c>
       <c r="K30" s="28" t="n"/>
@@ -1422,16 +1431,16 @@
       </c>
     </row>
     <row r="31">
-      <c r="G31" s="37" t="n"/>
-      <c r="H31" s="38" t="n"/>
-      <c r="J31" s="37" t="n"/>
-      <c r="L31" s="38" t="n"/>
+      <c r="G31" s="38" t="n"/>
+      <c r="H31" s="39" t="n"/>
+      <c r="J31" s="38" t="n"/>
+      <c r="L31" s="39" t="n"/>
     </row>
     <row r="32">
-      <c r="G32" s="37" t="n"/>
-      <c r="H32" s="38" t="n"/>
-      <c r="J32" s="37" t="n"/>
-      <c r="L32" s="38" t="n"/>
+      <c r="G32" s="38" t="n"/>
+      <c r="H32" s="39" t="n"/>
+      <c r="J32" s="38" t="n"/>
+      <c r="L32" s="39" t="n"/>
     </row>
     <row r="33">
       <c r="E33" s="16" t="inlineStr">
@@ -1453,7 +1462,7 @@
           <t>Achat vêtements sport - Tommy Hilfiger Maasmechelen</t>
         </is>
       </c>
-      <c r="J33" s="39" t="n">
+      <c r="J33" s="40" t="n">
         <v>210.49</v>
       </c>
       <c r="K33" s="28" t="inlineStr">
@@ -1487,7 +1496,7 @@
           <t>Achat vêtements sport - NIKE Maasmechelen</t>
         </is>
       </c>
-      <c r="J34" s="33" t="n">
+      <c r="J34" s="37" t="n">
         <v>141.47</v>
       </c>
       <c r="K34" s="28" t="inlineStr">
@@ -1511,7 +1520,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J35" s="33" t="n">
+      <c r="J35" s="37" t="n">
         <v>2.1</v>
       </c>
       <c r="K35" s="28" t="inlineStr">
@@ -1535,7 +1544,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J36" s="33" t="n">
+      <c r="J36" s="37" t="n">
         <v>256.99</v>
       </c>
       <c r="K36" s="28" t="inlineStr">
@@ -1559,7 +1568,7 @@
           <t>Telenet</t>
         </is>
       </c>
-      <c r="J37" s="33" t="n">
+      <c r="J37" s="37" t="n">
         <v>149.1</v>
       </c>
       <c r="K37" s="28" t="inlineStr">
@@ -1583,7 +1592,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J38" s="33" t="n">
+      <c r="J38" s="37" t="n">
         <v>65</v>
       </c>
       <c r="K38" s="28" t="inlineStr">
@@ -1607,7 +1616,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J39" s="33" t="n">
+      <c r="J39" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K39" s="28" t="inlineStr">
@@ -1627,7 +1636,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J40" s="33" t="n">
+      <c r="J40" s="37" t="n">
         <v>1.8</v>
       </c>
       <c r="K40" s="28" t="inlineStr">
@@ -1651,7 +1660,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J41" s="33" t="n">
+      <c r="J41" s="37" t="n">
         <v>6.2</v>
       </c>
       <c r="K41" s="28" t="inlineStr">
@@ -1675,7 +1684,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J42" s="33" t="n">
+      <c r="J42" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K42" s="28" t="inlineStr">
@@ -1699,7 +1708,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J43" s="33" t="n">
+      <c r="J43" s="37" t="n">
         <v>17.1</v>
       </c>
       <c r="K43" s="28" t="inlineStr">
@@ -1723,7 +1732,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J44" s="33" t="n">
+      <c r="J44" s="37" t="n">
         <v>69.47</v>
       </c>
       <c r="K44" s="28" t="inlineStr">
@@ -1747,7 +1756,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J45" s="33" t="n">
+      <c r="J45" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K45" s="28" t="inlineStr">
@@ -1767,7 +1776,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J46" s="33" t="n">
+      <c r="J46" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K46" s="28" t="inlineStr">
@@ -1787,7 +1796,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J47" s="33" t="n">
+      <c r="J47" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K47" s="28" t="inlineStr">
@@ -1811,7 +1820,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J48" s="33" t="n">
+      <c r="J48" s="37" t="n">
         <v>1.8</v>
       </c>
       <c r="K48" s="28" t="inlineStr">
@@ -1835,7 +1844,7 @@
           <t>Partena</t>
         </is>
       </c>
-      <c r="J49" s="33" t="n">
+      <c r="J49" s="37" t="n">
         <v>1441.87</v>
       </c>
       <c r="K49" s="28" t="inlineStr">
@@ -1859,7 +1868,7 @@
           <t>Farys (eau)</t>
         </is>
       </c>
-      <c r="J50" s="33" t="n">
+      <c r="J50" s="37" t="n">
         <v>290</v>
       </c>
       <c r="K50" s="28" t="inlineStr">
@@ -1883,7 +1892,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J51" s="33" t="n">
+      <c r="J51" s="37" t="n">
         <v>6.5</v>
       </c>
       <c r="K51" s="28" t="inlineStr">
@@ -1907,7 +1916,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J52" s="33" t="n">
+      <c r="J52" s="37" t="n">
         <v>68.61</v>
       </c>
       <c r="K52" s="28" t="inlineStr">
@@ -1931,7 +1940,7 @@
           <t>Repas Lunch Garden</t>
         </is>
       </c>
-      <c r="J53" s="33" t="n">
+      <c r="J53" s="37" t="n">
         <v>39.47</v>
       </c>
       <c r="K53" s="28" t="inlineStr">
@@ -1955,7 +1964,7 @@
           <t>Achat vêtement sport - DECATHLON</t>
         </is>
       </c>
-      <c r="J54" s="33" t="n">
+      <c r="J54" s="37" t="n">
         <v>140</v>
       </c>
       <c r="K54" s="28" t="inlineStr">
@@ -1979,7 +1988,7 @@
           <t>Précompte salarial février 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J55" s="33" t="n">
+      <c r="J55" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K55" s="28" t="inlineStr">
@@ -2003,7 +2012,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J56" s="33" t="n">
+      <c r="J56" s="37" t="n">
         <v>331.52</v>
       </c>
       <c r="K56" s="28" t="inlineStr">
@@ -2027,7 +2036,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J57" s="33" t="n">
+      <c r="J57" s="37" t="n">
         <v>66.06999999999999</v>
       </c>
       <c r="K57" s="28" t="inlineStr">
@@ -2051,7 +2060,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J58" s="33" t="n">
+      <c r="J58" s="37" t="n">
         <v>49.98</v>
       </c>
       <c r="K58" s="28" t="inlineStr">
@@ -2066,16 +2075,16 @@
       </c>
     </row>
     <row r="59">
-      <c r="G59" s="37" t="n"/>
-      <c r="H59" s="38" t="n"/>
-      <c r="J59" s="37" t="n"/>
-      <c r="L59" s="38" t="n"/>
+      <c r="G59" s="38" t="n"/>
+      <c r="H59" s="39" t="n"/>
+      <c r="J59" s="38" t="n"/>
+      <c r="L59" s="39" t="n"/>
     </row>
     <row r="60">
-      <c r="G60" s="37" t="n"/>
-      <c r="H60" s="38" t="n"/>
-      <c r="J60" s="37" t="n"/>
-      <c r="L60" s="38" t="n"/>
+      <c r="G60" s="38" t="n"/>
+      <c r="H60" s="39" t="n"/>
+      <c r="J60" s="38" t="n"/>
+      <c r="L60" s="39" t="n"/>
     </row>
     <row r="61">
       <c r="E61" s="16" t="inlineStr">
@@ -2097,7 +2106,7 @@
           <t>Achat vêtements de tennis - Bellissimo Sport</t>
         </is>
       </c>
-      <c r="J61" s="39" t="n">
+      <c r="J61" s="40" t="n">
         <v>290.5</v>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2127,7 +2136,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J62" s="33" t="n">
+      <c r="J62" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K62" s="28" t="inlineStr">
@@ -2147,7 +2156,7 @@
           <t>Repas Topogigio</t>
         </is>
       </c>
-      <c r="J63" s="33" t="n">
+      <c r="J63" s="37" t="n">
         <v>75.5</v>
       </c>
       <c r="K63" s="28" t="inlineStr">
@@ -2171,7 +2180,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J64" s="33" t="n">
+      <c r="J64" s="37" t="n">
         <v>6.3</v>
       </c>
       <c r="K64" s="28" t="inlineStr">
@@ -2195,7 +2204,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J65" s="33" t="n">
+      <c r="J65" s="37" t="n">
         <v>67.55</v>
       </c>
       <c r="K65" s="28" t="inlineStr">
@@ -2219,7 +2228,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J66" s="33" t="n">
+      <c r="J66" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K66" s="28" t="inlineStr">
@@ -2243,7 +2252,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J67" s="33" t="n">
+      <c r="J67" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K67" s="28" t="inlineStr">
@@ -2267,7 +2276,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J68" s="33" t="n">
+      <c r="J68" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K68" s="28" t="inlineStr">
@@ -2291,7 +2300,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J69" s="33" t="n">
+      <c r="J69" s="37" t="n">
         <v>256.99</v>
       </c>
       <c r="K69" s="28" t="inlineStr">
@@ -2315,7 +2324,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J70" s="33" t="n">
+      <c r="J70" s="37" t="n">
         <v>256.99</v>
       </c>
       <c r="K70" s="28" t="inlineStr">
@@ -2339,7 +2348,7 @@
           <t>Telenet</t>
         </is>
       </c>
-      <c r="J71" s="33" t="n">
+      <c r="J71" s="37" t="n">
         <v>149.4</v>
       </c>
       <c r="K71" s="28" t="inlineStr">
@@ -2363,7 +2372,7 @@
           <t>Amende de stationnement - Ville de Louvain</t>
         </is>
       </c>
-      <c r="J72" s="33" t="n">
+      <c r="J72" s="37" t="n">
         <v>58</v>
       </c>
       <c r="K72" s="28" t="n"/>
@@ -2383,7 +2392,7 @@
           <t>Amende de stationnement - Woluwe-Saint-Lambert</t>
         </is>
       </c>
-      <c r="J73" s="33" t="n">
+      <c r="J73" s="37" t="n">
         <v>45</v>
       </c>
       <c r="K73" s="28" t="n"/>
@@ -2403,7 +2412,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J74" s="33" t="n">
+      <c r="J74" s="37" t="n">
         <v>1.85</v>
       </c>
       <c r="K74" s="28" t="inlineStr">
@@ -2427,7 +2436,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J75" s="33" t="n">
+      <c r="J75" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K75" s="28" t="inlineStr">
@@ -2451,7 +2460,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J76" s="33" t="n">
+      <c r="J76" s="37" t="n">
         <v>60.74</v>
       </c>
       <c r="K76" s="28" t="inlineStr">
@@ -2475,7 +2484,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J77" s="33" t="n">
+      <c r="J77" s="37" t="n">
         <v>2.67</v>
       </c>
       <c r="K77" s="28" t="inlineStr">
@@ -2499,7 +2508,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J78" s="33" t="n">
+      <c r="J78" s="37" t="n">
         <v>50.2</v>
       </c>
       <c r="K78" s="28" t="inlineStr">
@@ -2523,7 +2532,7 @@
           <t>Partena</t>
         </is>
       </c>
-      <c r="J79" s="33" t="n">
+      <c r="J79" s="37" t="n">
         <v>3014</v>
       </c>
       <c r="K79" s="28" t="inlineStr">
@@ -2547,7 +2556,7 @@
           <t>Entretien voiture - Monsieur Pneus</t>
         </is>
       </c>
-      <c r="J80" s="33" t="n">
+      <c r="J80" s="37" t="n">
         <v>919.17</v>
       </c>
       <c r="K80" s="28" t="inlineStr">
@@ -2571,7 +2580,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J81" s="33" t="n">
+      <c r="J81" s="37" t="n">
         <v>70.68000000000001</v>
       </c>
       <c r="K81" s="28" t="inlineStr">
@@ -2595,7 +2604,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J82" s="33" t="n">
+      <c r="J82" s="37" t="n">
         <v>16</v>
       </c>
       <c r="K82" s="28" t="inlineStr">
@@ -2619,7 +2628,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J83" s="33" t="n">
+      <c r="J83" s="37" t="n">
         <v>16.2</v>
       </c>
       <c r="K83" s="28" t="inlineStr">
@@ -2643,7 +2652,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J84" s="33" t="n">
+      <c r="J84" s="37" t="n">
         <v>3.2</v>
       </c>
       <c r="K84" s="28" t="inlineStr">
@@ -2667,7 +2676,7 @@
           <t>Précompte salarial mars 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J85" s="33" t="n">
+      <c r="J85" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K85" s="28" t="inlineStr">
@@ -2691,7 +2700,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J86" s="33" t="n">
+      <c r="J86" s="37" t="n">
         <v>331.52</v>
       </c>
       <c r="K86" s="28" t="inlineStr">
@@ -2715,7 +2724,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J87" s="33" t="n">
+      <c r="J87" s="37" t="n">
         <v>70.48999999999999</v>
       </c>
       <c r="K87" s="28" t="inlineStr">
@@ -2730,16 +2739,16 @@
       </c>
     </row>
     <row r="88">
-      <c r="G88" s="37" t="n"/>
-      <c r="H88" s="38" t="n"/>
-      <c r="J88" s="37" t="n"/>
-      <c r="L88" s="38" t="n"/>
+      <c r="G88" s="38" t="n"/>
+      <c r="H88" s="39" t="n"/>
+      <c r="J88" s="38" t="n"/>
+      <c r="L88" s="39" t="n"/>
     </row>
     <row r="89">
-      <c r="G89" s="37" t="n"/>
-      <c r="H89" s="38" t="n"/>
-      <c r="J89" s="37" t="n"/>
-      <c r="L89" s="38" t="n"/>
+      <c r="G89" s="38" t="n"/>
+      <c r="H89" s="39" t="n"/>
+      <c r="J89" s="38" t="n"/>
+      <c r="L89" s="39" t="n"/>
     </row>
     <row r="90">
       <c r="E90" s="16" t="inlineStr">
@@ -2747,12 +2756,12 @@
           <t>Avril</t>
         </is>
       </c>
-      <c r="F90" s="40" t="inlineStr">
+      <c r="F90" s="41" t="inlineStr">
         <is>
           <t>Remboursement billet d'avion Lima-Bruxelles</t>
         </is>
       </c>
-      <c r="G90" s="41" t="n">
+      <c r="G90" s="42" t="n">
         <v>1683.78</v>
       </c>
       <c r="H90" s="36" t="inlineStr">
@@ -2765,7 +2774,7 @@
           <t>Repas Exki</t>
         </is>
       </c>
-      <c r="J90" s="39" t="n">
+      <c r="J90" s="40" t="n">
         <v>30.3</v>
       </c>
       <c r="K90" s="28" t="inlineStr">
@@ -2789,7 +2798,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J91" s="33" t="n">
+      <c r="J91" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K91" s="28" t="inlineStr">
@@ -2813,7 +2822,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J92" s="33" t="n">
+      <c r="J92" s="37" t="n">
         <v>18.4</v>
       </c>
       <c r="K92" s="28" t="inlineStr">
@@ -2837,7 +2846,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J93" s="33" t="n">
+      <c r="J93" s="37" t="n">
         <v>10.4</v>
       </c>
       <c r="K93" s="28" t="inlineStr">
@@ -2861,7 +2870,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J94" s="33" t="n">
+      <c r="J94" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K94" s="28" t="inlineStr">
@@ -2881,7 +2890,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J95" s="33" t="n">
+      <c r="J95" s="37" t="n">
         <v>23</v>
       </c>
       <c r="K95" s="28" t="inlineStr">
@@ -2905,7 +2914,7 @@
           <t>Frais bancaires trimestriels</t>
         </is>
       </c>
-      <c r="J96" s="33" t="n">
+      <c r="J96" s="37" t="n">
         <v>11.25</v>
       </c>
       <c r="K96" s="28" t="n"/>
@@ -2921,7 +2930,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J97" s="33" t="n">
+      <c r="J97" s="37" t="n">
         <v>87</v>
       </c>
       <c r="K97" s="28" t="inlineStr">
@@ -2945,7 +2954,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J98" s="33" t="n">
+      <c r="J98" s="37" t="n">
         <v>10.46</v>
       </c>
       <c r="K98" s="28" t="inlineStr">
@@ -2969,7 +2978,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J99" s="33" t="n">
+      <c r="J99" s="37" t="n">
         <v>9</v>
       </c>
       <c r="K99" s="28" t="inlineStr">
@@ -2993,7 +3002,7 @@
           <t>Achat vêtements - N.Z.A. Utrecht</t>
         </is>
       </c>
-      <c r="J100" s="33" t="n">
+      <c r="J100" s="37" t="n">
         <v>289.97</v>
       </c>
       <c r="K100" s="28" t="inlineStr">
@@ -3017,7 +3026,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J101" s="33" t="n">
+      <c r="J101" s="37" t="n">
         <v>141.5</v>
       </c>
       <c r="K101" s="28" t="inlineStr">
@@ -3041,7 +3050,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J102" s="33" t="n">
+      <c r="J102" s="37" t="n">
         <v>32.76</v>
       </c>
       <c r="K102" s="28" t="inlineStr">
@@ -3065,7 +3074,7 @@
           <t>Telenet</t>
         </is>
       </c>
-      <c r="J103" s="33" t="n">
+      <c r="J103" s="37" t="n">
         <v>149.1</v>
       </c>
       <c r="K103" s="28" t="inlineStr">
@@ -3089,7 +3098,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J104" s="33" t="n">
+      <c r="J104" s="37" t="n">
         <v>8</v>
       </c>
       <c r="K104" s="28" t="inlineStr">
@@ -3108,18 +3117,22 @@
       <c r="F105" s="17" t="n"/>
       <c r="G105" s="31" t="n"/>
       <c r="H105" s="32" t="n"/>
-      <c r="I105" s="34" t="inlineStr">
+      <c r="I105" s="33" t="inlineStr">
         <is>
           <t>Divers - Blitha Vereycken, Anvers</t>
         </is>
       </c>
-      <c r="J105" s="35" t="n">
+      <c r="J105" s="34" t="n">
         <v>2.5</v>
       </c>
-      <c r="K105" s="28" t="n"/>
+      <c r="K105" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L105" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 01-03 — décompte n° 091 du 10-04 — à identifier</t>
+          <t>Carte Visa 01-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3146,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J106" s="33" t="n">
+      <c r="J106" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K106" s="28" t="inlineStr">
@@ -3157,7 +3170,7 @@
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J107" s="33" t="n">
+      <c r="J107" s="37" t="n">
         <v>48.67</v>
       </c>
       <c r="K107" s="28" t="n"/>
@@ -3177,7 +3190,7 @@
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J108" s="33" t="n">
+      <c r="J108" s="37" t="n">
         <v>97.34</v>
       </c>
       <c r="K108" s="28" t="n"/>
@@ -3192,18 +3205,22 @@
       <c r="F109" s="17" t="n"/>
       <c r="G109" s="31" t="n"/>
       <c r="H109" s="32" t="n"/>
-      <c r="I109" s="13" t="inlineStr">
+      <c r="I109" s="33" t="inlineStr">
         <is>
           <t>Repas - Paul, métro Montgomery</t>
         </is>
       </c>
-      <c r="J109" s="33" t="n">
+      <c r="J109" s="34" t="n">
         <v>4.9</v>
       </c>
-      <c r="K109" s="28" t="n"/>
-      <c r="L109" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 10-03 — décompte n° 091 du 10-04</t>
+      <c r="K109" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L109" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 10-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3212,18 +3229,22 @@
       <c r="F110" s="17" t="n"/>
       <c r="G110" s="31" t="n"/>
       <c r="H110" s="32" t="n"/>
-      <c r="I110" s="13" t="inlineStr">
+      <c r="I110" s="33" t="inlineStr">
         <is>
           <t>Collation - Shop Metro Montgomery</t>
         </is>
       </c>
-      <c r="J110" s="33" t="n">
+      <c r="J110" s="34" t="n">
         <v>6.48</v>
       </c>
-      <c r="K110" s="28" t="n"/>
-      <c r="L110" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 10-03 — décompte n° 091 du 10-04</t>
+      <c r="K110" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L110" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 10-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3258,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J111" s="33" t="n">
+      <c r="J111" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K111" s="28" t="inlineStr">
@@ -3261,7 +3282,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J112" s="33" t="n">
+      <c r="J112" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K112" s="28" t="inlineStr">
@@ -3285,7 +3306,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J113" s="33" t="n">
+      <c r="J113" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K113" s="28" t="inlineStr">
@@ -3304,18 +3325,22 @@
       <c r="F114" s="17" t="n"/>
       <c r="G114" s="31" t="n"/>
       <c r="H114" s="32" t="n"/>
-      <c r="I114" s="34" t="inlineStr">
+      <c r="I114" s="33" t="inlineStr">
         <is>
           <t>Achat - Flying Tiger Bruxelles</t>
         </is>
       </c>
-      <c r="J114" s="35" t="n">
+      <c r="J114" s="34" t="n">
         <v>81</v>
       </c>
-      <c r="K114" s="28" t="n"/>
+      <c r="K114" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L114" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 12-03 — décompte n° 091 du 10-04 — nature de l'achat à préciser</t>
+          <t>Carte Visa 12-03 — décompte n° 091 du 10-04 — nature de l'achat à préciser — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3354,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J115" s="33" t="n">
+      <c r="J115" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K115" s="28" t="inlineStr">
@@ -3353,7 +3378,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J116" s="33" t="n">
+      <c r="J116" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K116" s="28" t="inlineStr">
@@ -3377,7 +3402,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J117" s="33" t="n">
+      <c r="J117" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K117" s="28" t="inlineStr">
@@ -3401,7 +3426,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J118" s="33" t="n">
+      <c r="J118" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K118" s="28" t="inlineStr">
@@ -3425,7 +3450,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J119" s="33" t="n">
+      <c r="J119" s="37" t="n">
         <v>5</v>
       </c>
       <c r="K119" s="28" t="inlineStr">
@@ -3449,7 +3474,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J120" s="33" t="n">
+      <c r="J120" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K120" s="28" t="inlineStr">
@@ -3468,18 +3493,22 @@
       <c r="F121" s="17" t="n"/>
       <c r="G121" s="31" t="n"/>
       <c r="H121" s="32" t="n"/>
-      <c r="I121" s="13" t="inlineStr">
+      <c r="I121" s="33" t="inlineStr">
         <is>
           <t>Divers - sanitaires autoroute</t>
         </is>
       </c>
-      <c r="J121" s="33" t="n">
+      <c r="J121" s="34" t="n">
         <v>1.5</v>
       </c>
-      <c r="K121" s="28" t="n"/>
-      <c r="L121" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 21-03 — décompte n° 091 du 10-04 — Valinsopay, Wijk en Aalburg (Pays-Bas)</t>
+      <c r="K121" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L121" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 21-03 — décompte n° 091 du 10-04 — Valinsopay, Wijk en Aalburg (Pays-Bas) — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3488,18 +3517,22 @@
       <c r="F122" s="17" t="n"/>
       <c r="G122" s="31" t="n"/>
       <c r="H122" s="32" t="n"/>
-      <c r="I122" s="13" t="inlineStr">
+      <c r="I122" s="33" t="inlineStr">
         <is>
           <t>Divers - sanitaires autoroute</t>
         </is>
       </c>
-      <c r="J122" s="33" t="n">
+      <c r="J122" s="34" t="n">
         <v>1.5</v>
       </c>
-      <c r="K122" s="28" t="n"/>
-      <c r="L122" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 21-03 — décompte n° 091 du 10-04 — Valinsopay, Wijk en Aalburg (Pays-Bas)</t>
+      <c r="K122" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L122" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 21-03 — décompte n° 091 du 10-04 — Valinsopay, Wijk en Aalburg (Pays-Bas) — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3546,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J123" s="33" t="n">
+      <c r="J123" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K123" s="28" t="inlineStr">
@@ -3537,7 +3570,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J124" s="33" t="n">
+      <c r="J124" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K124" s="28" t="inlineStr">
@@ -3561,7 +3594,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J125" s="33" t="n">
+      <c r="J125" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K125" s="28" t="inlineStr">
@@ -3585,7 +3618,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J126" s="33" t="n">
+      <c r="J126" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K126" s="28" t="inlineStr">
@@ -3609,7 +3642,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J127" s="33" t="n">
+      <c r="J127" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K127" s="28" t="inlineStr">
@@ -3628,18 +3661,22 @@
       <c r="F128" s="17" t="n"/>
       <c r="G128" s="31" t="n"/>
       <c r="H128" s="32" t="n"/>
-      <c r="I128" s="13" t="inlineStr">
+      <c r="I128" s="33" t="inlineStr">
         <is>
           <t>Collation - Intermarché Bruxelles</t>
         </is>
       </c>
-      <c r="J128" s="33" t="n">
+      <c r="J128" s="34" t="n">
         <v>3.58</v>
       </c>
-      <c r="K128" s="28" t="n"/>
-      <c r="L128" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04</t>
+      <c r="K128" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L128" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3648,18 +3685,22 @@
       <c r="F129" s="17" t="n"/>
       <c r="G129" s="31" t="n"/>
       <c r="H129" s="32" t="n"/>
-      <c r="I129" s="34" t="inlineStr">
+      <c r="I129" s="33" t="inlineStr">
         <is>
           <t>Achat - Oris Group, Waterloo</t>
         </is>
       </c>
-      <c r="J129" s="35" t="n">
+      <c r="J129" s="34" t="n">
         <v>25.63</v>
       </c>
-      <c r="K129" s="28" t="n"/>
+      <c r="K129" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L129" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — à identifier</t>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3668,18 +3709,22 @@
       <c r="F130" s="17" t="n"/>
       <c r="G130" s="31" t="n"/>
       <c r="H130" s="32" t="n"/>
-      <c r="I130" s="13" t="inlineStr">
+      <c r="I130" s="33" t="inlineStr">
         <is>
           <t>Achat - Fnac Woluwe</t>
         </is>
       </c>
-      <c r="J130" s="33" t="n">
+      <c r="J130" s="34" t="n">
         <v>1.09</v>
       </c>
-      <c r="K130" s="28" t="n"/>
-      <c r="L130" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04</t>
+      <c r="K130" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L130" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3688,18 +3733,22 @@
       <c r="F131" s="17" t="n"/>
       <c r="G131" s="31" t="n"/>
       <c r="H131" s="32" t="n"/>
-      <c r="I131" s="34" t="inlineStr">
+      <c r="I131" s="33" t="inlineStr">
         <is>
           <t>Achat vêtements - Zara Bruxelles</t>
         </is>
       </c>
-      <c r="J131" s="35" t="n">
+      <c r="J131" s="34" t="n">
         <v>84.05</v>
       </c>
-      <c r="K131" s="28" t="n"/>
+      <c r="K131" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L131" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — usage professionnel à confirmer</t>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — usage professionnel à confirmer — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3708,18 +3757,22 @@
       <c r="F132" s="17" t="n"/>
       <c r="G132" s="31" t="n"/>
       <c r="H132" s="32" t="n"/>
-      <c r="I132" s="34" t="inlineStr">
+      <c r="I132" s="33" t="inlineStr">
         <is>
           <t>Achat - commerçant 2419 Bruxelles</t>
         </is>
       </c>
-      <c r="J132" s="35" t="n">
+      <c r="J132" s="34" t="n">
         <v>2.89</v>
       </c>
-      <c r="K132" s="28" t="n"/>
+      <c r="K132" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L132" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — à identifier</t>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3728,18 +3781,22 @@
       <c r="F133" s="17" t="n"/>
       <c r="G133" s="31" t="n"/>
       <c r="H133" s="32" t="n"/>
-      <c r="I133" s="13" t="inlineStr">
+      <c r="I133" s="33" t="inlineStr">
         <is>
           <t>Repas Quick Kraainem</t>
         </is>
       </c>
-      <c r="J133" s="33" t="n">
+      <c r="J133" s="34" t="n">
         <v>10.45</v>
       </c>
-      <c r="K133" s="28" t="n"/>
-      <c r="L133" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04</t>
+      <c r="K133" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L133" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3748,18 +3805,22 @@
       <c r="F134" s="17" t="n"/>
       <c r="G134" s="31" t="n"/>
       <c r="H134" s="32" t="n"/>
-      <c r="I134" s="13" t="inlineStr">
+      <c r="I134" s="33" t="inlineStr">
         <is>
           <t>Collation - Naki Ixelles</t>
         </is>
       </c>
-      <c r="J134" s="33" t="n">
+      <c r="J134" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="K134" s="28" t="n"/>
-      <c r="L134" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04</t>
+      <c r="K134" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L134" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3834,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J135" s="33" t="n">
+      <c r="J135" s="37" t="n">
         <v>6.9</v>
       </c>
       <c r="K135" s="28" t="inlineStr">
@@ -3797,7 +3858,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J136" s="33" t="n">
+      <c r="J136" s="37" t="n">
         <v>2.5</v>
       </c>
       <c r="K136" s="28" t="inlineStr">
@@ -3821,7 +3882,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J137" s="33" t="n">
+      <c r="J137" s="37" t="n">
         <v>2</v>
       </c>
       <c r="K137" s="28" t="n"/>
@@ -3841,7 +3902,7 @@
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J138" s="33" t="n">
+      <c r="J138" s="37" t="n">
         <v>431.25</v>
       </c>
       <c r="K138" s="28" t="n"/>
@@ -3861,7 +3922,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J139" s="33" t="n">
+      <c r="J139" s="37" t="n">
         <v>72.18000000000001</v>
       </c>
       <c r="K139" s="28" t="inlineStr">
@@ -3885,7 +3946,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J140" s="33" t="n">
+      <c r="J140" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K140" s="28" t="inlineStr">
@@ -3909,7 +3970,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J141" s="33" t="n">
+      <c r="J141" s="37" t="n">
         <v>14</v>
       </c>
       <c r="K141" s="28" t="inlineStr">
@@ -3928,18 +3989,22 @@
       <c r="F142" s="17" t="n"/>
       <c r="G142" s="31" t="n"/>
       <c r="H142" s="32" t="n"/>
-      <c r="I142" s="13" t="inlineStr">
+      <c r="I142" s="33" t="inlineStr">
         <is>
           <t>Divers - sanitaires autoroute</t>
         </is>
       </c>
-      <c r="J142" s="33" t="n">
+      <c r="J142" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K142" s="28" t="n"/>
-      <c r="L142" s="32" t="inlineStr">
-        <is>
-          <t>2theloo, aire E40 Jabbeke</t>
+      <c r="K142" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L142" s="36" t="inlineStr">
+        <is>
+          <t>2theloo, aire E40 Jabbeke — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3948,18 +4013,22 @@
       <c r="F143" s="17" t="n"/>
       <c r="G143" s="31" t="n"/>
       <c r="H143" s="32" t="n"/>
-      <c r="I143" s="13" t="inlineStr">
+      <c r="I143" s="33" t="inlineStr">
         <is>
           <t>Divers - sanitaires autoroute</t>
         </is>
       </c>
-      <c r="J143" s="33" t="n">
+      <c r="J143" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K143" s="28" t="n"/>
-      <c r="L143" s="32" t="inlineStr">
-        <is>
-          <t>2theloo, aire E40 Jabbeke</t>
+      <c r="K143" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L143" s="36" t="inlineStr">
+        <is>
+          <t>2theloo, aire E40 Jabbeke — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -3973,7 +4042,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J144" s="33" t="n">
+      <c r="J144" s="37" t="n">
         <v>64.06999999999999</v>
       </c>
       <c r="K144" s="28" t="inlineStr">
@@ -3992,18 +4061,22 @@
       <c r="F145" s="17" t="n"/>
       <c r="G145" s="31" t="n"/>
       <c r="H145" s="32" t="n"/>
-      <c r="I145" s="13" t="inlineStr">
+      <c r="I145" s="33" t="inlineStr">
         <is>
           <t>Collation</t>
         </is>
       </c>
-      <c r="J145" s="33" t="n">
+      <c r="J145" s="34" t="n">
         <v>0.8</v>
       </c>
-      <c r="K145" s="28" t="n"/>
-      <c r="L145" s="32" t="inlineStr">
-        <is>
-          <t>AC Restaurants Wanlin</t>
+      <c r="K145" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L145" s="36" t="inlineStr">
+        <is>
+          <t>AC Restaurants Wanlin — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -4017,7 +4090,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J146" s="33" t="n">
+      <c r="J146" s="37" t="n">
         <v>256.99</v>
       </c>
       <c r="K146" s="28" t="inlineStr">
@@ -4041,7 +4114,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J147" s="33" t="n">
+      <c r="J147" s="37" t="n">
         <v>60.37</v>
       </c>
       <c r="K147" s="28" t="inlineStr">
@@ -4065,7 +4138,7 @@
           <t>Repas Topogigio</t>
         </is>
       </c>
-      <c r="J148" s="33" t="n">
+      <c r="J148" s="37" t="n">
         <v>26</v>
       </c>
       <c r="K148" s="28" t="inlineStr">
@@ -4089,7 +4162,7 @@
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J149" s="33" t="n">
+      <c r="J149" s="37" t="n">
         <v>84.2</v>
       </c>
       <c r="K149" s="28" t="inlineStr">
@@ -4108,32 +4181,36 @@
       <c r="F150" s="17" t="n"/>
       <c r="G150" s="31" t="n"/>
       <c r="H150" s="32" t="n"/>
-      <c r="I150" s="13" t="inlineStr">
+      <c r="I150" s="33" t="inlineStr">
         <is>
           <t>Achat Delhaize</t>
         </is>
       </c>
-      <c r="J150" s="33" t="n">
+      <c r="J150" s="34" t="n">
         <v>43.43</v>
       </c>
-      <c r="K150" s="28" t="n"/>
-      <c r="L150" s="32" t="inlineStr">
-        <is>
-          <t>Delhaize Sterrebeek</t>
+      <c r="K150" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L150" s="36" t="inlineStr">
+        <is>
+          <t>Delhaize Sterrebeek — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="G151" s="37" t="n"/>
-      <c r="H151" s="38" t="n"/>
-      <c r="J151" s="37" t="n"/>
-      <c r="L151" s="38" t="n"/>
+      <c r="G151" s="38" t="n"/>
+      <c r="H151" s="39" t="n"/>
+      <c r="J151" s="38" t="n"/>
+      <c r="L151" s="39" t="n"/>
     </row>
     <row r="152">
-      <c r="G152" s="37" t="n"/>
-      <c r="H152" s="38" t="n"/>
-      <c r="J152" s="37" t="n"/>
-      <c r="L152" s="38" t="n"/>
+      <c r="G152" s="38" t="n"/>
+      <c r="H152" s="39" t="n"/>
+      <c r="J152" s="38" t="n"/>
+      <c r="L152" s="39" t="n"/>
     </row>
     <row r="153">
       <c r="E153" s="16" t="inlineStr">
@@ -4155,7 +4232,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J153" s="39" t="n">
+      <c r="J153" s="40" t="n">
         <v>724.12</v>
       </c>
       <c r="K153" s="28" t="inlineStr">
@@ -4181,7 +4258,7 @@
           <t>Précompte salarial avril 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J154" s="33" t="n">
+      <c r="J154" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K154" s="28" t="inlineStr">
@@ -4205,7 +4282,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J155" s="33" t="n">
+      <c r="J155" s="37" t="n">
         <v>331.99</v>
       </c>
       <c r="K155" s="28" t="inlineStr">
@@ -4229,7 +4306,7 @@
           <t>Farys (eau)</t>
         </is>
       </c>
-      <c r="J156" s="33" t="n">
+      <c r="J156" s="37" t="n">
         <v>290</v>
       </c>
       <c r="K156" s="28" t="inlineStr">
@@ -4253,7 +4330,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J157" s="33" t="n">
+      <c r="J157" s="37" t="n">
         <v>71.54000000000001</v>
       </c>
       <c r="K157" s="28" t="inlineStr">
@@ -4277,7 +4354,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J158" s="33" t="n">
+      <c r="J158" s="37" t="n">
         <v>59.49</v>
       </c>
       <c r="K158" s="28" t="inlineStr">
@@ -4301,7 +4378,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J159" s="33" t="n">
+      <c r="J159" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K159" s="28" t="inlineStr">
@@ -4325,7 +4402,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J160" s="33" t="n">
+      <c r="J160" s="37" t="n">
         <v>2</v>
       </c>
       <c r="K160" s="28" t="n"/>
@@ -4345,7 +4422,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J161" s="33" t="n">
+      <c r="J161" s="37" t="n">
         <v>2</v>
       </c>
       <c r="K161" s="28" t="n"/>
@@ -4365,7 +4442,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J162" s="33" t="n">
+      <c r="J162" s="37" t="n">
         <v>2</v>
       </c>
       <c r="K162" s="28" t="n"/>
@@ -4385,7 +4462,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J163" s="33" t="n">
+      <c r="J163" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K163" s="28" t="n"/>
@@ -4405,7 +4482,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J164" s="33" t="n">
+      <c r="J164" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K164" s="28" t="n"/>
@@ -4425,7 +4502,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J165" s="33" t="n">
+      <c r="J165" s="37" t="n">
         <v>5</v>
       </c>
       <c r="K165" s="28" t="n"/>
@@ -4445,7 +4522,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J166" s="33" t="n">
+      <c r="J166" s="37" t="n">
         <v>8</v>
       </c>
       <c r="K166" s="28" t="n"/>
@@ -4465,7 +4542,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J167" s="33" t="n">
+      <c r="J167" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K167" s="28" t="n"/>
@@ -4485,7 +4562,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J168" s="33" t="n">
+      <c r="J168" s="37" t="n">
         <v>18</v>
       </c>
       <c r="K168" s="28" t="n"/>
@@ -4505,7 +4582,7 @@
           <t>Abonnement Shopify</t>
         </is>
       </c>
-      <c r="J169" s="33" t="n">
+      <c r="J169" s="37" t="n">
         <v>23.26</v>
       </c>
       <c r="K169" s="28" t="n"/>
@@ -4525,7 +4602,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J170" s="33" t="n">
+      <c r="J170" s="37" t="n">
         <v>18</v>
       </c>
       <c r="K170" s="28" t="n"/>
@@ -4545,7 +4622,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J171" s="33" t="n">
+      <c r="J171" s="37" t="n">
         <v>20</v>
       </c>
       <c r="K171" s="28" t="n"/>
@@ -4560,18 +4637,22 @@
       <c r="F172" s="17" t="n"/>
       <c r="G172" s="31" t="n"/>
       <c r="H172" s="32" t="n"/>
-      <c r="I172" s="34" t="inlineStr">
+      <c r="I172" s="33" t="inlineStr">
         <is>
           <t>Coiffure hommes, Schaerbeek</t>
         </is>
       </c>
-      <c r="J172" s="35" t="n">
+      <c r="J172" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="K172" s="28" t="n"/>
+      <c r="K172" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L172" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — dépense privée ? à valider</t>
+          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — dépense privée ? à valider — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -4580,18 +4661,22 @@
       <c r="F173" s="17" t="n"/>
       <c r="G173" s="31" t="n"/>
       <c r="H173" s="32" t="n"/>
-      <c r="I173" s="34" t="inlineStr">
+      <c r="I173" s="33" t="inlineStr">
         <is>
           <t>Achat - SumUp Schaerbeek</t>
         </is>
       </c>
-      <c r="J173" s="35" t="n">
+      <c r="J173" s="34" t="n">
         <v>7.9</v>
       </c>
-      <c r="K173" s="28" t="n"/>
+      <c r="K173" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L173" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — commerçant à identifier</t>
+          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — commerçant à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -4600,18 +4685,22 @@
       <c r="F174" s="17" t="n"/>
       <c r="G174" s="31" t="n"/>
       <c r="H174" s="32" t="n"/>
-      <c r="I174" s="34" t="inlineStr">
+      <c r="I174" s="33" t="inlineStr">
         <is>
           <t>Achat - Action Schaerbeek</t>
         </is>
       </c>
-      <c r="J174" s="35" t="n">
+      <c r="J174" s="34" t="n">
         <v>17.39</v>
       </c>
-      <c r="K174" s="28" t="n"/>
+      <c r="K174" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L174" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — nature de l'achat à préciser</t>
+          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — nature de l'achat à préciser — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -4625,7 +4714,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J175" s="33" t="n">
+      <c r="J175" s="37" t="n">
         <v>22</v>
       </c>
       <c r="K175" s="28" t="n"/>
@@ -4645,7 +4734,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J176" s="33" t="n">
+      <c r="J176" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K176" s="28" t="inlineStr">
@@ -4669,7 +4758,7 @@
           <t>Billet d'avion Lima-Bruxelles - Air Europa</t>
         </is>
       </c>
-      <c r="J177" s="33" t="n">
+      <c r="J177" s="37" t="n">
         <v>1683.78</v>
       </c>
       <c r="K177" s="28" t="inlineStr">
@@ -4693,7 +4782,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J178" s="33" t="n">
+      <c r="J178" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K178" s="28" t="inlineStr">
@@ -4717,7 +4806,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J179" s="33" t="n">
+      <c r="J179" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K179" s="28" t="inlineStr">
@@ -4741,7 +4830,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J180" s="33" t="n">
+      <c r="J180" s="37" t="n">
         <v>25</v>
       </c>
       <c r="K180" s="28" t="n"/>
@@ -4756,18 +4845,22 @@
       <c r="F181" s="17" t="n"/>
       <c r="G181" s="31" t="n"/>
       <c r="H181" s="32" t="n"/>
-      <c r="I181" s="34" t="inlineStr">
+      <c r="I181" s="33" t="inlineStr">
         <is>
           <t>Achat - Action Bruxelles</t>
         </is>
       </c>
-      <c r="J181" s="35" t="n">
+      <c r="J181" s="34" t="n">
         <v>24.46</v>
       </c>
-      <c r="K181" s="28" t="n"/>
+      <c r="K181" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L181" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 16-04 — décompte n° 121 du 12-05 — nature de l'achat à préciser</t>
+          <t>Carte Visa 16-04 — décompte n° 121 du 12-05 — nature de l'achat à préciser — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4874,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J182" s="33" t="n">
+      <c r="J182" s="37" t="n">
         <v>6.9</v>
       </c>
       <c r="K182" s="28" t="inlineStr">
@@ -4805,7 +4898,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J183" s="33" t="n">
+      <c r="J183" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K183" s="28" t="inlineStr">
@@ -4829,7 +4922,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J184" s="33" t="n">
+      <c r="J184" s="37" t="n">
         <v>28</v>
       </c>
       <c r="K184" s="28" t="n"/>
@@ -4849,7 +4942,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J185" s="33" t="n">
+      <c r="J185" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K185" s="28" t="inlineStr">
@@ -4873,7 +4966,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J186" s="33" t="n">
+      <c r="J186" s="37" t="n">
         <v>31</v>
       </c>
       <c r="K186" s="28" t="n"/>
@@ -4893,7 +4986,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J187" s="33" t="n">
+      <c r="J187" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K187" s="28" t="inlineStr">
@@ -4917,7 +5010,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J188" s="33" t="n">
+      <c r="J188" s="37" t="n">
         <v>35</v>
       </c>
       <c r="K188" s="28" t="n"/>
@@ -4937,7 +5030,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J189" s="33" t="n">
+      <c r="J189" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K189" s="28" t="inlineStr">
@@ -4961,7 +5054,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J190" s="33" t="n">
+      <c r="J190" s="37" t="n">
         <v>39</v>
       </c>
       <c r="K190" s="28" t="n"/>
@@ -4981,7 +5074,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J191" s="33" t="n">
+      <c r="J191" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K191" s="28" t="inlineStr">
@@ -5005,7 +5098,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J192" s="33" t="n">
+      <c r="J192" s="37" t="n">
         <v>43</v>
       </c>
       <c r="K192" s="28" t="n"/>
@@ -5025,7 +5118,7 @@
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J193" s="33" t="n">
+      <c r="J193" s="37" t="n">
         <v>50</v>
       </c>
       <c r="K193" s="28" t="inlineStr">
@@ -5049,7 +5142,7 @@
           <t>Telenet</t>
         </is>
       </c>
-      <c r="J194" s="33" t="n">
+      <c r="J194" s="37" t="n">
         <v>149.1</v>
       </c>
       <c r="K194" s="28" t="inlineStr">
@@ -5073,7 +5166,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J195" s="33" t="n">
+      <c r="J195" s="37" t="n">
         <v>66.09</v>
       </c>
       <c r="K195" s="28" t="inlineStr">
@@ -5092,18 +5185,22 @@
       <c r="F196" s="17" t="n"/>
       <c r="G196" s="31" t="n"/>
       <c r="H196" s="32" t="n"/>
-      <c r="I196" s="13" t="inlineStr">
+      <c r="I196" s="33" t="inlineStr">
         <is>
           <t>Divers - sanitaires autoroute</t>
         </is>
       </c>
-      <c r="J196" s="33" t="n">
+      <c r="J196" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K196" s="28" t="n"/>
-      <c r="L196" s="32" t="inlineStr">
-        <is>
-          <t>Tank und Rastanlage, Frechen (Allemagne)</t>
+      <c r="K196" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L196" s="36" t="inlineStr">
+        <is>
+          <t>Tank und Rastanlage, Frechen (Allemagne) — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -5112,18 +5209,22 @@
       <c r="F197" s="17" t="n"/>
       <c r="G197" s="31" t="n"/>
       <c r="H197" s="32" t="n"/>
-      <c r="I197" s="13" t="inlineStr">
+      <c r="I197" s="33" t="inlineStr">
         <is>
           <t>Divers - sanitaires autoroute</t>
         </is>
       </c>
-      <c r="J197" s="33" t="n">
+      <c r="J197" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="K197" s="28" t="n"/>
-      <c r="L197" s="32" t="inlineStr">
-        <is>
-          <t>Tank und Rastanlage, Frechen (Allemagne)</t>
+      <c r="K197" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L197" s="36" t="inlineStr">
+        <is>
+          <t>Tank und Rastanlage, Frechen (Allemagne) — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -5137,7 +5238,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J198" s="33" t="n">
+      <c r="J198" s="37" t="n">
         <v>16.5</v>
       </c>
       <c r="K198" s="28" t="inlineStr">
@@ -5161,7 +5262,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J199" s="33" t="n">
+      <c r="J199" s="37" t="n">
         <v>58.83</v>
       </c>
       <c r="K199" s="28" t="inlineStr">
@@ -5185,7 +5286,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J200" s="33" t="n">
+      <c r="J200" s="37" t="n">
         <v>1.85</v>
       </c>
       <c r="K200" s="28" t="inlineStr">
@@ -5209,7 +5310,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J201" s="33" t="n">
+      <c r="J201" s="37" t="n">
         <v>1.85</v>
       </c>
       <c r="K201" s="28" t="inlineStr">
@@ -5233,7 +5334,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J202" s="33" t="n">
+      <c r="J202" s="37" t="n">
         <v>256.99</v>
       </c>
       <c r="K202" s="28" t="inlineStr">
@@ -5257,7 +5358,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J203" s="33" t="n">
+      <c r="J203" s="37" t="n">
         <v>72.42</v>
       </c>
       <c r="K203" s="28" t="inlineStr">
@@ -5281,7 +5382,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J204" s="33" t="n">
+      <c r="J204" s="37" t="n">
         <v>1.5</v>
       </c>
       <c r="K204" s="28" t="inlineStr">
@@ -5296,16 +5397,16 @@
       </c>
     </row>
     <row r="205">
-      <c r="G205" s="37" t="n"/>
-      <c r="H205" s="38" t="n"/>
-      <c r="J205" s="37" t="n"/>
-      <c r="L205" s="38" t="n"/>
+      <c r="G205" s="38" t="n"/>
+      <c r="H205" s="39" t="n"/>
+      <c r="J205" s="38" t="n"/>
+      <c r="L205" s="39" t="n"/>
     </row>
     <row r="206">
-      <c r="G206" s="37" t="n"/>
-      <c r="H206" s="38" t="n"/>
-      <c r="J206" s="37" t="n"/>
-      <c r="L206" s="38" t="n"/>
+      <c r="G206" s="38" t="n"/>
+      <c r="H206" s="39" t="n"/>
+      <c r="J206" s="38" t="n"/>
+      <c r="L206" s="39" t="n"/>
     </row>
     <row r="207">
       <c r="E207" s="16" t="inlineStr">
@@ -5327,7 +5428,7 @@
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J207" s="39" t="n">
+      <c r="J207" s="40" t="n">
         <v>200</v>
       </c>
       <c r="K207" s="28" t="inlineStr">
@@ -5343,12 +5444,12 @@
     </row>
     <row r="208">
       <c r="E208" s="16" t="n"/>
-      <c r="F208" s="40" t="inlineStr">
+      <c r="F208" s="41" t="inlineStr">
         <is>
           <t>Approvisionnement compte - Thibault Duchène</t>
         </is>
       </c>
-      <c r="G208" s="41" t="n">
+      <c r="G208" s="42" t="n">
         <v>1500</v>
       </c>
       <c r="H208" s="36" t="inlineStr">
@@ -5361,7 +5462,7 @@
           <t>Précompte salarial mai 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J208" s="33" t="n">
+      <c r="J208" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K208" s="28" t="inlineStr">
@@ -5385,7 +5486,7 @@
           <t>Partena</t>
         </is>
       </c>
-      <c r="J209" s="33" t="n">
+      <c r="J209" s="37" t="n">
         <v>1441.87</v>
       </c>
       <c r="K209" s="28" t="inlineStr">
@@ -5409,7 +5510,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J210" s="33" t="n">
+      <c r="J210" s="37" t="n">
         <v>331.99</v>
       </c>
       <c r="K210" s="28" t="inlineStr">
@@ -5433,7 +5534,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J211" s="33" t="n">
+      <c r="J211" s="37" t="n">
         <v>55.61</v>
       </c>
       <c r="K211" s="28" t="inlineStr">
@@ -5457,7 +5558,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J212" s="33" t="n">
+      <c r="J212" s="37" t="n">
         <v>3.7</v>
       </c>
       <c r="K212" s="28" t="inlineStr">
@@ -5481,7 +5582,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J213" s="33" t="n">
+      <c r="J213" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K213" s="28" t="inlineStr">
@@ -5501,7 +5602,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J214" s="33" t="n">
+      <c r="J214" s="37" t="n">
         <v>15.8</v>
       </c>
       <c r="K214" s="28" t="inlineStr">
@@ -5525,7 +5626,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J215" s="33" t="n">
+      <c r="J215" s="37" t="n">
         <v>75.87</v>
       </c>
       <c r="K215" s="28" t="inlineStr">
@@ -5549,7 +5650,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J216" s="33" t="n">
+      <c r="J216" s="37" t="n">
         <v>31.05</v>
       </c>
       <c r="K216" s="28" t="inlineStr">
@@ -5573,7 +5674,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J217" s="33" t="n">
+      <c r="J217" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K217" s="28" t="inlineStr">
@@ -5597,7 +5698,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J218" s="33" t="n">
+      <c r="J218" s="37" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="K218" s="28" t="inlineStr">
@@ -5621,7 +5722,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J219" s="33" t="n">
+      <c r="J219" s="37" t="n">
         <v>4</v>
       </c>
       <c r="K219" s="28" t="inlineStr">
@@ -5645,7 +5746,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J220" s="33" t="n">
+      <c r="J220" s="37" t="n">
         <v>25.78</v>
       </c>
       <c r="K220" s="28" t="n"/>
@@ -5665,7 +5766,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J221" s="33" t="n">
+      <c r="J221" s="37" t="n">
         <v>48</v>
       </c>
       <c r="K221" s="28" t="n"/>
@@ -5685,7 +5786,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J222" s="33" t="n">
+      <c r="J222" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K222" s="28" t="inlineStr">
@@ -5709,7 +5810,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J223" s="33" t="n">
+      <c r="J223" s="37" t="n">
         <v>53</v>
       </c>
       <c r="K223" s="28" t="n"/>
@@ -5729,7 +5830,7 @@
           <t>Abonnement Shopify</t>
         </is>
       </c>
-      <c r="J224" s="33" t="n">
+      <c r="J224" s="37" t="n">
         <v>22.83</v>
       </c>
       <c r="K224" s="28" t="n"/>
@@ -5749,7 +5850,7 @@
           <t>Parking - AG Real Estate</t>
         </is>
       </c>
-      <c r="J225" s="33" t="n">
+      <c r="J225" s="37" t="n">
         <v>1</v>
       </c>
       <c r="K225" s="28" t="inlineStr">
@@ -5773,7 +5874,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J226" s="33" t="n">
+      <c r="J226" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K226" s="28" t="inlineStr">
@@ -5797,7 +5898,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J227" s="33" t="n">
+      <c r="J227" s="37" t="n">
         <v>59</v>
       </c>
       <c r="K227" s="28" t="n"/>
@@ -5817,7 +5918,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J228" s="33" t="n">
+      <c r="J228" s="37" t="n">
         <v>9</v>
       </c>
       <c r="K228" s="28" t="inlineStr">
@@ -5841,7 +5942,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J229" s="33" t="n">
+      <c r="J229" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K229" s="28" t="inlineStr">
@@ -5865,7 +5966,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J230" s="33" t="n">
+      <c r="J230" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K230" s="28" t="inlineStr">
@@ -5889,7 +5990,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J231" s="33" t="n">
+      <c r="J231" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K231" s="28" t="inlineStr">
@@ -5913,7 +6014,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J232" s="33" t="n">
+      <c r="J232" s="37" t="n">
         <v>65</v>
       </c>
       <c r="K232" s="28" t="n"/>
@@ -5933,7 +6034,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J233" s="33" t="n">
+      <c r="J233" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K233" s="28" t="inlineStr">
@@ -5957,7 +6058,7 @@
           <t>Parking - AG Real Estate</t>
         </is>
       </c>
-      <c r="J234" s="33" t="n">
+      <c r="J234" s="37" t="n">
         <v>1</v>
       </c>
       <c r="K234" s="28" t="inlineStr">
@@ -5981,7 +6082,7 @@
           <t>Parking - AG Real Estate</t>
         </is>
       </c>
-      <c r="J235" s="33" t="n">
+      <c r="J235" s="37" t="n">
         <v>1</v>
       </c>
       <c r="K235" s="28" t="inlineStr">
@@ -6005,7 +6106,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J236" s="33" t="n">
+      <c r="J236" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K236" s="28" t="inlineStr">
@@ -6029,7 +6130,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J237" s="33" t="n">
+      <c r="J237" s="37" t="n">
         <v>9</v>
       </c>
       <c r="K237" s="28" t="inlineStr">
@@ -6053,7 +6154,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J238" s="33" t="n">
+      <c r="J238" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K238" s="28" t="inlineStr">
@@ -6077,7 +6178,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J239" s="33" t="n">
+      <c r="J239" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K239" s="28" t="inlineStr">
@@ -6101,7 +6202,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J240" s="33" t="n">
+      <c r="J240" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K240" s="28" t="inlineStr">
@@ -6120,18 +6221,22 @@
       <c r="F241" s="17" t="n"/>
       <c r="G241" s="31" t="n"/>
       <c r="H241" s="32" t="n"/>
-      <c r="I241" s="34" t="inlineStr">
+      <c r="I241" s="33" t="inlineStr">
         <is>
           <t>Achat - Mood for Green SRL, Bruxelles</t>
         </is>
       </c>
-      <c r="J241" s="35" t="n">
+      <c r="J241" s="34" t="n">
         <v>17</v>
       </c>
-      <c r="K241" s="28" t="n"/>
+      <c r="K241" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L241" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 21-05 — décompte n° 152 du 10-06 — à identifier</t>
+          <t>Carte Visa 21-05 — décompte n° 152 du 10-06 — à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6250,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J242" s="33" t="n">
+      <c r="J242" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K242" s="28" t="inlineStr">
@@ -6169,7 +6274,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J243" s="33" t="n">
+      <c r="J243" s="37" t="n">
         <v>15</v>
       </c>
       <c r="K243" s="28" t="inlineStr">
@@ -6193,7 +6298,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J244" s="33" t="n">
+      <c r="J244" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K244" s="28" t="inlineStr">
@@ -6217,7 +6322,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J245" s="33" t="n">
+      <c r="J245" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K245" s="28" t="inlineStr">
@@ -6241,7 +6346,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J246" s="33" t="n">
+      <c r="J246" s="37" t="n">
         <v>6.9</v>
       </c>
       <c r="K246" s="28" t="inlineStr">
@@ -6265,7 +6370,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J247" s="33" t="n">
+      <c r="J247" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K247" s="28" t="inlineStr">
@@ -6289,7 +6394,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J248" s="33" t="n">
+      <c r="J248" s="37" t="n">
         <v>72</v>
       </c>
       <c r="K248" s="28" t="n"/>
@@ -6309,7 +6414,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J249" s="33" t="n">
+      <c r="J249" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K249" s="28" t="inlineStr">
@@ -6333,7 +6438,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J250" s="33" t="n">
+      <c r="J250" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K250" s="28" t="inlineStr">
@@ -6357,7 +6462,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J251" s="33" t="n">
+      <c r="J251" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K251" s="28" t="inlineStr">
@@ -6381,7 +6486,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J252" s="33" t="n">
+      <c r="J252" s="37" t="n">
         <v>24</v>
       </c>
       <c r="K252" s="28" t="inlineStr">
@@ -6405,7 +6510,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J253" s="33" t="n">
+      <c r="J253" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K253" s="28" t="inlineStr">
@@ -6429,7 +6534,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J254" s="33" t="n">
+      <c r="J254" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K254" s="28" t="inlineStr">
@@ -6453,7 +6558,7 @@
           <t>Telenet</t>
         </is>
       </c>
-      <c r="J255" s="33" t="n">
+      <c r="J255" s="37" t="n">
         <v>155.52</v>
       </c>
       <c r="K255" s="28" t="inlineStr">
@@ -6477,7 +6582,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J256" s="33" t="n">
+      <c r="J256" s="37" t="n">
         <v>64.94</v>
       </c>
       <c r="K256" s="28" t="inlineStr">
@@ -6501,7 +6606,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J257" s="33" t="n">
+      <c r="J257" s="37" t="n">
         <v>68.06</v>
       </c>
       <c r="K257" s="28" t="inlineStr">
@@ -6525,7 +6630,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J258" s="33" t="n">
+      <c r="J258" s="37" t="n">
         <v>9</v>
       </c>
       <c r="K258" s="28" t="inlineStr">
@@ -6549,7 +6654,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J259" s="33" t="n">
+      <c r="J259" s="37" t="n">
         <v>3.6</v>
       </c>
       <c r="K259" s="28" t="inlineStr">
@@ -6573,7 +6678,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J260" s="33" t="n">
+      <c r="J260" s="37" t="n">
         <v>5</v>
       </c>
       <c r="K260" s="28" t="inlineStr">
@@ -6597,7 +6702,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J261" s="33" t="n">
+      <c r="J261" s="37" t="n">
         <v>64.97</v>
       </c>
       <c r="K261" s="28" t="inlineStr">
@@ -6621,7 +6726,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J262" s="33" t="n">
+      <c r="J262" s="37" t="n">
         <v>256.99</v>
       </c>
       <c r="K262" s="28" t="inlineStr">
@@ -6645,7 +6750,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J263" s="33" t="n">
+      <c r="J263" s="37" t="n">
         <v>1.85</v>
       </c>
       <c r="K263" s="28" t="inlineStr">
@@ -6669,7 +6774,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J264" s="33" t="n">
+      <c r="J264" s="37" t="n">
         <v>54.33</v>
       </c>
       <c r="K264" s="28" t="inlineStr">
@@ -6693,7 +6798,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J265" s="33" t="n">
+      <c r="J265" s="37" t="n">
         <v>3.5</v>
       </c>
       <c r="K265" s="28" t="inlineStr">
@@ -6717,7 +6822,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J266" s="33" t="n">
+      <c r="J266" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K266" s="28" t="inlineStr">
@@ -6732,16 +6837,16 @@
       </c>
     </row>
     <row r="267">
-      <c r="G267" s="37" t="n"/>
-      <c r="H267" s="38" t="n"/>
-      <c r="J267" s="37" t="n"/>
-      <c r="L267" s="38" t="n"/>
+      <c r="G267" s="38" t="n"/>
+      <c r="H267" s="39" t="n"/>
+      <c r="J267" s="38" t="n"/>
+      <c r="L267" s="39" t="n"/>
     </row>
     <row r="268">
-      <c r="G268" s="37" t="n"/>
-      <c r="H268" s="38" t="n"/>
-      <c r="J268" s="37" t="n"/>
-      <c r="L268" s="38" t="n"/>
+      <c r="G268" s="38" t="n"/>
+      <c r="H268" s="39" t="n"/>
+      <c r="J268" s="38" t="n"/>
+      <c r="L268" s="39" t="n"/>
     </row>
     <row r="269">
       <c r="E269" s="16" t="inlineStr">
@@ -6749,12 +6854,12 @@
           <t>Juillet</t>
         </is>
       </c>
-      <c r="F269" s="40" t="inlineStr">
+      <c r="F269" s="41" t="inlineStr">
         <is>
           <t>Prise en charge par T. Duchène - facture Proximus 7504645054</t>
         </is>
       </c>
-      <c r="G269" s="41" t="n">
+      <c r="G269" s="42" t="n">
         <v>109.59</v>
       </c>
       <c r="H269" s="36" t="inlineStr">
@@ -6767,7 +6872,7 @@
           <t>Précompte salarial juin 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J269" s="39" t="n">
+      <c r="J269" s="40" t="n">
         <v>2250</v>
       </c>
       <c r="K269" s="28" t="inlineStr">
@@ -6783,12 +6888,12 @@
     </row>
     <row r="270">
       <c r="E270" s="16" t="n"/>
-      <c r="F270" s="40" t="inlineStr">
+      <c r="F270" s="41" t="inlineStr">
         <is>
           <t>Remboursement paiement à Sandaya</t>
         </is>
       </c>
-      <c r="G270" s="41" t="n">
+      <c r="G270" s="42" t="n">
         <v>1775.4</v>
       </c>
       <c r="H270" s="36" t="inlineStr">
@@ -6801,7 +6906,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J270" s="33" t="n">
+      <c r="J270" s="37" t="n">
         <v>331.99</v>
       </c>
       <c r="K270" s="28" t="inlineStr">
@@ -6835,7 +6940,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J271" s="33" t="n">
+      <c r="J271" s="37" t="n">
         <v>84.91</v>
       </c>
       <c r="K271" s="28" t="inlineStr">
@@ -6859,7 +6964,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J272" s="33" t="n">
+      <c r="J272" s="37" t="n">
         <v>109.59</v>
       </c>
       <c r="K272" s="28" t="inlineStr">
@@ -6883,7 +6988,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J273" s="33" t="n">
+      <c r="J273" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K273" s="28" t="inlineStr">
@@ -6903,7 +7008,7 @@
           <t>Frais bancaires trimestriels</t>
         </is>
       </c>
-      <c r="J274" s="33" t="n">
+      <c r="J274" s="37" t="n">
         <v>11.25</v>
       </c>
       <c r="K274" s="28" t="n"/>
@@ -6919,7 +7024,7 @@
           <t>Intérêt crédit</t>
         </is>
       </c>
-      <c r="J275" s="33" t="n">
+      <c r="J275" s="37" t="n">
         <v>0.51</v>
       </c>
       <c r="K275" s="28" t="n"/>
@@ -6939,7 +7044,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J276" s="33" t="n">
+      <c r="J276" s="37" t="n">
         <v>60.86</v>
       </c>
       <c r="K276" s="28" t="inlineStr">
@@ -6963,7 +7068,7 @@
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J277" s="33" t="n">
+      <c r="J277" s="37" t="n">
         <v>458.66</v>
       </c>
       <c r="K277" s="28" t="n"/>
@@ -6983,7 +7088,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J278" s="33" t="n">
+      <c r="J278" s="37" t="n">
         <v>20.78</v>
       </c>
       <c r="K278" s="28" t="n"/>
@@ -6998,18 +7103,22 @@
       <c r="F279" s="17" t="n"/>
       <c r="G279" s="31" t="n"/>
       <c r="H279" s="32" t="n"/>
-      <c r="I279" s="13" t="inlineStr">
+      <c r="I279" s="33" t="inlineStr">
         <is>
           <t>Achat Delhaize Wezembeek</t>
         </is>
       </c>
-      <c r="J279" s="33" t="n">
+      <c r="J279" s="34" t="n">
         <v>5.67</v>
       </c>
-      <c r="K279" s="28" t="n"/>
-      <c r="L279" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 03-06 — décompte n° 182 du 10-07</t>
+      <c r="K279" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L279" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 03-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -7018,18 +7127,22 @@
       <c r="F280" s="17" t="n"/>
       <c r="G280" s="31" t="n"/>
       <c r="H280" s="32" t="n"/>
-      <c r="I280" s="13" t="inlineStr">
+      <c r="I280" s="33" t="inlineStr">
         <is>
           <t>Achat Delhaize Wezembeek</t>
         </is>
       </c>
-      <c r="J280" s="33" t="n">
+      <c r="J280" s="34" t="n">
         <v>0.92</v>
       </c>
-      <c r="K280" s="28" t="n"/>
-      <c r="L280" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 03-06 — décompte n° 182 du 10-07</t>
+      <c r="K280" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L280" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 03-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7156,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J281" s="33" t="n">
+      <c r="J281" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K281" s="28" t="inlineStr">
@@ -7067,7 +7180,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J282" s="33" t="n">
+      <c r="J282" s="37" t="n">
         <v>9</v>
       </c>
       <c r="K282" s="28" t="inlineStr">
@@ -7091,7 +7204,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J283" s="33" t="n">
+      <c r="J283" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K283" s="28" t="inlineStr">
@@ -7115,7 +7228,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J284" s="33" t="n">
+      <c r="J284" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K284" s="28" t="inlineStr">
@@ -7139,7 +7252,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J285" s="33" t="n">
+      <c r="J285" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K285" s="28" t="inlineStr">
@@ -7163,7 +7276,7 @@
           <t>Abonnement Shopify</t>
         </is>
       </c>
-      <c r="J286" s="33" t="n">
+      <c r="J286" s="37" t="n">
         <v>27.96</v>
       </c>
       <c r="K286" s="28" t="n"/>
@@ -7183,7 +7296,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J287" s="33" t="n">
+      <c r="J287" s="37" t="n">
         <v>6.9</v>
       </c>
       <c r="K287" s="28" t="inlineStr">
@@ -7207,7 +7320,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J288" s="33" t="n">
+      <c r="J288" s="37" t="n">
         <v>18</v>
       </c>
       <c r="K288" s="28" t="inlineStr">
@@ -7226,18 +7339,22 @@
       <c r="F289" s="17" t="n"/>
       <c r="G289" s="31" t="n"/>
       <c r="H289" s="32" t="n"/>
-      <c r="I289" s="13" t="inlineStr">
+      <c r="I289" s="33" t="inlineStr">
         <is>
           <t>Achat - Carrefour Bruxelles</t>
         </is>
       </c>
-      <c r="J289" s="33" t="n">
+      <c r="J289" s="34" t="n">
         <v>4.79</v>
       </c>
-      <c r="K289" s="28" t="n"/>
-      <c r="L289" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 08-06 — décompte n° 182 du 10-07</t>
+      <c r="K289" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L289" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 08-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -7246,18 +7363,22 @@
       <c r="F290" s="17" t="n"/>
       <c r="G290" s="31" t="n"/>
       <c r="H290" s="32" t="n"/>
-      <c r="I290" s="13" t="inlineStr">
+      <c r="I290" s="33" t="inlineStr">
         <is>
           <t>Repas - Dal Long Yi, Bruxelles</t>
         </is>
       </c>
-      <c r="J290" s="33" t="n">
+      <c r="J290" s="34" t="n">
         <v>9.4</v>
       </c>
-      <c r="K290" s="28" t="n"/>
-      <c r="L290" s="32" t="inlineStr">
-        <is>
-          <t>Carte Visa 08-06 — décompte n° 182 du 10-07</t>
+      <c r="K290" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L290" s="36" t="inlineStr">
+        <is>
+          <t>Carte Visa 08-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -7266,18 +7387,22 @@
       <c r="F291" s="17" t="n"/>
       <c r="G291" s="31" t="n"/>
       <c r="H291" s="32" t="n"/>
-      <c r="I291" s="34" t="inlineStr">
+      <c r="I291" s="33" t="inlineStr">
         <is>
           <t>Achat - Proxy Meiser, Schaerbeek</t>
         </is>
       </c>
-      <c r="J291" s="35" t="n">
+      <c r="J291" s="34" t="n">
         <v>33.84</v>
       </c>
-      <c r="K291" s="28" t="n"/>
+      <c r="K291" s="35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L291" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 09-06 — décompte n° 182 du 10-07 — nature de l'achat à préciser</t>
+          <t>Carte Visa 09-06 — décompte n° 182 du 10-07 — nature de l'achat à préciser — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
         </is>
       </c>
     </row>
@@ -7291,7 +7416,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J292" s="33" t="n">
+      <c r="J292" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K292" s="28" t="inlineStr">
@@ -7315,7 +7440,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J293" s="33" t="n">
+      <c r="J293" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K293" s="28" t="inlineStr">
@@ -7339,7 +7464,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J294" s="33" t="n">
+      <c r="J294" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K294" s="28" t="inlineStr">
@@ -7363,7 +7488,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J295" s="33" t="n">
+      <c r="J295" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K295" s="28" t="inlineStr">
@@ -7387,7 +7512,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J296" s="33" t="n">
+      <c r="J296" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K296" s="28" t="inlineStr">
@@ -7411,7 +7536,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J297" s="33" t="n">
+      <c r="J297" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K297" s="28" t="inlineStr">
@@ -7435,7 +7560,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J298" s="33" t="n">
+      <c r="J298" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K298" s="28" t="inlineStr">
@@ -7459,7 +7584,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J299" s="33" t="n">
+      <c r="J299" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K299" s="28" t="inlineStr">
@@ -7483,7 +7608,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J300" s="33" t="n">
+      <c r="J300" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K300" s="28" t="inlineStr">
@@ -7507,7 +7632,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J301" s="33" t="n">
+      <c r="J301" s="37" t="n">
         <v>9</v>
       </c>
       <c r="K301" s="28" t="inlineStr">
@@ -7531,7 +7656,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J302" s="33" t="n">
+      <c r="J302" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K302" s="28" t="inlineStr">
@@ -7555,7 +7680,7 @@
           <t>Consommation club de tennis Orée</t>
         </is>
       </c>
-      <c r="J303" s="33" t="n">
+      <c r="J303" s="37" t="n">
         <v>8.5</v>
       </c>
       <c r="K303" s="28" t="inlineStr">
@@ -7579,7 +7704,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J304" s="33" t="n">
+      <c r="J304" s="37" t="n">
         <v>56.98</v>
       </c>
       <c r="K304" s="28" t="inlineStr">
@@ -7603,7 +7728,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J305" s="33" t="n">
+      <c r="J305" s="37" t="n">
         <v>62.27</v>
       </c>
       <c r="K305" s="28" t="inlineStr">
@@ -7627,7 +7752,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J306" s="33" t="n">
+      <c r="J306" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K306" s="28" t="inlineStr">
@@ -7651,7 +7776,7 @@
           <t>Péage autoroute France</t>
         </is>
       </c>
-      <c r="J307" s="33" t="n">
+      <c r="J307" s="37" t="n">
         <v>34.4</v>
       </c>
       <c r="K307" s="28" t="inlineStr">
@@ -7675,7 +7800,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J308" s="33" t="n">
+      <c r="J308" s="37" t="n">
         <v>356.79</v>
       </c>
       <c r="K308" s="28" t="inlineStr">
@@ -7699,7 +7824,7 @@
           <t>Telenet</t>
         </is>
       </c>
-      <c r="J309" s="33" t="n">
+      <c r="J309" s="37" t="n">
         <v>153.42</v>
       </c>
       <c r="K309" s="28" t="inlineStr">
@@ -7723,7 +7848,7 @@
           <t>Amende de stationnement - Saint-Josse</t>
         </is>
       </c>
-      <c r="J310" s="33" t="n">
+      <c r="J310" s="37" t="n">
         <v>100</v>
       </c>
       <c r="K310" s="28" t="n"/>
@@ -7743,7 +7868,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J311" s="33" t="n">
+      <c r="J311" s="37" t="n">
         <v>60.9</v>
       </c>
       <c r="K311" s="28" t="inlineStr">
@@ -7767,7 +7892,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J312" s="33" t="n">
+      <c r="J312" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K312" s="28" t="inlineStr">
@@ -7791,7 +7916,7 @@
           <t>Repas Topogigio</t>
         </is>
       </c>
-      <c r="J313" s="33" t="n">
+      <c r="J313" s="37" t="n">
         <v>231.5</v>
       </c>
       <c r="K313" s="28" t="inlineStr">
@@ -7815,7 +7940,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J314" s="33" t="n">
+      <c r="J314" s="37" t="n">
         <v>43.01</v>
       </c>
       <c r="K314" s="28" t="inlineStr">
@@ -7839,7 +7964,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J315" s="33" t="n">
+      <c r="J315" s="37" t="n">
         <v>1.7</v>
       </c>
       <c r="K315" s="28" t="inlineStr">
@@ -7863,7 +7988,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J316" s="33" t="n">
+      <c r="J316" s="37" t="n">
         <v>2.8</v>
       </c>
       <c r="K316" s="28" t="inlineStr">
@@ -7878,16 +8003,16 @@
       </c>
     </row>
     <row r="317">
-      <c r="G317" s="37" t="n"/>
-      <c r="H317" s="38" t="n"/>
-      <c r="J317" s="37" t="n"/>
-      <c r="L317" s="38" t="n"/>
+      <c r="G317" s="38" t="n"/>
+      <c r="H317" s="39" t="n"/>
+      <c r="J317" s="38" t="n"/>
+      <c r="L317" s="39" t="n"/>
     </row>
     <row r="318">
-      <c r="G318" s="37" t="n"/>
-      <c r="H318" s="38" t="n"/>
-      <c r="J318" s="37" t="n"/>
-      <c r="L318" s="38" t="n"/>
+      <c r="G318" s="38" t="n"/>
+      <c r="H318" s="39" t="n"/>
+      <c r="J318" s="38" t="n"/>
+      <c r="L318" s="39" t="n"/>
     </row>
     <row r="319">
       <c r="E319" s="16" t="inlineStr">
@@ -7913,7 +8038,7 @@
           <t>Précompte salarial juillet 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J319" s="39" t="n">
+      <c r="J319" s="40" t="n">
         <v>2250</v>
       </c>
       <c r="K319" s="28" t="inlineStr">
@@ -7937,7 +8062,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J320" s="33" t="n">
+      <c r="J320" s="37" t="n">
         <v>331.79</v>
       </c>
       <c r="K320" s="28" t="inlineStr">
@@ -7961,7 +8086,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J321" s="33" t="n">
+      <c r="J321" s="37" t="n">
         <v>87.43000000000001</v>
       </c>
       <c r="K321" s="28" t="inlineStr">
@@ -7985,7 +8110,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J322" s="33" t="n">
+      <c r="J322" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K322" s="28" t="inlineStr">
@@ -8005,7 +8130,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J323" s="33" t="n">
+      <c r="J323" s="37" t="n">
         <v>72.01000000000001</v>
       </c>
       <c r="K323" s="28" t="inlineStr">
@@ -8029,7 +8154,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J324" s="33" t="n">
+      <c r="J324" s="37" t="n">
         <v>77.28</v>
       </c>
       <c r="K324" s="28" t="inlineStr">
@@ -8053,7 +8178,7 @@
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J325" s="33" t="n">
+      <c r="J325" s="37" t="n">
         <v>18</v>
       </c>
       <c r="K325" s="28" t="inlineStr">
@@ -8077,7 +8202,7 @@
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J326" s="33" t="n">
+      <c r="J326" s="37" t="n">
         <v>26.47</v>
       </c>
       <c r="K326" s="28" t="n"/>
@@ -8097,7 +8222,7 @@
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J327" s="33" t="n">
+      <c r="J327" s="37" t="n">
         <v>5.51</v>
       </c>
       <c r="K327" s="28" t="n"/>
@@ -8117,7 +8242,7 @@
           <t>Abonnement Shopify</t>
         </is>
       </c>
-      <c r="J328" s="33" t="n">
+      <c r="J328" s="37" t="n">
         <v>22.48</v>
       </c>
       <c r="K328" s="28" t="n"/>
@@ -8137,7 +8262,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J329" s="33" t="n">
+      <c r="J329" s="37" t="n">
         <v>6</v>
       </c>
       <c r="K329" s="28" t="inlineStr">
@@ -8161,7 +8286,7 @@
           <t>Séjour Sandaya Lyon</t>
         </is>
       </c>
-      <c r="J330" s="33" t="n">
+      <c r="J330" s="37" t="n">
         <v>1775.4</v>
       </c>
       <c r="K330" s="28" t="inlineStr">
@@ -8185,7 +8310,7 @@
           <t>Transport - Uber</t>
         </is>
       </c>
-      <c r="J331" s="33" t="n">
+      <c r="J331" s="37" t="n">
         <v>42.66</v>
       </c>
       <c r="K331" s="28" t="inlineStr">
@@ -8209,7 +8334,7 @@
           <t>Transport - Uber</t>
         </is>
       </c>
-      <c r="J332" s="33" t="n">
+      <c r="J332" s="37" t="n">
         <v>48.18</v>
       </c>
       <c r="K332" s="28" t="inlineStr">
@@ -8233,7 +8358,7 @@
           <t>Transport - Uber</t>
         </is>
       </c>
-      <c r="J333" s="33" t="n">
+      <c r="J333" s="37" t="n">
         <v>111.19</v>
       </c>
       <c r="K333" s="28" t="inlineStr">
@@ -8257,7 +8382,7 @@
           <t>Transport - Uber</t>
         </is>
       </c>
-      <c r="J334" s="33" t="n">
+      <c r="J334" s="37" t="n">
         <v>91.52</v>
       </c>
       <c r="K334" s="28" t="inlineStr">
@@ -8281,7 +8406,7 @@
           <t>Transport - STIB</t>
         </is>
       </c>
-      <c r="J335" s="33" t="n">
+      <c r="J335" s="37" t="n">
         <v>2.3</v>
       </c>
       <c r="K335" s="28" t="inlineStr">
@@ -8305,7 +8430,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J336" s="33" t="n">
+      <c r="J336" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K336" s="28" t="inlineStr">
@@ -8329,7 +8454,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J337" s="33" t="n">
+      <c r="J337" s="37" t="n">
         <v>66.73999999999999</v>
       </c>
       <c r="K337" s="28" t="inlineStr">
@@ -8353,7 +8478,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J338" s="33" t="n">
+      <c r="J338" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K338" s="28" t="inlineStr">
@@ -8377,7 +8502,7 @@
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J339" s="33" t="n">
+      <c r="J339" s="37" t="n">
         <v>123</v>
       </c>
       <c r="K339" s="28" t="inlineStr">
@@ -8401,7 +8526,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J340" s="33" t="n">
+      <c r="J340" s="37" t="n">
         <v>62.86</v>
       </c>
       <c r="K340" s="28" t="inlineStr">
@@ -8425,7 +8550,7 @@
           <t>Péage autoroute France</t>
         </is>
       </c>
-      <c r="J341" s="33" t="n">
+      <c r="J341" s="37" t="n">
         <v>73.90000000000001</v>
       </c>
       <c r="K341" s="28" t="inlineStr">
@@ -8449,7 +8574,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J342" s="33" t="n">
+      <c r="J342" s="37" t="n">
         <v>72.59</v>
       </c>
       <c r="K342" s="28" t="inlineStr">
@@ -8473,7 +8598,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J343" s="33" t="n">
+      <c r="J343" s="37" t="n">
         <v>4.2</v>
       </c>
       <c r="K343" s="28" t="inlineStr">
@@ -8497,7 +8622,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J344" s="33" t="n">
+      <c r="J344" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K344" s="28" t="inlineStr">
@@ -8521,7 +8646,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J345" s="33" t="n">
+      <c r="J345" s="37" t="n">
         <v>2.8</v>
       </c>
       <c r="K345" s="28" t="inlineStr">
@@ -8545,7 +8670,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J346" s="33" t="n">
+      <c r="J346" s="37" t="n">
         <v>5</v>
       </c>
       <c r="K346" s="28" t="inlineStr">
@@ -8569,7 +8694,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J347" s="33" t="n">
+      <c r="J347" s="37" t="n">
         <v>5.55</v>
       </c>
       <c r="K347" s="28" t="inlineStr">
@@ -8593,7 +8718,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J348" s="33" t="n">
+      <c r="J348" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K348" s="28" t="inlineStr">
@@ -8617,7 +8742,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J349" s="33" t="n">
+      <c r="J349" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K349" s="28" t="inlineStr">
@@ -8632,16 +8757,16 @@
       </c>
     </row>
     <row r="350">
-      <c r="G350" s="37" t="n"/>
-      <c r="H350" s="38" t="n"/>
-      <c r="J350" s="37" t="n"/>
-      <c r="L350" s="38" t="n"/>
+      <c r="G350" s="38" t="n"/>
+      <c r="H350" s="39" t="n"/>
+      <c r="J350" s="38" t="n"/>
+      <c r="L350" s="39" t="n"/>
     </row>
     <row r="351">
-      <c r="G351" s="37" t="n"/>
-      <c r="H351" s="38" t="n"/>
-      <c r="J351" s="37" t="n"/>
-      <c r="L351" s="38" t="n"/>
+      <c r="G351" s="38" t="n"/>
+      <c r="H351" s="39" t="n"/>
+      <c r="J351" s="38" t="n"/>
+      <c r="L351" s="39" t="n"/>
     </row>
     <row r="352">
       <c r="E352" s="16" t="inlineStr">
@@ -8663,7 +8788,7 @@
           <t>Partena</t>
         </is>
       </c>
-      <c r="J352" s="39" t="n">
+      <c r="J352" s="40" t="n">
         <v>1441.87</v>
       </c>
       <c r="K352" s="28" t="inlineStr">
@@ -8687,7 +8812,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J353" s="33" t="n">
+      <c r="J353" s="37" t="n">
         <v>263.44</v>
       </c>
       <c r="K353" s="28" t="inlineStr">
@@ -8711,7 +8836,7 @@
           <t>Telenet</t>
         </is>
       </c>
-      <c r="J354" s="33" t="n">
+      <c r="J354" s="37" t="n">
         <v>153.42</v>
       </c>
       <c r="K354" s="28" t="inlineStr">
@@ -8735,7 +8860,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J355" s="33" t="n">
+      <c r="J355" s="37" t="n">
         <v>65.14</v>
       </c>
       <c r="K355" s="28" t="inlineStr">
@@ -8759,7 +8884,7 @@
           <t>Précompte salarial août 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J356" s="33" t="n">
+      <c r="J356" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K356" s="28" t="inlineStr">
@@ -8783,7 +8908,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J357" s="33" t="n">
+      <c r="J357" s="37" t="n">
         <v>331.79</v>
       </c>
       <c r="K357" s="28" t="inlineStr">
@@ -8807,7 +8932,7 @@
           <t>Farys (eau)</t>
         </is>
       </c>
-      <c r="J358" s="33" t="n">
+      <c r="J358" s="37" t="n">
         <v>300</v>
       </c>
       <c r="K358" s="28" t="inlineStr">
@@ -8831,7 +8956,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J359" s="33" t="n">
+      <c r="J359" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K359" s="28" t="inlineStr">
@@ -8851,7 +8976,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J360" s="33" t="n">
+      <c r="J360" s="37" t="n">
         <v>70.62</v>
       </c>
       <c r="K360" s="28" t="inlineStr">
@@ -8875,7 +9000,7 @@
           <t>Vlaamse Belastingsdienst - taxe de circulation</t>
         </is>
       </c>
-      <c r="J361" s="33" t="n">
+      <c r="J361" s="37" t="n">
         <v>161.02</v>
       </c>
       <c r="K361" s="28" t="inlineStr">
@@ -8899,7 +9024,7 @@
           <t>Transport - De Lijn</t>
         </is>
       </c>
-      <c r="J362" s="33" t="n">
+      <c r="J362" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K362" s="28" t="inlineStr">
@@ -8923,7 +9048,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J363" s="33" t="n">
+      <c r="J363" s="37" t="n">
         <v>3.2</v>
       </c>
       <c r="K363" s="28" t="inlineStr">
@@ -8947,7 +9072,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J364" s="33" t="n">
+      <c r="J364" s="37" t="n">
         <v>66.73999999999999</v>
       </c>
       <c r="K364" s="28" t="inlineStr">
@@ -8971,7 +9096,7 @@
           <t>Repas Lunch Garden</t>
         </is>
       </c>
-      <c r="J365" s="33" t="n">
+      <c r="J365" s="37" t="n">
         <v>45.77</v>
       </c>
       <c r="K365" s="28" t="inlineStr">
@@ -8995,7 +9120,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J366" s="33" t="n">
+      <c r="J366" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K366" s="28" t="inlineStr">
@@ -9019,7 +9144,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J367" s="33" t="n">
+      <c r="J367" s="37" t="n">
         <v>161.83</v>
       </c>
       <c r="K367" s="28" t="inlineStr">
@@ -9043,7 +9168,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J368" s="33" t="n">
+      <c r="J368" s="37" t="n">
         <v>0.9</v>
       </c>
       <c r="K368" s="28" t="inlineStr">
@@ -9067,7 +9192,7 @@
           <t>Péage autoroute France</t>
         </is>
       </c>
-      <c r="J369" s="33" t="n">
+      <c r="J369" s="37" t="n">
         <v>101.2</v>
       </c>
       <c r="K369" s="28" t="inlineStr">
@@ -9091,7 +9216,7 @@
           <t>Repas Exki</t>
         </is>
       </c>
-      <c r="J370" s="33" t="n">
+      <c r="J370" s="37" t="n">
         <v>35.4</v>
       </c>
       <c r="K370" s="28" t="inlineStr">
@@ -9115,7 +9240,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J371" s="33" t="n">
+      <c r="J371" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K371" s="28" t="inlineStr">
@@ -9139,7 +9264,7 @@
           <t>Formation Indigo Nails Lab Belgium</t>
         </is>
       </c>
-      <c r="J372" s="33" t="n">
+      <c r="J372" s="37" t="n">
         <v>630</v>
       </c>
       <c r="K372" s="28" t="inlineStr">
@@ -9163,7 +9288,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J373" s="33" t="n">
+      <c r="J373" s="37" t="n">
         <v>59.4</v>
       </c>
       <c r="K373" s="28" t="inlineStr">
@@ -9187,7 +9312,7 @@
           <t>Repas - Chez Ji SPRL</t>
         </is>
       </c>
-      <c r="J374" s="33" t="n">
+      <c r="J374" s="37" t="n">
         <v>47</v>
       </c>
       <c r="K374" s="28" t="inlineStr">
@@ -9211,7 +9336,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J375" s="33" t="n">
+      <c r="J375" s="37" t="n">
         <v>58.45</v>
       </c>
       <c r="K375" s="28" t="inlineStr">
@@ -9235,7 +9360,7 @@
           <t>Repas - TotalEnergies Nivelles</t>
         </is>
       </c>
-      <c r="J376" s="33" t="n">
+      <c r="J376" s="37" t="n">
         <v>13.65</v>
       </c>
       <c r="K376" s="28" t="inlineStr">
@@ -9259,7 +9384,7 @@
           <t>Achat matériel sportif - Bellissimo Sport</t>
         </is>
       </c>
-      <c r="J377" s="33" t="n">
+      <c r="J377" s="37" t="n">
         <v>40</v>
       </c>
       <c r="K377" s="28" t="inlineStr">
@@ -9274,16 +9399,16 @@
       </c>
     </row>
     <row r="378">
-      <c r="G378" s="37" t="n"/>
-      <c r="H378" s="38" t="n"/>
-      <c r="J378" s="37" t="n"/>
-      <c r="L378" s="38" t="n"/>
+      <c r="G378" s="38" t="n"/>
+      <c r="H378" s="39" t="n"/>
+      <c r="J378" s="38" t="n"/>
+      <c r="L378" s="39" t="n"/>
     </row>
     <row r="379">
-      <c r="G379" s="37" t="n"/>
-      <c r="H379" s="38" t="n"/>
-      <c r="J379" s="37" t="n"/>
-      <c r="L379" s="38" t="n"/>
+      <c r="G379" s="38" t="n"/>
+      <c r="H379" s="39" t="n"/>
+      <c r="J379" s="38" t="n"/>
+      <c r="L379" s="39" t="n"/>
     </row>
     <row r="380">
       <c r="E380" s="16" t="inlineStr">
@@ -9305,7 +9430,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J380" s="39" t="n">
+      <c r="J380" s="40" t="n">
         <v>724.12</v>
       </c>
       <c r="K380" s="28" t="inlineStr">
@@ -9331,7 +9456,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J381" s="33" t="n">
+      <c r="J381" s="37" t="n">
         <v>68.23</v>
       </c>
       <c r="K381" s="28" t="inlineStr">
@@ -9361,7 +9486,7 @@
           <t>Précompte salarial septembre 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J382" s="33" t="n">
+      <c r="J382" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K382" s="28" t="inlineStr">
@@ -9385,7 +9510,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J383" s="33" t="n">
+      <c r="J383" s="37" t="n">
         <v>331.79</v>
       </c>
       <c r="K383" s="28" t="inlineStr">
@@ -9409,7 +9534,7 @@
           <t>Farys (eau)</t>
         </is>
       </c>
-      <c r="J384" s="33" t="n">
+      <c r="J384" s="37" t="n">
         <v>172.14</v>
       </c>
       <c r="K384" s="28" t="inlineStr">
@@ -9433,7 +9558,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J385" s="33" t="n">
+      <c r="J385" s="37" t="n">
         <v>10</v>
       </c>
       <c r="K385" s="28" t="inlineStr">
@@ -9457,7 +9582,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J386" s="33" t="n">
+      <c r="J386" s="37" t="n">
         <v>1</v>
       </c>
       <c r="K386" s="28" t="inlineStr">
@@ -9481,7 +9606,7 @@
           <t>Frais bancaires trimestriels</t>
         </is>
       </c>
-      <c r="J387" s="33" t="n">
+      <c r="J387" s="37" t="n">
         <v>11.25</v>
       </c>
       <c r="K387" s="28" t="n"/>
@@ -9497,7 +9622,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J388" s="33" t="n">
+      <c r="J388" s="37" t="n">
         <v>1.85</v>
       </c>
       <c r="K388" s="28" t="inlineStr">
@@ -9521,7 +9646,7 @@
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J389" s="33" t="n">
+      <c r="J389" s="37" t="n">
         <v>458.66</v>
       </c>
       <c r="K389" s="28" t="n"/>
@@ -9541,7 +9666,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J390" s="33" t="n">
+      <c r="J390" s="37" t="n">
         <v>263.44</v>
       </c>
       <c r="K390" s="28" t="inlineStr">
@@ -9565,7 +9690,7 @@
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J391" s="33" t="n">
+      <c r="J391" s="37" t="n">
         <v>17.37</v>
       </c>
       <c r="K391" s="28" t="inlineStr">
@@ -9589,7 +9714,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J392" s="33" t="n">
+      <c r="J392" s="37" t="n">
         <v>5</v>
       </c>
       <c r="K392" s="28" t="inlineStr">
@@ -9613,7 +9738,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J393" s="33" t="n">
+      <c r="J393" s="37" t="n">
         <v>64.26000000000001</v>
       </c>
       <c r="K393" s="28" t="inlineStr">
@@ -9637,7 +9762,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J394" s="33" t="n">
+      <c r="J394" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K394" s="28" t="inlineStr">
@@ -9661,7 +9786,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J395" s="33" t="n">
+      <c r="J395" s="37" t="n">
         <v>12</v>
       </c>
       <c r="K395" s="28" t="inlineStr">
@@ -9685,7 +9810,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J396" s="33" t="n">
+      <c r="J396" s="37" t="n">
         <v>67.14</v>
       </c>
       <c r="K396" s="28" t="inlineStr">
@@ -9709,7 +9834,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J397" s="33" t="n">
+      <c r="J397" s="37" t="n">
         <v>7.7</v>
       </c>
       <c r="K397" s="28" t="inlineStr">
@@ -9733,7 +9858,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J398" s="33" t="n">
+      <c r="J398" s="37" t="n">
         <v>3.2</v>
       </c>
       <c r="K398" s="28" t="inlineStr">
@@ -9757,7 +9882,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J399" s="33" t="n">
+      <c r="J399" s="37" t="n">
         <v>3</v>
       </c>
       <c r="K399" s="28" t="inlineStr">
@@ -9781,7 +9906,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J400" s="33" t="n">
+      <c r="J400" s="37" t="n">
         <v>81.39</v>
       </c>
       <c r="K400" s="28" t="inlineStr">
@@ -9805,7 +9930,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J401" s="33" t="n">
+      <c r="J401" s="37" t="n">
         <v>9.199999999999999</v>
       </c>
       <c r="K401" s="28" t="inlineStr">
@@ -9829,7 +9954,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J402" s="33" t="n">
+      <c r="J402" s="37" t="n">
         <v>1.8</v>
       </c>
       <c r="K402" s="28" t="inlineStr">
@@ -9853,7 +9978,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J403" s="33" t="n">
+      <c r="J403" s="37" t="n">
         <v>70.66</v>
       </c>
       <c r="K403" s="28" t="inlineStr">
@@ -9877,7 +10002,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J404" s="33" t="n">
+      <c r="J404" s="37" t="n">
         <v>5</v>
       </c>
       <c r="K404" s="28" t="inlineStr">
@@ -9901,7 +10026,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J405" s="33" t="n">
+      <c r="J405" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K405" s="28" t="inlineStr">
@@ -9925,7 +10050,7 @@
           <t>Versement impôts anticipé</t>
         </is>
       </c>
-      <c r="J406" s="33" t="n">
+      <c r="J406" s="37" t="n">
         <v>5500</v>
       </c>
       <c r="K406" s="28" t="inlineStr">
@@ -9944,12 +10069,12 @@
       <c r="F407" s="17" t="n"/>
       <c r="G407" s="31" t="n"/>
       <c r="H407" s="32" t="n"/>
-      <c r="I407" s="34" t="inlineStr">
+      <c r="I407" s="33" t="inlineStr">
         <is>
           <t>Précompte mobilier</t>
         </is>
       </c>
-      <c r="J407" s="35" t="n">
+      <c r="J407" s="34" t="n">
         <v>2100</v>
       </c>
       <c r="K407" s="28" t="inlineStr">
@@ -9973,7 +10098,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J408" s="33" t="n">
+      <c r="J408" s="37" t="n">
         <v>148.72</v>
       </c>
       <c r="K408" s="28" t="inlineStr">
@@ -9997,7 +10122,7 @@
           <t>Consommation Lambermont</t>
         </is>
       </c>
-      <c r="J409" s="33" t="n">
+      <c r="J409" s="37" t="n">
         <v>58</v>
       </c>
       <c r="K409" s="28" t="inlineStr">
@@ -10012,16 +10137,16 @@
       </c>
     </row>
     <row r="410">
-      <c r="G410" s="37" t="n"/>
-      <c r="H410" s="38" t="n"/>
-      <c r="J410" s="37" t="n"/>
-      <c r="L410" s="38" t="n"/>
+      <c r="G410" s="38" t="n"/>
+      <c r="H410" s="39" t="n"/>
+      <c r="J410" s="38" t="n"/>
+      <c r="L410" s="39" t="n"/>
     </row>
     <row r="411">
-      <c r="G411" s="37" t="n"/>
-      <c r="H411" s="38" t="n"/>
-      <c r="J411" s="37" t="n"/>
-      <c r="L411" s="38" t="n"/>
+      <c r="G411" s="38" t="n"/>
+      <c r="H411" s="39" t="n"/>
+      <c r="J411" s="38" t="n"/>
+      <c r="L411" s="39" t="n"/>
     </row>
     <row r="412">
       <c r="E412" s="16" t="inlineStr">
@@ -10037,7 +10162,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J412" s="39" t="n">
+      <c r="J412" s="40" t="n">
         <v>65.29000000000001</v>
       </c>
       <c r="K412" s="28" t="inlineStr">
@@ -10056,12 +10181,12 @@
       <c r="F413" s="17" t="n"/>
       <c r="G413" s="31" t="n"/>
       <c r="H413" s="32" t="n"/>
-      <c r="I413" s="34" t="inlineStr">
+      <c r="I413" s="33" t="inlineStr">
         <is>
           <t>Achat - Media Markt</t>
         </is>
       </c>
-      <c r="J413" s="35" t="n">
+      <c r="J413" s="34" t="n">
         <v>748</v>
       </c>
       <c r="K413" s="28" t="inlineStr">
@@ -10080,12 +10205,12 @@
       <c r="F414" s="17" t="n"/>
       <c r="G414" s="31" t="n"/>
       <c r="H414" s="32" t="n"/>
-      <c r="I414" s="34" t="inlineStr">
+      <c r="I414" s="33" t="inlineStr">
         <is>
           <t>Achat - Media Markt</t>
         </is>
       </c>
-      <c r="J414" s="35" t="n">
+      <c r="J414" s="34" t="n">
         <v>39</v>
       </c>
       <c r="K414" s="28" t="inlineStr">
@@ -10109,7 +10234,7 @@
           <t>Précompte salarial octobre 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J415" s="33" t="n">
+      <c r="J415" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K415" s="28" t="inlineStr">
@@ -10133,7 +10258,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J416" s="33" t="n">
+      <c r="J416" s="37" t="n">
         <v>331.85</v>
       </c>
       <c r="K416" s="28" t="inlineStr">
@@ -10157,7 +10282,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J417" s="33" t="n">
+      <c r="J417" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K417" s="28" t="inlineStr">
@@ -10177,7 +10302,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J418" s="33" t="n">
+      <c r="J418" s="37" t="n">
         <v>2.72</v>
       </c>
       <c r="K418" s="28" t="inlineStr">
@@ -10201,7 +10326,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J419" s="33" t="n">
+      <c r="J419" s="37" t="n">
         <v>70.44</v>
       </c>
       <c r="K419" s="28" t="inlineStr">
@@ -10225,7 +10350,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J420" s="33" t="n">
+      <c r="J420" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K420" s="28" t="inlineStr">
@@ -10249,7 +10374,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J421" s="33" t="n">
+      <c r="J421" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K421" s="28" t="inlineStr">
@@ -10273,7 +10398,7 @@
           <t>Partena</t>
         </is>
       </c>
-      <c r="J422" s="33" t="n">
+      <c r="J422" s="37" t="n">
         <v>1441.87</v>
       </c>
       <c r="K422" s="28" t="inlineStr">
@@ -10297,7 +10422,7 @@
           <t>Frais comptable BDH - publication BNB</t>
         </is>
       </c>
-      <c r="J423" s="33" t="n">
+      <c r="J423" s="37" t="n">
         <v>287.7</v>
       </c>
       <c r="K423" s="28" t="inlineStr">
@@ -10321,7 +10446,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J424" s="33" t="n">
+      <c r="J424" s="37" t="n">
         <v>270.94</v>
       </c>
       <c r="K424" s="28" t="inlineStr">
@@ -10345,7 +10470,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J425" s="33" t="n">
+      <c r="J425" s="37" t="n">
         <v>263.44</v>
       </c>
       <c r="K425" s="28" t="inlineStr">
@@ -10369,7 +10494,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J426" s="33" t="n">
+      <c r="J426" s="37" t="n">
         <v>143.48</v>
       </c>
       <c r="K426" s="28" t="inlineStr">
@@ -10393,7 +10518,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J427" s="33" t="n">
+      <c r="J427" s="37" t="n">
         <v>65.52</v>
       </c>
       <c r="K427" s="28" t="inlineStr">
@@ -10417,7 +10542,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J428" s="33" t="n">
+      <c r="J428" s="37" t="n">
         <v>0.9</v>
       </c>
       <c r="K428" s="28" t="inlineStr">
@@ -10441,7 +10566,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J429" s="33" t="n">
+      <c r="J429" s="37" t="n">
         <v>2.68</v>
       </c>
       <c r="K429" s="28" t="inlineStr">
@@ -10460,12 +10585,12 @@
       <c r="F430" s="17" t="n"/>
       <c r="G430" s="31" t="n"/>
       <c r="H430" s="32" t="n"/>
-      <c r="I430" s="34" t="inlineStr">
+      <c r="I430" s="33" t="inlineStr">
         <is>
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J430" s="35" t="n">
+      <c r="J430" s="34" t="n">
         <v>118.5</v>
       </c>
       <c r="K430" s="28" t="inlineStr">
@@ -10489,7 +10614,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J431" s="33" t="n">
+      <c r="J431" s="37" t="n">
         <v>12.6</v>
       </c>
       <c r="K431" s="28" t="inlineStr">
@@ -10513,7 +10638,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J432" s="33" t="n">
+      <c r="J432" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K432" s="28" t="inlineStr">
@@ -10537,7 +10662,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J433" s="33" t="n">
+      <c r="J433" s="37" t="n">
         <v>69.11</v>
       </c>
       <c r="K433" s="28" t="inlineStr">
@@ -10561,7 +10686,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J434" s="33" t="n">
+      <c r="J434" s="37" t="n">
         <v>1.85</v>
       </c>
       <c r="K434" s="28" t="inlineStr">
@@ -10585,7 +10710,7 @@
           <t>Semelles orthopédiques de travail - Podomed</t>
         </is>
       </c>
-      <c r="J435" s="33" t="n">
+      <c r="J435" s="37" t="n">
         <v>65</v>
       </c>
       <c r="K435" s="28" t="inlineStr">
@@ -10609,7 +10734,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J436" s="33" t="n">
+      <c r="J436" s="37" t="n">
         <v>5.55</v>
       </c>
       <c r="K436" s="28" t="inlineStr">
@@ -10633,7 +10758,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J437" s="33" t="n">
+      <c r="J437" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K437" s="28" t="inlineStr">
@@ -10648,16 +10773,16 @@
       </c>
     </row>
     <row r="438">
-      <c r="G438" s="37" t="n"/>
-      <c r="H438" s="38" t="n"/>
-      <c r="J438" s="37" t="n"/>
-      <c r="L438" s="38" t="n"/>
+      <c r="G438" s="38" t="n"/>
+      <c r="H438" s="39" t="n"/>
+      <c r="J438" s="38" t="n"/>
+      <c r="L438" s="39" t="n"/>
     </row>
     <row r="439">
-      <c r="G439" s="37" t="n"/>
-      <c r="H439" s="38" t="n"/>
-      <c r="J439" s="37" t="n"/>
-      <c r="L439" s="38" t="n"/>
+      <c r="G439" s="38" t="n"/>
+      <c r="H439" s="39" t="n"/>
+      <c r="J439" s="38" t="n"/>
+      <c r="L439" s="39" t="n"/>
     </row>
     <row r="440">
       <c r="E440" s="16" t="inlineStr">
@@ -10679,7 +10804,7 @@
           <t>Précompte salarial novembre 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J440" s="39" t="n">
+      <c r="J440" s="40" t="n">
         <v>2250</v>
       </c>
       <c r="K440" s="28" t="inlineStr">
@@ -10709,7 +10834,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J441" s="33" t="n">
+      <c r="J441" s="37" t="n">
         <v>331.85</v>
       </c>
       <c r="K441" s="28" t="inlineStr">
@@ -10733,7 +10858,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J442" s="33" t="n">
+      <c r="J442" s="37" t="n">
         <v>63.61</v>
       </c>
       <c r="K442" s="28" t="inlineStr">
@@ -10757,7 +10882,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J443" s="33" t="n">
+      <c r="J443" s="37" t="n">
         <v>724.12</v>
       </c>
       <c r="K443" s="28" t="inlineStr">
@@ -10777,7 +10902,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J444" s="33" t="n">
+      <c r="J444" s="37" t="n">
         <v>4.6</v>
       </c>
       <c r="K444" s="28" t="inlineStr">
@@ -10801,7 +10926,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J445" s="33" t="n">
+      <c r="J445" s="37" t="n">
         <v>3.2</v>
       </c>
       <c r="K445" s="28" t="inlineStr">
@@ -10825,7 +10950,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J446" s="33" t="n">
+      <c r="J446" s="37" t="n">
         <v>63.8</v>
       </c>
       <c r="K446" s="28" t="inlineStr">
@@ -10849,7 +10974,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J447" s="33" t="n">
+      <c r="J447" s="37" t="n">
         <v>6.97</v>
       </c>
       <c r="K447" s="28" t="inlineStr">
@@ -10873,7 +10998,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J448" s="33" t="n">
+      <c r="J448" s="37" t="n">
         <v>7</v>
       </c>
       <c r="K448" s="28" t="inlineStr">
@@ -10892,12 +11017,12 @@
       <c r="F449" s="17" t="n"/>
       <c r="G449" s="31" t="n"/>
       <c r="H449" s="32" t="n"/>
-      <c r="I449" s="34" t="inlineStr">
+      <c r="I449" s="33" t="inlineStr">
         <is>
           <t>Xerius</t>
         </is>
       </c>
-      <c r="J449" s="35" t="n">
+      <c r="J449" s="34" t="n">
         <v>399.73</v>
       </c>
       <c r="K449" s="28" t="n"/>
@@ -10917,7 +11042,7 @@
           <t>Electrabel</t>
         </is>
       </c>
-      <c r="J450" s="33" t="n">
+      <c r="J450" s="37" t="n">
         <v>263.44</v>
       </c>
       <c r="K450" s="28" t="inlineStr">
@@ -10941,7 +11066,7 @@
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J451" s="33" t="n">
+      <c r="J451" s="37" t="n">
         <v>153.79</v>
       </c>
       <c r="K451" s="28" t="inlineStr">
@@ -10965,7 +11090,7 @@
           <t>Assurance RC - LRS Insurance</t>
         </is>
       </c>
-      <c r="J452" s="33" t="n">
+      <c r="J452" s="37" t="n">
         <v>55.04</v>
       </c>
       <c r="K452" s="28" t="n"/>
@@ -10985,7 +11110,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J453" s="33" t="n">
+      <c r="J453" s="37" t="n">
         <v>63.2</v>
       </c>
       <c r="K453" s="28" t="inlineStr">
@@ -11009,7 +11134,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J454" s="33" t="n">
+      <c r="J454" s="37" t="n">
         <v>3.7</v>
       </c>
       <c r="K454" s="28" t="inlineStr">
@@ -11033,7 +11158,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J455" s="33" t="n">
+      <c r="J455" s="37" t="n">
         <v>1.6</v>
       </c>
       <c r="K455" s="28" t="inlineStr">
@@ -11057,7 +11182,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J456" s="33" t="n">
+      <c r="J456" s="37" t="n">
         <v>14</v>
       </c>
       <c r="K456" s="28" t="inlineStr">
@@ -11081,7 +11206,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J457" s="33" t="n">
+      <c r="J457" s="37" t="n">
         <v>2.6</v>
       </c>
       <c r="K457" s="28" t="inlineStr">
@@ -11105,7 +11230,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J458" s="33" t="n">
+      <c r="J458" s="37" t="n">
         <v>63.32</v>
       </c>
       <c r="K458" s="28" t="inlineStr">
@@ -11129,7 +11254,7 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="J459" s="33" t="n">
+      <c r="J459" s="37" t="n">
         <v>3.4</v>
       </c>
       <c r="K459" s="28" t="inlineStr">
@@ -11153,7 +11278,7 @@
           <t>Semelles orthopédiques de travail - Podomed</t>
         </is>
       </c>
-      <c r="J460" s="33" t="n">
+      <c r="J460" s="37" t="n">
         <v>210</v>
       </c>
       <c r="K460" s="28" t="inlineStr">
@@ -11177,7 +11302,7 @@
           <t>Frais comptable BDH</t>
         </is>
       </c>
-      <c r="J461" s="33" t="n">
+      <c r="J461" s="37" t="n">
         <v>304.92</v>
       </c>
       <c r="K461" s="28" t="inlineStr">
@@ -11201,7 +11326,7 @@
           <t>Frais comptable BDH</t>
         </is>
       </c>
-      <c r="J462" s="33" t="n">
+      <c r="J462" s="37" t="n">
         <v>1179.75</v>
       </c>
       <c r="K462" s="28" t="inlineStr">
@@ -11225,7 +11350,7 @@
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J463" s="33" t="n">
+      <c r="J463" s="37" t="n">
         <v>11.84</v>
       </c>
       <c r="K463" s="28" t="inlineStr">
@@ -11249,7 +11374,7 @@
           <t>Précompte salarial décembre 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J464" s="33" t="n">
+      <c r="J464" s="37" t="n">
         <v>2250</v>
       </c>
       <c r="K464" s="28" t="inlineStr">
@@ -11273,7 +11398,7 @@
           <t>SD Worx</t>
         </is>
       </c>
-      <c r="J465" s="33" t="n">
+      <c r="J465" s="37" t="n">
         <v>331.85</v>
       </c>
       <c r="K465" s="28" t="inlineStr">
@@ -11288,28 +11413,28 @@
       </c>
     </row>
     <row r="466">
-      <c r="G466" s="37" t="n"/>
-      <c r="H466" s="38" t="n"/>
-      <c r="J466" s="37" t="n"/>
-      <c r="L466" s="38" t="n"/>
+      <c r="G466" s="38" t="n"/>
+      <c r="H466" s="39" t="n"/>
+      <c r="J466" s="38" t="n"/>
+      <c r="L466" s="39" t="n"/>
     </row>
     <row r="467">
-      <c r="G467" s="37" t="n"/>
-      <c r="H467" s="38" t="n"/>
-      <c r="J467" s="37" t="n"/>
-      <c r="L467" s="38" t="n"/>
+      <c r="G467" s="38" t="n"/>
+      <c r="H467" s="39" t="n"/>
+      <c r="J467" s="38" t="n"/>
+      <c r="L467" s="39" t="n"/>
     </row>
     <row r="468">
-      <c r="G468" s="37">
+      <c r="G468" s="38">
         <f>SUM(G6:G467)</f>
         <v/>
       </c>
-      <c r="H468" s="38" t="n"/>
-      <c r="J468" s="37">
+      <c r="H468" s="39" t="n"/>
+      <c r="J468" s="38">
         <f>SUM(J6:J467)</f>
         <v/>
       </c>
-      <c r="L468" s="38" t="n"/>
+      <c r="L468" s="39" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bilan 2025 : deux couleurs au lieu d'une
Jaune = il manque une piece, orange = arbitrage a trancher avec BDH. Le
surlignage se decide desormais apres le remplissage de la colonne Facture,
puisqu'il en depend. Une ligne qui est les deux part en orange : la piece
manquante se voit deja a la colonne Facture restee vide.

68 pieces manquantes, 22 arbitrages. La legende est en D5.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ESFU2FaojwQMriXAPdRnAL
</commit_message>
<xml_diff>
--- a/Bilan_2025_MTCB.xlsx
+++ b/Bilan_2025_MTCB.xlsx
@@ -39,7 +39,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
   </fills>
@@ -318,7 +323,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -361,13 +366,19 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="5" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -806,7 +817,7 @@
     <row r="5" ht="15.75" customHeight="1" thickBot="1">
       <c r="D5" t="inlineStr">
         <is>
-          <t>Surligné en jaune = à trancher avec le comptable</t>
+          <t>Jaune = pièce manquante  ·  Orange = à trancher avec le comptable</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -880,7 +891,7 @@
       </c>
       <c r="L6" s="36" t="inlineStr">
         <is>
-          <t>Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -919,16 +930,16 @@
       <c r="F8" s="17" t="n"/>
       <c r="G8" s="31" t="n"/>
       <c r="H8" s="32" t="n"/>
-      <c r="I8" s="13" t="inlineStr">
+      <c r="I8" s="33" t="inlineStr">
         <is>
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J8" s="37" t="n">
+      <c r="J8" s="34" t="n">
         <v>5.69</v>
       </c>
-      <c r="K8" s="28" t="n"/>
-      <c r="L8" s="32" t="n"/>
+      <c r="K8" s="35" t="n"/>
+      <c r="L8" s="36" t="n"/>
     </row>
     <row r="9">
       <c r="E9" s="16" t="n"/>
@@ -999,32 +1010,32 @@
       <c r="F12" s="17" t="n"/>
       <c r="G12" s="31" t="n"/>
       <c r="H12" s="32" t="n"/>
-      <c r="I12" s="13" t="inlineStr">
+      <c r="I12" s="33" t="inlineStr">
         <is>
           <t>Frais bancaires trimestriels</t>
         </is>
       </c>
-      <c r="J12" s="37" t="n">
+      <c r="J12" s="34" t="n">
         <v>11.25</v>
       </c>
-      <c r="K12" s="28" t="n"/>
-      <c r="L12" s="32" t="n"/>
+      <c r="K12" s="35" t="n"/>
+      <c r="L12" s="36" t="n"/>
     </row>
     <row r="13">
       <c r="E13" s="16" t="n"/>
       <c r="F13" s="17" t="n"/>
       <c r="G13" s="31" t="n"/>
       <c r="H13" s="32" t="n"/>
-      <c r="I13" s="13" t="inlineStr">
+      <c r="I13" s="33" t="inlineStr">
         <is>
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J13" s="37" t="n">
+      <c r="J13" s="34" t="n">
         <v>431.25</v>
       </c>
-      <c r="K13" s="28" t="n"/>
-      <c r="L13" s="32" t="inlineStr">
+      <c r="K13" s="35" t="n"/>
+      <c r="L13" s="36" t="inlineStr">
         <is>
           <t>Paiement par domiciliation (AG Insurance)</t>
         </is>
@@ -1271,20 +1282,20 @@
       <c r="F24" s="17" t="n"/>
       <c r="G24" s="31" t="n"/>
       <c r="H24" s="32" t="n"/>
-      <c r="I24" s="33" t="inlineStr">
+      <c r="I24" s="38" t="inlineStr">
         <is>
           <t>Billets d'avion Pérou - Translatina Travel</t>
         </is>
       </c>
-      <c r="J24" s="34" t="n">
+      <c r="J24" s="39" t="n">
         <v>1100</v>
       </c>
-      <c r="K24" s="28" t="inlineStr">
+      <c r="K24" s="40" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L24" s="36" t="inlineStr">
+      <c r="L24" s="41" t="inlineStr">
         <is>
           <t>Avance - remboursé plus tard — Facture Translatina Travel en main — rattachement privé/société à trancher</t>
         </is>
@@ -1319,20 +1330,20 @@
       <c r="F26" s="17" t="n"/>
       <c r="G26" s="31" t="n"/>
       <c r="H26" s="32" t="n"/>
-      <c r="I26" s="33" t="inlineStr">
+      <c r="I26" s="38" t="inlineStr">
         <is>
           <t>Billets d'avion Pérou - Translatina Travel</t>
         </is>
       </c>
-      <c r="J26" s="34" t="n">
+      <c r="J26" s="39" t="n">
         <v>42</v>
       </c>
-      <c r="K26" s="28" t="inlineStr">
+      <c r="K26" s="40" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L26" s="36" t="inlineStr">
+      <c r="L26" s="41" t="inlineStr">
         <is>
           <t>Avance - remboursé plus tard — Facture Translatina Travel en main — rattachement privé/société à trancher</t>
         </is>
@@ -1415,32 +1426,32 @@
       <c r="F30" s="17" t="n"/>
       <c r="G30" s="31" t="n"/>
       <c r="H30" s="32" t="n"/>
-      <c r="I30" s="13" t="inlineStr">
+      <c r="I30" s="33" t="inlineStr">
         <is>
           <t>Proximus</t>
         </is>
       </c>
-      <c r="J30" s="37" t="n">
+      <c r="J30" s="34" t="n">
         <v>70.18000000000001</v>
       </c>
-      <c r="K30" s="28" t="n"/>
-      <c r="L30" s="32" t="inlineStr">
+      <c r="K30" s="35" t="n"/>
+      <c r="L30" s="36" t="inlineStr">
         <is>
           <t>Facture 750/1364/96037</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="G31" s="38" t="n"/>
-      <c r="H31" s="39" t="n"/>
-      <c r="J31" s="38" t="n"/>
-      <c r="L31" s="39" t="n"/>
+      <c r="G31" s="42" t="n"/>
+      <c r="H31" s="43" t="n"/>
+      <c r="J31" s="42" t="n"/>
+      <c r="L31" s="43" t="n"/>
     </row>
     <row r="32">
-      <c r="G32" s="38" t="n"/>
-      <c r="H32" s="39" t="n"/>
-      <c r="J32" s="38" t="n"/>
-      <c r="L32" s="39" t="n"/>
+      <c r="G32" s="42" t="n"/>
+      <c r="H32" s="43" t="n"/>
+      <c r="J32" s="42" t="n"/>
+      <c r="L32" s="43" t="n"/>
     </row>
     <row r="33">
       <c r="E33" s="16" t="inlineStr">
@@ -1462,7 +1473,7 @@
           <t>Achat vêtements sport - Tommy Hilfiger Maasmechelen</t>
         </is>
       </c>
-      <c r="J33" s="40" t="n">
+      <c r="J33" s="44" t="n">
         <v>210.49</v>
       </c>
       <c r="K33" s="28" t="inlineStr">
@@ -2075,16 +2086,16 @@
       </c>
     </row>
     <row r="59">
-      <c r="G59" s="38" t="n"/>
-      <c r="H59" s="39" t="n"/>
-      <c r="J59" s="38" t="n"/>
-      <c r="L59" s="39" t="n"/>
+      <c r="G59" s="42" t="n"/>
+      <c r="H59" s="43" t="n"/>
+      <c r="J59" s="42" t="n"/>
+      <c r="L59" s="43" t="n"/>
     </row>
     <row r="60">
-      <c r="G60" s="38" t="n"/>
-      <c r="H60" s="39" t="n"/>
-      <c r="J60" s="38" t="n"/>
-      <c r="L60" s="39" t="n"/>
+      <c r="G60" s="42" t="n"/>
+      <c r="H60" s="43" t="n"/>
+      <c r="J60" s="42" t="n"/>
+      <c r="L60" s="43" t="n"/>
     </row>
     <row r="61">
       <c r="E61" s="16" t="inlineStr">
@@ -2106,7 +2117,7 @@
           <t>Achat vêtements de tennis - Bellissimo Sport</t>
         </is>
       </c>
-      <c r="J61" s="40" t="n">
+      <c r="J61" s="44" t="n">
         <v>290.5</v>
       </c>
       <c r="K61" s="28" t="inlineStr">
@@ -2367,16 +2378,16 @@
       <c r="F72" s="17" t="n"/>
       <c r="G72" s="31" t="n"/>
       <c r="H72" s="32" t="n"/>
-      <c r="I72" s="13" t="inlineStr">
+      <c r="I72" s="33" t="inlineStr">
         <is>
           <t>Amende de stationnement - Ville de Louvain</t>
         </is>
       </c>
-      <c r="J72" s="37" t="n">
+      <c r="J72" s="34" t="n">
         <v>58</v>
       </c>
-      <c r="K72" s="28" t="n"/>
-      <c r="L72" s="32" t="inlineStr">
+      <c r="K72" s="35" t="n"/>
+      <c r="L72" s="36" t="inlineStr">
         <is>
           <t>Amende — dépense non admise, comm. 194/3769/90294</t>
         </is>
@@ -2387,16 +2398,16 @@
       <c r="F73" s="17" t="n"/>
       <c r="G73" s="31" t="n"/>
       <c r="H73" s="32" t="n"/>
-      <c r="I73" s="13" t="inlineStr">
+      <c r="I73" s="33" t="inlineStr">
         <is>
           <t>Amende de stationnement - Woluwe-Saint-Lambert</t>
         </is>
       </c>
-      <c r="J73" s="37" t="n">
+      <c r="J73" s="34" t="n">
         <v>45</v>
       </c>
-      <c r="K73" s="28" t="n"/>
-      <c r="L73" s="32" t="inlineStr">
+      <c r="K73" s="35" t="n"/>
+      <c r="L73" s="36" t="inlineStr">
         <is>
           <t>Amende — dépense non admise, comm. 602/2505/46621</t>
         </is>
@@ -2739,16 +2750,16 @@
       </c>
     </row>
     <row r="88">
-      <c r="G88" s="38" t="n"/>
-      <c r="H88" s="39" t="n"/>
-      <c r="J88" s="38" t="n"/>
-      <c r="L88" s="39" t="n"/>
+      <c r="G88" s="42" t="n"/>
+      <c r="H88" s="43" t="n"/>
+      <c r="J88" s="42" t="n"/>
+      <c r="L88" s="43" t="n"/>
     </row>
     <row r="89">
-      <c r="G89" s="38" t="n"/>
-      <c r="H89" s="39" t="n"/>
-      <c r="J89" s="38" t="n"/>
-      <c r="L89" s="39" t="n"/>
+      <c r="G89" s="42" t="n"/>
+      <c r="H89" s="43" t="n"/>
+      <c r="J89" s="42" t="n"/>
+      <c r="L89" s="43" t="n"/>
     </row>
     <row r="90">
       <c r="E90" s="16" t="inlineStr">
@@ -2756,15 +2767,15 @@
           <t>Avril</t>
         </is>
       </c>
-      <c r="F90" s="41" t="inlineStr">
+      <c r="F90" s="45" t="inlineStr">
         <is>
           <t>Remboursement billet d'avion Lima-Bruxelles</t>
         </is>
       </c>
-      <c r="G90" s="42" t="n">
+      <c r="G90" s="46" t="n">
         <v>1683.78</v>
       </c>
-      <c r="H90" s="36" t="inlineStr">
+      <c r="H90" s="41" t="inlineStr">
         <is>
           <t>Versement de Thibault Duchène (contrepartie du billet Air Europa du 13-04) — produit ou compte courant, à trancher</t>
         </is>
@@ -2774,7 +2785,7 @@
           <t>Repas Exki</t>
         </is>
       </c>
-      <c r="J90" s="40" t="n">
+      <c r="J90" s="44" t="n">
         <v>30.3</v>
       </c>
       <c r="K90" s="28" t="inlineStr">
@@ -2909,16 +2920,16 @@
       <c r="F96" s="17" t="n"/>
       <c r="G96" s="31" t="n"/>
       <c r="H96" s="32" t="n"/>
-      <c r="I96" s="13" t="inlineStr">
+      <c r="I96" s="33" t="inlineStr">
         <is>
           <t>Frais bancaires trimestriels</t>
         </is>
       </c>
-      <c r="J96" s="37" t="n">
+      <c r="J96" s="34" t="n">
         <v>11.25</v>
       </c>
-      <c r="K96" s="28" t="n"/>
-      <c r="L96" s="32" t="n"/>
+      <c r="K96" s="35" t="n"/>
+      <c r="L96" s="36" t="n"/>
     </row>
     <row r="97">
       <c r="E97" s="16" t="n"/>
@@ -3117,22 +3128,22 @@
       <c r="F105" s="17" t="n"/>
       <c r="G105" s="31" t="n"/>
       <c r="H105" s="32" t="n"/>
-      <c r="I105" s="33" t="inlineStr">
+      <c r="I105" s="38" t="inlineStr">
         <is>
           <t>Divers - Blitha Vereycken, Anvers</t>
         </is>
       </c>
-      <c r="J105" s="34" t="n">
+      <c r="J105" s="39" t="n">
         <v>2.5</v>
       </c>
-      <c r="K105" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L105" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 01-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K105" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L105" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 01-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3165,16 +3176,16 @@
       <c r="F107" s="17" t="n"/>
       <c r="G107" s="31" t="n"/>
       <c r="H107" s="32" t="n"/>
-      <c r="I107" s="13" t="inlineStr">
+      <c r="I107" s="33" t="inlineStr">
         <is>
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J107" s="37" t="n">
+      <c r="J107" s="34" t="n">
         <v>48.67</v>
       </c>
-      <c r="K107" s="28" t="n"/>
-      <c r="L107" s="32" t="inlineStr">
+      <c r="K107" s="35" t="n"/>
+      <c r="L107" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 05-03 — décompte n° 091 du 10-04 — Envoi 798748628</t>
         </is>
@@ -3185,16 +3196,16 @@
       <c r="F108" s="17" t="n"/>
       <c r="G108" s="31" t="n"/>
       <c r="H108" s="32" t="n"/>
-      <c r="I108" s="13" t="inlineStr">
+      <c r="I108" s="33" t="inlineStr">
         <is>
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J108" s="37" t="n">
+      <c r="J108" s="34" t="n">
         <v>97.34</v>
       </c>
-      <c r="K108" s="28" t="n"/>
-      <c r="L108" s="32" t="inlineStr">
+      <c r="K108" s="35" t="n"/>
+      <c r="L108" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 10-03 — décompte n° 091 du 10-04 — Envoi 798752501</t>
         </is>
@@ -3220,7 +3231,7 @@
       </c>
       <c r="L109" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 10-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 10-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3255,7 @@
       </c>
       <c r="L110" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 10-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 10-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3325,22 +3336,22 @@
       <c r="F114" s="17" t="n"/>
       <c r="G114" s="31" t="n"/>
       <c r="H114" s="32" t="n"/>
-      <c r="I114" s="33" t="inlineStr">
+      <c r="I114" s="38" t="inlineStr">
         <is>
           <t>Achat - Flying Tiger Bruxelles</t>
         </is>
       </c>
-      <c r="J114" s="34" t="n">
+      <c r="J114" s="39" t="n">
         <v>81</v>
       </c>
-      <c r="K114" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L114" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 12-03 — décompte n° 091 du 10-04 — nature de l'achat à préciser — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K114" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L114" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 12-03 — décompte n° 091 du 10-04 — nature de l'achat à préciser — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3508,7 +3519,7 @@
       </c>
       <c r="L121" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 21-03 — décompte n° 091 du 10-04 — Valinsopay, Wijk en Aalburg (Pays-Bas) — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 21-03 — décompte n° 091 du 10-04 — Valinsopay, Wijk en Aalburg (Pays-Bas) — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3543,7 @@
       </c>
       <c r="L122" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 21-03 — décompte n° 091 du 10-04 — Valinsopay, Wijk en Aalburg (Pays-Bas) — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 21-03 — décompte n° 091 du 10-04 — Valinsopay, Wijk en Aalburg (Pays-Bas) — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3687,7 @@
       </c>
       <c r="L128" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3685,22 +3696,22 @@
       <c r="F129" s="17" t="n"/>
       <c r="G129" s="31" t="n"/>
       <c r="H129" s="32" t="n"/>
-      <c r="I129" s="33" t="inlineStr">
+      <c r="I129" s="38" t="inlineStr">
         <is>
           <t>Achat - Oris Group, Waterloo</t>
         </is>
       </c>
-      <c r="J129" s="34" t="n">
+      <c r="J129" s="39" t="n">
         <v>25.63</v>
       </c>
-      <c r="K129" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L129" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K129" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L129" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3735,7 @@
       </c>
       <c r="L130" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3733,22 +3744,22 @@
       <c r="F131" s="17" t="n"/>
       <c r="G131" s="31" t="n"/>
       <c r="H131" s="32" t="n"/>
-      <c r="I131" s="33" t="inlineStr">
+      <c r="I131" s="38" t="inlineStr">
         <is>
           <t>Achat vêtements - Zara Bruxelles</t>
         </is>
       </c>
-      <c r="J131" s="34" t="n">
+      <c r="J131" s="39" t="n">
         <v>84.05</v>
       </c>
-      <c r="K131" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L131" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — usage professionnel à confirmer — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K131" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L131" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — usage professionnel à confirmer — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3757,22 +3768,22 @@
       <c r="F132" s="17" t="n"/>
       <c r="G132" s="31" t="n"/>
       <c r="H132" s="32" t="n"/>
-      <c r="I132" s="33" t="inlineStr">
+      <c r="I132" s="38" t="inlineStr">
         <is>
           <t>Achat - commerçant 2419 Bruxelles</t>
         </is>
       </c>
-      <c r="J132" s="34" t="n">
+      <c r="J132" s="39" t="n">
         <v>2.89</v>
       </c>
-      <c r="K132" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L132" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K132" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L132" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — à identifier — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3796,7 +3807,7 @@
       </c>
       <c r="L133" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3831,7 @@
       </c>
       <c r="L134" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 29-03 — décompte n° 091 du 10-04 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -3877,16 +3888,16 @@
       <c r="F137" s="17" t="n"/>
       <c r="G137" s="31" t="n"/>
       <c r="H137" s="32" t="n"/>
-      <c r="I137" s="13" t="inlineStr">
+      <c r="I137" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J137" s="37" t="n">
+      <c r="J137" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="K137" s="28" t="n"/>
-      <c r="L137" s="32" t="inlineStr">
+      <c r="K137" s="35" t="n"/>
+      <c r="L137" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 01-04 — décompte n° 091 du 10-04</t>
         </is>
@@ -3897,16 +3908,16 @@
       <c r="F138" s="17" t="n"/>
       <c r="G138" s="31" t="n"/>
       <c r="H138" s="32" t="n"/>
-      <c r="I138" s="13" t="inlineStr">
+      <c r="I138" s="33" t="inlineStr">
         <is>
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J138" s="37" t="n">
+      <c r="J138" s="34" t="n">
         <v>431.25</v>
       </c>
-      <c r="K138" s="28" t="n"/>
-      <c r="L138" s="32" t="inlineStr">
+      <c r="K138" s="35" t="n"/>
+      <c r="L138" s="36" t="inlineStr">
         <is>
           <t>Paiement par domiciliation (AG Insurance)</t>
         </is>
@@ -4004,7 +4015,7 @@
       </c>
       <c r="L142" s="36" t="inlineStr">
         <is>
-          <t>2theloo, aire E40 Jabbeke — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>2theloo, aire E40 Jabbeke — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -4028,7 +4039,7 @@
       </c>
       <c r="L143" s="36" t="inlineStr">
         <is>
-          <t>2theloo, aire E40 Jabbeke — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>2theloo, aire E40 Jabbeke — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4087,7 @@
       </c>
       <c r="L145" s="36" t="inlineStr">
         <is>
-          <t>AC Restaurants Wanlin — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>AC Restaurants Wanlin — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -4196,21 +4207,21 @@
       </c>
       <c r="L150" s="36" t="inlineStr">
         <is>
-          <t>Delhaize Sterrebeek — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Delhaize Sterrebeek — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="G151" s="38" t="n"/>
-      <c r="H151" s="39" t="n"/>
-      <c r="J151" s="38" t="n"/>
-      <c r="L151" s="39" t="n"/>
+      <c r="G151" s="42" t="n"/>
+      <c r="H151" s="43" t="n"/>
+      <c r="J151" s="42" t="n"/>
+      <c r="L151" s="43" t="n"/>
     </row>
     <row r="152">
-      <c r="G152" s="38" t="n"/>
-      <c r="H152" s="39" t="n"/>
-      <c r="J152" s="38" t="n"/>
-      <c r="L152" s="39" t="n"/>
+      <c r="G152" s="42" t="n"/>
+      <c r="H152" s="43" t="n"/>
+      <c r="J152" s="42" t="n"/>
+      <c r="L152" s="43" t="n"/>
     </row>
     <row r="153">
       <c r="E153" s="16" t="inlineStr">
@@ -4232,7 +4243,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J153" s="40" t="n">
+      <c r="J153" s="44" t="n">
         <v>724.12</v>
       </c>
       <c r="K153" s="28" t="inlineStr">
@@ -4397,16 +4408,16 @@
       <c r="F160" s="17" t="n"/>
       <c r="G160" s="31" t="n"/>
       <c r="H160" s="32" t="n"/>
-      <c r="I160" s="13" t="inlineStr">
+      <c r="I160" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J160" s="37" t="n">
+      <c r="J160" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="K160" s="28" t="n"/>
-      <c r="L160" s="32" t="inlineStr">
+      <c r="K160" s="35" t="n"/>
+      <c r="L160" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 01-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4417,16 +4428,16 @@
       <c r="F161" s="17" t="n"/>
       <c r="G161" s="31" t="n"/>
       <c r="H161" s="32" t="n"/>
-      <c r="I161" s="13" t="inlineStr">
+      <c r="I161" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J161" s="37" t="n">
+      <c r="J161" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="K161" s="28" t="n"/>
-      <c r="L161" s="32" t="inlineStr">
+      <c r="K161" s="35" t="n"/>
+      <c r="L161" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 01-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4437,16 +4448,16 @@
       <c r="F162" s="17" t="n"/>
       <c r="G162" s="31" t="n"/>
       <c r="H162" s="32" t="n"/>
-      <c r="I162" s="13" t="inlineStr">
+      <c r="I162" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J162" s="37" t="n">
+      <c r="J162" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="K162" s="28" t="n"/>
-      <c r="L162" s="32" t="inlineStr">
+      <c r="K162" s="35" t="n"/>
+      <c r="L162" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 02-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4457,16 +4468,16 @@
       <c r="F163" s="17" t="n"/>
       <c r="G163" s="31" t="n"/>
       <c r="H163" s="32" t="n"/>
-      <c r="I163" s="13" t="inlineStr">
+      <c r="I163" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J163" s="37" t="n">
+      <c r="J163" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="K163" s="28" t="n"/>
-      <c r="L163" s="32" t="inlineStr">
+      <c r="K163" s="35" t="n"/>
+      <c r="L163" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 02-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4477,16 +4488,16 @@
       <c r="F164" s="17" t="n"/>
       <c r="G164" s="31" t="n"/>
       <c r="H164" s="32" t="n"/>
-      <c r="I164" s="13" t="inlineStr">
+      <c r="I164" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J164" s="37" t="n">
+      <c r="J164" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="K164" s="28" t="n"/>
-      <c r="L164" s="32" t="inlineStr">
+      <c r="K164" s="35" t="n"/>
+      <c r="L164" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 02-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4497,16 +4508,16 @@
       <c r="F165" s="17" t="n"/>
       <c r="G165" s="31" t="n"/>
       <c r="H165" s="32" t="n"/>
-      <c r="I165" s="13" t="inlineStr">
+      <c r="I165" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J165" s="37" t="n">
+      <c r="J165" s="34" t="n">
         <v>5</v>
       </c>
-      <c r="K165" s="28" t="n"/>
-      <c r="L165" s="32" t="inlineStr">
+      <c r="K165" s="35" t="n"/>
+      <c r="L165" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 03-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4517,16 +4528,16 @@
       <c r="F166" s="17" t="n"/>
       <c r="G166" s="31" t="n"/>
       <c r="H166" s="32" t="n"/>
-      <c r="I166" s="13" t="inlineStr">
+      <c r="I166" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J166" s="37" t="n">
+      <c r="J166" s="34" t="n">
         <v>8</v>
       </c>
-      <c r="K166" s="28" t="n"/>
-      <c r="L166" s="32" t="inlineStr">
+      <c r="K166" s="35" t="n"/>
+      <c r="L166" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 03-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4537,16 +4548,16 @@
       <c r="F167" s="17" t="n"/>
       <c r="G167" s="31" t="n"/>
       <c r="H167" s="32" t="n"/>
-      <c r="I167" s="13" t="inlineStr">
+      <c r="I167" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J167" s="37" t="n">
+      <c r="J167" s="34" t="n">
         <v>12</v>
       </c>
-      <c r="K167" s="28" t="n"/>
-      <c r="L167" s="32" t="inlineStr">
+      <c r="K167" s="35" t="n"/>
+      <c r="L167" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 05-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4557,16 +4568,16 @@
       <c r="F168" s="17" t="n"/>
       <c r="G168" s="31" t="n"/>
       <c r="H168" s="32" t="n"/>
-      <c r="I168" s="13" t="inlineStr">
+      <c r="I168" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J168" s="37" t="n">
+      <c r="J168" s="34" t="n">
         <v>18</v>
       </c>
-      <c r="K168" s="28" t="n"/>
-      <c r="L168" s="32" t="inlineStr">
+      <c r="K168" s="35" t="n"/>
+      <c r="L168" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 06-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4577,16 +4588,16 @@
       <c r="F169" s="17" t="n"/>
       <c r="G169" s="31" t="n"/>
       <c r="H169" s="32" t="n"/>
-      <c r="I169" s="13" t="inlineStr">
+      <c r="I169" s="33" t="inlineStr">
         <is>
           <t>Abonnement Shopify</t>
         </is>
       </c>
-      <c r="J169" s="37" t="n">
+      <c r="J169" s="34" t="n">
         <v>23.26</v>
       </c>
-      <c r="K169" s="28" t="n"/>
-      <c r="L169" s="32" t="inlineStr">
+      <c r="K169" s="35" t="n"/>
+      <c r="L169" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 07-04 — décompte n° 121 du 12-05 — 25,00 USD - facture 351488651</t>
         </is>
@@ -4597,16 +4608,16 @@
       <c r="F170" s="17" t="n"/>
       <c r="G170" s="31" t="n"/>
       <c r="H170" s="32" t="n"/>
-      <c r="I170" s="13" t="inlineStr">
+      <c r="I170" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J170" s="37" t="n">
+      <c r="J170" s="34" t="n">
         <v>18</v>
       </c>
-      <c r="K170" s="28" t="n"/>
-      <c r="L170" s="32" t="inlineStr">
+      <c r="K170" s="35" t="n"/>
+      <c r="L170" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 08-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4617,16 +4628,16 @@
       <c r="F171" s="17" t="n"/>
       <c r="G171" s="31" t="n"/>
       <c r="H171" s="32" t="n"/>
-      <c r="I171" s="13" t="inlineStr">
+      <c r="I171" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J171" s="37" t="n">
+      <c r="J171" s="34" t="n">
         <v>20</v>
       </c>
-      <c r="K171" s="28" t="n"/>
-      <c r="L171" s="32" t="inlineStr">
+      <c r="K171" s="35" t="n"/>
+      <c r="L171" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 10-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4637,22 +4648,22 @@
       <c r="F172" s="17" t="n"/>
       <c r="G172" s="31" t="n"/>
       <c r="H172" s="32" t="n"/>
-      <c r="I172" s="33" t="inlineStr">
+      <c r="I172" s="38" t="inlineStr">
         <is>
           <t>Coiffure hommes, Schaerbeek</t>
         </is>
       </c>
-      <c r="J172" s="34" t="n">
+      <c r="J172" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="K172" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L172" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — dépense privée ? à valider — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K172" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L172" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — dépense privée ? à valider — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -4661,22 +4672,22 @@
       <c r="F173" s="17" t="n"/>
       <c r="G173" s="31" t="n"/>
       <c r="H173" s="32" t="n"/>
-      <c r="I173" s="33" t="inlineStr">
+      <c r="I173" s="38" t="inlineStr">
         <is>
           <t>Achat - SumUp Schaerbeek</t>
         </is>
       </c>
-      <c r="J173" s="34" t="n">
+      <c r="J173" s="39" t="n">
         <v>7.9</v>
       </c>
-      <c r="K173" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L173" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — commerçant à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K173" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L173" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — commerçant à identifier — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -4685,22 +4696,22 @@
       <c r="F174" s="17" t="n"/>
       <c r="G174" s="31" t="n"/>
       <c r="H174" s="32" t="n"/>
-      <c r="I174" s="33" t="inlineStr">
+      <c r="I174" s="38" t="inlineStr">
         <is>
           <t>Achat - Action Schaerbeek</t>
         </is>
       </c>
-      <c r="J174" s="34" t="n">
+      <c r="J174" s="39" t="n">
         <v>17.39</v>
       </c>
-      <c r="K174" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L174" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — nature de l'achat à préciser — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K174" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L174" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 11-04 — décompte n° 121 du 12-05 — nature de l'achat à préciser — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -4709,16 +4720,16 @@
       <c r="F175" s="17" t="n"/>
       <c r="G175" s="31" t="n"/>
       <c r="H175" s="32" t="n"/>
-      <c r="I175" s="13" t="inlineStr">
+      <c r="I175" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J175" s="37" t="n">
+      <c r="J175" s="34" t="n">
         <v>22</v>
       </c>
-      <c r="K175" s="28" t="n"/>
-      <c r="L175" s="32" t="inlineStr">
+      <c r="K175" s="35" t="n"/>
+      <c r="L175" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 12-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4825,16 +4836,16 @@
       <c r="F180" s="17" t="n"/>
       <c r="G180" s="31" t="n"/>
       <c r="H180" s="32" t="n"/>
-      <c r="I180" s="13" t="inlineStr">
+      <c r="I180" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J180" s="37" t="n">
+      <c r="J180" s="34" t="n">
         <v>25</v>
       </c>
-      <c r="K180" s="28" t="n"/>
-      <c r="L180" s="32" t="inlineStr">
+      <c r="K180" s="35" t="n"/>
+      <c r="L180" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 15-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4845,22 +4856,22 @@
       <c r="F181" s="17" t="n"/>
       <c r="G181" s="31" t="n"/>
       <c r="H181" s="32" t="n"/>
-      <c r="I181" s="33" t="inlineStr">
+      <c r="I181" s="38" t="inlineStr">
         <is>
           <t>Achat - Action Bruxelles</t>
         </is>
       </c>
-      <c r="J181" s="34" t="n">
+      <c r="J181" s="39" t="n">
         <v>24.46</v>
       </c>
-      <c r="K181" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L181" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 16-04 — décompte n° 121 du 12-05 — nature de l'achat à préciser — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K181" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L181" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 16-04 — décompte n° 121 du 12-05 — nature de l'achat à préciser — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -4917,16 +4928,16 @@
       <c r="F184" s="17" t="n"/>
       <c r="G184" s="31" t="n"/>
       <c r="H184" s="32" t="n"/>
-      <c r="I184" s="13" t="inlineStr">
+      <c r="I184" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J184" s="37" t="n">
+      <c r="J184" s="34" t="n">
         <v>28</v>
       </c>
-      <c r="K184" s="28" t="n"/>
-      <c r="L184" s="32" t="inlineStr">
+      <c r="K184" s="35" t="n"/>
+      <c r="L184" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 17-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -4961,16 +4972,16 @@
       <c r="F186" s="17" t="n"/>
       <c r="G186" s="31" t="n"/>
       <c r="H186" s="32" t="n"/>
-      <c r="I186" s="13" t="inlineStr">
+      <c r="I186" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J186" s="37" t="n">
+      <c r="J186" s="34" t="n">
         <v>31</v>
       </c>
-      <c r="K186" s="28" t="n"/>
-      <c r="L186" s="32" t="inlineStr">
+      <c r="K186" s="35" t="n"/>
+      <c r="L186" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 19-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -5005,16 +5016,16 @@
       <c r="F188" s="17" t="n"/>
       <c r="G188" s="31" t="n"/>
       <c r="H188" s="32" t="n"/>
-      <c r="I188" s="13" t="inlineStr">
+      <c r="I188" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J188" s="37" t="n">
+      <c r="J188" s="34" t="n">
         <v>35</v>
       </c>
-      <c r="K188" s="28" t="n"/>
-      <c r="L188" s="32" t="inlineStr">
+      <c r="K188" s="35" t="n"/>
+      <c r="L188" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 21-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -5049,16 +5060,16 @@
       <c r="F190" s="17" t="n"/>
       <c r="G190" s="31" t="n"/>
       <c r="H190" s="32" t="n"/>
-      <c r="I190" s="13" t="inlineStr">
+      <c r="I190" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J190" s="37" t="n">
+      <c r="J190" s="34" t="n">
         <v>39</v>
       </c>
-      <c r="K190" s="28" t="n"/>
-      <c r="L190" s="32" t="inlineStr">
+      <c r="K190" s="35" t="n"/>
+      <c r="L190" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 24-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -5093,16 +5104,16 @@
       <c r="F192" s="17" t="n"/>
       <c r="G192" s="31" t="n"/>
       <c r="H192" s="32" t="n"/>
-      <c r="I192" s="13" t="inlineStr">
+      <c r="I192" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J192" s="37" t="n">
+      <c r="J192" s="34" t="n">
         <v>43</v>
       </c>
-      <c r="K192" s="28" t="n"/>
-      <c r="L192" s="32" t="inlineStr">
+      <c r="K192" s="35" t="n"/>
+      <c r="L192" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 29-04 — décompte n° 121 du 12-05</t>
         </is>
@@ -5200,7 +5211,7 @@
       </c>
       <c r="L196" s="36" t="inlineStr">
         <is>
-          <t>Tank und Rastanlage, Frechen (Allemagne) — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Tank und Rastanlage, Frechen (Allemagne) — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -5224,7 +5235,7 @@
       </c>
       <c r="L197" s="36" t="inlineStr">
         <is>
-          <t>Tank und Rastanlage, Frechen (Allemagne) — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Tank und Rastanlage, Frechen (Allemagne) — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -5397,16 +5408,16 @@
       </c>
     </row>
     <row r="205">
-      <c r="G205" s="38" t="n"/>
-      <c r="H205" s="39" t="n"/>
-      <c r="J205" s="38" t="n"/>
-      <c r="L205" s="39" t="n"/>
+      <c r="G205" s="42" t="n"/>
+      <c r="H205" s="43" t="n"/>
+      <c r="J205" s="42" t="n"/>
+      <c r="L205" s="43" t="n"/>
     </row>
     <row r="206">
-      <c r="G206" s="38" t="n"/>
-      <c r="H206" s="39" t="n"/>
-      <c r="J206" s="38" t="n"/>
-      <c r="L206" s="39" t="n"/>
+      <c r="G206" s="42" t="n"/>
+      <c r="H206" s="43" t="n"/>
+      <c r="J206" s="42" t="n"/>
+      <c r="L206" s="43" t="n"/>
     </row>
     <row r="207">
       <c r="E207" s="16" t="inlineStr">
@@ -5428,7 +5439,7 @@
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J207" s="40" t="n">
+      <c r="J207" s="44" t="n">
         <v>200</v>
       </c>
       <c r="K207" s="28" t="inlineStr">
@@ -5444,15 +5455,15 @@
     </row>
     <row r="208">
       <c r="E208" s="16" t="n"/>
-      <c r="F208" s="41" t="inlineStr">
+      <c r="F208" s="45" t="inlineStr">
         <is>
           <t>Approvisionnement compte - Thibault Duchène</t>
         </is>
       </c>
-      <c r="G208" s="42" t="n">
+      <c r="G208" s="46" t="n">
         <v>1500</v>
       </c>
-      <c r="H208" s="36" t="inlineStr">
+      <c r="H208" s="41" t="inlineStr">
         <is>
           <t>Apport du gérant, pas un produit — à traiter en compte courant</t>
         </is>
@@ -5741,16 +5752,16 @@
       <c r="F220" s="17" t="n"/>
       <c r="G220" s="31" t="n"/>
       <c r="H220" s="32" t="n"/>
-      <c r="I220" s="13" t="inlineStr">
+      <c r="I220" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J220" s="37" t="n">
+      <c r="J220" s="34" t="n">
         <v>25.78</v>
       </c>
-      <c r="K220" s="28" t="n"/>
-      <c r="L220" s="32" t="inlineStr">
+      <c r="K220" s="35" t="n"/>
+      <c r="L220" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 01-05 — décompte n° 152 du 10-06</t>
         </is>
@@ -5761,16 +5772,16 @@
       <c r="F221" s="17" t="n"/>
       <c r="G221" s="31" t="n"/>
       <c r="H221" s="32" t="n"/>
-      <c r="I221" s="13" t="inlineStr">
+      <c r="I221" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J221" s="37" t="n">
+      <c r="J221" s="34" t="n">
         <v>48</v>
       </c>
-      <c r="K221" s="28" t="n"/>
-      <c r="L221" s="32" t="inlineStr">
+      <c r="K221" s="35" t="n"/>
+      <c r="L221" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 03-05 — décompte n° 152 du 10-06</t>
         </is>
@@ -5805,16 +5816,16 @@
       <c r="F223" s="17" t="n"/>
       <c r="G223" s="31" t="n"/>
       <c r="H223" s="32" t="n"/>
-      <c r="I223" s="13" t="inlineStr">
+      <c r="I223" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J223" s="37" t="n">
+      <c r="J223" s="34" t="n">
         <v>53</v>
       </c>
-      <c r="K223" s="28" t="n"/>
-      <c r="L223" s="32" t="inlineStr">
+      <c r="K223" s="35" t="n"/>
+      <c r="L223" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 06-05 — décompte n° 152 du 10-06</t>
         </is>
@@ -5825,16 +5836,16 @@
       <c r="F224" s="17" t="n"/>
       <c r="G224" s="31" t="n"/>
       <c r="H224" s="32" t="n"/>
-      <c r="I224" s="13" t="inlineStr">
+      <c r="I224" s="33" t="inlineStr">
         <is>
           <t>Abonnement Shopify</t>
         </is>
       </c>
-      <c r="J224" s="37" t="n">
+      <c r="J224" s="34" t="n">
         <v>22.83</v>
       </c>
-      <c r="K224" s="28" t="n"/>
-      <c r="L224" s="32" t="inlineStr">
+      <c r="K224" s="35" t="n"/>
+      <c r="L224" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 07-05 — décompte n° 152 du 10-06 — 25,34 USD - facture 363251007</t>
         </is>
@@ -5893,16 +5904,16 @@
       <c r="F227" s="17" t="n"/>
       <c r="G227" s="31" t="n"/>
       <c r="H227" s="32" t="n"/>
-      <c r="I227" s="13" t="inlineStr">
+      <c r="I227" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J227" s="37" t="n">
+      <c r="J227" s="34" t="n">
         <v>59</v>
       </c>
-      <c r="K227" s="28" t="n"/>
-      <c r="L227" s="32" t="inlineStr">
+      <c r="K227" s="35" t="n"/>
+      <c r="L227" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 09-05 — décompte n° 152 du 10-06</t>
         </is>
@@ -6009,16 +6020,16 @@
       <c r="F232" s="17" t="n"/>
       <c r="G232" s="31" t="n"/>
       <c r="H232" s="32" t="n"/>
-      <c r="I232" s="13" t="inlineStr">
+      <c r="I232" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J232" s="37" t="n">
+      <c r="J232" s="34" t="n">
         <v>65</v>
       </c>
-      <c r="K232" s="28" t="n"/>
-      <c r="L232" s="32" t="inlineStr">
+      <c r="K232" s="35" t="n"/>
+      <c r="L232" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 13-05 — décompte n° 152 du 10-06</t>
         </is>
@@ -6221,22 +6232,22 @@
       <c r="F241" s="17" t="n"/>
       <c r="G241" s="31" t="n"/>
       <c r="H241" s="32" t="n"/>
-      <c r="I241" s="33" t="inlineStr">
+      <c r="I241" s="38" t="inlineStr">
         <is>
           <t>Achat - Mood for Green SRL, Bruxelles</t>
         </is>
       </c>
-      <c r="J241" s="34" t="n">
+      <c r="J241" s="39" t="n">
         <v>17</v>
       </c>
-      <c r="K241" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L241" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 21-05 — décompte n° 152 du 10-06 — à identifier — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K241" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L241" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 21-05 — décompte n° 152 du 10-06 — à identifier — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -6389,16 +6400,16 @@
       <c r="F248" s="17" t="n"/>
       <c r="G248" s="31" t="n"/>
       <c r="H248" s="32" t="n"/>
-      <c r="I248" s="13" t="inlineStr">
+      <c r="I248" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J248" s="37" t="n">
+      <c r="J248" s="34" t="n">
         <v>72</v>
       </c>
-      <c r="K248" s="28" t="n"/>
-      <c r="L248" s="32" t="inlineStr">
+      <c r="K248" s="35" t="n"/>
+      <c r="L248" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 27-05 — décompte n° 152 du 10-06</t>
         </is>
@@ -6837,16 +6848,16 @@
       </c>
     </row>
     <row r="267">
-      <c r="G267" s="38" t="n"/>
-      <c r="H267" s="39" t="n"/>
-      <c r="J267" s="38" t="n"/>
-      <c r="L267" s="39" t="n"/>
+      <c r="G267" s="42" t="n"/>
+      <c r="H267" s="43" t="n"/>
+      <c r="J267" s="42" t="n"/>
+      <c r="L267" s="43" t="n"/>
     </row>
     <row r="268">
-      <c r="G268" s="38" t="n"/>
-      <c r="H268" s="39" t="n"/>
-      <c r="J268" s="38" t="n"/>
-      <c r="L268" s="39" t="n"/>
+      <c r="G268" s="42" t="n"/>
+      <c r="H268" s="43" t="n"/>
+      <c r="J268" s="42" t="n"/>
+      <c r="L268" s="43" t="n"/>
     </row>
     <row r="269">
       <c r="E269" s="16" t="inlineStr">
@@ -6854,15 +6865,15 @@
           <t>Juillet</t>
         </is>
       </c>
-      <c r="F269" s="41" t="inlineStr">
+      <c r="F269" s="45" t="inlineStr">
         <is>
           <t>Prise en charge par T. Duchène - facture Proximus 7504645054</t>
         </is>
       </c>
-      <c r="G269" s="42" t="n">
+      <c r="G269" s="46" t="n">
         <v>109.59</v>
       </c>
-      <c r="H269" s="36" t="inlineStr">
+      <c r="H269" s="41" t="inlineStr">
         <is>
           <t>Contrepartie de la facture payée à titre privé — à traiter en compte courant</t>
         </is>
@@ -6872,7 +6883,7 @@
           <t>Précompte salarial juin 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J269" s="40" t="n">
+      <c r="J269" s="44" t="n">
         <v>2250</v>
       </c>
       <c r="K269" s="28" t="inlineStr">
@@ -6888,15 +6899,15 @@
     </row>
     <row r="270">
       <c r="E270" s="16" t="n"/>
-      <c r="F270" s="41" t="inlineStr">
+      <c r="F270" s="45" t="inlineStr">
         <is>
           <t>Remboursement paiement à Sandaya</t>
         </is>
       </c>
-      <c r="G270" s="42" t="n">
+      <c r="G270" s="46" t="n">
         <v>1775.4</v>
       </c>
-      <c r="H270" s="36" t="inlineStr">
+      <c r="H270" s="41" t="inlineStr">
         <is>
           <t>Versement de Thibault Duchène — dépense privée payée par la société ?</t>
         </is>
@@ -7003,32 +7014,32 @@
       <c r="F274" s="17" t="n"/>
       <c r="G274" s="31" t="n"/>
       <c r="H274" s="32" t="n"/>
-      <c r="I274" s="13" t="inlineStr">
+      <c r="I274" s="33" t="inlineStr">
         <is>
           <t>Frais bancaires trimestriels</t>
         </is>
       </c>
-      <c r="J274" s="37" t="n">
+      <c r="J274" s="34" t="n">
         <v>11.25</v>
       </c>
-      <c r="K274" s="28" t="n"/>
-      <c r="L274" s="32" t="n"/>
+      <c r="K274" s="35" t="n"/>
+      <c r="L274" s="36" t="n"/>
     </row>
     <row r="275">
       <c r="E275" s="16" t="n"/>
       <c r="F275" s="17" t="n"/>
       <c r="G275" s="31" t="n"/>
       <c r="H275" s="32" t="n"/>
-      <c r="I275" s="13" t="inlineStr">
+      <c r="I275" s="33" t="inlineStr">
         <is>
           <t>Intérêt crédit</t>
         </is>
       </c>
-      <c r="J275" s="37" t="n">
+      <c r="J275" s="34" t="n">
         <v>0.51</v>
       </c>
-      <c r="K275" s="28" t="n"/>
-      <c r="L275" s="32" t="inlineStr">
+      <c r="K275" s="35" t="n"/>
+      <c r="L275" s="36" t="inlineStr">
         <is>
           <t>Intérêts nets au 01-07</t>
         </is>
@@ -7063,16 +7074,16 @@
       <c r="F277" s="17" t="n"/>
       <c r="G277" s="31" t="n"/>
       <c r="H277" s="32" t="n"/>
-      <c r="I277" s="13" t="inlineStr">
+      <c r="I277" s="33" t="inlineStr">
         <is>
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J277" s="37" t="n">
+      <c r="J277" s="34" t="n">
         <v>458.66</v>
       </c>
-      <c r="K277" s="28" t="n"/>
-      <c r="L277" s="32" t="inlineStr">
+      <c r="K277" s="35" t="n"/>
+      <c r="L277" s="36" t="inlineStr">
         <is>
           <t>Domiciliation AG Insurance — prime passée de 431,25 à 458,66</t>
         </is>
@@ -7083,16 +7094,16 @@
       <c r="F278" s="17" t="n"/>
       <c r="G278" s="31" t="n"/>
       <c r="H278" s="32" t="n"/>
-      <c r="I278" s="13" t="inlineStr">
+      <c r="I278" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J278" s="37" t="n">
+      <c r="J278" s="34" t="n">
         <v>20.78</v>
       </c>
-      <c r="K278" s="28" t="n"/>
-      <c r="L278" s="32" t="inlineStr">
+      <c r="K278" s="35" t="n"/>
+      <c r="L278" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 01-06 — décompte n° 182 du 10-07</t>
         </is>
@@ -7118,7 +7129,7 @@
       </c>
       <c r="L279" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 03-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 03-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -7142,7 +7153,7 @@
       </c>
       <c r="L280" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 03-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 03-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -7271,16 +7282,16 @@
       <c r="F286" s="17" t="n"/>
       <c r="G286" s="31" t="n"/>
       <c r="H286" s="32" t="n"/>
-      <c r="I286" s="13" t="inlineStr">
+      <c r="I286" s="33" t="inlineStr">
         <is>
           <t>Abonnement Shopify</t>
         </is>
       </c>
-      <c r="J286" s="37" t="n">
+      <c r="J286" s="34" t="n">
         <v>27.96</v>
       </c>
-      <c r="K286" s="28" t="n"/>
-      <c r="L286" s="32" t="inlineStr">
+      <c r="K286" s="35" t="n"/>
+      <c r="L286" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 06-06 — décompte n° 182 du 10-07 — 31,38 USD - facture 375321628</t>
         </is>
@@ -7354,7 +7365,7 @@
       </c>
       <c r="L289" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 08-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 08-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -7378,7 +7389,7 @@
       </c>
       <c r="L290" s="36" t="inlineStr">
         <is>
-          <t>Carte Visa 08-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+          <t>Carte Visa 08-06 — décompte n° 182 du 10-07 — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -7387,22 +7398,22 @@
       <c r="F291" s="17" t="n"/>
       <c r="G291" s="31" t="n"/>
       <c r="H291" s="32" t="n"/>
-      <c r="I291" s="33" t="inlineStr">
+      <c r="I291" s="38" t="inlineStr">
         <is>
           <t>Achat - Proxy Meiser, Schaerbeek</t>
         </is>
       </c>
-      <c r="J291" s="34" t="n">
+      <c r="J291" s="39" t="n">
         <v>33.84</v>
       </c>
-      <c r="K291" s="35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L291" s="36" t="inlineStr">
-        <is>
-          <t>Carte Visa 09-06 — décompte n° 182 du 10-07 — nature de l'achat à préciser — Ticket non conservé — pièce manquante, à trancher avec le comptable</t>
+      <c r="K291" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L291" s="41" t="inlineStr">
+        <is>
+          <t>Carte Visa 09-06 — décompte n° 182 du 10-07 — nature de l'achat à préciser — Ticket non conservé — pièce manquante</t>
         </is>
       </c>
     </row>
@@ -7843,16 +7854,16 @@
       <c r="F310" s="17" t="n"/>
       <c r="G310" s="31" t="n"/>
       <c r="H310" s="32" t="n"/>
-      <c r="I310" s="13" t="inlineStr">
+      <c r="I310" s="33" t="inlineStr">
         <is>
           <t>Amende de stationnement - Saint-Josse</t>
         </is>
       </c>
-      <c r="J310" s="37" t="n">
+      <c r="J310" s="34" t="n">
         <v>100</v>
       </c>
-      <c r="K310" s="28" t="n"/>
-      <c r="L310" s="32" t="inlineStr">
+      <c r="K310" s="35" t="n"/>
+      <c r="L310" s="36" t="inlineStr">
         <is>
           <t>Amende — dépense non admise, comm. 500/2300/37391</t>
         </is>
@@ -8003,16 +8014,16 @@
       </c>
     </row>
     <row r="317">
-      <c r="G317" s="38" t="n"/>
-      <c r="H317" s="39" t="n"/>
-      <c r="J317" s="38" t="n"/>
-      <c r="L317" s="39" t="n"/>
+      <c r="G317" s="42" t="n"/>
+      <c r="H317" s="43" t="n"/>
+      <c r="J317" s="42" t="n"/>
+      <c r="L317" s="43" t="n"/>
     </row>
     <row r="318">
-      <c r="G318" s="38" t="n"/>
-      <c r="H318" s="39" t="n"/>
-      <c r="J318" s="38" t="n"/>
-      <c r="L318" s="39" t="n"/>
+      <c r="G318" s="42" t="n"/>
+      <c r="H318" s="43" t="n"/>
+      <c r="J318" s="42" t="n"/>
+      <c r="L318" s="43" t="n"/>
     </row>
     <row r="319">
       <c r="E319" s="16" t="inlineStr">
@@ -8038,7 +8049,7 @@
           <t>Précompte salarial juillet 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J319" s="40" t="n">
+      <c r="J319" s="44" t="n">
         <v>2250</v>
       </c>
       <c r="K319" s="28" t="inlineStr">
@@ -8197,16 +8208,16 @@
       <c r="F326" s="17" t="n"/>
       <c r="G326" s="31" t="n"/>
       <c r="H326" s="32" t="n"/>
-      <c r="I326" s="13" t="inlineStr">
+      <c r="I326" s="33" t="inlineStr">
         <is>
           <t>Publicité Facebook</t>
         </is>
       </c>
-      <c r="J326" s="37" t="n">
+      <c r="J326" s="34" t="n">
         <v>26.47</v>
       </c>
-      <c r="K326" s="28" t="n"/>
-      <c r="L326" s="32" t="inlineStr">
+      <c r="K326" s="35" t="n"/>
+      <c r="L326" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 01-07 — décompte n° 213 du 11-08</t>
         </is>
@@ -8217,16 +8228,16 @@
       <c r="F327" s="17" t="n"/>
       <c r="G327" s="31" t="n"/>
       <c r="H327" s="32" t="n"/>
-      <c r="I327" s="13" t="inlineStr">
+      <c r="I327" s="33" t="inlineStr">
         <is>
           <t>Réception marchandise - FEDEX</t>
         </is>
       </c>
-      <c r="J327" s="37" t="n">
+      <c r="J327" s="34" t="n">
         <v>5.51</v>
       </c>
-      <c r="K327" s="28" t="n"/>
-      <c r="L327" s="32" t="inlineStr">
+      <c r="K327" s="35" t="n"/>
+      <c r="L327" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 04-07 — décompte n° 213 du 11-08 — Envoi 798875231</t>
         </is>
@@ -8237,16 +8248,16 @@
       <c r="F328" s="17" t="n"/>
       <c r="G328" s="31" t="n"/>
       <c r="H328" s="32" t="n"/>
-      <c r="I328" s="13" t="inlineStr">
+      <c r="I328" s="33" t="inlineStr">
         <is>
           <t>Abonnement Shopify</t>
         </is>
       </c>
-      <c r="J328" s="37" t="n">
+      <c r="J328" s="34" t="n">
         <v>22.48</v>
       </c>
-      <c r="K328" s="28" t="n"/>
-      <c r="L328" s="32" t="inlineStr">
+      <c r="K328" s="35" t="n"/>
+      <c r="L328" s="36" t="inlineStr">
         <is>
           <t>Carte Visa 06-07 — décompte n° 213 du 11-08 — 26,00 USD - facture 387615031</t>
         </is>
@@ -8757,16 +8768,16 @@
       </c>
     </row>
     <row r="350">
-      <c r="G350" s="38" t="n"/>
-      <c r="H350" s="39" t="n"/>
-      <c r="J350" s="38" t="n"/>
-      <c r="L350" s="39" t="n"/>
+      <c r="G350" s="42" t="n"/>
+      <c r="H350" s="43" t="n"/>
+      <c r="J350" s="42" t="n"/>
+      <c r="L350" s="43" t="n"/>
     </row>
     <row r="351">
-      <c r="G351" s="38" t="n"/>
-      <c r="H351" s="39" t="n"/>
-      <c r="J351" s="38" t="n"/>
-      <c r="L351" s="39" t="n"/>
+      <c r="G351" s="42" t="n"/>
+      <c r="H351" s="43" t="n"/>
+      <c r="J351" s="42" t="n"/>
+      <c r="L351" s="43" t="n"/>
     </row>
     <row r="352">
       <c r="E352" s="16" t="inlineStr">
@@ -8788,7 +8799,7 @@
           <t>Partena</t>
         </is>
       </c>
-      <c r="J352" s="40" t="n">
+      <c r="J352" s="44" t="n">
         <v>1441.87</v>
       </c>
       <c r="K352" s="28" t="inlineStr">
@@ -9399,16 +9410,16 @@
       </c>
     </row>
     <row r="378">
-      <c r="G378" s="38" t="n"/>
-      <c r="H378" s="39" t="n"/>
-      <c r="J378" s="38" t="n"/>
-      <c r="L378" s="39" t="n"/>
+      <c r="G378" s="42" t="n"/>
+      <c r="H378" s="43" t="n"/>
+      <c r="J378" s="42" t="n"/>
+      <c r="L378" s="43" t="n"/>
     </row>
     <row r="379">
-      <c r="G379" s="38" t="n"/>
-      <c r="H379" s="39" t="n"/>
-      <c r="J379" s="38" t="n"/>
-      <c r="L379" s="39" t="n"/>
+      <c r="G379" s="42" t="n"/>
+      <c r="H379" s="43" t="n"/>
+      <c r="J379" s="42" t="n"/>
+      <c r="L379" s="43" t="n"/>
     </row>
     <row r="380">
       <c r="E380" s="16" t="inlineStr">
@@ -9430,7 +9441,7 @@
           <t>Crédit voiture</t>
         </is>
       </c>
-      <c r="J380" s="40" t="n">
+      <c r="J380" s="44" t="n">
         <v>724.12</v>
       </c>
       <c r="K380" s="28" t="inlineStr">
@@ -9601,16 +9612,16 @@
       <c r="F387" s="17" t="n"/>
       <c r="G387" s="31" t="n"/>
       <c r="H387" s="32" t="n"/>
-      <c r="I387" s="13" t="inlineStr">
+      <c r="I387" s="33" t="inlineStr">
         <is>
           <t>Frais bancaires trimestriels</t>
         </is>
       </c>
-      <c r="J387" s="37" t="n">
+      <c r="J387" s="34" t="n">
         <v>11.25</v>
       </c>
-      <c r="K387" s="28" t="n"/>
-      <c r="L387" s="32" t="n"/>
+      <c r="K387" s="35" t="n"/>
+      <c r="L387" s="36" t="n"/>
     </row>
     <row r="388">
       <c r="E388" s="16" t="n"/>
@@ -9641,16 +9652,16 @@
       <c r="F389" s="17" t="n"/>
       <c r="G389" s="31" t="n"/>
       <c r="H389" s="32" t="n"/>
-      <c r="I389" s="13" t="inlineStr">
+      <c r="I389" s="33" t="inlineStr">
         <is>
           <t>Assurance voiture</t>
         </is>
       </c>
-      <c r="J389" s="37" t="n">
+      <c r="J389" s="34" t="n">
         <v>458.66</v>
       </c>
-      <c r="K389" s="28" t="n"/>
-      <c r="L389" s="32" t="inlineStr">
+      <c r="K389" s="35" t="n"/>
+      <c r="L389" s="36" t="inlineStr">
         <is>
           <t>Paiement par domiciliation (AG Insurance)</t>
         </is>
@@ -10069,20 +10080,20 @@
       <c r="F407" s="17" t="n"/>
       <c r="G407" s="31" t="n"/>
       <c r="H407" s="32" t="n"/>
-      <c r="I407" s="33" t="inlineStr">
+      <c r="I407" s="38" t="inlineStr">
         <is>
           <t>Précompte mobilier</t>
         </is>
       </c>
-      <c r="J407" s="34" t="n">
+      <c r="J407" s="39" t="n">
         <v>2100</v>
       </c>
-      <c r="K407" s="28" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="L407" s="36" t="inlineStr">
+      <c r="K407" s="40" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L407" s="41" t="inlineStr">
         <is>
           <t>Comm. 204/0596/50233 — lié à une distribution de dividendes ?</t>
         </is>
@@ -10137,16 +10148,16 @@
       </c>
     </row>
     <row r="410">
-      <c r="G410" s="38" t="n"/>
-      <c r="H410" s="39" t="n"/>
-      <c r="J410" s="38" t="n"/>
-      <c r="L410" s="39" t="n"/>
+      <c r="G410" s="42" t="n"/>
+      <c r="H410" s="43" t="n"/>
+      <c r="J410" s="42" t="n"/>
+      <c r="L410" s="43" t="n"/>
     </row>
     <row r="411">
-      <c r="G411" s="38" t="n"/>
-      <c r="H411" s="39" t="n"/>
-      <c r="J411" s="38" t="n"/>
-      <c r="L411" s="39" t="n"/>
+      <c r="G411" s="42" t="n"/>
+      <c r="H411" s="43" t="n"/>
+      <c r="J411" s="42" t="n"/>
+      <c r="L411" s="43" t="n"/>
     </row>
     <row r="412">
       <c r="E412" s="16" t="inlineStr">
@@ -10162,7 +10173,7 @@
           <t>Carburant</t>
         </is>
       </c>
-      <c r="J412" s="40" t="n">
+      <c r="J412" s="44" t="n">
         <v>65.29000000000001</v>
       </c>
       <c r="K412" s="28" t="inlineStr">
@@ -10181,20 +10192,20 @@
       <c r="F413" s="17" t="n"/>
       <c r="G413" s="31" t="n"/>
       <c r="H413" s="32" t="n"/>
-      <c r="I413" s="33" t="inlineStr">
+      <c r="I413" s="38" t="inlineStr">
         <is>
           <t>Achat - Media Markt</t>
         </is>
       </c>
-      <c r="J413" s="34" t="n">
+      <c r="J413" s="39" t="n">
         <v>748</v>
       </c>
-      <c r="K413" s="28" t="inlineStr">
+      <c r="K413" s="40" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L413" s="36" t="inlineStr">
+      <c r="L413" s="41" t="inlineStr">
         <is>
           <t>Ordinateur acheté le 03-11-2025 à 12:33 — investissement à amortir plutôt que charge de l'exercice, à trancher avec BDH — Facture Media Markt en main (achat du 03-11-2025)</t>
         </is>
@@ -10205,20 +10216,20 @@
       <c r="F414" s="17" t="n"/>
       <c r="G414" s="31" t="n"/>
       <c r="H414" s="32" t="n"/>
-      <c r="I414" s="33" t="inlineStr">
+      <c r="I414" s="38" t="inlineStr">
         <is>
           <t>Achat - Media Markt</t>
         </is>
       </c>
-      <c r="J414" s="34" t="n">
+      <c r="J414" s="39" t="n">
         <v>39</v>
       </c>
-      <c r="K414" s="28" t="inlineStr">
+      <c r="K414" s="40" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L414" s="36" t="inlineStr">
+      <c r="L414" s="41" t="inlineStr">
         <is>
           <t>Même passage en caisse, à 12:35 — accessoire ou garantie : à trancher avec le PC — intégré à sa valeur ou laissé en charge — Facture Media Markt en main (achat du 03-11-2025)</t>
         </is>
@@ -10585,20 +10596,20 @@
       <c r="F430" s="17" t="n"/>
       <c r="G430" s="31" t="n"/>
       <c r="H430" s="32" t="n"/>
-      <c r="I430" s="33" t="inlineStr">
+      <c r="I430" s="38" t="inlineStr">
         <is>
           <t>Achat matériel sportif - DECATHLON</t>
         </is>
       </c>
-      <c r="J430" s="34" t="n">
+      <c r="J430" s="39" t="n">
         <v>118.5</v>
       </c>
-      <c r="K430" s="28" t="inlineStr">
+      <c r="K430" s="40" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="L430" s="36" t="inlineStr">
+      <c r="L430" s="41" t="inlineStr">
         <is>
           <t>Decathlon Evere — 10 articles dont masque de ski, luge et vêtements enfant : usage professionnel à confirmer — Justificatif : 2025-11-22_Decathlon-Evere_118.50.pdf</t>
         </is>
@@ -10773,16 +10784,16 @@
       </c>
     </row>
     <row r="438">
-      <c r="G438" s="38" t="n"/>
-      <c r="H438" s="39" t="n"/>
-      <c r="J438" s="38" t="n"/>
-      <c r="L438" s="39" t="n"/>
+      <c r="G438" s="42" t="n"/>
+      <c r="H438" s="43" t="n"/>
+      <c r="J438" s="42" t="n"/>
+      <c r="L438" s="43" t="n"/>
     </row>
     <row r="439">
-      <c r="G439" s="38" t="n"/>
-      <c r="H439" s="39" t="n"/>
-      <c r="J439" s="38" t="n"/>
-      <c r="L439" s="39" t="n"/>
+      <c r="G439" s="42" t="n"/>
+      <c r="H439" s="43" t="n"/>
+      <c r="J439" s="42" t="n"/>
+      <c r="L439" s="43" t="n"/>
     </row>
     <row r="440">
       <c r="E440" s="16" t="inlineStr">
@@ -10804,7 +10815,7 @@
           <t>Précompte salarial novembre 2025 Thibault Duchène</t>
         </is>
       </c>
-      <c r="J440" s="40" t="n">
+      <c r="J440" s="44" t="n">
         <v>2250</v>
       </c>
       <c r="K440" s="28" t="inlineStr">
@@ -11017,16 +11028,16 @@
       <c r="F449" s="17" t="n"/>
       <c r="G449" s="31" t="n"/>
       <c r="H449" s="32" t="n"/>
-      <c r="I449" s="33" t="inlineStr">
+      <c r="I449" s="38" t="inlineStr">
         <is>
           <t>Xerius</t>
         </is>
       </c>
-      <c r="J449" s="34" t="n">
+      <c r="J449" s="39" t="n">
         <v>399.73</v>
       </c>
-      <c r="K449" s="28" t="n"/>
-      <c r="L449" s="36" t="inlineStr">
+      <c r="K449" s="40" t="n"/>
+      <c r="L449" s="41" t="inlineStr">
         <is>
           <t>Cotisation annuelle à charge des sociétés ('taxe société') — communication 925/3695/86745, payée le 16-12-2025. Base 347,50 : le surplus de 52,23 est à vérifier — indexation ou majoration de retard ?</t>
         </is>
@@ -11085,16 +11096,16 @@
       <c r="F452" s="17" t="n"/>
       <c r="G452" s="31" t="n"/>
       <c r="H452" s="32" t="n"/>
-      <c r="I452" s="13" t="inlineStr">
+      <c r="I452" s="33" t="inlineStr">
         <is>
           <t>Assurance RC - LRS Insurance</t>
         </is>
       </c>
-      <c r="J452" s="37" t="n">
+      <c r="J452" s="34" t="n">
         <v>55.04</v>
       </c>
-      <c r="K452" s="28" t="n"/>
-      <c r="L452" s="32" t="inlineStr">
+      <c r="K452" s="35" t="n"/>
+      <c r="L452" s="36" t="inlineStr">
         <is>
           <t>RC professionnelle — prime annuelle payée le 16-12-2025, communication 025/0074/58347. Même montant qu'en 2024, où le courtier était Liantis</t>
         </is>
@@ -11413,28 +11424,28 @@
       </c>
     </row>
     <row r="466">
-      <c r="G466" s="38" t="n"/>
-      <c r="H466" s="39" t="n"/>
-      <c r="J466" s="38" t="n"/>
-      <c r="L466" s="39" t="n"/>
+      <c r="G466" s="42" t="n"/>
+      <c r="H466" s="43" t="n"/>
+      <c r="J466" s="42" t="n"/>
+      <c r="L466" s="43" t="n"/>
     </row>
     <row r="467">
-      <c r="G467" s="38" t="n"/>
-      <c r="H467" s="39" t="n"/>
-      <c r="J467" s="38" t="n"/>
-      <c r="L467" s="39" t="n"/>
+      <c r="G467" s="42" t="n"/>
+      <c r="H467" s="43" t="n"/>
+      <c r="J467" s="42" t="n"/>
+      <c r="L467" s="43" t="n"/>
     </row>
     <row r="468">
-      <c r="G468" s="38">
+      <c r="G468" s="42">
         <f>SUM(G6:G467)</f>
         <v/>
       </c>
-      <c r="H468" s="39" t="n"/>
-      <c r="J468" s="38">
+      <c r="H468" s="43" t="n"/>
+      <c r="J468" s="42">
         <f>SUM(J6:J467)</f>
         <v/>
       </c>
-      <c r="L468" s="39" t="n"/>
+      <c r="L468" s="43" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>